<commit_message>
Sync data files (2026-09-14T21:45:09Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -14649,30 +14649,74 @@
       <c r="C77" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="D77" s="52"/>
-      <c r="E77" s="52"/>
-      <c r="F77" s="52"/>
-      <c r="G77" s="53"/>
-      <c r="H77" s="52"/>
-      <c r="I77" s="52"/>
-      <c r="J77" s="52"/>
-      <c r="K77" s="52"/>
-      <c r="L77" s="52"/>
-      <c r="M77" s="53"/>
+      <c r="D77" s="52">
+        <v>78753.07</v>
+      </c>
+      <c r="E77" s="52">
+        <v>44764.99</v>
+      </c>
+      <c r="F77" s="52">
+        <v>33988.08000000001</v>
+      </c>
+      <c r="G77" s="53">
+        <v>0.4315778419812714</v>
+      </c>
+      <c r="H77" s="52">
+        <v>55589.78</v>
+      </c>
+      <c r="I77" s="52">
+        <v>32417.98</v>
+      </c>
+      <c r="J77" s="52">
+        <v>32594.75</v>
+      </c>
+      <c r="K77" s="52">
+        <v>24016.8</v>
+      </c>
+      <c r="L77" s="52">
+        <v>8577.95</v>
+      </c>
+      <c r="M77" s="53">
+        <v>0.26316968223410214</v>
+      </c>
       <c r="N77" s="53"/>
-      <c r="O77" s="52"/>
-      <c r="P77" s="52"/>
-      <c r="Q77" s="52"/>
-      <c r="R77" s="53"/>
-      <c r="S77" s="54"/>
-      <c r="T77" s="54"/>
-      <c r="U77" s="54"/>
-      <c r="V77" s="53"/>
+      <c r="O77" s="52">
+        <v>22995.03</v>
+      </c>
+      <c r="P77" s="52">
+        <v>8401.18</v>
+      </c>
+      <c r="Q77" s="52">
+        <v>14593.849999999999</v>
+      </c>
+      <c r="R77" s="53">
+        <v>0.6346523574876832</v>
+      </c>
+      <c r="S77" s="54">
+        <v>472.14</v>
+      </c>
+      <c r="T77" s="54">
+        <v>167.25</v>
+      </c>
+      <c r="U77" s="54">
+        <v>304.89</v>
+      </c>
+      <c r="V77" s="53">
+        <v>0.6457618502986402</v>
+      </c>
       <c r="W77" s="53"/>
-      <c r="X77" s="55"/>
-      <c r="Y77" s="55"/>
-      <c r="Z77" s="53"/>
-      <c r="AA77" s="56"/>
+      <c r="X77" s="55">
+        <v>73.82367713004484</v>
+      </c>
+      <c r="Y77" s="55">
+        <v>49.060202993773025</v>
+      </c>
+      <c r="Z77" s="53">
+        <v>0.2758</v>
+      </c>
+      <c r="AA77" s="56">
+        <v>0.2941</v>
+      </c>
       <c r="AB77" s="57"/>
       <c r="AD77" s="35" t="s">
         <v>101</v>
@@ -21955,30 +21999,74 @@
       <c r="C196" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="D196" s="52"/>
-      <c r="E196" s="52"/>
-      <c r="F196" s="52"/>
-      <c r="G196" s="53"/>
-      <c r="H196" s="52"/>
-      <c r="I196" s="52"/>
-      <c r="J196" s="52"/>
-      <c r="K196" s="52"/>
-      <c r="L196" s="52"/>
-      <c r="M196" s="53"/>
+      <c r="D196" s="52">
+        <v>23770.95</v>
+      </c>
+      <c r="E196" s="52">
+        <v>10204.54</v>
+      </c>
+      <c r="F196" s="52">
+        <v>13566.41</v>
+      </c>
+      <c r="G196" s="53">
+        <v>0.5707138334816235</v>
+      </c>
+      <c r="H196" s="52">
+        <v>14310.96</v>
+      </c>
+      <c r="I196" s="52">
+        <v>7116.73</v>
+      </c>
+      <c r="J196" s="52">
+        <v>7389.339999999999</v>
+      </c>
+      <c r="K196" s="52">
+        <v>6605.049999999999</v>
+      </c>
+      <c r="L196" s="52">
+        <v>784.29</v>
+      </c>
+      <c r="M196" s="53">
+        <v>0.10613803127207573</v>
+      </c>
       <c r="N196" s="53"/>
-      <c r="O196" s="52"/>
-      <c r="P196" s="52"/>
-      <c r="Q196" s="52"/>
-      <c r="R196" s="53"/>
-      <c r="S196" s="54"/>
-      <c r="T196" s="54"/>
-      <c r="U196" s="54"/>
-      <c r="V196" s="53"/>
+      <c r="O196" s="52">
+        <v>6921.62</v>
+      </c>
+      <c r="P196" s="52">
+        <v>511.68</v>
+      </c>
+      <c r="Q196" s="52">
+        <v>6409.94</v>
+      </c>
+      <c r="R196" s="53">
+        <v>0.9260751095841725</v>
+      </c>
+      <c r="S196" s="54">
+        <v>140.15</v>
+      </c>
+      <c r="T196" s="54">
+        <v>9.25</v>
+      </c>
+      <c r="U196" s="54">
+        <v>130.9</v>
+      </c>
+      <c r="V196" s="53">
+        <v>0.9339992864787727</v>
+      </c>
       <c r="W196" s="53"/>
-      <c r="X196" s="55"/>
-      <c r="Y196" s="55"/>
-      <c r="Z196" s="53"/>
-      <c r="AA196" s="56"/>
+      <c r="X196" s="55">
+        <v>333.8172972972973</v>
+      </c>
+      <c r="Y196" s="55">
+        <v>67.49902570438813</v>
+      </c>
+      <c r="Z196" s="53">
+        <v>0.30260000000000004</v>
+      </c>
+      <c r="AA196" s="56">
+        <v>0.398</v>
+      </c>
       <c r="AB196" s="57"/>
       <c r="AD196" s="35" t="s">
         <v>101</v>
@@ -25344,30 +25432,74 @@
       <c r="C259" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="D259" s="52"/>
-      <c r="E259" s="52"/>
-      <c r="F259" s="52"/>
-      <c r="G259" s="53"/>
-      <c r="H259" s="52"/>
-      <c r="I259" s="52"/>
-      <c r="J259" s="52"/>
-      <c r="K259" s="52"/>
-      <c r="L259" s="52"/>
-      <c r="M259" s="53"/>
+      <c r="D259" s="52">
+        <v>239296.88</v>
+      </c>
+      <c r="E259" s="52">
+        <v>10598.48</v>
+      </c>
+      <c r="F259" s="52">
+        <v>228698.4</v>
+      </c>
+      <c r="G259" s="53">
+        <v>0.9557099114706384</v>
+      </c>
+      <c r="H259" s="52">
+        <v>203192.69</v>
+      </c>
+      <c r="I259" s="52">
+        <v>18229.7</v>
+      </c>
+      <c r="J259" s="52">
+        <v>175849.53</v>
+      </c>
+      <c r="K259" s="52">
+        <v>16839.61</v>
+      </c>
+      <c r="L259" s="52">
+        <v>159009.91999999998</v>
+      </c>
+      <c r="M259" s="53">
+        <v>0.9042385271089436</v>
+      </c>
       <c r="N259" s="53"/>
-      <c r="O259" s="52"/>
-      <c r="P259" s="52"/>
-      <c r="Q259" s="52"/>
-      <c r="R259" s="53"/>
-      <c r="S259" s="54"/>
-      <c r="T259" s="54"/>
-      <c r="U259" s="54"/>
-      <c r="V259" s="53"/>
+      <c r="O259" s="52">
+        <v>27343.16</v>
+      </c>
+      <c r="P259" s="52">
+        <v>1390.09</v>
+      </c>
+      <c r="Q259" s="52">
+        <v>25953.07</v>
+      </c>
+      <c r="R259" s="53">
+        <v>0.9491613259038092</v>
+      </c>
+      <c r="S259" s="54">
+        <v>547.57</v>
+      </c>
+      <c r="T259" s="54">
+        <v>27.84</v>
+      </c>
+      <c r="U259" s="54">
+        <v>519.73</v>
+      </c>
+      <c r="V259" s="53">
+        <v>0.9491571853826908</v>
+      </c>
       <c r="W259" s="53"/>
-      <c r="X259" s="55"/>
-      <c r="Y259" s="55"/>
-      <c r="Z259" s="53"/>
-      <c r="AA259" s="56"/>
+      <c r="X259" s="55">
+        <v>-274.10991379310343</v>
+      </c>
+      <c r="Y259" s="55">
+        <v>65.93529946112827</v>
+      </c>
+      <c r="Z259" s="53">
+        <v>-0.72</v>
+      </c>
+      <c r="AA259" s="56">
+        <v>0.1509</v>
+      </c>
       <c r="AB259" s="57"/>
       <c r="AD259" s="35"/>
       <c r="AE259" s="36"/>
@@ -26756,10 +26888,10 @@
         <v>0</v>
       </c>
       <c r="D24" s="52">
-        <v>-249.79000000000087</v>
+        <v>499.0499999999993</v>
       </c>
       <c r="E24" s="52">
-        <v>249.79000000000087</v>
+        <v>-499.0499999999993</v>
       </c>
       <c r="F24" s="52">
         <v>3</v>
@@ -26777,7 +26909,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="52">
-        <v>252.79000000000087</v>
+        <v>-496.0499999999993</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="58">
@@ -27777,10 +27909,10 @@
         <v>0</v>
       </c>
       <c r="D58" s="99">
-        <v>178.1800000000003</v>
+        <v>180.76999999999953</v>
       </c>
       <c r="E58" s="99">
-        <v>-178.1800000000003</v>
+        <v>-180.76999999999953</v>
       </c>
       <c r="F58" s="99"/>
       <c r="G58" s="100">
@@ -27796,7 +27928,7 @@
         <v>0</v>
       </c>
       <c r="M58" s="99">
-        <v>-178.1800000000003</v>
+        <v>-180.76999999999953</v>
       </c>
       <c r="N58" s="98"/>
       <c r="O58" s="60">
@@ -28235,22 +28367,22 @@
         <v>98702.24999999996</v>
       </c>
       <c r="D74" s="104">
-        <v>89783.35999999996</v>
+        <v>90534.78999999996</v>
       </c>
       <c r="E74" s="105">
-        <v>8918.890000000003</v>
+        <v>8167.459999999994</v>
       </c>
       <c r="F74" s="106" t="s">
         <v>127</v>
       </c>
       <c r="G74" s="107">
-        <v>0.09036156723884214</v>
+        <v>0.08274846824667115</v>
       </c>
       <c r="H74" s="108" t="s">
         <v>128</v>
       </c>
       <c r="I74" s="109">
-        <v>-0.6211987062098385</v>
+        <v>-0.6288118052020095</v>
       </c>
       <c r="J74" s="36"/>
       <c r="K74" s="36"/>
@@ -29357,10 +29489,10 @@
         <v>472.14</v>
       </c>
       <c r="D24" s="54">
-        <v>156</v>
+        <v>167.25</v>
       </c>
       <c r="E24" s="54">
-        <v>316.14</v>
+        <v>304.89</v>
       </c>
       <c r="F24" s="54"/>
       <c r="G24" s="54"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-14T21:45:55Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -14649,30 +14649,74 @@
       <c r="C77" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="D77" s="52"/>
-      <c r="E77" s="52"/>
-      <c r="F77" s="52"/>
-      <c r="G77" s="53"/>
-      <c r="H77" s="52"/>
-      <c r="I77" s="52"/>
-      <c r="J77" s="52"/>
-      <c r="K77" s="52"/>
-      <c r="L77" s="52"/>
-      <c r="M77" s="53"/>
+      <c r="D77" s="52">
+        <v>78753.07</v>
+      </c>
+      <c r="E77" s="52">
+        <v>44764.99</v>
+      </c>
+      <c r="F77" s="52">
+        <v>33988.08000000001</v>
+      </c>
+      <c r="G77" s="53">
+        <v>0.4315778419812714</v>
+      </c>
+      <c r="H77" s="52">
+        <v>55589.78</v>
+      </c>
+      <c r="I77" s="52">
+        <v>32417.98</v>
+      </c>
+      <c r="J77" s="52">
+        <v>32594.75</v>
+      </c>
+      <c r="K77" s="52">
+        <v>24016.8</v>
+      </c>
+      <c r="L77" s="52">
+        <v>8577.95</v>
+      </c>
+      <c r="M77" s="53">
+        <v>0.26316968223410214</v>
+      </c>
       <c r="N77" s="53"/>
-      <c r="O77" s="52"/>
-      <c r="P77" s="52"/>
-      <c r="Q77" s="52"/>
-      <c r="R77" s="53"/>
-      <c r="S77" s="54"/>
-      <c r="T77" s="54"/>
-      <c r="U77" s="54"/>
-      <c r="V77" s="53"/>
+      <c r="O77" s="52">
+        <v>22995.03</v>
+      </c>
+      <c r="P77" s="52">
+        <v>8401.18</v>
+      </c>
+      <c r="Q77" s="52">
+        <v>14593.849999999999</v>
+      </c>
+      <c r="R77" s="53">
+        <v>0.6346523574876832</v>
+      </c>
+      <c r="S77" s="54">
+        <v>472.14</v>
+      </c>
+      <c r="T77" s="54">
+        <v>167.25</v>
+      </c>
+      <c r="U77" s="54">
+        <v>304.89</v>
+      </c>
+      <c r="V77" s="53">
+        <v>0.6457618502986402</v>
+      </c>
       <c r="W77" s="53"/>
-      <c r="X77" s="55"/>
-      <c r="Y77" s="55"/>
-      <c r="Z77" s="53"/>
-      <c r="AA77" s="56"/>
+      <c r="X77" s="55">
+        <v>73.82367713004484</v>
+      </c>
+      <c r="Y77" s="55">
+        <v>49.060202993773025</v>
+      </c>
+      <c r="Z77" s="53">
+        <v>0.2758</v>
+      </c>
+      <c r="AA77" s="56">
+        <v>0.2941</v>
+      </c>
       <c r="AB77" s="57"/>
       <c r="AD77" s="35" t="s">
         <v>101</v>
@@ -21955,30 +21999,74 @@
       <c r="C196" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="D196" s="52"/>
-      <c r="E196" s="52"/>
-      <c r="F196" s="52"/>
-      <c r="G196" s="53"/>
-      <c r="H196" s="52"/>
-      <c r="I196" s="52"/>
-      <c r="J196" s="52"/>
-      <c r="K196" s="52"/>
-      <c r="L196" s="52"/>
-      <c r="M196" s="53"/>
+      <c r="D196" s="52">
+        <v>23770.95</v>
+      </c>
+      <c r="E196" s="52">
+        <v>10204.54</v>
+      </c>
+      <c r="F196" s="52">
+        <v>13566.41</v>
+      </c>
+      <c r="G196" s="53">
+        <v>0.5707138334816235</v>
+      </c>
+      <c r="H196" s="52">
+        <v>14310.96</v>
+      </c>
+      <c r="I196" s="52">
+        <v>7116.73</v>
+      </c>
+      <c r="J196" s="52">
+        <v>7389.339999999999</v>
+      </c>
+      <c r="K196" s="52">
+        <v>6605.049999999999</v>
+      </c>
+      <c r="L196" s="52">
+        <v>784.29</v>
+      </c>
+      <c r="M196" s="53">
+        <v>0.10613803127207573</v>
+      </c>
       <c r="N196" s="53"/>
-      <c r="O196" s="52"/>
-      <c r="P196" s="52"/>
-      <c r="Q196" s="52"/>
-      <c r="R196" s="53"/>
-      <c r="S196" s="54"/>
-      <c r="T196" s="54"/>
-      <c r="U196" s="54"/>
-      <c r="V196" s="53"/>
+      <c r="O196" s="52">
+        <v>6921.62</v>
+      </c>
+      <c r="P196" s="52">
+        <v>511.68</v>
+      </c>
+      <c r="Q196" s="52">
+        <v>6409.94</v>
+      </c>
+      <c r="R196" s="53">
+        <v>0.9260751095841725</v>
+      </c>
+      <c r="S196" s="54">
+        <v>140.15</v>
+      </c>
+      <c r="T196" s="54">
+        <v>9.25</v>
+      </c>
+      <c r="U196" s="54">
+        <v>130.9</v>
+      </c>
+      <c r="V196" s="53">
+        <v>0.9339992864787727</v>
+      </c>
       <c r="W196" s="53"/>
-      <c r="X196" s="55"/>
-      <c r="Y196" s="55"/>
-      <c r="Z196" s="53"/>
-      <c r="AA196" s="56"/>
+      <c r="X196" s="55">
+        <v>333.8172972972973</v>
+      </c>
+      <c r="Y196" s="55">
+        <v>67.49902570438813</v>
+      </c>
+      <c r="Z196" s="53">
+        <v>0.30260000000000004</v>
+      </c>
+      <c r="AA196" s="56">
+        <v>0.398</v>
+      </c>
       <c r="AB196" s="57"/>
       <c r="AD196" s="35" t="s">
         <v>101</v>
@@ -25344,30 +25432,74 @@
       <c r="C259" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="D259" s="52"/>
-      <c r="E259" s="52"/>
-      <c r="F259" s="52"/>
-      <c r="G259" s="53"/>
-      <c r="H259" s="52"/>
-      <c r="I259" s="52"/>
-      <c r="J259" s="52"/>
-      <c r="K259" s="52"/>
-      <c r="L259" s="52"/>
-      <c r="M259" s="53"/>
+      <c r="D259" s="52">
+        <v>239296.88</v>
+      </c>
+      <c r="E259" s="52">
+        <v>10598.48</v>
+      </c>
+      <c r="F259" s="52">
+        <v>228698.4</v>
+      </c>
+      <c r="G259" s="53">
+        <v>0.9557099114706384</v>
+      </c>
+      <c r="H259" s="52">
+        <v>203192.69</v>
+      </c>
+      <c r="I259" s="52">
+        <v>18229.7</v>
+      </c>
+      <c r="J259" s="52">
+        <v>175849.53</v>
+      </c>
+      <c r="K259" s="52">
+        <v>16839.61</v>
+      </c>
+      <c r="L259" s="52">
+        <v>159009.91999999998</v>
+      </c>
+      <c r="M259" s="53">
+        <v>0.9042385271089436</v>
+      </c>
       <c r="N259" s="53"/>
-      <c r="O259" s="52"/>
-      <c r="P259" s="52"/>
-      <c r="Q259" s="52"/>
-      <c r="R259" s="53"/>
-      <c r="S259" s="54"/>
-      <c r="T259" s="54"/>
-      <c r="U259" s="54"/>
-      <c r="V259" s="53"/>
+      <c r="O259" s="52">
+        <v>27343.16</v>
+      </c>
+      <c r="P259" s="52">
+        <v>1390.09</v>
+      </c>
+      <c r="Q259" s="52">
+        <v>25953.07</v>
+      </c>
+      <c r="R259" s="53">
+        <v>0.9491613259038092</v>
+      </c>
+      <c r="S259" s="54">
+        <v>547.57</v>
+      </c>
+      <c r="T259" s="54">
+        <v>27.84</v>
+      </c>
+      <c r="U259" s="54">
+        <v>519.73</v>
+      </c>
+      <c r="V259" s="53">
+        <v>0.9491571853826908</v>
+      </c>
       <c r="W259" s="53"/>
-      <c r="X259" s="55"/>
-      <c r="Y259" s="55"/>
-      <c r="Z259" s="53"/>
-      <c r="AA259" s="56"/>
+      <c r="X259" s="55">
+        <v>-274.10991379310343</v>
+      </c>
+      <c r="Y259" s="55">
+        <v>65.93529946112827</v>
+      </c>
+      <c r="Z259" s="53">
+        <v>-0.72</v>
+      </c>
+      <c r="AA259" s="56">
+        <v>0.1509</v>
+      </c>
       <c r="AB259" s="57"/>
       <c r="AD259" s="35"/>
       <c r="AE259" s="36"/>
@@ -26756,10 +26888,10 @@
         <v>0</v>
       </c>
       <c r="D24" s="52">
-        <v>-249.79000000000087</v>
+        <v>499.0499999999993</v>
       </c>
       <c r="E24" s="52">
-        <v>249.79000000000087</v>
+        <v>-499.0499999999993</v>
       </c>
       <c r="F24" s="52">
         <v>3</v>
@@ -26777,7 +26909,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="52">
-        <v>252.79000000000087</v>
+        <v>-496.0499999999993</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="58">
@@ -27777,10 +27909,10 @@
         <v>0</v>
       </c>
       <c r="D58" s="99">
-        <v>178.1800000000003</v>
+        <v>180.76999999999953</v>
       </c>
       <c r="E58" s="99">
-        <v>-178.1800000000003</v>
+        <v>-180.76999999999953</v>
       </c>
       <c r="F58" s="99"/>
       <c r="G58" s="100">
@@ -27796,7 +27928,7 @@
         <v>0</v>
       </c>
       <c r="M58" s="99">
-        <v>-178.1800000000003</v>
+        <v>-180.76999999999953</v>
       </c>
       <c r="N58" s="98"/>
       <c r="O58" s="60">
@@ -28235,22 +28367,22 @@
         <v>98702.24999999996</v>
       </c>
       <c r="D74" s="104">
-        <v>89783.35999999996</v>
+        <v>90534.78999999996</v>
       </c>
       <c r="E74" s="105">
-        <v>8918.890000000003</v>
+        <v>8167.459999999994</v>
       </c>
       <c r="F74" s="106" t="s">
         <v>127</v>
       </c>
       <c r="G74" s="107">
-        <v>0.09036156723884214</v>
+        <v>0.08274846824667115</v>
       </c>
       <c r="H74" s="108" t="s">
         <v>128</v>
       </c>
       <c r="I74" s="109">
-        <v>-0.6211987062098385</v>
+        <v>-0.6288118052020095</v>
       </c>
       <c r="J74" s="36"/>
       <c r="K74" s="36"/>
@@ -29357,10 +29489,10 @@
         <v>472.14</v>
       </c>
       <c r="D24" s="54">
-        <v>156</v>
+        <v>167.25</v>
       </c>
       <c r="E24" s="54">
-        <v>316.14</v>
+        <v>304.89</v>
       </c>
       <c r="F24" s="54"/>
       <c r="G24" s="54"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-15T18:55:34Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -18143,7 +18143,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>100</v>
@@ -26146,7 +26146,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD75"/>
+  <dimension ref="A1:R75"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -26160,7 +26160,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -26182,7 +26182,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>105</v>
       </c>
@@ -26230,7 +26230,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -26248,7 +26248,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -26295,7 +26295,7 @@
         <v>-100.50142857142866</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -26312,7 +26312,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -26362,7 +26362,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -26379,7 +26379,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -26422,7 +26422,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -26439,7 +26439,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -26486,7 +26486,7 @@
         <v>27.80091109478323</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -26503,7 +26503,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -26553,7 +26553,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -26570,7 +26570,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -26617,7 +26617,7 @@
         <v>110.61624999999997</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -26634,7 +26634,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -26679,7 +26679,7 @@
         <v>40.952161383285286</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -26696,7 +26696,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -26746,7 +26746,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -26763,7 +26763,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -26802,7 +26802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -26819,7 +26819,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -26860,7 +26860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -26877,7 +26877,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -26916,7 +26916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -26933,7 +26933,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -26978,7 +26978,7 @@
         <v>-3.0733682373472964</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -26995,7 +26995,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -27038,7 +27038,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -27055,7 +27055,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -27098,7 +27098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -27115,7 +27115,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -27162,7 +27162,7 @@
         <v>13.90219151036525</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -27179,7 +27179,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -27224,7 +27224,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -27241,7 +27241,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -27284,7 +27284,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -27301,7 +27301,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -27342,7 +27342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -27359,7 +27359,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -27404,7 +27404,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -27421,7 +27421,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -27464,7 +27464,7 @@
         <v>-0.05012183692595682</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -27481,7 +27481,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -27518,7 +27518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -27535,7 +27535,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27576,7 +27576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -27593,7 +27593,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -27636,7 +27636,7 @@
         <v>95.15307262569829</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -27653,7 +27653,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -27695,7 +27695,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -27712,7 +27712,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -27757,7 +27757,7 @@
         <v>14.869587534372164</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -27774,7 +27774,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -27819,7 +27819,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -27836,7 +27836,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -27881,7 +27881,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -27898,7 +27898,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -27935,7 +27935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -27952,7 +27952,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -27969,7 +27969,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -27986,7 +27986,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -28007,7 +28007,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -28024,7 +28024,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -28065,7 +28065,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -28082,7 +28082,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -28127,7 +28127,7 @@
         <v>-15.917709392560841</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <v>9437</v>
       </c>
@@ -28166,7 +28166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="102">
         <v>7480</v>
       </c>
@@ -28205,7 +28205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="102">
         <v>8829</v>
       </c>
@@ -28244,7 +28244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="102">
         <v>8386</v>
       </c>
@@ -28283,7 +28283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" s="102">
         <v>8530</v>
       </c>
@@ -28322,7 +28322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A72" s="35"/>
       <c r="B72" s="35"/>
       <c r="C72" s="36"/>
@@ -28339,7 +28339,7 @@
       <c r="N72" s="35"/>
       <c r="O72" s="36"/>
     </row>
-    <row r="73" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A73" s="35"/>
       <c r="B73" s="35"/>
       <c r="C73" s="36"/>
@@ -28356,7 +28356,7 @@
       <c r="N73" s="35"/>
       <c r="O73" s="35"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A74" s="49" t="s">
         <v>125</v>
       </c>
@@ -28391,7 +28391,7 @@
       <c r="N74" s="35"/>
       <c r="O74" s="35"/>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A75" s="59"/>
       <c r="B75" s="98" t="s">
         <v>129</v>
@@ -28774,7 +28774,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD114"/>
+  <dimension ref="A1:AB114"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -28785,7 +28785,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -28806,7 +28806,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>130</v>
@@ -28868,7 +28868,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>146</v>
       </c>
@@ -28926,7 +28926,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -28966,7 +28966,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -28985,7 +28985,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -29021,7 +29021,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -29040,7 +29040,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -29076,7 +29076,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -29095,7 +29095,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -29133,7 +29133,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -29152,7 +29152,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -29192,7 +29192,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -29211,7 +29211,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -29249,7 +29249,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -29268,7 +29268,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -29301,7 +29301,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -29320,7 +29320,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -29353,7 +29353,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -29372,7 +29372,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -29403,7 +29403,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -29422,7 +29422,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -29459,7 +29459,7 @@
       </c>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -29478,7 +29478,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -29513,7 +29513,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -29532,7 +29532,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -29563,7 +29563,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -29582,7 +29582,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -29614,7 +29614,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -29633,7 +29633,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -29671,7 +29671,7 @@
       </c>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -29690,7 +29690,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -29719,7 +29719,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -29738,7 +29738,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -29769,7 +29769,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -29788,7 +29788,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -29825,7 +29825,7 @@
       </c>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -29844,7 +29844,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -29880,7 +29880,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -29899,7 +29899,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -29934,7 +29934,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -29953,7 +29953,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -29983,7 +29983,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -30002,7 +30002,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -30042,7 +30042,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -30061,7 +30061,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -30090,7 +30090,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -30109,7 +30109,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -30144,7 +30144,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -30163,7 +30163,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -30198,7 +30198,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -30217,7 +30217,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -30253,7 +30253,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -30272,7 +30272,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -30310,7 +30310,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -30329,7 +30329,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -30367,7 +30367,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -30386,7 +30386,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -30421,7 +30421,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -30440,7 +30440,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -30459,7 +30459,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -30478,7 +30478,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -30499,7 +30499,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -30518,7 +30518,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -30555,7 +30555,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -30574,7 +30574,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -30613,7 +30613,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <v>9437</v>
       </c>
@@ -30629,7 +30629,9 @@
       <c r="E67" s="54">
         <v>519.73</v>
       </c>
-      <c r="F67" s="54"/>
+      <c r="F67" s="54">
+        <v>240</v>
+      </c>
       <c r="G67" s="54"/>
       <c r="H67" s="54"/>
       <c r="I67" s="54"/>
@@ -30638,15 +30640,17 @@
       <c r="L67" s="54"/>
       <c r="M67" s="54"/>
       <c r="N67" s="54"/>
-      <c r="O67" s="54"/>
+      <c r="O67" s="54">
+        <v>0</v>
+      </c>
       <c r="P67" s="54">
-        <v>160</v>
+        <v>0</v>
       </c>
       <c r="Q67" s="54">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="19">
         <v>7480</v>
       </c>
@@ -30675,7 +30679,7 @@
       <c r="P68" s="54"/>
       <c r="Q68" s="54"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="19">
         <v>8829</v>
       </c>
@@ -30708,7 +30712,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="19">
         <v>8386</v>
       </c>
@@ -30743,7 +30747,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="19">
         <v>8530</v>
       </c>
@@ -30772,7 +30776,7 @@
       <c r="P71" s="54"/>
       <c r="Q71" s="54"/>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="143"/>
       <c r="C72" s="35"/>
@@ -30791,7 +30795,7 @@
       <c r="P72" s="35"/>
       <c r="Q72" s="144"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="143"/>
       <c r="C73" s="35"/>
@@ -30810,7 +30814,7 @@
       <c r="P73" s="35"/>
       <c r="Q73" s="144"/>
     </row>
-    <row r="74" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="145"/>
       <c r="B74" s="145"/>
       <c r="C74" s="145"/>
@@ -30829,7 +30833,7 @@
       <c r="P74" s="145"/>
       <c r="Q74" s="145"/>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="146" t="s">
         <v>150</v>
@@ -30874,7 +30878,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="77" t="s">
         <v>151</v>
@@ -30913,7 +30917,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="77" t="s">
         <v>152</v>
@@ -30942,7 +30946,7 @@
       <c r="P77" s="20"/>
       <c r="Q77" s="20"/>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="142"/>
       <c r="B78" s="148" t="s">
         <v>153</v>
@@ -30987,7 +30991,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="142"/>
       <c r="B79" s="151" t="s">
         <v>154</v>
@@ -31032,7 +31036,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="142"/>
       <c r="B80" s="35"/>
       <c r="C80" s="35"/>
@@ -31051,7 +31055,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="144"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="142"/>
       <c r="B81" s="156" t="s">
         <v>155</v>
@@ -31098,7 +31102,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="161"/>
       <c r="B82" s="162" t="s">
         <v>157</v>
@@ -31143,7 +31147,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="83" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="35"/>
       <c r="C83" s="35"/>
@@ -31162,7 +31166,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="164" t="s">
         <v>158</v>
@@ -31185,7 +31189,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="167" t="s">
         <v>160</v>
@@ -31208,7 +31212,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>161</v>
@@ -31231,7 +31235,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>162</v>
@@ -31254,7 +31258,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>163</v>
@@ -31277,7 +31281,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>164</v>
@@ -31300,7 +31304,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>165</v>
@@ -31323,7 +31327,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>166</v>
@@ -31346,7 +31350,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19" t="s">
         <v>167</v>
@@ -31369,7 +31373,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19" t="s">
         <v>168</v>
@@ -31392,7 +31396,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19" t="s">
         <v>169</v>
@@ -31415,7 +31419,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19" t="s">
         <v>170</v>
@@ -31438,7 +31442,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -31459,7 +31463,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -31480,7 +31484,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -31501,7 +31505,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19"/>
       <c r="C99" s="131">
@@ -31522,7 +31526,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19"/>
       <c r="C100" s="131">
@@ -31543,7 +31547,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19"/>
       <c r="C101" s="131">
@@ -31564,7 +31568,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19"/>
       <c r="C102" s="131">
@@ -31585,7 +31589,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>171</v>
@@ -31608,7 +31612,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>172</v>
@@ -31631,7 +31635,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>173</v>
@@ -31654,7 +31658,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19" t="s">
         <v>174</v>
@@ -31677,7 +31681,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19" t="s">
         <v>175</v>
@@ -31700,7 +31704,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19" t="s">
         <v>176</v>
@@ -31723,7 +31727,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="19" t="s">
         <v>177</v>
@@ -31746,7 +31750,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="19"/>
       <c r="C110" s="131"/>
@@ -31765,7 +31769,7 @@
       <c r="P110" s="35"/>
       <c r="Q110" s="35"/>
     </row>
-    <row r="111" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="111" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A111" s="35"/>
       <c r="B111" s="19"/>
       <c r="C111" s="131"/>
@@ -31784,7 +31788,7 @@
       <c r="P111" s="35"/>
       <c r="Q111" s="35"/>
     </row>
-    <row r="112" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="112" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A112" s="35"/>
       <c r="B112" s="19"/>
       <c r="C112" s="131"/>
@@ -31803,7 +31807,7 @@
       <c r="P112" s="35"/>
       <c r="Q112" s="35"/>
     </row>
-    <row r="113" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="113" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A113" s="35"/>
       <c r="B113" s="169"/>
       <c r="C113" s="150"/>
@@ -31822,7 +31826,7 @@
       <c r="P113" s="35"/>
       <c r="Q113" s="35"/>
     </row>
-    <row r="114" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="114" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A114" s="35"/>
       <c r="B114" s="164" t="s">
         <v>178</v>
@@ -31896,11 +31900,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>179</v>
       </c>
@@ -31932,7 +31935,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>180</v>
       </c>
@@ -31965,7 +31968,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>181</v>
       </c>
@@ -31998,7 +32001,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>182</v>
       </c>
@@ -32031,7 +32034,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>183</v>
       </c>
@@ -32064,7 +32067,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>184</v>
       </c>
@@ -32097,7 +32100,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>185</v>
       </c>
@@ -32130,7 +32133,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>186</v>
       </c>
@@ -32163,7 +32166,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -32194,7 +32197,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -32225,7 +32228,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>187</v>
       </c>
@@ -32258,7 +32261,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>188</v>
       </c>
@@ -32291,7 +32294,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>189</v>
       </c>
@@ -32324,7 +32327,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>190</v>
       </c>
@@ -32357,7 +32360,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>191</v>
       </c>
@@ -32390,7 +32393,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>192</v>
       </c>
@@ -32423,7 +32426,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>193</v>
       </c>
@@ -32456,7 +32459,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>194</v>
       </c>
@@ -32489,7 +32492,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>195</v>
       </c>
@@ -32522,7 +32525,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>196</v>
       </c>
@@ -32555,7 +32558,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>197</v>
       </c>
@@ -32588,7 +32591,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>198</v>
       </c>
@@ -32621,7 +32624,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>199</v>
       </c>
@@ -32654,7 +32657,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>200</v>
       </c>
@@ -32687,7 +32690,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>201</v>
       </c>
@@ -32720,7 +32723,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>202</v>
       </c>
@@ -32753,7 +32756,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>203</v>
       </c>
@@ -32785,7 +32788,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>204</v>
       </c>
@@ -32817,7 +32820,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>205</v>
       </c>
@@ -32849,7 +32852,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>206</v>
       </c>
@@ -32881,7 +32884,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>207</v>
       </c>
@@ -32913,7 +32916,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -32943,7 +32946,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -32973,7 +32976,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>208</v>
       </c>
@@ -33005,7 +33008,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>209</v>
       </c>
@@ -33037,7 +33040,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>210</v>
       </c>
@@ -33069,7 +33072,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>211</v>
       </c>
@@ -33101,7 +33104,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>212</v>
       </c>
@@ -33133,7 +33136,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -33163,7 +33166,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>213</v>
       </c>
@@ -33195,7 +33198,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>214</v>
       </c>
@@ -33227,7 +33230,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>215</v>
       </c>
@@ -33259,7 +33262,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>216</v>
       </c>
@@ -33291,7 +33294,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -33321,7 +33324,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -33351,7 +33354,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -33381,7 +33384,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -33411,7 +33414,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>217</v>
       </c>
@@ -33443,7 +33446,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>218</v>
       </c>
@@ -33475,7 +33478,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -33505,7 +33508,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -33535,7 +33538,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -33565,7 +33568,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -33595,7 +33598,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -33625,7 +33628,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -33720,11 +33723,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>219</v>
       </c>
@@ -33756,7 +33758,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -33787,7 +33789,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -33818,7 +33820,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -33849,7 +33851,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -33880,7 +33882,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -33911,7 +33913,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -33942,7 +33944,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -33973,7 +33975,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -34004,7 +34006,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -34035,7 +34037,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -34066,7 +34068,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -34097,7 +34099,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -34128,7 +34130,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -34159,7 +34161,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -34190,7 +34192,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -34221,7 +34223,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -34252,7 +34254,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -34283,7 +34285,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -34314,7 +34316,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -34345,7 +34347,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -34375,7 +34377,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -34405,7 +34407,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -34435,7 +34437,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -34465,7 +34467,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -34495,7 +34497,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -34525,7 +34527,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -34555,7 +34557,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -34585,7 +34587,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -34615,7 +34617,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -34645,7 +34647,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -34675,7 +34677,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -34705,7 +34707,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -34735,7 +34737,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -34765,7 +34767,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -34795,7 +34797,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -34825,7 +34827,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>217</v>
       </c>
@@ -34857,7 +34859,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>218</v>
       </c>
@@ -34889,7 +34891,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -34919,7 +34921,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -34949,7 +34951,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -34979,7 +34981,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -35009,7 +35011,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -35039,7 +35041,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -56782,19 +56784,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -56808,7 +56810,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>226</v>
       </c>
@@ -56820,7 +56822,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>227</v>
       </c>
@@ -56831,7 +56833,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>228</v>
       </c>
@@ -56842,7 +56844,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>229</v>
       </c>
@@ -56853,13 +56855,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Sync data files (2026-09-15T18:56:19Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -29182,14 +29182,14 @@
         <v>0</v>
       </c>
       <c r="O12" s="86">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="P12" s="54">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="131"/>
       <c r="S12" s="35" t="s">
-        <v>148</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Sync data files (2026-09-15T18:59:33Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -29242,7 +29242,9 @@
       <c r="N14" s="54">
         <v>0</v>
       </c>
-      <c r="O14" s="54"/>
+      <c r="O14" s="54">
+        <v>30</v>
+      </c>
       <c r="P14" s="54"/>
       <c r="Q14" s="131"/>
       <c r="S14" s="35" t="s">
@@ -30738,13 +30740,13 @@
       <c r="M70" s="54"/>
       <c r="N70" s="54"/>
       <c r="O70" s="54">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="P70" s="54">
-        <v>72</v>
+        <v>18</v>
       </c>
       <c r="Q70" s="54">
-        <v>16</v>
+        <v>90</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Sync data files (2026-09-15T19:00:46Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -29663,13 +29663,13 @@
         <v>0</v>
       </c>
       <c r="O30" s="54">
+        <v>0</v>
+      </c>
+      <c r="P30" s="54">
         <v>48</v>
       </c>
-      <c r="P30" s="54">
+      <c r="Q30" s="131">
         <v>16</v>
-      </c>
-      <c r="Q30" s="131">
-        <v>64</v>
       </c>
       <c r="S30" s="139"/>
     </row>
@@ -29932,9 +29932,15 @@
       <c r="L40" s="54"/>
       <c r="M40" s="54"/>
       <c r="N40" s="54"/>
-      <c r="O40" s="54"/>
-      <c r="P40" s="54"/>
-      <c r="Q40" s="131"/>
+      <c r="O40" s="54">
+        <v>58</v>
+      </c>
+      <c r="P40" s="54">
+        <v>16</v>
+      </c>
+      <c r="Q40" s="131">
+        <v>72</v>
+      </c>
     </row>
     <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-15T19:01:31Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -30683,9 +30683,15 @@
       <c r="L68" s="54"/>
       <c r="M68" s="54"/>
       <c r="N68" s="54"/>
-      <c r="O68" s="54"/>
-      <c r="P68" s="54"/>
-      <c r="Q68" s="54"/>
+      <c r="O68" s="54">
+        <v>56</v>
+      </c>
+      <c r="P68" s="54">
+        <v>16</v>
+      </c>
+      <c r="Q68" s="54">
+        <v>68</v>
+      </c>
     </row>
     <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="19">

</xml_diff>

<commit_message>
Sync data files (2026-09-15T19:02:55Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -30786,8 +30786,12 @@
       <c r="L71" s="54"/>
       <c r="M71" s="54"/>
       <c r="N71" s="54"/>
-      <c r="O71" s="54"/>
-      <c r="P71" s="54"/>
+      <c r="O71" s="54">
+        <v>20</v>
+      </c>
+      <c r="P71" s="54">
+        <v>16</v>
+      </c>
       <c r="Q71" s="54"/>
     </row>
     <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Sync data files (2026-09-16T20:45:20Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -18143,7 +18143,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>100</v>
@@ -26146,7 +26146,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R75"/>
+  <dimension ref="A1:AD75"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -26160,7 +26160,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -26182,7 +26182,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>105</v>
       </c>
@@ -26230,7 +26230,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -26248,7 +26248,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -26295,7 +26295,7 @@
         <v>-100.50142857142866</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -26312,7 +26312,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -26362,7 +26362,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -26379,7 +26379,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -26422,7 +26422,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -26439,7 +26439,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -26486,7 +26486,7 @@
         <v>27.80091109478323</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -26503,7 +26503,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -26553,7 +26553,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -26570,7 +26570,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -26617,7 +26617,7 @@
         <v>110.61624999999997</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -26634,7 +26634,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -26679,7 +26679,7 @@
         <v>40.952161383285286</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -26696,7 +26696,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -26746,7 +26746,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -26763,7 +26763,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -26802,7 +26802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -26819,7 +26819,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -26860,7 +26860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -26877,7 +26877,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -26916,7 +26916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -26933,7 +26933,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -26978,7 +26978,7 @@
         <v>-3.0733682373472964</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -26995,7 +26995,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -27038,7 +27038,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -27055,7 +27055,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -27098,7 +27098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -27115,7 +27115,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -27162,7 +27162,7 @@
         <v>13.90219151036525</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -27179,7 +27179,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -27224,7 +27224,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -27241,7 +27241,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -27284,7 +27284,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -27301,7 +27301,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -27342,7 +27342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -27359,7 +27359,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -27404,7 +27404,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -27421,7 +27421,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -27464,7 +27464,7 @@
         <v>-0.05012183692595682</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -27481,7 +27481,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -27518,7 +27518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -27535,7 +27535,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27576,7 +27576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -27593,7 +27593,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -27636,7 +27636,7 @@
         <v>95.15307262569829</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -27653,7 +27653,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -27695,7 +27695,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -27712,7 +27712,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -27757,7 +27757,7 @@
         <v>14.869587534372164</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -27774,7 +27774,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -27819,7 +27819,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -27836,7 +27836,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -27881,7 +27881,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -27898,7 +27898,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -27935,7 +27935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -27952,7 +27952,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -27969,7 +27969,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -27986,7 +27986,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -28007,7 +28007,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -28024,7 +28024,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -28065,7 +28065,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -28082,7 +28082,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -28127,7 +28127,7 @@
         <v>-15.917709392560841</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <v>9437</v>
       </c>
@@ -28166,7 +28166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="102">
         <v>7480</v>
       </c>
@@ -28205,7 +28205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="102">
         <v>8829</v>
       </c>
@@ -28244,7 +28244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="102">
         <v>8386</v>
       </c>
@@ -28283,7 +28283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="102">
         <v>8530</v>
       </c>
@@ -28322,7 +28322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="35"/>
       <c r="B72" s="35"/>
       <c r="C72" s="36"/>
@@ -28339,7 +28339,7 @@
       <c r="N72" s="35"/>
       <c r="O72" s="36"/>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="35"/>
       <c r="B73" s="35"/>
       <c r="C73" s="36"/>
@@ -28356,7 +28356,7 @@
       <c r="N73" s="35"/>
       <c r="O73" s="35"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="49" t="s">
         <v>125</v>
       </c>
@@ -28391,7 +28391,7 @@
       <c r="N74" s="35"/>
       <c r="O74" s="35"/>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="59"/>
       <c r="B75" s="98" t="s">
         <v>129</v>
@@ -28774,7 +28774,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB114"/>
+  <dimension ref="A1:AD114"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -28785,7 +28785,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -28806,7 +28806,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>130</v>
@@ -28868,7 +28868,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>146</v>
       </c>
@@ -28926,7 +28926,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -28966,7 +28966,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -28985,7 +28985,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -29021,7 +29021,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -29040,7 +29040,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -29076,7 +29076,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -29095,7 +29095,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -29133,7 +29133,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -29152,7 +29152,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -29192,7 +29192,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -29211,7 +29211,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -29251,7 +29251,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -29270,7 +29270,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -29303,7 +29303,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -29322,7 +29322,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -29355,7 +29355,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -29374,7 +29374,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -29405,7 +29405,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -29424,7 +29424,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -29461,7 +29461,7 @@
       </c>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -29480,7 +29480,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -29515,7 +29515,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -29534,7 +29534,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -29565,7 +29565,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -29584,7 +29584,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -29616,7 +29616,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -29635,7 +29635,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -29673,7 +29673,7 @@
       </c>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -29692,7 +29692,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -29721,7 +29721,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -29740,7 +29740,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -29771,7 +29771,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -29790,7 +29790,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -29827,7 +29827,7 @@
       </c>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -29846,7 +29846,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -29882,7 +29882,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -29901,7 +29901,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -29942,7 +29942,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -29961,7 +29961,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -29991,7 +29991,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -30010,7 +30010,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -30050,7 +30050,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -30069,7 +30069,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -30098,7 +30098,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -30117,7 +30117,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -30152,7 +30152,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -30171,7 +30171,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -30206,7 +30206,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -30225,7 +30225,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -30261,7 +30261,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -30280,7 +30280,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -30318,7 +30318,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -30337,7 +30337,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -30375,7 +30375,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -30394,7 +30394,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -30429,7 +30429,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -30448,7 +30448,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -30467,7 +30467,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -30486,7 +30486,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -30507,7 +30507,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -30526,7 +30526,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -30563,7 +30563,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -30582,7 +30582,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -30621,7 +30621,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <v>9437</v>
       </c>
@@ -30658,7 +30658,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="19">
         <v>7480</v>
       </c>
@@ -30693,7 +30693,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="19">
         <v>8829</v>
       </c>
@@ -30726,7 +30726,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="19">
         <v>8386</v>
       </c>
@@ -30761,7 +30761,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="19">
         <v>8530</v>
       </c>
@@ -30794,7 +30794,7 @@
       </c>
       <c r="Q71" s="54"/>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="143"/>
       <c r="C72" s="35"/>
@@ -30813,7 +30813,7 @@
       <c r="P72" s="35"/>
       <c r="Q72" s="144"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="143"/>
       <c r="C73" s="35"/>
@@ -30832,7 +30832,7 @@
       <c r="P73" s="35"/>
       <c r="Q73" s="144"/>
     </row>
-    <row r="74" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="145"/>
       <c r="B74" s="145"/>
       <c r="C74" s="145"/>
@@ -30851,7 +30851,7 @@
       <c r="P74" s="145"/>
       <c r="Q74" s="145"/>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="146" t="s">
         <v>150</v>
@@ -30896,7 +30896,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="77" t="s">
         <v>151</v>
@@ -30935,7 +30935,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="77" t="s">
         <v>152</v>
@@ -30964,7 +30964,7 @@
       <c r="P77" s="20"/>
       <c r="Q77" s="20"/>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="142"/>
       <c r="B78" s="148" t="s">
         <v>153</v>
@@ -31009,7 +31009,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="142"/>
       <c r="B79" s="151" t="s">
         <v>154</v>
@@ -31054,7 +31054,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="142"/>
       <c r="B80" s="35"/>
       <c r="C80" s="35"/>
@@ -31073,7 +31073,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="144"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="142"/>
       <c r="B81" s="156" t="s">
         <v>155</v>
@@ -31120,7 +31120,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="161"/>
       <c r="B82" s="162" t="s">
         <v>157</v>
@@ -31165,7 +31165,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="35"/>
       <c r="C83" s="35"/>
@@ -31184,7 +31184,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="164" t="s">
         <v>158</v>
@@ -31207,7 +31207,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="167" t="s">
         <v>160</v>
@@ -31230,7 +31230,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>161</v>
@@ -31253,7 +31253,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>162</v>
@@ -31276,7 +31276,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>163</v>
@@ -31299,7 +31299,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>164</v>
@@ -31322,7 +31322,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>165</v>
@@ -31345,7 +31345,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>166</v>
@@ -31368,7 +31368,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19" t="s">
         <v>167</v>
@@ -31391,7 +31391,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19" t="s">
         <v>168</v>
@@ -31414,7 +31414,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19" t="s">
         <v>169</v>
@@ -31437,7 +31437,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19" t="s">
         <v>170</v>
@@ -31460,7 +31460,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -31481,7 +31481,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -31502,7 +31502,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -31523,7 +31523,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19"/>
       <c r="C99" s="131">
@@ -31544,7 +31544,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19"/>
       <c r="C100" s="131">
@@ -31565,7 +31565,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19"/>
       <c r="C101" s="131">
@@ -31586,7 +31586,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19"/>
       <c r="C102" s="131">
@@ -31607,7 +31607,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>171</v>
@@ -31630,7 +31630,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>172</v>
@@ -31653,7 +31653,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>173</v>
@@ -31676,7 +31676,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19" t="s">
         <v>174</v>
@@ -31699,7 +31699,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19" t="s">
         <v>175</v>
@@ -31722,7 +31722,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19" t="s">
         <v>176</v>
@@ -31745,7 +31745,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="19" t="s">
         <v>177</v>
@@ -31768,7 +31768,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="19"/>
       <c r="C110" s="131"/>
@@ -31787,7 +31787,7 @@
       <c r="P110" s="35"/>
       <c r="Q110" s="35"/>
     </row>
-    <row r="111" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="111" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A111" s="35"/>
       <c r="B111" s="19"/>
       <c r="C111" s="131"/>
@@ -31806,7 +31806,7 @@
       <c r="P111" s="35"/>
       <c r="Q111" s="35"/>
     </row>
-    <row r="112" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="112" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A112" s="35"/>
       <c r="B112" s="19"/>
       <c r="C112" s="131"/>
@@ -31825,7 +31825,7 @@
       <c r="P112" s="35"/>
       <c r="Q112" s="35"/>
     </row>
-    <row r="113" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="113" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A113" s="35"/>
       <c r="B113" s="169"/>
       <c r="C113" s="150"/>
@@ -31844,7 +31844,7 @@
       <c r="P113" s="35"/>
       <c r="Q113" s="35"/>
     </row>
-    <row r="114" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="114" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A114" s="35"/>
       <c r="B114" s="164" t="s">
         <v>178</v>
@@ -31918,10 +31918,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>179</v>
       </c>
@@ -31953,7 +31954,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>180</v>
       </c>
@@ -31986,7 +31987,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>181</v>
       </c>
@@ -32019,7 +32020,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>182</v>
       </c>
@@ -32052,7 +32053,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>183</v>
       </c>
@@ -32085,7 +32086,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>184</v>
       </c>
@@ -32118,7 +32119,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>185</v>
       </c>
@@ -32151,7 +32152,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>186</v>
       </c>
@@ -32184,7 +32185,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -32215,7 +32216,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -32246,7 +32247,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>187</v>
       </c>
@@ -32279,7 +32280,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>188</v>
       </c>
@@ -32312,7 +32313,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>189</v>
       </c>
@@ -32345,7 +32346,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>190</v>
       </c>
@@ -32378,7 +32379,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>191</v>
       </c>
@@ -32411,7 +32412,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>192</v>
       </c>
@@ -32444,7 +32445,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>193</v>
       </c>
@@ -32477,7 +32478,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>194</v>
       </c>
@@ -32510,7 +32511,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>195</v>
       </c>
@@ -32543,7 +32544,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>196</v>
       </c>
@@ -32576,7 +32577,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>197</v>
       </c>
@@ -32609,7 +32610,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>198</v>
       </c>
@@ -32642,7 +32643,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>199</v>
       </c>
@@ -32675,7 +32676,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>200</v>
       </c>
@@ -32708,7 +32709,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>201</v>
       </c>
@@ -32741,7 +32742,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>202</v>
       </c>
@@ -32774,7 +32775,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>203</v>
       </c>
@@ -32806,7 +32807,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>204</v>
       </c>
@@ -32838,7 +32839,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>205</v>
       </c>
@@ -32870,7 +32871,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>206</v>
       </c>
@@ -32902,7 +32903,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>207</v>
       </c>
@@ -32934,7 +32935,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -32964,7 +32965,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -32994,7 +32995,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>208</v>
       </c>
@@ -33026,7 +33027,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>209</v>
       </c>
@@ -33058,7 +33059,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>210</v>
       </c>
@@ -33090,7 +33091,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>211</v>
       </c>
@@ -33122,7 +33123,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>212</v>
       </c>
@@ -33154,7 +33155,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -33184,7 +33185,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>213</v>
       </c>
@@ -33216,7 +33217,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>214</v>
       </c>
@@ -33248,7 +33249,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>215</v>
       </c>
@@ -33280,7 +33281,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>216</v>
       </c>
@@ -33312,7 +33313,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -33342,7 +33343,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -33372,7 +33373,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -33402,7 +33403,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -33432,7 +33433,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>217</v>
       </c>
@@ -33464,7 +33465,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>218</v>
       </c>
@@ -33496,7 +33497,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -33526,7 +33527,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -33556,7 +33557,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -33586,7 +33587,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -33616,7 +33617,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -33646,7 +33647,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -33741,10 +33742,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>219</v>
       </c>
@@ -33776,7 +33778,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -33807,7 +33809,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -33838,7 +33840,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -33869,7 +33871,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -33900,7 +33902,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -33931,7 +33933,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -33962,7 +33964,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -33993,7 +33995,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -34024,7 +34026,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -34055,7 +34057,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -34086,7 +34088,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -34117,7 +34119,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -34148,7 +34150,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -34179,7 +34181,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -34210,7 +34212,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -34241,7 +34243,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -34272,7 +34274,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -34303,7 +34305,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -34334,7 +34336,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -34365,7 +34367,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -34395,7 +34397,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -34425,7 +34427,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -34455,7 +34457,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -34485,7 +34487,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -34515,7 +34517,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -34545,7 +34547,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -34575,7 +34577,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -34605,7 +34607,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -34635,7 +34637,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -34665,7 +34667,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -34695,7 +34697,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -34725,7 +34727,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -34755,7 +34757,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -34785,7 +34787,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -34815,7 +34817,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -34845,7 +34847,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>217</v>
       </c>
@@ -34877,7 +34879,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>218</v>
       </c>
@@ -34909,7 +34911,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -34939,7 +34941,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -34969,7 +34971,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -34999,7 +35001,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -35029,7 +35031,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -35059,7 +35061,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -56802,19 +56804,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -56828,7 +56830,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>226</v>
       </c>
@@ -56840,7 +56842,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>227</v>
       </c>
@@ -56851,7 +56853,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>228</v>
       </c>
@@ -56862,7 +56864,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>229</v>
       </c>
@@ -56873,13 +56875,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Sync data files (2026-09-16T21:05:56Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1185" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1186" uniqueCount="230">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -7609,7 +7609,9 @@
       <c r="L52" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="M52" s="13"/>
+      <c r="M52" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="N52" s="14"/>
       <c r="O52" s="13" t="s">
         <v>33</v>
@@ -18143,7 +18145,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>100</v>
@@ -26146,7 +26148,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD75"/>
+  <dimension ref="A1:R75"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -26160,7 +26162,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -26182,7 +26184,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>105</v>
       </c>
@@ -26230,7 +26232,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -26248,7 +26250,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -26295,7 +26297,7 @@
         <v>-100.50142857142866</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -26312,7 +26314,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -26362,7 +26364,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -26379,7 +26381,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -26422,7 +26424,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -26439,7 +26441,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -26486,7 +26488,7 @@
         <v>27.80091109478323</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -26503,7 +26505,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -26553,7 +26555,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -26570,7 +26572,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -26617,7 +26619,7 @@
         <v>110.61624999999997</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -26634,7 +26636,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -26679,7 +26681,7 @@
         <v>40.952161383285286</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -26696,7 +26698,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -26746,7 +26748,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -26763,7 +26765,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -26802,7 +26804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -26819,7 +26821,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -26860,7 +26862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -26877,7 +26879,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -26916,7 +26918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -26933,7 +26935,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -26978,7 +26980,7 @@
         <v>-3.0733682373472964</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -26995,7 +26997,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -27038,7 +27040,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -27055,7 +27057,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -27098,7 +27100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -27115,7 +27117,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -27162,7 +27164,7 @@
         <v>13.90219151036525</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -27179,7 +27181,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -27224,7 +27226,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -27241,7 +27243,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -27284,7 +27286,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -27301,7 +27303,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -27342,7 +27344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -27359,7 +27361,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -27404,7 +27406,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -27421,7 +27423,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -27464,7 +27466,7 @@
         <v>-0.05012183692595682</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -27481,7 +27483,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -27518,7 +27520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -27535,7 +27537,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27576,7 +27578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -27593,7 +27595,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -27636,7 +27638,7 @@
         <v>95.15307262569829</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -27653,7 +27655,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -27695,7 +27697,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -27712,7 +27714,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -27757,7 +27759,7 @@
         <v>14.869587534372164</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -27774,7 +27776,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -27819,7 +27821,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -27836,7 +27838,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -27881,7 +27883,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -27898,7 +27900,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -27935,7 +27937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -27952,7 +27954,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -27969,7 +27971,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -27986,7 +27988,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -28007,7 +28009,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -28024,7 +28026,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -28065,7 +28067,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -28082,7 +28084,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -28127,7 +28129,7 @@
         <v>-15.917709392560841</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <v>9437</v>
       </c>
@@ -28166,7 +28168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="102">
         <v>7480</v>
       </c>
@@ -28205,7 +28207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="102">
         <v>8829</v>
       </c>
@@ -28244,7 +28246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="102">
         <v>8386</v>
       </c>
@@ -28283,7 +28285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" s="102">
         <v>8530</v>
       </c>
@@ -28322,7 +28324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A72" s="35"/>
       <c r="B72" s="35"/>
       <c r="C72" s="36"/>
@@ -28339,7 +28341,7 @@
       <c r="N72" s="35"/>
       <c r="O72" s="36"/>
     </row>
-    <row r="73" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A73" s="35"/>
       <c r="B73" s="35"/>
       <c r="C73" s="36"/>
@@ -28356,7 +28358,7 @@
       <c r="N73" s="35"/>
       <c r="O73" s="35"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A74" s="49" t="s">
         <v>125</v>
       </c>
@@ -28391,7 +28393,7 @@
       <c r="N74" s="35"/>
       <c r="O74" s="35"/>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A75" s="59"/>
       <c r="B75" s="98" t="s">
         <v>129</v>
@@ -28774,7 +28776,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD114"/>
+  <dimension ref="A1:AB114"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -28785,7 +28787,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -28806,7 +28808,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>130</v>
@@ -28868,7 +28870,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>146</v>
       </c>
@@ -28926,7 +28928,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -28966,7 +28968,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -28985,7 +28987,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -29021,7 +29023,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -29040,7 +29042,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -29076,7 +29078,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -29095,7 +29097,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -29133,7 +29135,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -29152,7 +29154,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -29192,7 +29194,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -29211,7 +29213,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -29251,7 +29253,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -29270,7 +29272,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -29303,7 +29305,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -29322,7 +29324,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -29355,7 +29357,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -29374,7 +29376,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -29405,7 +29407,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -29424,7 +29426,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -29461,7 +29463,7 @@
       </c>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -29480,7 +29482,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -29515,7 +29517,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -29534,7 +29536,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -29565,7 +29567,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -29584,7 +29586,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -29616,7 +29618,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -29635,7 +29637,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -29673,7 +29675,7 @@
       </c>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -29692,7 +29694,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -29721,7 +29723,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -29740,7 +29742,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -29771,7 +29773,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -29790,7 +29792,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -29827,7 +29829,7 @@
       </c>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -29846,7 +29848,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -29882,7 +29884,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -29901,7 +29903,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -29942,7 +29944,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -29961,7 +29963,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -29991,7 +29993,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -30010,7 +30012,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -30050,7 +30052,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -30069,7 +30071,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -30098,7 +30100,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -30117,7 +30119,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -30152,7 +30154,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -30171,7 +30173,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -30206,7 +30208,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -30225,7 +30227,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -30261,7 +30263,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -30280,7 +30282,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -30318,7 +30320,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -30337,7 +30339,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -30375,7 +30377,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -30394,7 +30396,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -30429,7 +30431,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -30448,7 +30450,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -30467,7 +30469,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -30486,7 +30488,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -30507,7 +30509,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -30526,7 +30528,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -30563,7 +30565,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -30582,7 +30584,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -30621,7 +30623,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <v>9437</v>
       </c>
@@ -30658,7 +30660,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="19">
         <v>7480</v>
       </c>
@@ -30693,7 +30695,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="19">
         <v>8829</v>
       </c>
@@ -30726,7 +30728,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="19">
         <v>8386</v>
       </c>
@@ -30761,7 +30763,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="19">
         <v>8530</v>
       </c>
@@ -30794,7 +30796,7 @@
       </c>
       <c r="Q71" s="54"/>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="143"/>
       <c r="C72" s="35"/>
@@ -30813,7 +30815,7 @@
       <c r="P72" s="35"/>
       <c r="Q72" s="144"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="143"/>
       <c r="C73" s="35"/>
@@ -30832,7 +30834,7 @@
       <c r="P73" s="35"/>
       <c r="Q73" s="144"/>
     </row>
-    <row r="74" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="145"/>
       <c r="B74" s="145"/>
       <c r="C74" s="145"/>
@@ -30851,7 +30853,7 @@
       <c r="P74" s="145"/>
       <c r="Q74" s="145"/>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="146" t="s">
         <v>150</v>
@@ -30896,7 +30898,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="77" t="s">
         <v>151</v>
@@ -30935,7 +30937,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="77" t="s">
         <v>152</v>
@@ -30964,7 +30966,7 @@
       <c r="P77" s="20"/>
       <c r="Q77" s="20"/>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="142"/>
       <c r="B78" s="148" t="s">
         <v>153</v>
@@ -31009,7 +31011,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="142"/>
       <c r="B79" s="151" t="s">
         <v>154</v>
@@ -31054,7 +31056,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="142"/>
       <c r="B80" s="35"/>
       <c r="C80" s="35"/>
@@ -31073,7 +31075,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="144"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="142"/>
       <c r="B81" s="156" t="s">
         <v>155</v>
@@ -31120,7 +31122,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="161"/>
       <c r="B82" s="162" t="s">
         <v>157</v>
@@ -31165,7 +31167,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="83" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="35"/>
       <c r="C83" s="35"/>
@@ -31184,7 +31186,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="164" t="s">
         <v>158</v>
@@ -31207,7 +31209,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="167" t="s">
         <v>160</v>
@@ -31230,7 +31232,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>161</v>
@@ -31253,7 +31255,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>162</v>
@@ -31276,7 +31278,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>163</v>
@@ -31299,7 +31301,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>164</v>
@@ -31322,7 +31324,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>165</v>
@@ -31345,7 +31347,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>166</v>
@@ -31368,7 +31370,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19" t="s">
         <v>167</v>
@@ -31391,7 +31393,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19" t="s">
         <v>168</v>
@@ -31414,7 +31416,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19" t="s">
         <v>169</v>
@@ -31437,7 +31439,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19" t="s">
         <v>170</v>
@@ -31460,7 +31462,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -31481,7 +31483,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -31502,7 +31504,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -31523,7 +31525,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19"/>
       <c r="C99" s="131">
@@ -31544,7 +31546,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19"/>
       <c r="C100" s="131">
@@ -31565,7 +31567,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19"/>
       <c r="C101" s="131">
@@ -31586,7 +31588,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19"/>
       <c r="C102" s="131">
@@ -31607,7 +31609,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>171</v>
@@ -31630,7 +31632,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>172</v>
@@ -31653,7 +31655,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>173</v>
@@ -31676,7 +31678,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19" t="s">
         <v>174</v>
@@ -31699,7 +31701,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19" t="s">
         <v>175</v>
@@ -31722,7 +31724,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19" t="s">
         <v>176</v>
@@ -31745,7 +31747,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="19" t="s">
         <v>177</v>
@@ -31768,7 +31770,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="19"/>
       <c r="C110" s="131"/>
@@ -31787,7 +31789,7 @@
       <c r="P110" s="35"/>
       <c r="Q110" s="35"/>
     </row>
-    <row r="111" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="111" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A111" s="35"/>
       <c r="B111" s="19"/>
       <c r="C111" s="131"/>
@@ -31806,7 +31808,7 @@
       <c r="P111" s="35"/>
       <c r="Q111" s="35"/>
     </row>
-    <row r="112" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="112" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A112" s="35"/>
       <c r="B112" s="19"/>
       <c r="C112" s="131"/>
@@ -31825,7 +31827,7 @@
       <c r="P112" s="35"/>
       <c r="Q112" s="35"/>
     </row>
-    <row r="113" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="113" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A113" s="35"/>
       <c r="B113" s="169"/>
       <c r="C113" s="150"/>
@@ -31844,7 +31846,7 @@
       <c r="P113" s="35"/>
       <c r="Q113" s="35"/>
     </row>
-    <row r="114" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="114" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A114" s="35"/>
       <c r="B114" s="164" t="s">
         <v>178</v>
@@ -31918,11 +31920,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>179</v>
       </c>
@@ -31954,7 +31955,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>180</v>
       </c>
@@ -31987,7 +31988,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>181</v>
       </c>
@@ -32020,7 +32021,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>182</v>
       </c>
@@ -32053,7 +32054,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>183</v>
       </c>
@@ -32086,7 +32087,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>184</v>
       </c>
@@ -32119,7 +32120,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>185</v>
       </c>
@@ -32152,7 +32153,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>186</v>
       </c>
@@ -32185,7 +32186,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -32216,7 +32217,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -32247,7 +32248,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>187</v>
       </c>
@@ -32280,7 +32281,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>188</v>
       </c>
@@ -32313,7 +32314,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>189</v>
       </c>
@@ -32346,7 +32347,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>190</v>
       </c>
@@ -32379,7 +32380,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>191</v>
       </c>
@@ -32412,7 +32413,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>192</v>
       </c>
@@ -32445,7 +32446,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>193</v>
       </c>
@@ -32478,7 +32479,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>194</v>
       </c>
@@ -32511,7 +32512,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>195</v>
       </c>
@@ -32544,7 +32545,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>196</v>
       </c>
@@ -32577,7 +32578,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>197</v>
       </c>
@@ -32610,7 +32611,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>198</v>
       </c>
@@ -32643,7 +32644,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>199</v>
       </c>
@@ -32676,7 +32677,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>200</v>
       </c>
@@ -32709,7 +32710,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>201</v>
       </c>
@@ -32742,7 +32743,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>202</v>
       </c>
@@ -32775,7 +32776,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>203</v>
       </c>
@@ -32807,7 +32808,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>204</v>
       </c>
@@ -32839,7 +32840,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>205</v>
       </c>
@@ -32871,7 +32872,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>206</v>
       </c>
@@ -32903,7 +32904,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>207</v>
       </c>
@@ -32935,7 +32936,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -32965,7 +32966,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -32995,7 +32996,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>208</v>
       </c>
@@ -33027,7 +33028,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>209</v>
       </c>
@@ -33059,7 +33060,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>210</v>
       </c>
@@ -33091,7 +33092,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>211</v>
       </c>
@@ -33123,7 +33124,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>212</v>
       </c>
@@ -33155,7 +33156,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -33185,7 +33186,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>213</v>
       </c>
@@ -33217,7 +33218,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>214</v>
       </c>
@@ -33249,7 +33250,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>215</v>
       </c>
@@ -33281,7 +33282,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>216</v>
       </c>
@@ -33313,7 +33314,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -33343,7 +33344,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -33373,7 +33374,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -33403,7 +33404,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -33433,7 +33434,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>217</v>
       </c>
@@ -33465,7 +33466,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>218</v>
       </c>
@@ -33497,7 +33498,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -33527,7 +33528,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -33557,7 +33558,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -33587,7 +33588,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -33617,7 +33618,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -33647,7 +33648,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -33742,11 +33743,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>219</v>
       </c>
@@ -33778,7 +33778,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -33809,7 +33809,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -33840,7 +33840,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -33871,7 +33871,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -33902,7 +33902,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -33933,7 +33933,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -33964,7 +33964,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -33995,7 +33995,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -34026,7 +34026,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -34057,7 +34057,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -34088,7 +34088,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -34119,7 +34119,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -34150,7 +34150,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -34181,7 +34181,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -34212,7 +34212,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -34243,7 +34243,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -34274,7 +34274,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -34305,7 +34305,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -34336,7 +34336,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -34367,7 +34367,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -34397,7 +34397,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -34427,7 +34427,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -34457,7 +34457,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -34487,7 +34487,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -34517,7 +34517,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -34547,7 +34547,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -34577,7 +34577,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -34607,7 +34607,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -34637,7 +34637,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -34667,7 +34667,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -34697,7 +34697,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -34727,7 +34727,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -34757,7 +34757,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -34787,7 +34787,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -34817,7 +34817,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -34847,7 +34847,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>217</v>
       </c>
@@ -34879,7 +34879,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>218</v>
       </c>
@@ -34911,7 +34911,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -34941,7 +34941,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -34971,7 +34971,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -35001,7 +35001,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -35031,7 +35031,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -35061,7 +35061,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -56804,19 +56804,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -56830,7 +56830,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>226</v>
       </c>
@@ -56842,7 +56842,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>227</v>
       </c>
@@ -56853,7 +56853,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>228</v>
       </c>
@@ -56864,7 +56864,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>229</v>
       </c>
@@ -56875,13 +56875,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Sync data files (2026-09-16T22:47:52Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1186" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1187" uniqueCount="230">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -7617,7 +7617,9 @@
         <v>33</v>
       </c>
       <c r="P52" s="18"/>
-      <c r="Q52" s="15"/>
+      <c r="Q52" s="15" t="s">
+        <v>30</v>
+      </c>
       <c r="R52" s="13"/>
       <c r="S52" s="13"/>
       <c r="T52" s="16"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-16T22:52:05Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -18147,7 +18147,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>100</v>
@@ -26150,7 +26150,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R75"/>
+  <dimension ref="A1:AD75"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -26164,7 +26164,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -26186,7 +26186,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>105</v>
       </c>
@@ -26234,7 +26234,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -26252,7 +26252,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -26299,7 +26299,7 @@
         <v>-100.50142857142866</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -26316,7 +26316,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -26366,7 +26366,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -26383,7 +26383,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -26426,7 +26426,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -26443,7 +26443,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -26490,7 +26490,7 @@
         <v>27.80091109478323</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -26507,7 +26507,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -26557,7 +26557,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -26574,7 +26574,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -26621,7 +26621,7 @@
         <v>110.61624999999997</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -26638,7 +26638,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -26683,7 +26683,7 @@
         <v>40.952161383285286</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -26700,7 +26700,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -26750,7 +26750,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -26767,7 +26767,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -26806,7 +26806,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -26823,7 +26823,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -26864,7 +26864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -26881,7 +26881,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -26920,7 +26920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -26937,7 +26937,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -26982,7 +26982,7 @@
         <v>-3.0733682373472964</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -26999,7 +26999,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -27042,7 +27042,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -27059,7 +27059,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -27102,7 +27102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -27119,7 +27119,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -27166,7 +27166,7 @@
         <v>13.90219151036525</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -27183,7 +27183,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -27228,7 +27228,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -27245,7 +27245,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -27288,7 +27288,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -27305,7 +27305,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -27346,7 +27346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -27363,7 +27363,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -27408,7 +27408,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -27425,7 +27425,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -27468,7 +27468,7 @@
         <v>-0.05012183692595682</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -27485,7 +27485,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -27522,7 +27522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -27539,7 +27539,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27580,7 +27580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -27597,7 +27597,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -27640,7 +27640,7 @@
         <v>95.15307262569829</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -27657,7 +27657,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -27699,7 +27699,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -27716,7 +27716,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -27761,7 +27761,7 @@
         <v>14.869587534372164</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -27778,7 +27778,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -27823,7 +27823,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -27840,7 +27840,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -27885,7 +27885,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -27902,7 +27902,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -27939,7 +27939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -27956,7 +27956,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -27973,7 +27973,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -27990,7 +27990,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -28011,7 +28011,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -28028,7 +28028,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -28069,7 +28069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -28086,7 +28086,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -28131,7 +28131,7 @@
         <v>-15.917709392560841</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <v>9437</v>
       </c>
@@ -28170,7 +28170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="102">
         <v>7480</v>
       </c>
@@ -28209,7 +28209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="102">
         <v>8829</v>
       </c>
@@ -28248,7 +28248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="102">
         <v>8386</v>
       </c>
@@ -28287,7 +28287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="102">
         <v>8530</v>
       </c>
@@ -28326,7 +28326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="35"/>
       <c r="B72" s="35"/>
       <c r="C72" s="36"/>
@@ -28343,7 +28343,7 @@
       <c r="N72" s="35"/>
       <c r="O72" s="36"/>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="35"/>
       <c r="B73" s="35"/>
       <c r="C73" s="36"/>
@@ -28360,7 +28360,7 @@
       <c r="N73" s="35"/>
       <c r="O73" s="35"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="49" t="s">
         <v>125</v>
       </c>
@@ -28395,7 +28395,7 @@
       <c r="N74" s="35"/>
       <c r="O74" s="35"/>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="59"/>
       <c r="B75" s="98" t="s">
         <v>129</v>
@@ -28778,7 +28778,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB114"/>
+  <dimension ref="A1:AD114"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -28789,7 +28789,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -28810,7 +28810,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>130</v>
@@ -28872,7 +28872,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>146</v>
       </c>
@@ -28930,7 +28930,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -28970,7 +28970,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -28989,7 +28989,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -29025,7 +29025,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -29044,7 +29044,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -29080,7 +29080,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -29099,7 +29099,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -29137,7 +29137,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -29156,7 +29156,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -29196,7 +29196,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -29215,7 +29215,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -29255,7 +29255,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -29274,7 +29274,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -29307,7 +29307,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -29326,7 +29326,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -29359,7 +29359,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -29378,7 +29378,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -29409,7 +29409,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -29428,7 +29428,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -29465,7 +29465,7 @@
       </c>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -29484,7 +29484,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -29519,7 +29519,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -29538,7 +29538,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -29569,7 +29569,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -29588,7 +29588,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -29620,7 +29620,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -29639,7 +29639,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -29677,7 +29677,7 @@
       </c>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -29696,7 +29696,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -29725,7 +29725,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -29744,7 +29744,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -29775,7 +29775,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -29794,7 +29794,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -29831,7 +29831,7 @@
       </c>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -29850,7 +29850,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -29886,7 +29886,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -29905,7 +29905,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -29946,7 +29946,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -29965,7 +29965,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -29995,7 +29995,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -30014,7 +30014,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -30054,7 +30054,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -30073,7 +30073,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -30102,7 +30102,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -30121,7 +30121,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -30156,7 +30156,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -30175,7 +30175,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -30210,7 +30210,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -30229,7 +30229,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -30265,7 +30265,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -30284,7 +30284,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -30322,7 +30322,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -30341,7 +30341,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -30379,7 +30379,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -30398,7 +30398,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -30433,7 +30433,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -30452,7 +30452,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -30471,7 +30471,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -30490,7 +30490,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -30511,7 +30511,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -30530,7 +30530,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -30567,7 +30567,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -30586,7 +30586,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -30625,7 +30625,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <v>9437</v>
       </c>
@@ -30662,7 +30662,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="19">
         <v>7480</v>
       </c>
@@ -30697,7 +30697,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="19">
         <v>8829</v>
       </c>
@@ -30730,7 +30730,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="19">
         <v>8386</v>
       </c>
@@ -30765,7 +30765,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="19">
         <v>8530</v>
       </c>
@@ -30798,7 +30798,7 @@
       </c>
       <c r="Q71" s="54"/>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="143"/>
       <c r="C72" s="35"/>
@@ -30817,7 +30817,7 @@
       <c r="P72" s="35"/>
       <c r="Q72" s="144"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="143"/>
       <c r="C73" s="35"/>
@@ -30836,7 +30836,7 @@
       <c r="P73" s="35"/>
       <c r="Q73" s="144"/>
     </row>
-    <row r="74" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="145"/>
       <c r="B74" s="145"/>
       <c r="C74" s="145"/>
@@ -30855,7 +30855,7 @@
       <c r="P74" s="145"/>
       <c r="Q74" s="145"/>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="146" t="s">
         <v>150</v>
@@ -30900,7 +30900,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="77" t="s">
         <v>151</v>
@@ -30939,7 +30939,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="77" t="s">
         <v>152</v>
@@ -30968,7 +30968,7 @@
       <c r="P77" s="20"/>
       <c r="Q77" s="20"/>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="142"/>
       <c r="B78" s="148" t="s">
         <v>153</v>
@@ -31013,7 +31013,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="142"/>
       <c r="B79" s="151" t="s">
         <v>154</v>
@@ -31058,7 +31058,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="142"/>
       <c r="B80" s="35"/>
       <c r="C80" s="35"/>
@@ -31077,7 +31077,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="144"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="142"/>
       <c r="B81" s="156" t="s">
         <v>155</v>
@@ -31124,7 +31124,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="161"/>
       <c r="B82" s="162" t="s">
         <v>157</v>
@@ -31169,7 +31169,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="35"/>
       <c r="C83" s="35"/>
@@ -31188,7 +31188,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="164" t="s">
         <v>158</v>
@@ -31211,7 +31211,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="167" t="s">
         <v>160</v>
@@ -31234,7 +31234,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>161</v>
@@ -31257,7 +31257,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>162</v>
@@ -31280,7 +31280,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>163</v>
@@ -31303,7 +31303,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>164</v>
@@ -31326,7 +31326,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>165</v>
@@ -31349,7 +31349,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>166</v>
@@ -31372,7 +31372,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19" t="s">
         <v>167</v>
@@ -31395,7 +31395,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19" t="s">
         <v>168</v>
@@ -31418,7 +31418,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19" t="s">
         <v>169</v>
@@ -31441,7 +31441,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19" t="s">
         <v>170</v>
@@ -31464,7 +31464,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -31485,7 +31485,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -31506,7 +31506,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -31527,7 +31527,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19"/>
       <c r="C99" s="131">
@@ -31548,7 +31548,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19"/>
       <c r="C100" s="131">
@@ -31569,7 +31569,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19"/>
       <c r="C101" s="131">
@@ -31590,7 +31590,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19"/>
       <c r="C102" s="131">
@@ -31611,7 +31611,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>171</v>
@@ -31634,7 +31634,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>172</v>
@@ -31657,7 +31657,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>173</v>
@@ -31680,7 +31680,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19" t="s">
         <v>174</v>
@@ -31703,7 +31703,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19" t="s">
         <v>175</v>
@@ -31726,7 +31726,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19" t="s">
         <v>176</v>
@@ -31749,7 +31749,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="19" t="s">
         <v>177</v>
@@ -31772,7 +31772,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="19"/>
       <c r="C110" s="131"/>
@@ -31791,7 +31791,7 @@
       <c r="P110" s="35"/>
       <c r="Q110" s="35"/>
     </row>
-    <row r="111" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="111" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A111" s="35"/>
       <c r="B111" s="19"/>
       <c r="C111" s="131"/>
@@ -31810,7 +31810,7 @@
       <c r="P111" s="35"/>
       <c r="Q111" s="35"/>
     </row>
-    <row r="112" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="112" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A112" s="35"/>
       <c r="B112" s="19"/>
       <c r="C112" s="131"/>
@@ -31829,7 +31829,7 @@
       <c r="P112" s="35"/>
       <c r="Q112" s="35"/>
     </row>
-    <row r="113" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="113" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A113" s="35"/>
       <c r="B113" s="169"/>
       <c r="C113" s="150"/>
@@ -31848,7 +31848,7 @@
       <c r="P113" s="35"/>
       <c r="Q113" s="35"/>
     </row>
-    <row r="114" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="114" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A114" s="35"/>
       <c r="B114" s="164" t="s">
         <v>178</v>
@@ -31922,10 +31922,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>179</v>
       </c>
@@ -31957,7 +31958,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>180</v>
       </c>
@@ -31990,7 +31991,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>181</v>
       </c>
@@ -32023,7 +32024,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>182</v>
       </c>
@@ -32056,7 +32057,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>183</v>
       </c>
@@ -32089,7 +32090,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>184</v>
       </c>
@@ -32122,7 +32123,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>185</v>
       </c>
@@ -32155,7 +32156,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>186</v>
       </c>
@@ -32188,7 +32189,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -32219,7 +32220,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -32250,7 +32251,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>187</v>
       </c>
@@ -32283,7 +32284,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>188</v>
       </c>
@@ -32316,7 +32317,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>189</v>
       </c>
@@ -32349,7 +32350,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>190</v>
       </c>
@@ -32382,7 +32383,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>191</v>
       </c>
@@ -32415,7 +32416,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>192</v>
       </c>
@@ -32448,7 +32449,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>193</v>
       </c>
@@ -32481,7 +32482,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>194</v>
       </c>
@@ -32514,7 +32515,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>195</v>
       </c>
@@ -32547,7 +32548,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>196</v>
       </c>
@@ -32580,7 +32581,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>197</v>
       </c>
@@ -32613,7 +32614,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>198</v>
       </c>
@@ -32646,7 +32647,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>199</v>
       </c>
@@ -32679,7 +32680,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>200</v>
       </c>
@@ -32712,7 +32713,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>201</v>
       </c>
@@ -32745,7 +32746,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>202</v>
       </c>
@@ -32778,7 +32779,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>203</v>
       </c>
@@ -32810,7 +32811,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>204</v>
       </c>
@@ -32842,7 +32843,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>205</v>
       </c>
@@ -32874,7 +32875,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>206</v>
       </c>
@@ -32906,7 +32907,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>207</v>
       </c>
@@ -32938,7 +32939,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -32968,7 +32969,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -32998,7 +32999,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>208</v>
       </c>
@@ -33030,7 +33031,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>209</v>
       </c>
@@ -33062,7 +33063,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>210</v>
       </c>
@@ -33094,7 +33095,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>211</v>
       </c>
@@ -33126,7 +33127,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>212</v>
       </c>
@@ -33158,7 +33159,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -33188,7 +33189,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>213</v>
       </c>
@@ -33220,7 +33221,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>214</v>
       </c>
@@ -33252,7 +33253,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>215</v>
       </c>
@@ -33284,7 +33285,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>216</v>
       </c>
@@ -33316,7 +33317,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -33346,7 +33347,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -33376,7 +33377,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -33406,7 +33407,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -33436,7 +33437,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>217</v>
       </c>
@@ -33468,7 +33469,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>218</v>
       </c>
@@ -33500,7 +33501,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -33530,7 +33531,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -33560,7 +33561,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -33590,7 +33591,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -33620,7 +33621,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -33650,7 +33651,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -33745,10 +33746,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>219</v>
       </c>
@@ -33780,7 +33782,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -33811,7 +33813,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -33842,7 +33844,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -33873,7 +33875,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -33904,7 +33906,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -33935,7 +33937,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -33966,7 +33968,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -33997,7 +33999,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -34028,7 +34030,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -34059,7 +34061,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -34090,7 +34092,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -34121,7 +34123,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -34152,7 +34154,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -34183,7 +34185,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -34214,7 +34216,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -34245,7 +34247,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -34276,7 +34278,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -34307,7 +34309,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -34338,7 +34340,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -34369,7 +34371,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -34399,7 +34401,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -34429,7 +34431,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -34459,7 +34461,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -34489,7 +34491,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -34519,7 +34521,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -34549,7 +34551,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -34579,7 +34581,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -34609,7 +34611,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -34639,7 +34641,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -34669,7 +34671,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -34699,7 +34701,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -34729,7 +34731,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -34759,7 +34761,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -34789,7 +34791,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -34819,7 +34821,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -34849,7 +34851,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>217</v>
       </c>
@@ -34881,7 +34883,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>218</v>
       </c>
@@ -34913,7 +34915,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -34943,7 +34945,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -34973,7 +34975,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -35003,7 +35005,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -35033,7 +35035,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -35063,7 +35065,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -56806,19 +56808,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -56832,7 +56834,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>226</v>
       </c>
@@ -56844,7 +56846,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>227</v>
       </c>
@@ -56855,7 +56857,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>228</v>
       </c>
@@ -56866,7 +56868,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>229</v>
       </c>
@@ -56877,13 +56879,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Sync data files (2026-09-17T00:12:51Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1187" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1188" uniqueCount="230">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -7067,7 +7067,9 @@
       <c r="B38" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="C38" s="13"/>
+      <c r="C38" s="13" t="s">
+        <v>42</v>
+      </c>
       <c r="D38" s="13"/>
       <c r="E38" s="13"/>
       <c r="F38" s="13"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-17T00:21:02Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1189" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1191" uniqueCount="231">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -7002,7 +7002,9 @@
       <c r="B36" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="C36" s="13"/>
+      <c r="C36" s="13" t="s">
+        <v>42</v>
+      </c>
       <c r="D36" s="13"/>
       <c r="E36" s="13"/>
       <c r="F36" s="13"/>
@@ -7140,7 +7142,9 @@
       <c r="B40" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="C40" s="13"/>
+      <c r="C40" s="13" t="s">
+        <v>42</v>
+      </c>
       <c r="D40" s="13"/>
       <c r="E40" s="13"/>
       <c r="F40" s="13"/>
@@ -8383,7 +8387,7 @@
         <v>66</v>
       </c>
       <c r="C72" s="29" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D72" s="29"/>
       <c r="E72" s="13"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-21T21:24:49Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -18158,7 +18158,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>101</v>
@@ -26161,7 +26161,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R75"/>
+  <dimension ref="A1:AD75"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -26175,7 +26175,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -26197,7 +26197,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>106</v>
       </c>
@@ -26245,7 +26245,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -26263,7 +26263,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -26310,7 +26310,7 @@
         <v>-100.50142857142866</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -26327,7 +26327,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -26377,7 +26377,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -26394,7 +26394,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -26437,7 +26437,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -26454,7 +26454,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -26501,7 +26501,7 @@
         <v>27.80091109478323</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -26518,7 +26518,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -26568,7 +26568,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -26585,7 +26585,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -26632,7 +26632,7 @@
         <v>110.61624999999997</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -26649,7 +26649,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -26694,7 +26694,7 @@
         <v>40.952161383285286</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -26711,7 +26711,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -26761,7 +26761,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -26778,7 +26778,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -26817,7 +26817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -26834,7 +26834,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -26875,7 +26875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -26892,7 +26892,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -26931,7 +26931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -26948,7 +26948,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -26993,7 +26993,7 @@
         <v>-3.0733682373472964</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -27010,7 +27010,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -27053,7 +27053,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -27070,7 +27070,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -27113,7 +27113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -27130,7 +27130,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -27177,7 +27177,7 @@
         <v>13.90219151036525</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -27194,7 +27194,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -27239,7 +27239,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -27256,7 +27256,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -27299,7 +27299,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -27316,7 +27316,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -27357,7 +27357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -27374,7 +27374,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -27419,7 +27419,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -27436,7 +27436,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -27479,7 +27479,7 @@
         <v>-0.05012183692595682</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -27496,7 +27496,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -27533,7 +27533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -27550,7 +27550,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27591,7 +27591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -27608,7 +27608,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -27651,7 +27651,7 @@
         <v>95.15307262569829</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -27668,7 +27668,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -27710,7 +27710,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -27727,7 +27727,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -27772,7 +27772,7 @@
         <v>14.869587534372164</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -27789,7 +27789,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -27834,7 +27834,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -27851,7 +27851,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -27896,7 +27896,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -27913,7 +27913,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -27950,7 +27950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -27967,7 +27967,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -27984,7 +27984,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -28001,7 +28001,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -28022,7 +28022,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -28039,7 +28039,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -28080,7 +28080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -28097,7 +28097,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -28142,7 +28142,7 @@
         <v>-15.917709392560841</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <v>9437</v>
       </c>
@@ -28181,7 +28181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="102">
         <v>7480</v>
       </c>
@@ -28220,7 +28220,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="102">
         <v>8829</v>
       </c>
@@ -28259,7 +28259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="102">
         <v>8386</v>
       </c>
@@ -28298,7 +28298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="102">
         <v>8530</v>
       </c>
@@ -28337,7 +28337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="35"/>
       <c r="B72" s="35"/>
       <c r="C72" s="36"/>
@@ -28354,7 +28354,7 @@
       <c r="N72" s="35"/>
       <c r="O72" s="36"/>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="35"/>
       <c r="B73" s="35"/>
       <c r="C73" s="36"/>
@@ -28371,7 +28371,7 @@
       <c r="N73" s="35"/>
       <c r="O73" s="35"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="49" t="s">
         <v>126</v>
       </c>
@@ -28406,7 +28406,7 @@
       <c r="N74" s="35"/>
       <c r="O74" s="35"/>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="59"/>
       <c r="B75" s="98" t="s">
         <v>130</v>
@@ -28789,7 +28789,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB114"/>
+  <dimension ref="A1:AD114"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -28800,7 +28800,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -28821,7 +28821,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>131</v>
@@ -28883,7 +28883,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>147</v>
       </c>
@@ -28941,7 +28941,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -28981,7 +28981,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -29000,7 +29000,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -29036,7 +29036,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -29055,7 +29055,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -29091,7 +29091,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -29110,7 +29110,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -29148,7 +29148,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -29167,7 +29167,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -29207,7 +29207,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -29226,7 +29226,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -29266,7 +29266,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -29285,7 +29285,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -29318,7 +29318,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -29337,7 +29337,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -29370,7 +29370,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -29389,7 +29389,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -29420,7 +29420,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -29439,7 +29439,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -29476,7 +29476,7 @@
       </c>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -29495,7 +29495,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -29530,7 +29530,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -29549,7 +29549,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -29580,7 +29580,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -29599,7 +29599,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -29631,7 +29631,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -29650,7 +29650,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -29688,7 +29688,7 @@
       </c>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -29707,7 +29707,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -29736,7 +29736,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -29755,7 +29755,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -29786,7 +29786,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -29805,7 +29805,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -29842,7 +29842,7 @@
       </c>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -29861,7 +29861,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -29897,7 +29897,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -29916,7 +29916,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -29957,7 +29957,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -29976,7 +29976,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -30006,7 +30006,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -30025,7 +30025,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -30065,7 +30065,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -30084,7 +30084,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -30113,7 +30113,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -30132,7 +30132,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -30167,7 +30167,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -30186,7 +30186,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -30221,7 +30221,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -30240,7 +30240,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -30276,7 +30276,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -30295,7 +30295,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -30333,7 +30333,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -30352,7 +30352,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -30390,7 +30390,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -30409,7 +30409,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -30444,7 +30444,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -30463,7 +30463,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -30482,7 +30482,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -30501,7 +30501,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -30522,7 +30522,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -30541,7 +30541,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -30578,7 +30578,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -30597,7 +30597,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -30636,7 +30636,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <v>9437</v>
       </c>
@@ -30673,7 +30673,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="19">
         <v>7480</v>
       </c>
@@ -30708,7 +30708,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="19">
         <v>8829</v>
       </c>
@@ -30741,7 +30741,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="19">
         <v>8386</v>
       </c>
@@ -30776,7 +30776,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="19">
         <v>8530</v>
       </c>
@@ -30809,7 +30809,7 @@
       </c>
       <c r="Q71" s="54"/>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="143"/>
       <c r="C72" s="35"/>
@@ -30828,7 +30828,7 @@
       <c r="P72" s="35"/>
       <c r="Q72" s="144"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="143"/>
       <c r="C73" s="35"/>
@@ -30847,7 +30847,7 @@
       <c r="P73" s="35"/>
       <c r="Q73" s="144"/>
     </row>
-    <row r="74" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="145"/>
       <c r="B74" s="145"/>
       <c r="C74" s="145"/>
@@ -30866,7 +30866,7 @@
       <c r="P74" s="145"/>
       <c r="Q74" s="145"/>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="146" t="s">
         <v>151</v>
@@ -30911,7 +30911,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="77" t="s">
         <v>152</v>
@@ -30950,7 +30950,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="77" t="s">
         <v>153</v>
@@ -30979,7 +30979,7 @@
       <c r="P77" s="20"/>
       <c r="Q77" s="20"/>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="142"/>
       <c r="B78" s="148" t="s">
         <v>154</v>
@@ -31024,7 +31024,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="142"/>
       <c r="B79" s="151" t="s">
         <v>155</v>
@@ -31069,7 +31069,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="142"/>
       <c r="B80" s="35"/>
       <c r="C80" s="35"/>
@@ -31088,7 +31088,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="144"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="142"/>
       <c r="B81" s="156" t="s">
         <v>156</v>
@@ -31135,7 +31135,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="161"/>
       <c r="B82" s="162" t="s">
         <v>158</v>
@@ -31180,7 +31180,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="35"/>
       <c r="C83" s="35"/>
@@ -31199,7 +31199,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="164" t="s">
         <v>159</v>
@@ -31222,7 +31222,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="167" t="s">
         <v>161</v>
@@ -31245,7 +31245,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -31268,7 +31268,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -31291,7 +31291,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -31314,7 +31314,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -31337,7 +31337,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -31360,7 +31360,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>167</v>
@@ -31383,7 +31383,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19" t="s">
         <v>168</v>
@@ -31406,7 +31406,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19" t="s">
         <v>169</v>
@@ -31429,7 +31429,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19" t="s">
         <v>170</v>
@@ -31452,7 +31452,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19" t="s">
         <v>171</v>
@@ -31475,7 +31475,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -31496,7 +31496,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -31517,7 +31517,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -31538,7 +31538,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19"/>
       <c r="C99" s="131">
@@ -31559,7 +31559,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19"/>
       <c r="C100" s="131">
@@ -31580,7 +31580,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19"/>
       <c r="C101" s="131">
@@ -31601,7 +31601,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19"/>
       <c r="C102" s="131">
@@ -31622,7 +31622,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -31645,7 +31645,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -31668,7 +31668,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>174</v>
@@ -31691,7 +31691,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19" t="s">
         <v>175</v>
@@ -31714,7 +31714,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19" t="s">
         <v>176</v>
@@ -31737,7 +31737,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19" t="s">
         <v>177</v>
@@ -31760,7 +31760,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="19" t="s">
         <v>178</v>
@@ -31783,7 +31783,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="19"/>
       <c r="C110" s="131"/>
@@ -31802,7 +31802,7 @@
       <c r="P110" s="35"/>
       <c r="Q110" s="35"/>
     </row>
-    <row r="111" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="111" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A111" s="35"/>
       <c r="B111" s="19"/>
       <c r="C111" s="131"/>
@@ -31821,7 +31821,7 @@
       <c r="P111" s="35"/>
       <c r="Q111" s="35"/>
     </row>
-    <row r="112" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="112" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A112" s="35"/>
       <c r="B112" s="19"/>
       <c r="C112" s="131"/>
@@ -31840,7 +31840,7 @@
       <c r="P112" s="35"/>
       <c r="Q112" s="35"/>
     </row>
-    <row r="113" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="113" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A113" s="35"/>
       <c r="B113" s="169"/>
       <c r="C113" s="150"/>
@@ -31859,7 +31859,7 @@
       <c r="P113" s="35"/>
       <c r="Q113" s="35"/>
     </row>
-    <row r="114" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="114" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A114" s="35"/>
       <c r="B114" s="164" t="s">
         <v>179</v>
@@ -31933,10 +31933,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>180</v>
       </c>
@@ -31968,7 +31969,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>181</v>
       </c>
@@ -32001,7 +32002,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>182</v>
       </c>
@@ -32034,7 +32035,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>183</v>
       </c>
@@ -32067,7 +32068,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>184</v>
       </c>
@@ -32100,7 +32101,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>185</v>
       </c>
@@ -32133,7 +32134,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>186</v>
       </c>
@@ -32166,7 +32167,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>187</v>
       </c>
@@ -32199,7 +32200,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -32230,7 +32231,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -32261,7 +32262,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>188</v>
       </c>
@@ -32294,7 +32295,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>189</v>
       </c>
@@ -32327,7 +32328,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>190</v>
       </c>
@@ -32360,7 +32361,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>191</v>
       </c>
@@ -32393,7 +32394,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>192</v>
       </c>
@@ -32426,7 +32427,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>193</v>
       </c>
@@ -32459,7 +32460,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>194</v>
       </c>
@@ -32492,7 +32493,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>195</v>
       </c>
@@ -32525,7 +32526,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>196</v>
       </c>
@@ -32558,7 +32559,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>197</v>
       </c>
@@ -32591,7 +32592,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>198</v>
       </c>
@@ -32624,7 +32625,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>199</v>
       </c>
@@ -32657,7 +32658,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>200</v>
       </c>
@@ -32690,7 +32691,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>201</v>
       </c>
@@ -32723,7 +32724,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>202</v>
       </c>
@@ -32756,7 +32757,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>203</v>
       </c>
@@ -32789,7 +32790,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>204</v>
       </c>
@@ -32821,7 +32822,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>205</v>
       </c>
@@ -32853,7 +32854,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>206</v>
       </c>
@@ -32885,7 +32886,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>207</v>
       </c>
@@ -32917,7 +32918,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>208</v>
       </c>
@@ -32949,7 +32950,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -32979,7 +32980,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -33009,7 +33010,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>209</v>
       </c>
@@ -33041,7 +33042,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>210</v>
       </c>
@@ -33073,7 +33074,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>211</v>
       </c>
@@ -33105,7 +33106,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>212</v>
       </c>
@@ -33137,7 +33138,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>213</v>
       </c>
@@ -33169,7 +33170,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -33199,7 +33200,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>214</v>
       </c>
@@ -33231,7 +33232,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>215</v>
       </c>
@@ -33263,7 +33264,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>216</v>
       </c>
@@ -33295,7 +33296,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>217</v>
       </c>
@@ -33327,7 +33328,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -33357,7 +33358,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -33387,7 +33388,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -33417,7 +33418,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -33447,7 +33448,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>218</v>
       </c>
@@ -33479,7 +33480,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>219</v>
       </c>
@@ -33511,7 +33512,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -33541,7 +33542,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -33571,7 +33572,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -33601,7 +33602,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -33631,7 +33632,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -33661,7 +33662,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -33756,10 +33757,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>220</v>
       </c>
@@ -33791,7 +33793,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -33822,7 +33824,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -33853,7 +33855,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -33884,7 +33886,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -33915,7 +33917,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -33946,7 +33948,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -33977,7 +33979,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -34008,7 +34010,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -34039,7 +34041,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -34070,7 +34072,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -34101,7 +34103,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -34132,7 +34134,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -34163,7 +34165,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -34194,7 +34196,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -34225,7 +34227,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -34256,7 +34258,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -34287,7 +34289,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -34318,7 +34320,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -34349,7 +34351,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -34380,7 +34382,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -34410,7 +34412,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -34440,7 +34442,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -34470,7 +34472,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -34500,7 +34502,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -34530,7 +34532,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -34560,7 +34562,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -34590,7 +34592,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -34620,7 +34622,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -34650,7 +34652,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -34680,7 +34682,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -34710,7 +34712,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -34740,7 +34742,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -34770,7 +34772,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -34800,7 +34802,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -34830,7 +34832,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -34860,7 +34862,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>218</v>
       </c>
@@ -34892,7 +34894,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>219</v>
       </c>
@@ -34924,7 +34926,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -34954,7 +34956,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -34984,7 +34986,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -35014,7 +35016,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -35044,7 +35046,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -35074,7 +35076,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -56817,19 +56819,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -56843,7 +56845,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>227</v>
       </c>
@@ -56855,7 +56857,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>228</v>
       </c>
@@ -56866,7 +56868,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>229</v>
       </c>
@@ -56877,7 +56879,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>230</v>
       </c>
@@ -56888,13 +56890,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Sync data files (2026-09-21T21:25:58Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -18158,7 +18158,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>101</v>
@@ -26161,7 +26161,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R75"/>
+  <dimension ref="A1:AD75"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -26175,7 +26175,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -26197,7 +26197,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>106</v>
       </c>
@@ -26245,7 +26245,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -26263,7 +26263,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -26310,7 +26310,7 @@
         <v>-100.50142857142866</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -26327,7 +26327,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -26377,7 +26377,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -26394,7 +26394,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -26437,7 +26437,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -26454,7 +26454,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -26501,7 +26501,7 @@
         <v>27.80091109478323</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -26518,7 +26518,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -26568,7 +26568,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -26585,7 +26585,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -26632,7 +26632,7 @@
         <v>110.61624999999997</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -26649,7 +26649,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -26694,7 +26694,7 @@
         <v>40.952161383285286</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -26711,7 +26711,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -26761,7 +26761,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -26778,7 +26778,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -26817,7 +26817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -26834,7 +26834,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -26875,7 +26875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -26892,7 +26892,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -26931,7 +26931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -26948,7 +26948,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -26993,7 +26993,7 @@
         <v>-3.0733682373472964</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -27010,7 +27010,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -27053,7 +27053,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -27070,7 +27070,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -27113,7 +27113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -27130,7 +27130,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -27177,7 +27177,7 @@
         <v>13.90219151036525</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -27194,7 +27194,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -27239,7 +27239,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -27256,7 +27256,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -27299,7 +27299,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -27316,7 +27316,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -27357,7 +27357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -27374,7 +27374,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -27419,7 +27419,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -27436,7 +27436,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -27479,7 +27479,7 @@
         <v>-0.05012183692595682</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -27496,7 +27496,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -27533,7 +27533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -27550,7 +27550,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27591,7 +27591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -27608,7 +27608,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -27651,7 +27651,7 @@
         <v>95.15307262569829</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -27668,7 +27668,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -27710,7 +27710,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -27727,7 +27727,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -27772,7 +27772,7 @@
         <v>14.869587534372164</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -27789,7 +27789,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -27834,7 +27834,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -27851,7 +27851,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -27896,7 +27896,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -27913,7 +27913,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -27950,7 +27950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -27967,7 +27967,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -27984,7 +27984,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -28001,7 +28001,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -28022,7 +28022,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -28039,7 +28039,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -28080,7 +28080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -28097,7 +28097,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -28142,7 +28142,7 @@
         <v>-15.917709392560841</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <v>9437</v>
       </c>
@@ -28181,7 +28181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="102">
         <v>7480</v>
       </c>
@@ -28220,7 +28220,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="102">
         <v>8829</v>
       </c>
@@ -28259,7 +28259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="102">
         <v>8386</v>
       </c>
@@ -28298,7 +28298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="102">
         <v>8530</v>
       </c>
@@ -28337,7 +28337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="35"/>
       <c r="B72" s="35"/>
       <c r="C72" s="36"/>
@@ -28354,7 +28354,7 @@
       <c r="N72" s="35"/>
       <c r="O72" s="36"/>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="35"/>
       <c r="B73" s="35"/>
       <c r="C73" s="36"/>
@@ -28371,7 +28371,7 @@
       <c r="N73" s="35"/>
       <c r="O73" s="35"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="49" t="s">
         <v>126</v>
       </c>
@@ -28406,7 +28406,7 @@
       <c r="N74" s="35"/>
       <c r="O74" s="35"/>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="59"/>
       <c r="B75" s="98" t="s">
         <v>130</v>
@@ -28789,7 +28789,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB114"/>
+  <dimension ref="A1:AD114"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -28800,7 +28800,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -28821,7 +28821,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>131</v>
@@ -28883,7 +28883,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>147</v>
       </c>
@@ -28941,7 +28941,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -28981,7 +28981,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -29000,7 +29000,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -29036,7 +29036,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -29055,7 +29055,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -29091,7 +29091,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -29110,7 +29110,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -29148,7 +29148,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -29167,7 +29167,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -29207,7 +29207,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -29226,7 +29226,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -29266,7 +29266,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -29285,7 +29285,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -29318,7 +29318,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -29337,7 +29337,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -29370,7 +29370,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -29389,7 +29389,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -29420,7 +29420,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -29439,7 +29439,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -29476,7 +29476,7 @@
       </c>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -29495,7 +29495,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -29530,7 +29530,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -29549,7 +29549,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -29580,7 +29580,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -29599,7 +29599,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -29631,7 +29631,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -29650,7 +29650,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -29688,7 +29688,7 @@
       </c>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -29707,7 +29707,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -29736,7 +29736,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -29755,7 +29755,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -29786,7 +29786,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -29805,7 +29805,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -29842,7 +29842,7 @@
       </c>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -29861,7 +29861,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -29897,7 +29897,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -29916,7 +29916,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -29957,7 +29957,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -29976,7 +29976,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -30006,7 +30006,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -30025,7 +30025,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -30065,7 +30065,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -30084,7 +30084,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -30113,7 +30113,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -30132,7 +30132,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -30167,7 +30167,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -30186,7 +30186,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -30221,7 +30221,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -30240,7 +30240,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -30276,7 +30276,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -30295,7 +30295,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -30333,7 +30333,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -30352,7 +30352,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -30390,7 +30390,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -30409,7 +30409,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -30444,7 +30444,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -30463,7 +30463,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -30482,7 +30482,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -30501,7 +30501,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -30522,7 +30522,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -30541,7 +30541,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -30578,7 +30578,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -30597,7 +30597,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -30636,7 +30636,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <v>9437</v>
       </c>
@@ -30673,7 +30673,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="19">
         <v>7480</v>
       </c>
@@ -30708,7 +30708,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="19">
         <v>8829</v>
       </c>
@@ -30741,7 +30741,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="19">
         <v>8386</v>
       </c>
@@ -30776,7 +30776,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="19">
         <v>8530</v>
       </c>
@@ -30809,7 +30809,7 @@
       </c>
       <c r="Q71" s="54"/>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="143"/>
       <c r="C72" s="35"/>
@@ -30828,7 +30828,7 @@
       <c r="P72" s="35"/>
       <c r="Q72" s="144"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="143"/>
       <c r="C73" s="35"/>
@@ -30847,7 +30847,7 @@
       <c r="P73" s="35"/>
       <c r="Q73" s="144"/>
     </row>
-    <row r="74" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="145"/>
       <c r="B74" s="145"/>
       <c r="C74" s="145"/>
@@ -30866,7 +30866,7 @@
       <c r="P74" s="145"/>
       <c r="Q74" s="145"/>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="146" t="s">
         <v>151</v>
@@ -30911,7 +30911,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="77" t="s">
         <v>152</v>
@@ -30950,7 +30950,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="77" t="s">
         <v>153</v>
@@ -30979,7 +30979,7 @@
       <c r="P77" s="20"/>
       <c r="Q77" s="20"/>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="142"/>
       <c r="B78" s="148" t="s">
         <v>154</v>
@@ -31024,7 +31024,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="142"/>
       <c r="B79" s="151" t="s">
         <v>155</v>
@@ -31069,7 +31069,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="142"/>
       <c r="B80" s="35"/>
       <c r="C80" s="35"/>
@@ -31088,7 +31088,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="144"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="142"/>
       <c r="B81" s="156" t="s">
         <v>156</v>
@@ -31135,7 +31135,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="161"/>
       <c r="B82" s="162" t="s">
         <v>158</v>
@@ -31180,7 +31180,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="35"/>
       <c r="C83" s="35"/>
@@ -31199,7 +31199,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="164" t="s">
         <v>159</v>
@@ -31222,7 +31222,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="167" t="s">
         <v>161</v>
@@ -31245,7 +31245,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -31268,7 +31268,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -31291,7 +31291,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -31314,7 +31314,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -31337,7 +31337,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -31360,7 +31360,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>167</v>
@@ -31383,7 +31383,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19" t="s">
         <v>168</v>
@@ -31406,7 +31406,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19" t="s">
         <v>169</v>
@@ -31429,7 +31429,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19" t="s">
         <v>170</v>
@@ -31452,7 +31452,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19" t="s">
         <v>171</v>
@@ -31475,7 +31475,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -31496,7 +31496,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -31517,7 +31517,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -31538,7 +31538,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19"/>
       <c r="C99" s="131">
@@ -31559,7 +31559,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19"/>
       <c r="C100" s="131">
@@ -31580,7 +31580,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19"/>
       <c r="C101" s="131">
@@ -31601,7 +31601,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19"/>
       <c r="C102" s="131">
@@ -31622,7 +31622,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -31645,7 +31645,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -31668,7 +31668,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>174</v>
@@ -31691,7 +31691,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19" t="s">
         <v>175</v>
@@ -31714,7 +31714,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19" t="s">
         <v>176</v>
@@ -31737,7 +31737,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19" t="s">
         <v>177</v>
@@ -31760,7 +31760,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="19" t="s">
         <v>178</v>
@@ -31783,7 +31783,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="19"/>
       <c r="C110" s="131"/>
@@ -31802,7 +31802,7 @@
       <c r="P110" s="35"/>
       <c r="Q110" s="35"/>
     </row>
-    <row r="111" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="111" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A111" s="35"/>
       <c r="B111" s="19"/>
       <c r="C111" s="131"/>
@@ -31821,7 +31821,7 @@
       <c r="P111" s="35"/>
       <c r="Q111" s="35"/>
     </row>
-    <row r="112" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="112" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A112" s="35"/>
       <c r="B112" s="19"/>
       <c r="C112" s="131"/>
@@ -31840,7 +31840,7 @@
       <c r="P112" s="35"/>
       <c r="Q112" s="35"/>
     </row>
-    <row r="113" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="113" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A113" s="35"/>
       <c r="B113" s="169"/>
       <c r="C113" s="150"/>
@@ -31859,7 +31859,7 @@
       <c r="P113" s="35"/>
       <c r="Q113" s="35"/>
     </row>
-    <row r="114" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="114" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A114" s="35"/>
       <c r="B114" s="164" t="s">
         <v>179</v>
@@ -31933,10 +31933,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>180</v>
       </c>
@@ -31968,7 +31969,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>181</v>
       </c>
@@ -32001,7 +32002,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>182</v>
       </c>
@@ -32034,7 +32035,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>183</v>
       </c>
@@ -32067,7 +32068,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>184</v>
       </c>
@@ -32100,7 +32101,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>185</v>
       </c>
@@ -32133,7 +32134,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>186</v>
       </c>
@@ -32166,7 +32167,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>187</v>
       </c>
@@ -32199,7 +32200,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -32230,7 +32231,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -32261,7 +32262,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>188</v>
       </c>
@@ -32294,7 +32295,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>189</v>
       </c>
@@ -32327,7 +32328,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>190</v>
       </c>
@@ -32360,7 +32361,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>191</v>
       </c>
@@ -32393,7 +32394,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>192</v>
       </c>
@@ -32426,7 +32427,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>193</v>
       </c>
@@ -32459,7 +32460,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>194</v>
       </c>
@@ -32492,7 +32493,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>195</v>
       </c>
@@ -32525,7 +32526,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>196</v>
       </c>
@@ -32558,7 +32559,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>197</v>
       </c>
@@ -32591,7 +32592,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>198</v>
       </c>
@@ -32624,7 +32625,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>199</v>
       </c>
@@ -32657,7 +32658,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>200</v>
       </c>
@@ -32690,7 +32691,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>201</v>
       </c>
@@ -32723,7 +32724,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>202</v>
       </c>
@@ -32756,7 +32757,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>203</v>
       </c>
@@ -32789,7 +32790,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>204</v>
       </c>
@@ -32821,7 +32822,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>205</v>
       </c>
@@ -32853,7 +32854,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>206</v>
       </c>
@@ -32885,7 +32886,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>207</v>
       </c>
@@ -32917,7 +32918,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>208</v>
       </c>
@@ -32949,7 +32950,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -32979,7 +32980,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -33009,7 +33010,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>209</v>
       </c>
@@ -33041,7 +33042,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>210</v>
       </c>
@@ -33073,7 +33074,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>211</v>
       </c>
@@ -33105,7 +33106,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>212</v>
       </c>
@@ -33137,7 +33138,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>213</v>
       </c>
@@ -33169,7 +33170,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -33199,7 +33200,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>214</v>
       </c>
@@ -33231,7 +33232,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>215</v>
       </c>
@@ -33263,7 +33264,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>216</v>
       </c>
@@ -33295,7 +33296,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>217</v>
       </c>
@@ -33327,7 +33328,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -33357,7 +33358,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -33387,7 +33388,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -33417,7 +33418,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -33447,7 +33448,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>218</v>
       </c>
@@ -33479,7 +33480,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>219</v>
       </c>
@@ -33511,7 +33512,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -33541,7 +33542,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -33571,7 +33572,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -33601,7 +33602,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -33631,7 +33632,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -33661,7 +33662,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -33756,10 +33757,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>220</v>
       </c>
@@ -33791,7 +33793,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -33822,7 +33824,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -33853,7 +33855,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -33884,7 +33886,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -33915,7 +33917,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -33946,7 +33948,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -33977,7 +33979,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -34008,7 +34010,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -34039,7 +34041,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -34070,7 +34072,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -34101,7 +34103,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -34132,7 +34134,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -34163,7 +34165,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -34194,7 +34196,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -34225,7 +34227,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -34256,7 +34258,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -34287,7 +34289,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -34318,7 +34320,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -34349,7 +34351,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -34380,7 +34382,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -34410,7 +34412,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -34440,7 +34442,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -34470,7 +34472,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -34500,7 +34502,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -34530,7 +34532,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -34560,7 +34562,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -34590,7 +34592,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -34620,7 +34622,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -34650,7 +34652,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -34680,7 +34682,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -34710,7 +34712,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -34740,7 +34742,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -34770,7 +34772,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -34800,7 +34802,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -34830,7 +34832,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -34860,7 +34862,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>218</v>
       </c>
@@ -34892,7 +34894,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>219</v>
       </c>
@@ -34924,7 +34926,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -34954,7 +34956,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -34984,7 +34986,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -35014,7 +35016,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -35044,7 +35046,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -35074,7 +35076,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -56817,19 +56819,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -56843,7 +56845,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>227</v>
       </c>
@@ -56855,7 +56857,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>228</v>
       </c>
@@ -56866,7 +56868,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>229</v>
       </c>
@@ -56877,7 +56879,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>230</v>
       </c>
@@ -56888,13 +56890,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Sync data files (2026-09-21T22:02:39Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -10338,30 +10338,74 @@
       <c r="C8" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D8" s="52"/>
-      <c r="E8" s="52"/>
-      <c r="F8" s="52"/>
-      <c r="G8" s="53"/>
-      <c r="H8" s="52"/>
-      <c r="I8" s="52"/>
-      <c r="J8" s="52"/>
-      <c r="K8" s="52"/>
-      <c r="L8" s="52"/>
-      <c r="M8" s="53"/>
+      <c r="D8" s="52">
+        <v>267886.84883856</v>
+      </c>
+      <c r="E8" s="52">
+        <v>216530.08</v>
+      </c>
+      <c r="F8" s="52">
+        <v>51356.768838560005</v>
+      </c>
+      <c r="G8" s="53">
+        <v>0.19171067583653492</v>
+      </c>
+      <c r="H8" s="52">
+        <v>225410.5455298</v>
+      </c>
+      <c r="I8" s="52">
+        <v>168279</v>
+      </c>
+      <c r="J8" s="52">
+        <v>193787.2413298</v>
+      </c>
+      <c r="K8" s="52">
+        <v>138094.41999999998</v>
+      </c>
+      <c r="L8" s="52">
+        <v>55692.821329800005</v>
+      </c>
+      <c r="M8" s="53">
+        <v>0.2873915792785257</v>
+      </c>
       <c r="N8" s="53"/>
-      <c r="O8" s="52"/>
-      <c r="P8" s="52"/>
-      <c r="Q8" s="52"/>
-      <c r="R8" s="53"/>
-      <c r="S8" s="54"/>
-      <c r="T8" s="54"/>
-      <c r="U8" s="54"/>
-      <c r="V8" s="53"/>
+      <c r="O8" s="52">
+        <v>31623.3042</v>
+      </c>
+      <c r="P8" s="52">
+        <v>30184.58</v>
+      </c>
+      <c r="Q8" s="52">
+        <v>1438.724199999997</v>
+      </c>
+      <c r="R8" s="53">
+        <v>0.045495694912234916</v>
+      </c>
+      <c r="S8" s="54">
+        <v>638.02</v>
+      </c>
+      <c r="T8" s="54">
+        <v>605.75</v>
+      </c>
+      <c r="U8" s="54">
+        <v>32.26999999999998</v>
+      </c>
+      <c r="V8" s="53">
+        <v>0.05057835177580637</v>
+      </c>
       <c r="W8" s="53"/>
-      <c r="X8" s="55"/>
-      <c r="Y8" s="55"/>
-      <c r="Z8" s="53"/>
-      <c r="AA8" s="56"/>
+      <c r="X8" s="55">
+        <v>79.65510524143625</v>
+      </c>
+      <c r="Y8" s="55">
+        <v>66.57519091683645</v>
+      </c>
+      <c r="Z8" s="53">
+        <v>0.2228</v>
+      </c>
+      <c r="AA8" s="56">
+        <v>0.1586</v>
+      </c>
       <c r="AB8" s="57"/>
       <c r="AD8" s="35"/>
       <c r="AE8" s="35"/>
@@ -10789,30 +10833,74 @@
       <c r="C15" s="63" t="s">
         <v>103</v>
       </c>
-      <c r="D15" s="52"/>
-      <c r="E15" s="62"/>
-      <c r="F15" s="52"/>
-      <c r="G15" s="53"/>
-      <c r="H15" s="52"/>
-      <c r="I15" s="52"/>
-      <c r="J15" s="52"/>
-      <c r="K15" s="52"/>
-      <c r="L15" s="52"/>
-      <c r="M15" s="53"/>
+      <c r="D15" s="52">
+        <v>129996.91589078</v>
+      </c>
+      <c r="E15" s="62">
+        <v>85864.08</v>
+      </c>
+      <c r="F15" s="52">
+        <v>44132.83589078</v>
+      </c>
+      <c r="G15" s="53">
+        <v>0.3394914070719897</v>
+      </c>
+      <c r="H15" s="52">
+        <v>101885.523895</v>
+      </c>
+      <c r="I15" s="52">
+        <v>90641.75</v>
+      </c>
+      <c r="J15" s="52">
+        <v>83735.424895</v>
+      </c>
+      <c r="K15" s="52">
+        <v>80523.92</v>
+      </c>
+      <c r="L15" s="52">
+        <v>3211.5048950000055</v>
+      </c>
+      <c r="M15" s="53">
+        <v>0.03835300171972699</v>
+      </c>
       <c r="N15" s="53"/>
-      <c r="O15" s="52"/>
-      <c r="P15" s="52"/>
-      <c r="Q15" s="52"/>
-      <c r="R15" s="53"/>
-      <c r="S15" s="54"/>
-      <c r="T15" s="54"/>
-      <c r="U15" s="54"/>
-      <c r="V15" s="53"/>
+      <c r="O15" s="52">
+        <v>18150.099</v>
+      </c>
+      <c r="P15" s="52">
+        <v>10117.83</v>
+      </c>
+      <c r="Q15" s="52">
+        <v>8032.268999999998</v>
+      </c>
+      <c r="R15" s="53">
+        <v>0.44254684230647995</v>
+      </c>
+      <c r="S15" s="54">
+        <v>363.57</v>
+      </c>
+      <c r="T15" s="54">
+        <v>217</v>
+      </c>
+      <c r="U15" s="54">
+        <v>146.57</v>
+      </c>
+      <c r="V15" s="53">
+        <v>0.40314107324586734</v>
+      </c>
       <c r="W15" s="53"/>
-      <c r="X15" s="55"/>
-      <c r="Y15" s="55"/>
-      <c r="Z15" s="53"/>
-      <c r="AA15" s="56"/>
+      <c r="X15" s="55">
+        <v>-22.016912442396315</v>
+      </c>
+      <c r="Y15" s="55">
+        <v>77.32043896850674</v>
+      </c>
+      <c r="Z15" s="53">
+        <v>-0.0556</v>
+      </c>
+      <c r="AA15" s="56">
+        <v>0.2162</v>
+      </c>
       <c r="AB15" s="57"/>
       <c r="AD15" s="35"/>
       <c r="AE15" s="35"/>
@@ -11240,30 +11328,74 @@
       <c r="C22" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D22" s="52"/>
-      <c r="E22" s="52"/>
-      <c r="F22" s="52"/>
-      <c r="G22" s="53"/>
-      <c r="H22" s="52"/>
-      <c r="I22" s="52"/>
-      <c r="J22" s="52"/>
-      <c r="K22" s="52"/>
-      <c r="L22" s="52"/>
-      <c r="M22" s="53"/>
+      <c r="D22" s="52">
+        <v>27500.3157</v>
+      </c>
+      <c r="E22" s="52">
+        <v>11999.08</v>
+      </c>
+      <c r="F22" s="52">
+        <v>15501.2357</v>
+      </c>
+      <c r="G22" s="53">
+        <v>0.563674827194802</v>
+      </c>
+      <c r="H22" s="52">
+        <v>19565.829</v>
+      </c>
+      <c r="I22" s="52">
+        <v>8083.92</v>
+      </c>
+      <c r="J22" s="52">
+        <v>13767.337200000002</v>
+      </c>
+      <c r="K22" s="52">
+        <v>6373.24</v>
+      </c>
+      <c r="L22" s="52">
+        <v>7394.097200000002</v>
+      </c>
+      <c r="M22" s="53">
+        <v>0.5370753321855152</v>
+      </c>
       <c r="N22" s="53"/>
-      <c r="O22" s="52"/>
-      <c r="P22" s="52"/>
-      <c r="Q22" s="52"/>
-      <c r="R22" s="53"/>
-      <c r="S22" s="54"/>
-      <c r="T22" s="54"/>
-      <c r="U22" s="54"/>
-      <c r="V22" s="53"/>
+      <c r="O22" s="52">
+        <v>5798.4918</v>
+      </c>
+      <c r="P22" s="52">
+        <v>1710.68</v>
+      </c>
+      <c r="Q22" s="52">
+        <v>4087.8117999999995</v>
+      </c>
+      <c r="R22" s="53">
+        <v>0.7049784566393626</v>
+      </c>
+      <c r="S22" s="54">
+        <v>125.39</v>
+      </c>
+      <c r="T22" s="54">
+        <v>34.75</v>
+      </c>
+      <c r="U22" s="54">
+        <v>90.64</v>
+      </c>
+      <c r="V22" s="53">
+        <v>0.7228646622537682</v>
+      </c>
       <c r="W22" s="53"/>
-      <c r="X22" s="55"/>
-      <c r="Y22" s="55"/>
-      <c r="Z22" s="53"/>
-      <c r="AA22" s="56"/>
+      <c r="X22" s="55">
+        <v>112.66647482014388</v>
+      </c>
+      <c r="Y22" s="55">
+        <v>63.27846478985563</v>
+      </c>
+      <c r="Z22" s="53">
+        <v>0.32630000000000003</v>
+      </c>
+      <c r="AA22" s="56">
+        <v>0.2885</v>
+      </c>
       <c r="AB22" s="57"/>
       <c r="AD22" s="35"/>
       <c r="AE22" s="35"/>
@@ -12100,30 +12232,74 @@
       <c r="C36" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D36" s="52"/>
-      <c r="E36" s="52"/>
-      <c r="F36" s="52"/>
-      <c r="G36" s="53"/>
-      <c r="H36" s="52"/>
-      <c r="I36" s="52"/>
-      <c r="J36" s="52"/>
-      <c r="K36" s="52"/>
-      <c r="L36" s="52"/>
-      <c r="M36" s="53"/>
+      <c r="D36" s="52">
+        <v>397238.61073204</v>
+      </c>
+      <c r="E36" s="52">
+        <v>259347.71</v>
+      </c>
+      <c r="F36" s="52">
+        <v>137890.90073204003</v>
+      </c>
+      <c r="G36" s="53">
+        <v>0.3471236103608651</v>
+      </c>
+      <c r="H36" s="52">
+        <v>328046.93216</v>
+      </c>
+      <c r="I36" s="52">
+        <v>276899.86</v>
+      </c>
+      <c r="J36" s="52">
+        <v>271925.57216000004</v>
+      </c>
+      <c r="K36" s="52">
+        <v>244422.38999999998</v>
+      </c>
+      <c r="L36" s="52">
+        <v>27503.182160000055</v>
+      </c>
+      <c r="M36" s="53">
+        <v>0.10114231604454355</v>
+      </c>
       <c r="N36" s="53"/>
-      <c r="O36" s="52"/>
-      <c r="P36" s="52"/>
-      <c r="Q36" s="52"/>
-      <c r="R36" s="53"/>
-      <c r="S36" s="54"/>
-      <c r="T36" s="54"/>
-      <c r="U36" s="54"/>
-      <c r="V36" s="53"/>
+      <c r="O36" s="52">
+        <v>56121.36</v>
+      </c>
+      <c r="P36" s="52">
+        <v>32477.47</v>
+      </c>
+      <c r="Q36" s="52">
+        <v>23643.89</v>
+      </c>
+      <c r="R36" s="53">
+        <v>0.4212993056476179</v>
+      </c>
+      <c r="S36" s="54">
+        <v>1124.47</v>
+      </c>
+      <c r="T36" s="54">
+        <v>750.5</v>
+      </c>
+      <c r="U36" s="54">
+        <v>373.97</v>
+      </c>
+      <c r="V36" s="53">
+        <v>0.3325744572998835</v>
+      </c>
       <c r="W36" s="53"/>
-      <c r="X36" s="55"/>
-      <c r="Y36" s="55"/>
-      <c r="Z36" s="53"/>
-      <c r="AA36" s="56"/>
+      <c r="X36" s="55">
+        <v>-23.38727514990007</v>
+      </c>
+      <c r="Y36" s="55">
+        <v>61.532703026350184</v>
+      </c>
+      <c r="Z36" s="53">
+        <v>-0.0677</v>
+      </c>
+      <c r="AA36" s="56">
+        <v>0.1742</v>
+      </c>
       <c r="AB36" s="57"/>
       <c r="AD36" s="35"/>
       <c r="AE36" s="35"/>
@@ -12551,30 +12727,74 @@
       <c r="C43" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D43" s="52"/>
-      <c r="E43" s="52"/>
-      <c r="F43" s="52"/>
-      <c r="G43" s="53"/>
-      <c r="H43" s="52"/>
-      <c r="I43" s="52"/>
-      <c r="J43" s="52"/>
-      <c r="K43" s="52"/>
-      <c r="L43" s="52"/>
-      <c r="M43" s="53"/>
+      <c r="D43" s="52">
+        <v>128258.49930985</v>
+      </c>
+      <c r="E43" s="52">
+        <v>53944.83</v>
+      </c>
+      <c r="F43" s="52">
+        <v>74313.66930985</v>
+      </c>
+      <c r="G43" s="53">
+        <v>0.5794054172606622</v>
+      </c>
+      <c r="H43" s="52">
+        <v>94098.31685</v>
+      </c>
+      <c r="I43" s="52">
+        <v>56107.33</v>
+      </c>
+      <c r="J43" s="52">
+        <v>69042.08885</v>
+      </c>
+      <c r="K43" s="52">
+        <v>40219.090000000004</v>
+      </c>
+      <c r="L43" s="52">
+        <v>28822.998849999996</v>
+      </c>
+      <c r="M43" s="53">
+        <v>0.41746997128983876</v>
+      </c>
       <c r="N43" s="53"/>
-      <c r="O43" s="52"/>
-      <c r="P43" s="52"/>
-      <c r="Q43" s="52"/>
-      <c r="R43" s="53"/>
-      <c r="S43" s="54"/>
-      <c r="T43" s="54"/>
-      <c r="U43" s="54"/>
-      <c r="V43" s="53"/>
+      <c r="O43" s="52">
+        <v>25056.228</v>
+      </c>
+      <c r="P43" s="52">
+        <v>15888.24</v>
+      </c>
+      <c r="Q43" s="52">
+        <v>9167.988</v>
+      </c>
+      <c r="R43" s="53">
+        <v>0.3658965746959199</v>
+      </c>
+      <c r="S43" s="54">
+        <v>501.83</v>
+      </c>
+      <c r="T43" s="54">
+        <v>358.75</v>
+      </c>
+      <c r="U43" s="54">
+        <v>143.07999999999998</v>
+      </c>
+      <c r="V43" s="53">
+        <v>0.28511647370623516</v>
+      </c>
       <c r="W43" s="53"/>
-      <c r="X43" s="55"/>
-      <c r="Y43" s="55"/>
-      <c r="Z43" s="53"/>
-      <c r="AA43" s="56"/>
+      <c r="X43" s="55">
+        <v>-6.02787456445993</v>
+      </c>
+      <c r="Y43" s="55">
+        <v>68.07122423898531</v>
+      </c>
+      <c r="Z43" s="53">
+        <v>-0.0401</v>
+      </c>
+      <c r="AA43" s="56">
+        <v>0.2663</v>
+      </c>
       <c r="AB43" s="57"/>
       <c r="AD43" s="35"/>
       <c r="AE43" s="35"/>
@@ -13004,30 +13224,74 @@
       <c r="C50" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D50" s="52"/>
-      <c r="E50" s="52"/>
-      <c r="F50" s="52"/>
-      <c r="G50" s="53"/>
-      <c r="H50" s="52"/>
-      <c r="I50" s="52"/>
-      <c r="J50" s="52"/>
-      <c r="K50" s="52"/>
-      <c r="L50" s="52"/>
-      <c r="M50" s="53"/>
+      <c r="D50" s="52">
+        <v>65693.35850319</v>
+      </c>
+      <c r="E50" s="52">
+        <v>33326.49</v>
+      </c>
+      <c r="F50" s="52">
+        <v>32366.868503190002</v>
+      </c>
+      <c r="G50" s="53">
+        <v>0.49269620614111703</v>
+      </c>
+      <c r="H50" s="52">
+        <v>50582.36785</v>
+      </c>
+      <c r="I50" s="52">
+        <v>29574.96</v>
+      </c>
+      <c r="J50" s="52">
+        <v>39438.99025</v>
+      </c>
+      <c r="K50" s="52">
+        <v>20218.23</v>
+      </c>
+      <c r="L50" s="52">
+        <v>19220.760250000003</v>
+      </c>
+      <c r="M50" s="53">
+        <v>0.48735426866056747</v>
+      </c>
       <c r="N50" s="53"/>
-      <c r="O50" s="52"/>
-      <c r="P50" s="52"/>
-      <c r="Q50" s="52"/>
-      <c r="R50" s="53"/>
-      <c r="S50" s="54"/>
-      <c r="T50" s="54"/>
-      <c r="U50" s="54"/>
-      <c r="V50" s="53"/>
+      <c r="O50" s="52">
+        <v>11143.3776</v>
+      </c>
+      <c r="P50" s="52">
+        <v>9356.73</v>
+      </c>
+      <c r="Q50" s="52">
+        <v>1786.6476000000002</v>
+      </c>
+      <c r="R50" s="53">
+        <v>0.1603326804612634</v>
+      </c>
+      <c r="S50" s="54">
+        <v>223.22</v>
+      </c>
+      <c r="T50" s="54">
+        <v>216.5</v>
+      </c>
+      <c r="U50" s="54">
+        <v>6.719999999999999</v>
+      </c>
+      <c r="V50" s="53">
+        <v>0.030104829316369496</v>
+      </c>
       <c r="W50" s="53"/>
-      <c r="X50" s="55"/>
-      <c r="Y50" s="55"/>
-      <c r="Z50" s="53"/>
-      <c r="AA50" s="56"/>
+      <c r="X50" s="55">
+        <v>17.3280831408776</v>
+      </c>
+      <c r="Y50" s="55">
+        <v>67.69550512136009</v>
+      </c>
+      <c r="Z50" s="53">
+        <v>0.11259999999999999</v>
+      </c>
+      <c r="AA50" s="56">
+        <v>0.23</v>
+      </c>
       <c r="AB50" s="57"/>
       <c r="AD50" s="35"/>
       <c r="AE50" s="35"/>
@@ -13455,30 +13719,74 @@
       <c r="C57" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D57" s="52"/>
-      <c r="E57" s="52"/>
-      <c r="F57" s="52"/>
-      <c r="G57" s="53"/>
-      <c r="H57" s="52"/>
-      <c r="I57" s="52"/>
-      <c r="J57" s="52"/>
-      <c r="K57" s="52"/>
-      <c r="L57" s="52"/>
-      <c r="M57" s="53"/>
+      <c r="D57" s="52">
+        <v>155296.79012754</v>
+      </c>
+      <c r="E57" s="52">
+        <v>127814.48</v>
+      </c>
+      <c r="F57" s="52">
+        <v>27482.31012754001</v>
+      </c>
+      <c r="G57" s="53">
+        <v>0.17696637583410268</v>
+      </c>
+      <c r="H57" s="52">
+        <v>109364.9721</v>
+      </c>
+      <c r="I57" s="52">
+        <v>109618.36</v>
+      </c>
+      <c r="J57" s="52">
+        <v>75135.0159</v>
+      </c>
+      <c r="K57" s="52">
+        <v>78027.66</v>
+      </c>
+      <c r="L57" s="52">
+        <v>-2892.644100000005</v>
+      </c>
+      <c r="M57" s="53">
+        <v>-0.03849928113211466</v>
+      </c>
       <c r="N57" s="53"/>
-      <c r="O57" s="52"/>
-      <c r="P57" s="52"/>
-      <c r="Q57" s="52"/>
-      <c r="R57" s="53"/>
-      <c r="S57" s="54"/>
-      <c r="T57" s="54"/>
-      <c r="U57" s="54"/>
-      <c r="V57" s="53"/>
+      <c r="O57" s="52">
+        <v>34229.9562</v>
+      </c>
+      <c r="P57" s="52">
+        <v>31590.7</v>
+      </c>
+      <c r="Q57" s="52">
+        <v>2639.2562</v>
+      </c>
+      <c r="R57" s="53">
+        <v>0.07710369784230106</v>
+      </c>
+      <c r="S57" s="54">
+        <v>685.48</v>
+      </c>
+      <c r="T57" s="54">
+        <v>660.25</v>
+      </c>
+      <c r="U57" s="54">
+        <v>25.230000000000018</v>
+      </c>
+      <c r="V57" s="53">
+        <v>0.036806325494544</v>
+      </c>
       <c r="W57" s="53"/>
-      <c r="X57" s="55"/>
-      <c r="Y57" s="55"/>
-      <c r="Z57" s="53"/>
-      <c r="AA57" s="56"/>
+      <c r="X57" s="55">
+        <v>27.559439606209768</v>
+      </c>
+      <c r="Y57" s="55">
+        <v>67.00679527854935</v>
+      </c>
+      <c r="Z57" s="53">
+        <v>0.1424</v>
+      </c>
+      <c r="AA57" s="56">
+        <v>0.2958</v>
+      </c>
       <c r="AB57" s="57"/>
       <c r="AD57" s="35"/>
       <c r="AE57" s="35"/>
@@ -14307,30 +14615,74 @@
       <c r="C71" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D71" s="52"/>
-      <c r="E71" s="52"/>
-      <c r="F71" s="52"/>
-      <c r="G71" s="53"/>
-      <c r="H71" s="52"/>
-      <c r="I71" s="52"/>
-      <c r="J71" s="52"/>
-      <c r="K71" s="52"/>
-      <c r="L71" s="52"/>
-      <c r="M71" s="53"/>
+      <c r="D71" s="52">
+        <v>53029.71458947</v>
+      </c>
+      <c r="E71" s="52">
+        <v>10650.43</v>
+      </c>
+      <c r="F71" s="52">
+        <v>42379.28458947</v>
+      </c>
+      <c r="G71" s="53">
+        <v>0.7991610914286378</v>
+      </c>
+      <c r="H71" s="52">
+        <v>39055.77825</v>
+      </c>
+      <c r="I71" s="52">
+        <v>20931.54</v>
+      </c>
+      <c r="J71" s="52">
+        <v>29537.289750000004</v>
+      </c>
+      <c r="K71" s="52">
+        <v>19627.920000000002</v>
+      </c>
+      <c r="L71" s="52">
+        <v>9909.369750000002</v>
+      </c>
+      <c r="M71" s="53">
+        <v>0.3354867638118355</v>
+      </c>
       <c r="N71" s="53"/>
-      <c r="O71" s="52"/>
-      <c r="P71" s="52"/>
-      <c r="Q71" s="52"/>
-      <c r="R71" s="53"/>
-      <c r="S71" s="54"/>
-      <c r="T71" s="54"/>
-      <c r="U71" s="54"/>
-      <c r="V71" s="53"/>
+      <c r="O71" s="52">
+        <v>9518.4885</v>
+      </c>
+      <c r="P71" s="52">
+        <v>1303.62</v>
+      </c>
+      <c r="Q71" s="52">
+        <v>8214.8685</v>
+      </c>
+      <c r="R71" s="53">
+        <v>0.8630433813099634</v>
+      </c>
+      <c r="S71" s="54">
+        <v>193.32</v>
+      </c>
+      <c r="T71" s="54">
+        <v>27.25</v>
+      </c>
+      <c r="U71" s="54">
+        <v>166.07</v>
+      </c>
+      <c r="V71" s="53">
+        <v>0.8590420028967515</v>
+      </c>
       <c r="W71" s="53"/>
-      <c r="X71" s="55"/>
-      <c r="Y71" s="55"/>
-      <c r="Z71" s="53"/>
-      <c r="AA71" s="56"/>
+      <c r="X71" s="55">
+        <v>-377.2884403669725</v>
+      </c>
+      <c r="Y71" s="55">
+        <v>72.28396616733912</v>
+      </c>
+      <c r="Z71" s="53">
+        <v>-0.9653</v>
+      </c>
+      <c r="AA71" s="56">
+        <v>0.2635</v>
+      </c>
       <c r="AB71" s="57"/>
       <c r="AD71" s="35"/>
       <c r="AE71" s="35"/>
@@ -14748,30 +15100,74 @@
       <c r="C78" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D78" s="52"/>
-      <c r="E78" s="52"/>
-      <c r="F78" s="52"/>
-      <c r="G78" s="53"/>
-      <c r="H78" s="52"/>
-      <c r="I78" s="52"/>
-      <c r="J78" s="52"/>
-      <c r="K78" s="52"/>
-      <c r="L78" s="52"/>
-      <c r="M78" s="53"/>
+      <c r="D78" s="52">
+        <v>78753.06644148</v>
+      </c>
+      <c r="E78" s="52">
+        <v>44764.99</v>
+      </c>
+      <c r="F78" s="52">
+        <v>33988.07644148</v>
+      </c>
+      <c r="G78" s="53">
+        <v>0.43157781629666364</v>
+      </c>
+      <c r="H78" s="52">
+        <v>55589.7822</v>
+      </c>
+      <c r="I78" s="52">
+        <v>41397.62</v>
+      </c>
+      <c r="J78" s="52">
+        <v>32594.7534</v>
+      </c>
+      <c r="K78" s="52">
+        <v>32996.44</v>
+      </c>
+      <c r="L78" s="52">
+        <v>-401.6866000000009</v>
+      </c>
+      <c r="M78" s="53">
+        <v>-0.01232365819954327</v>
+      </c>
       <c r="N78" s="53"/>
-      <c r="O78" s="52"/>
-      <c r="P78" s="52"/>
-      <c r="Q78" s="52"/>
-      <c r="R78" s="53"/>
-      <c r="S78" s="54"/>
-      <c r="T78" s="54"/>
-      <c r="U78" s="54"/>
-      <c r="V78" s="53"/>
+      <c r="O78" s="52">
+        <v>22995.0288</v>
+      </c>
+      <c r="P78" s="52">
+        <v>8401.18</v>
+      </c>
+      <c r="Q78" s="52">
+        <v>14593.8488</v>
+      </c>
+      <c r="R78" s="53">
+        <v>0.6346523384219462</v>
+      </c>
+      <c r="S78" s="54">
+        <v>472.14</v>
+      </c>
+      <c r="T78" s="54">
+        <v>167.25</v>
+      </c>
+      <c r="U78" s="54">
+        <v>304.89</v>
+      </c>
+      <c r="V78" s="53">
+        <v>0.6457618502986402</v>
+      </c>
       <c r="W78" s="53"/>
-      <c r="X78" s="55"/>
-      <c r="Y78" s="55"/>
-      <c r="Z78" s="53"/>
-      <c r="AA78" s="56"/>
+      <c r="X78" s="55">
+        <v>20.133751868460386</v>
+      </c>
+      <c r="Y78" s="55">
+        <v>49.060202993773025</v>
+      </c>
+      <c r="Z78" s="53">
+        <v>0.07519999999999999</v>
+      </c>
+      <c r="AA78" s="56">
+        <v>0.2941</v>
+      </c>
       <c r="AB78" s="57"/>
       <c r="AD78" s="35"/>
       <c r="AE78" s="35"/>
@@ -15195,30 +15591,74 @@
       <c r="C85" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D85" s="52"/>
-      <c r="E85" s="52"/>
-      <c r="F85" s="52"/>
-      <c r="G85" s="53"/>
-      <c r="H85" s="52"/>
-      <c r="I85" s="52"/>
-      <c r="J85" s="52"/>
-      <c r="K85" s="52"/>
-      <c r="L85" s="52"/>
-      <c r="M85" s="53"/>
+      <c r="D85" s="52">
+        <v>25467.8441072</v>
+      </c>
+      <c r="E85" s="52">
+        <v>19598.41</v>
+      </c>
+      <c r="F85" s="52">
+        <v>5869.434107199999</v>
+      </c>
+      <c r="G85" s="53">
+        <v>0.23046450584879521</v>
+      </c>
+      <c r="H85" s="52">
+        <v>16606.829916</v>
+      </c>
+      <c r="I85" s="52">
+        <v>14118.07</v>
+      </c>
+      <c r="J85" s="52">
+        <v>9659.986716</v>
+      </c>
+      <c r="K85" s="52">
+        <v>5298.48</v>
+      </c>
+      <c r="L85" s="52">
+        <v>4361.506716</v>
+      </c>
+      <c r="M85" s="53">
+        <v>0.4515023513206248</v>
+      </c>
       <c r="N85" s="53"/>
-      <c r="O85" s="52"/>
-      <c r="P85" s="52"/>
-      <c r="Q85" s="52"/>
-      <c r="R85" s="53"/>
-      <c r="S85" s="54"/>
-      <c r="T85" s="54"/>
-      <c r="U85" s="54"/>
-      <c r="V85" s="53"/>
+      <c r="O85" s="52">
+        <v>6946.8432</v>
+      </c>
+      <c r="P85" s="52">
+        <v>8819.59</v>
+      </c>
+      <c r="Q85" s="52">
+        <v>-1872.7468</v>
+      </c>
+      <c r="R85" s="53">
+        <v>-0.26958241982487813</v>
+      </c>
+      <c r="S85" s="54">
+        <v>139.07</v>
+      </c>
+      <c r="T85" s="54">
+        <v>167.75</v>
+      </c>
+      <c r="U85" s="54">
+        <v>-28.680000000000007</v>
+      </c>
+      <c r="V85" s="53">
+        <v>-0.20622707988782632</v>
+      </c>
       <c r="W85" s="53"/>
-      <c r="X85" s="55"/>
-      <c r="Y85" s="55"/>
-      <c r="Z85" s="53"/>
-      <c r="AA85" s="56"/>
+      <c r="X85" s="55">
+        <v>32.669687034277196</v>
+      </c>
+      <c r="Y85" s="55">
+        <v>63.7162162306752</v>
+      </c>
+      <c r="Z85" s="53">
+        <v>0.2796</v>
+      </c>
+      <c r="AA85" s="56">
+        <v>0.3479</v>
+      </c>
       <c r="AB85" s="57"/>
       <c r="AD85" s="35"/>
       <c r="AE85" s="35"/>
@@ -15646,30 +16086,74 @@
       <c r="C92" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D92" s="67"/>
-      <c r="E92" s="67"/>
-      <c r="F92" s="52"/>
-      <c r="G92" s="53"/>
-      <c r="H92" s="52"/>
-      <c r="I92" s="52"/>
-      <c r="J92" s="52"/>
-      <c r="K92" s="52"/>
-      <c r="L92" s="52"/>
-      <c r="M92" s="53"/>
+      <c r="D92" s="67">
+        <v>37083.0313712</v>
+      </c>
+      <c r="E92" s="67">
+        <v>36381.33</v>
+      </c>
+      <c r="F92" s="52">
+        <v>701.7013711999971</v>
+      </c>
+      <c r="G92" s="53">
+        <v>0.018922438248804095</v>
+      </c>
+      <c r="H92" s="52">
+        <v>27002.93286</v>
+      </c>
+      <c r="I92" s="52">
+        <v>25103.82</v>
+      </c>
+      <c r="J92" s="52">
+        <v>15440.324460000002</v>
+      </c>
+      <c r="K92" s="52">
+        <v>13974.73</v>
+      </c>
+      <c r="L92" s="52">
+        <v>1465.594460000002</v>
+      </c>
+      <c r="M92" s="53">
+        <v>0.0949199263135175</v>
+      </c>
       <c r="N92" s="53"/>
-      <c r="O92" s="52"/>
-      <c r="P92" s="52"/>
-      <c r="Q92" s="52"/>
-      <c r="R92" s="53"/>
-      <c r="S92" s="68"/>
-      <c r="T92" s="68"/>
-      <c r="U92" s="54"/>
-      <c r="V92" s="53"/>
+      <c r="O92" s="52">
+        <v>11562.6084</v>
+      </c>
+      <c r="P92" s="52">
+        <v>11129.09</v>
+      </c>
+      <c r="Q92" s="52">
+        <v>433.518399999999</v>
+      </c>
+      <c r="R92" s="53">
+        <v>0.03749313174006646</v>
+      </c>
+      <c r="S92" s="68">
+        <v>231.75</v>
+      </c>
+      <c r="T92" s="68">
+        <v>225.5</v>
+      </c>
+      <c r="U92" s="54">
+        <v>6.25</v>
+      </c>
+      <c r="V92" s="53">
+        <v>0.02696871628910464</v>
+      </c>
       <c r="W92" s="53"/>
-      <c r="X92" s="55"/>
-      <c r="Y92" s="55"/>
-      <c r="Z92" s="53"/>
-      <c r="AA92" s="56"/>
+      <c r="X92" s="55">
+        <v>50.01113082039912</v>
+      </c>
+      <c r="Y92" s="55">
+        <v>43.49557070636461</v>
+      </c>
+      <c r="Z92" s="53">
+        <v>0.31</v>
+      </c>
+      <c r="AA92" s="56">
+        <v>0.2718</v>
+      </c>
       <c r="AB92" s="57"/>
       <c r="AD92" s="35"/>
       <c r="AE92" s="35"/>
@@ -16097,30 +16581,74 @@
       <c r="C99" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D99" s="52"/>
-      <c r="E99" s="52"/>
-      <c r="F99" s="52"/>
-      <c r="G99" s="53"/>
-      <c r="H99" s="52"/>
-      <c r="I99" s="52"/>
-      <c r="J99" s="52"/>
-      <c r="K99" s="52"/>
-      <c r="L99" s="52"/>
-      <c r="M99" s="53"/>
+      <c r="D99" s="52">
+        <v>26186.1354</v>
+      </c>
+      <c r="E99" s="52">
+        <v>5762.27</v>
+      </c>
+      <c r="F99" s="52">
+        <v>20423.8654</v>
+      </c>
+      <c r="G99" s="53">
+        <v>0.7799495835494686</v>
+      </c>
+      <c r="H99" s="52">
+        <v>19428.9760178</v>
+      </c>
+      <c r="I99" s="52">
+        <v>8019.36</v>
+      </c>
+      <c r="J99" s="52">
+        <v>12051.3142178</v>
+      </c>
+      <c r="K99" s="52">
+        <v>7687.129999999999</v>
+      </c>
+      <c r="L99" s="52">
+        <v>4364.184217800001</v>
+      </c>
+      <c r="M99" s="53">
+        <v>0.3621334685103493</v>
+      </c>
       <c r="N99" s="53"/>
-      <c r="O99" s="52"/>
-      <c r="P99" s="52"/>
-      <c r="Q99" s="52"/>
-      <c r="R99" s="53"/>
-      <c r="S99" s="54"/>
-      <c r="T99" s="54"/>
-      <c r="U99" s="54"/>
-      <c r="V99" s="53"/>
+      <c r="O99" s="52">
+        <v>7377.6618</v>
+      </c>
+      <c r="P99" s="52">
+        <v>332.23</v>
+      </c>
+      <c r="Q99" s="52">
+        <v>7045.4318</v>
+      </c>
+      <c r="R99" s="53">
+        <v>0.954968117405436</v>
+      </c>
+      <c r="S99" s="54">
+        <v>147.9</v>
+      </c>
+      <c r="T99" s="54">
+        <v>6.5</v>
+      </c>
+      <c r="U99" s="54">
+        <v>141.4</v>
+      </c>
+      <c r="V99" s="53">
+        <v>0.9560513860716701</v>
+      </c>
       <c r="W99" s="53"/>
-      <c r="X99" s="55"/>
-      <c r="Y99" s="55"/>
-      <c r="Z99" s="53"/>
-      <c r="AA99" s="56"/>
+      <c r="X99" s="55">
+        <v>-347.24461538461543</v>
+      </c>
+      <c r="Y99" s="55">
+        <v>45.687352144692355</v>
+      </c>
+      <c r="Z99" s="53">
+        <v>-0.3917</v>
+      </c>
+      <c r="AA99" s="56">
+        <v>0.258</v>
+      </c>
       <c r="AB99" s="57"/>
       <c r="AD99" s="35"/>
       <c r="AE99" s="35"/>
@@ -17358,30 +17886,74 @@
       <c r="C120" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D120" s="52"/>
-      <c r="E120" s="52"/>
-      <c r="F120" s="52"/>
-      <c r="G120" s="53"/>
-      <c r="H120" s="52"/>
-      <c r="I120" s="52"/>
-      <c r="J120" s="52"/>
-      <c r="K120" s="52"/>
-      <c r="L120" s="52"/>
-      <c r="M120" s="53"/>
+      <c r="D120" s="52">
+        <v>21404.8192765</v>
+      </c>
+      <c r="E120" s="52">
+        <v>0</v>
+      </c>
+      <c r="F120" s="52">
+        <v>21404.8192765</v>
+      </c>
+      <c r="G120" s="53">
+        <v>1</v>
+      </c>
+      <c r="H120" s="52">
+        <v>17514.092529</v>
+      </c>
+      <c r="I120" s="52">
+        <v>0</v>
+      </c>
+      <c r="J120" s="52">
+        <v>13318.886529000001</v>
+      </c>
+      <c r="K120" s="52">
+        <v>0</v>
+      </c>
+      <c r="L120" s="52">
+        <v>13318.886529000001</v>
+      </c>
+      <c r="M120" s="53">
+        <v>1</v>
+      </c>
       <c r="N120" s="53"/>
-      <c r="O120" s="52"/>
-      <c r="P120" s="52"/>
-      <c r="Q120" s="52"/>
-      <c r="R120" s="53"/>
-      <c r="S120" s="54"/>
-      <c r="T120" s="54"/>
-      <c r="U120" s="54"/>
-      <c r="V120" s="53"/>
+      <c r="O120" s="52">
+        <v>4195.206</v>
+      </c>
+      <c r="P120" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q120" s="52">
+        <v>4195.206</v>
+      </c>
+      <c r="R120" s="53">
+        <v>1</v>
+      </c>
+      <c r="S120" s="54">
+        <v>84.05</v>
+      </c>
+      <c r="T120" s="54">
+        <v>0</v>
+      </c>
+      <c r="U120" s="54">
+        <v>84.05</v>
+      </c>
+      <c r="V120" s="53">
+        <v>1</v>
+      </c>
       <c r="W120" s="53"/>
-      <c r="X120" s="55"/>
-      <c r="Y120" s="55"/>
-      <c r="Z120" s="53"/>
-      <c r="AA120" s="56"/>
+      <c r="X120" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y120" s="55">
+        <v>46.29062162403328</v>
+      </c>
+      <c r="Z120" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA120" s="56">
+        <v>0.1818</v>
+      </c>
       <c r="AB120" s="57"/>
       <c r="AD120" s="35"/>
       <c r="AE120" s="35"/>
@@ -17799,30 +18371,74 @@
       <c r="C127" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D127" s="52"/>
-      <c r="E127" s="52"/>
-      <c r="F127" s="52"/>
-      <c r="G127" s="53"/>
-      <c r="H127" s="52"/>
-      <c r="I127" s="52"/>
-      <c r="J127" s="52"/>
-      <c r="K127" s="52"/>
-      <c r="L127" s="52"/>
-      <c r="M127" s="53"/>
+      <c r="D127" s="52">
+        <v>105896.9567712</v>
+      </c>
+      <c r="E127" s="52">
+        <v>67407.3</v>
+      </c>
+      <c r="F127" s="52">
+        <v>38489.656771199996</v>
+      </c>
+      <c r="G127" s="53">
+        <v>0.3634632943641657</v>
+      </c>
+      <c r="H127" s="52">
+        <v>85934.2000148</v>
+      </c>
+      <c r="I127" s="52">
+        <v>66541.03</v>
+      </c>
+      <c r="J127" s="52">
+        <v>70065.71561479999</v>
+      </c>
+      <c r="K127" s="52">
+        <v>61659.44</v>
+      </c>
+      <c r="L127" s="52">
+        <v>8406.27561479999</v>
+      </c>
+      <c r="M127" s="53">
+        <v>0.11997701787583442</v>
+      </c>
       <c r="N127" s="53"/>
-      <c r="O127" s="52"/>
-      <c r="P127" s="52"/>
-      <c r="Q127" s="52"/>
-      <c r="R127" s="53"/>
-      <c r="S127" s="54"/>
-      <c r="T127" s="54"/>
-      <c r="U127" s="54"/>
-      <c r="V127" s="53"/>
+      <c r="O127" s="52">
+        <v>15868.4844</v>
+      </c>
+      <c r="P127" s="52">
+        <v>4881.59</v>
+      </c>
+      <c r="Q127" s="52">
+        <v>10986.8944</v>
+      </c>
+      <c r="R127" s="53">
+        <v>0.6923720074993425</v>
+      </c>
+      <c r="S127" s="54">
+        <v>317.92</v>
+      </c>
+      <c r="T127" s="54">
+        <v>106</v>
+      </c>
+      <c r="U127" s="54">
+        <v>211.92000000000002</v>
+      </c>
+      <c r="V127" s="53">
+        <v>0.6665827881227983</v>
+      </c>
       <c r="W127" s="53"/>
-      <c r="X127" s="55"/>
-      <c r="Y127" s="55"/>
-      <c r="Z127" s="53"/>
-      <c r="AA127" s="56"/>
+      <c r="X127" s="55">
+        <v>8.172358490566037</v>
+      </c>
+      <c r="Y127" s="55">
+        <v>62.79176131227983</v>
+      </c>
+      <c r="Z127" s="53">
+        <v>0.0129</v>
+      </c>
+      <c r="AA127" s="56">
+        <v>0.1885</v>
+      </c>
       <c r="AB127" s="57"/>
       <c r="AD127" s="35"/>
       <c r="AE127" s="35"/>
@@ -18247,30 +18863,74 @@
       <c r="C134" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D134" s="52"/>
-      <c r="E134" s="52"/>
-      <c r="F134" s="52"/>
-      <c r="G134" s="53"/>
-      <c r="H134" s="52"/>
-      <c r="I134" s="52"/>
-      <c r="J134" s="52"/>
-      <c r="K134" s="52"/>
-      <c r="L134" s="52"/>
-      <c r="M134" s="53"/>
+      <c r="D134" s="52">
+        <v>31802.4136956</v>
+      </c>
+      <c r="E134" s="52">
+        <v>16498.64</v>
+      </c>
+      <c r="F134" s="52">
+        <v>15303.7736956</v>
+      </c>
+      <c r="G134" s="53">
+        <v>0.48121421984134943</v>
+      </c>
+      <c r="H134" s="52">
+        <v>23448.14263</v>
+      </c>
+      <c r="I134" s="52">
+        <v>12360.83</v>
+      </c>
+      <c r="J134" s="52">
+        <v>15632.028429999998</v>
+      </c>
+      <c r="K134" s="52">
+        <v>11772.08</v>
+      </c>
+      <c r="L134" s="52">
+        <v>3859.9484299999986</v>
+      </c>
+      <c r="M134" s="53">
+        <v>0.24692562755273845</v>
+      </c>
       <c r="N134" s="53"/>
-      <c r="O134" s="52"/>
-      <c r="P134" s="52"/>
-      <c r="Q134" s="52"/>
-      <c r="R134" s="53"/>
-      <c r="S134" s="54"/>
-      <c r="T134" s="54"/>
-      <c r="U134" s="54"/>
-      <c r="V134" s="53"/>
+      <c r="O134" s="52">
+        <v>7816.1142</v>
+      </c>
+      <c r="P134" s="52">
+        <v>588.75</v>
+      </c>
+      <c r="Q134" s="52">
+        <v>7227.3642</v>
+      </c>
+      <c r="R134" s="53">
+        <v>0.92467484674162</v>
+      </c>
+      <c r="S134" s="54">
+        <v>156.69</v>
+      </c>
+      <c r="T134" s="54">
+        <v>11.5</v>
+      </c>
+      <c r="U134" s="54">
+        <v>145.19</v>
+      </c>
+      <c r="V134" s="53">
+        <v>0.9266066756015061</v>
+      </c>
       <c r="W134" s="53"/>
-      <c r="X134" s="55"/>
-      <c r="Y134" s="55"/>
-      <c r="Z134" s="53"/>
-      <c r="AA134" s="56"/>
+      <c r="X134" s="55">
+        <v>359.80956521739137</v>
+      </c>
+      <c r="Y134" s="55">
+        <v>53.31719360265494</v>
+      </c>
+      <c r="Z134" s="53">
+        <v>0.25079999999999997</v>
+      </c>
+      <c r="AA134" s="56">
+        <v>0.2627</v>
+      </c>
       <c r="AB134" s="57"/>
       <c r="AD134" s="35"/>
       <c r="AE134" s="35"/>
@@ -19897,30 +20557,74 @@
       <c r="C162" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D162" s="52"/>
-      <c r="E162" s="52"/>
-      <c r="F162" s="52"/>
-      <c r="G162" s="53"/>
-      <c r="H162" s="52"/>
-      <c r="I162" s="52"/>
-      <c r="J162" s="52"/>
-      <c r="K162" s="52"/>
-      <c r="L162" s="52"/>
-      <c r="M162" s="53"/>
+      <c r="D162" s="52">
+        <v>17899.333054</v>
+      </c>
+      <c r="E162" s="52">
+        <v>13424.5</v>
+      </c>
+      <c r="F162" s="52">
+        <v>4474.833053999999</v>
+      </c>
+      <c r="G162" s="53">
+        <v>0.24999998829565323</v>
+      </c>
+      <c r="H162" s="52">
+        <v>13919.4012884</v>
+      </c>
+      <c r="I162" s="52">
+        <v>12620.62</v>
+      </c>
+      <c r="J162" s="52">
+        <v>8410.9272884</v>
+      </c>
+      <c r="K162" s="52">
+        <v>7749.860000000001</v>
+      </c>
+      <c r="L162" s="52">
+        <v>661.0672883999996</v>
+      </c>
+      <c r="M162" s="53">
+        <v>0.07859624340252186</v>
+      </c>
       <c r="N162" s="53"/>
-      <c r="O162" s="52"/>
-      <c r="P162" s="52"/>
-      <c r="Q162" s="52"/>
-      <c r="R162" s="53"/>
-      <c r="S162" s="54"/>
-      <c r="T162" s="54"/>
-      <c r="U162" s="54"/>
-      <c r="V162" s="53"/>
+      <c r="O162" s="52">
+        <v>5508.474</v>
+      </c>
+      <c r="P162" s="52">
+        <v>4870.76</v>
+      </c>
+      <c r="Q162" s="52">
+        <v>637.7139999999999</v>
+      </c>
+      <c r="R162" s="53">
+        <v>0.11576963057282287</v>
+      </c>
+      <c r="S162" s="54">
+        <v>110.44</v>
+      </c>
+      <c r="T162" s="54">
+        <v>95.5</v>
+      </c>
+      <c r="U162" s="54">
+        <v>14.939999999999998</v>
+      </c>
+      <c r="V162" s="53">
+        <v>0.13527707352408547</v>
+      </c>
       <c r="W162" s="53"/>
-      <c r="X162" s="55"/>
-      <c r="Y162" s="55"/>
-      <c r="Z162" s="53"/>
-      <c r="AA162" s="56"/>
+      <c r="X162" s="55">
+        <v>8.41759162303665</v>
+      </c>
+      <c r="Y162" s="55">
+        <v>36.03704967040926</v>
+      </c>
+      <c r="Z162" s="53">
+        <v>0.0599</v>
+      </c>
+      <c r="AA162" s="56">
+        <v>0.2224</v>
+      </c>
       <c r="AB162" s="57"/>
       <c r="AD162" s="35"/>
       <c r="AE162" s="35"/>
@@ -20324,30 +21028,74 @@
       <c r="C169" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D169" s="52"/>
-      <c r="E169" s="52"/>
-      <c r="F169" s="52"/>
-      <c r="G169" s="53"/>
-      <c r="H169" s="52"/>
-      <c r="I169" s="52"/>
-      <c r="J169" s="52"/>
-      <c r="K169" s="52"/>
-      <c r="L169" s="52"/>
-      <c r="M169" s="53"/>
+      <c r="D169" s="52">
+        <v>10827.20261235</v>
+      </c>
+      <c r="E169" s="52">
+        <v>0</v>
+      </c>
+      <c r="F169" s="52">
+        <v>10827.20261235</v>
+      </c>
+      <c r="G169" s="53">
+        <v>1</v>
+      </c>
+      <c r="H169" s="52">
+        <v>7687.765097</v>
+      </c>
+      <c r="I169" s="52">
+        <v>2116.21</v>
+      </c>
+      <c r="J169" s="52">
+        <v>4437.133697</v>
+      </c>
+      <c r="K169" s="52">
+        <v>1029.51</v>
+      </c>
+      <c r="L169" s="52">
+        <v>3407.623697</v>
+      </c>
+      <c r="M169" s="53">
+        <v>0.7679785937719064</v>
+      </c>
       <c r="N169" s="53"/>
-      <c r="O169" s="52"/>
-      <c r="P169" s="52"/>
-      <c r="Q169" s="52"/>
-      <c r="R169" s="53"/>
-      <c r="S169" s="54"/>
-      <c r="T169" s="54"/>
-      <c r="U169" s="54"/>
-      <c r="V169" s="53"/>
+      <c r="O169" s="52">
+        <v>3250.6314</v>
+      </c>
+      <c r="P169" s="52">
+        <v>1086.7</v>
+      </c>
+      <c r="Q169" s="52">
+        <v>2163.9314000000004</v>
+      </c>
+      <c r="R169" s="53">
+        <v>0.6656957168382734</v>
+      </c>
+      <c r="S169" s="54">
+        <v>65.13</v>
+      </c>
+      <c r="T169" s="54">
+        <v>24.33</v>
+      </c>
+      <c r="U169" s="54">
+        <v>40.8</v>
+      </c>
+      <c r="V169" s="53">
+        <v>0.6264394288346384</v>
+      </c>
       <c r="W169" s="53"/>
-      <c r="X169" s="55"/>
-      <c r="Y169" s="55"/>
-      <c r="Z169" s="53"/>
-      <c r="AA169" s="56"/>
+      <c r="X169" s="55">
+        <v>-86.97944923962187</v>
+      </c>
+      <c r="Y169" s="55">
+        <v>48.202633430830645</v>
+      </c>
+      <c r="Z169" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA169" s="56">
+        <v>0.29</v>
+      </c>
       <c r="AB169" s="57"/>
       <c r="AD169" s="35"/>
       <c r="AE169" s="35"/>
@@ -20765,30 +21513,74 @@
       <c r="C176" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D176" s="52"/>
-      <c r="E176" s="52"/>
-      <c r="F176" s="52"/>
-      <c r="G176" s="53"/>
-      <c r="H176" s="52"/>
-      <c r="I176" s="52"/>
-      <c r="J176" s="52"/>
-      <c r="K176" s="52"/>
-      <c r="L176" s="52"/>
-      <c r="M176" s="53"/>
+      <c r="D176" s="52">
+        <v>146237.1072</v>
+      </c>
+      <c r="E176" s="52">
+        <v>125386.21</v>
+      </c>
+      <c r="F176" s="52">
+        <v>20850.897199999992</v>
+      </c>
+      <c r="G176" s="53">
+        <v>0.14258280678024784</v>
+      </c>
+      <c r="H176" s="52">
+        <v>114651.8653946</v>
+      </c>
+      <c r="I176" s="52">
+        <v>105824.3</v>
+      </c>
+      <c r="J176" s="52">
+        <v>82888.0783946</v>
+      </c>
+      <c r="K176" s="52">
+        <v>78304.64</v>
+      </c>
+      <c r="L176" s="52">
+        <v>4583.438394600002</v>
+      </c>
+      <c r="M176" s="53">
+        <v>0.055296714357159035</v>
+      </c>
       <c r="N176" s="53"/>
-      <c r="O176" s="52"/>
-      <c r="P176" s="52"/>
-      <c r="Q176" s="52"/>
-      <c r="R176" s="53"/>
-      <c r="S176" s="54"/>
-      <c r="T176" s="54"/>
-      <c r="U176" s="54"/>
-      <c r="V176" s="53"/>
+      <c r="O176" s="52">
+        <v>31763.787</v>
+      </c>
+      <c r="P176" s="52">
+        <v>27519.66</v>
+      </c>
+      <c r="Q176" s="52">
+        <v>4244.127</v>
+      </c>
+      <c r="R176" s="53">
+        <v>0.1336152707484155</v>
+      </c>
+      <c r="S176" s="54">
+        <v>659.73</v>
+      </c>
+      <c r="T176" s="54">
+        <v>548.75</v>
+      </c>
+      <c r="U176" s="54">
+        <v>110.98000000000002</v>
+      </c>
+      <c r="V176" s="53">
+        <v>0.16822033256028984</v>
+      </c>
       <c r="W176" s="53"/>
-      <c r="X176" s="55"/>
-      <c r="Y176" s="55"/>
-      <c r="Z176" s="53"/>
-      <c r="AA176" s="56"/>
+      <c r="X176" s="55">
+        <v>35.648127562642365</v>
+      </c>
+      <c r="Y176" s="55">
+        <v>47.87601261940491</v>
+      </c>
+      <c r="Z176" s="53">
+        <v>0.156</v>
+      </c>
+      <c r="AA176" s="56">
+        <v>0.216</v>
+      </c>
       <c r="AB176" s="57"/>
       <c r="AD176" s="35"/>
       <c r="AE176" s="35"/>
@@ -21214,30 +22006,74 @@
       <c r="C183" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D183" s="52"/>
-      <c r="E183" s="52"/>
-      <c r="F183" s="52"/>
-      <c r="G183" s="53"/>
-      <c r="H183" s="52"/>
-      <c r="I183" s="52"/>
-      <c r="J183" s="52"/>
-      <c r="K183" s="52"/>
-      <c r="L183" s="52"/>
-      <c r="M183" s="53"/>
+      <c r="D183" s="52">
+        <v>16897.52982004</v>
+      </c>
+      <c r="E183" s="52">
+        <v>5491.7</v>
+      </c>
+      <c r="F183" s="52">
+        <v>11405.829820039999</v>
+      </c>
+      <c r="G183" s="53">
+        <v>0.6749998337930436</v>
+      </c>
+      <c r="H183" s="52">
+        <v>9226.2731</v>
+      </c>
+      <c r="I183" s="52">
+        <v>4727.04</v>
+      </c>
+      <c r="J183" s="52">
+        <v>2977.1135000000004</v>
+      </c>
+      <c r="K183" s="52">
+        <v>2842.2799999999997</v>
+      </c>
+      <c r="L183" s="52">
+        <v>134.83350000000064</v>
+      </c>
+      <c r="M183" s="53">
+        <v>0.04529000993747824</v>
+      </c>
       <c r="N183" s="53"/>
-      <c r="O183" s="52"/>
-      <c r="P183" s="52"/>
-      <c r="Q183" s="52"/>
-      <c r="R183" s="53"/>
-      <c r="S183" s="54"/>
-      <c r="T183" s="54"/>
-      <c r="U183" s="54"/>
-      <c r="V183" s="53"/>
+      <c r="O183" s="52">
+        <v>6249.1596</v>
+      </c>
+      <c r="P183" s="52">
+        <v>1884.76</v>
+      </c>
+      <c r="Q183" s="52">
+        <v>4364.3996</v>
+      </c>
+      <c r="R183" s="53">
+        <v>0.6983978453678795</v>
+      </c>
+      <c r="S183" s="54">
+        <v>125.17</v>
+      </c>
+      <c r="T183" s="54">
+        <v>32.75</v>
+      </c>
+      <c r="U183" s="54">
+        <v>92.42</v>
+      </c>
+      <c r="V183" s="53">
+        <v>0.7383558360629544</v>
+      </c>
       <c r="W183" s="53"/>
-      <c r="X183" s="55"/>
-      <c r="Y183" s="55"/>
-      <c r="Z183" s="53"/>
-      <c r="AA183" s="56"/>
+      <c r="X183" s="55">
+        <v>23.348396946564886</v>
+      </c>
+      <c r="Y183" s="55">
+        <v>61.286703843093385</v>
+      </c>
+      <c r="Z183" s="53">
+        <v>0.1392</v>
+      </c>
+      <c r="AA183" s="56">
+        <v>0.454</v>
+      </c>
       <c r="AB183" s="57"/>
       <c r="AD183" s="35"/>
       <c r="AE183" s="35"/>
@@ -21659,30 +22495,74 @@
       <c r="C190" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D190" s="52"/>
-      <c r="E190" s="52"/>
-      <c r="F190" s="52"/>
-      <c r="G190" s="53"/>
-      <c r="H190" s="52"/>
-      <c r="I190" s="52"/>
-      <c r="J190" s="52"/>
-      <c r="K190" s="52"/>
-      <c r="L190" s="52"/>
-      <c r="M190" s="53"/>
+      <c r="D190" s="52">
+        <v>20992.11525559</v>
+      </c>
+      <c r="E190" s="52">
+        <v>14169.68</v>
+      </c>
+      <c r="F190" s="52">
+        <v>6822.43525559</v>
+      </c>
+      <c r="G190" s="53">
+        <v>0.3249998950807614</v>
+      </c>
+      <c r="H190" s="52">
+        <v>16299.085174</v>
+      </c>
+      <c r="I190" s="52">
+        <v>9699.51</v>
+      </c>
+      <c r="J190" s="52">
+        <v>9784.324774</v>
+      </c>
+      <c r="K190" s="52">
+        <v>8137.88</v>
+      </c>
+      <c r="L190" s="52">
+        <v>1646.4447740000005</v>
+      </c>
+      <c r="M190" s="53">
+        <v>0.16827372476178604</v>
+      </c>
       <c r="N190" s="53"/>
-      <c r="O190" s="52"/>
-      <c r="P190" s="52"/>
-      <c r="Q190" s="52"/>
-      <c r="R190" s="53"/>
-      <c r="S190" s="54"/>
-      <c r="T190" s="54"/>
-      <c r="U190" s="54"/>
-      <c r="V190" s="53"/>
+      <c r="O190" s="52">
+        <v>6514.7604</v>
+      </c>
+      <c r="P190" s="52">
+        <v>1561.63</v>
+      </c>
+      <c r="Q190" s="52">
+        <v>4953.1304</v>
+      </c>
+      <c r="R190" s="53">
+        <v>0.7602935635207705</v>
+      </c>
+      <c r="S190" s="54">
+        <v>130.62</v>
+      </c>
+      <c r="T190" s="54">
+        <v>34.75</v>
+      </c>
+      <c r="U190" s="54">
+        <v>95.87</v>
+      </c>
+      <c r="V190" s="53">
+        <v>0.7339611085591793</v>
+      </c>
       <c r="W190" s="53"/>
-      <c r="X190" s="55"/>
-      <c r="Y190" s="55"/>
-      <c r="Z190" s="53"/>
-      <c r="AA190" s="56"/>
+      <c r="X190" s="55">
+        <v>128.6379856115108</v>
+      </c>
+      <c r="Y190" s="55">
+        <v>35.92887828502527</v>
+      </c>
+      <c r="Z190" s="53">
+        <v>0.3155</v>
+      </c>
+      <c r="AA190" s="56">
+        <v>0.2236</v>
+      </c>
       <c r="AB190" s="57"/>
       <c r="AD190" s="35"/>
       <c r="AE190" s="35"/>
@@ -22098,30 +22978,74 @@
       <c r="C197" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D197" s="52"/>
-      <c r="E197" s="52"/>
-      <c r="F197" s="52"/>
-      <c r="G197" s="53"/>
-      <c r="H197" s="52"/>
-      <c r="I197" s="52"/>
-      <c r="J197" s="52"/>
-      <c r="K197" s="52"/>
-      <c r="L197" s="52"/>
-      <c r="M197" s="53"/>
+      <c r="D197" s="52">
+        <v>23770.94615247</v>
+      </c>
+      <c r="E197" s="52">
+        <v>10204.54</v>
+      </c>
+      <c r="F197" s="52">
+        <v>13566.406152469997</v>
+      </c>
+      <c r="G197" s="53">
+        <v>0.5707137639980029</v>
+      </c>
+      <c r="H197" s="52">
+        <v>14310.9577</v>
+      </c>
+      <c r="I197" s="52">
+        <v>7116.73</v>
+      </c>
+      <c r="J197" s="52">
+        <v>7389.335500000001</v>
+      </c>
+      <c r="K197" s="52">
+        <v>6605.049999999999</v>
+      </c>
+      <c r="L197" s="52">
+        <v>784.2855000000018</v>
+      </c>
+      <c r="M197" s="53">
+        <v>0.10613748692287713</v>
+      </c>
       <c r="N197" s="53"/>
-      <c r="O197" s="52"/>
-      <c r="P197" s="52"/>
-      <c r="Q197" s="52"/>
-      <c r="R197" s="53"/>
-      <c r="S197" s="54"/>
-      <c r="T197" s="54"/>
-      <c r="U197" s="54"/>
-      <c r="V197" s="53"/>
+      <c r="O197" s="52">
+        <v>6921.6222</v>
+      </c>
+      <c r="P197" s="52">
+        <v>511.68</v>
+      </c>
+      <c r="Q197" s="52">
+        <v>6409.9421999999995</v>
+      </c>
+      <c r="R197" s="53">
+        <v>0.9260751330807971</v>
+      </c>
+      <c r="S197" s="54">
+        <v>140.15</v>
+      </c>
+      <c r="T197" s="54">
+        <v>9.25</v>
+      </c>
+      <c r="U197" s="54">
+        <v>130.9</v>
+      </c>
+      <c r="V197" s="53">
+        <v>0.9339992864787727</v>
+      </c>
       <c r="W197" s="53"/>
-      <c r="X197" s="55"/>
-      <c r="Y197" s="55"/>
-      <c r="Z197" s="53"/>
-      <c r="AA197" s="56"/>
+      <c r="X197" s="55">
+        <v>333.8172972972973</v>
+      </c>
+      <c r="Y197" s="55">
+        <v>67.49902570438813</v>
+      </c>
+      <c r="Z197" s="53">
+        <v>0.30260000000000004</v>
+      </c>
+      <c r="AA197" s="56">
+        <v>0.398</v>
+      </c>
       <c r="AB197" s="57"/>
       <c r="AD197" s="35"/>
       <c r="AE197" s="35"/>
@@ -23115,30 +24039,74 @@
       <c r="C218" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D218" s="52"/>
-      <c r="E218" s="52"/>
-      <c r="F218" s="52"/>
-      <c r="G218" s="53"/>
-      <c r="H218" s="52"/>
-      <c r="I218" s="52"/>
-      <c r="J218" s="52"/>
-      <c r="K218" s="52"/>
-      <c r="L218" s="52"/>
-      <c r="M218" s="53"/>
+      <c r="D218" s="52">
+        <v>137109.56054889</v>
+      </c>
+      <c r="E218" s="52">
+        <v>30174.75</v>
+      </c>
+      <c r="F218" s="52">
+        <v>106934.81054889</v>
+      </c>
+      <c r="G218" s="53">
+        <v>0.7799223491111664</v>
+      </c>
+      <c r="H218" s="52">
+        <v>117394.569232</v>
+      </c>
+      <c r="I218" s="52">
+        <v>37161.14</v>
+      </c>
+      <c r="J218" s="52">
+        <v>99479.615032</v>
+      </c>
+      <c r="K218" s="52">
+        <v>37161.14</v>
+      </c>
+      <c r="L218" s="52">
+        <v>62318.475032</v>
+      </c>
+      <c r="M218" s="53">
+        <v>0.6264446742375689</v>
+      </c>
       <c r="N218" s="53"/>
-      <c r="O218" s="52"/>
-      <c r="P218" s="52"/>
-      <c r="Q218" s="52"/>
-      <c r="R218" s="53"/>
-      <c r="S218" s="54"/>
-      <c r="T218" s="54"/>
-      <c r="U218" s="54"/>
-      <c r="V218" s="53"/>
+      <c r="O218" s="52">
+        <v>17914.9542</v>
+      </c>
+      <c r="P218" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q218" s="52">
+        <v>17914.9542</v>
+      </c>
+      <c r="R218" s="53">
+        <v>1</v>
+      </c>
+      <c r="S218" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="T218" s="54">
+        <v>0</v>
+      </c>
+      <c r="U218" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="V218" s="53">
+        <v>1</v>
+      </c>
       <c r="W218" s="53"/>
-      <c r="X218" s="55"/>
-      <c r="Y218" s="55"/>
-      <c r="Z218" s="53"/>
-      <c r="AA218" s="56"/>
+      <c r="X218" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y218" s="55">
+        <v>54.93783457863793</v>
+      </c>
+      <c r="Z218" s="53">
+        <v>-0.23149999999999998</v>
+      </c>
+      <c r="AA218" s="56">
+        <v>0.1438</v>
+      </c>
       <c r="AB218" s="57"/>
       <c r="AD218" s="35"/>
       <c r="AE218" s="35"/>
@@ -23556,30 +24524,74 @@
       <c r="C225" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D225" s="52"/>
-      <c r="E225" s="52"/>
-      <c r="F225" s="52"/>
-      <c r="G225" s="53"/>
-      <c r="H225" s="52"/>
-      <c r="I225" s="52"/>
-      <c r="J225" s="52"/>
-      <c r="K225" s="52"/>
-      <c r="L225" s="52"/>
-      <c r="M225" s="53"/>
+      <c r="D225" s="52">
+        <v>412300.73261827</v>
+      </c>
+      <c r="E225" s="52">
+        <v>306038.55</v>
+      </c>
+      <c r="F225" s="52">
+        <v>106262.18261826999</v>
+      </c>
+      <c r="G225" s="53">
+        <v>0.257729793356087</v>
+      </c>
+      <c r="H225" s="52">
+        <v>306356.278672</v>
+      </c>
+      <c r="I225" s="52">
+        <v>255995.88</v>
+      </c>
+      <c r="J225" s="52">
+        <v>186357.488872</v>
+      </c>
+      <c r="K225" s="52">
+        <v>184261.79</v>
+      </c>
+      <c r="L225" s="52">
+        <v>2095.698871999979</v>
+      </c>
+      <c r="M225" s="53">
+        <v>0.011245584412437613</v>
+      </c>
       <c r="N225" s="53"/>
-      <c r="O225" s="52"/>
-      <c r="P225" s="52"/>
-      <c r="Q225" s="52"/>
-      <c r="R225" s="53"/>
-      <c r="S225" s="54"/>
-      <c r="T225" s="54"/>
-      <c r="U225" s="54"/>
-      <c r="V225" s="53"/>
+      <c r="O225" s="52">
+        <v>119998.7898</v>
+      </c>
+      <c r="P225" s="52">
+        <v>71734.09</v>
+      </c>
+      <c r="Q225" s="52">
+        <v>48264.6998</v>
+      </c>
+      <c r="R225" s="53">
+        <v>0.4022098879533867</v>
+      </c>
+      <c r="S225" s="54">
+        <v>2412.45</v>
+      </c>
+      <c r="T225" s="54">
+        <v>1531.67</v>
+      </c>
+      <c r="U225" s="54">
+        <v>880.7799999999997</v>
+      </c>
+      <c r="V225" s="53">
+        <v>0.3650977222325851</v>
+      </c>
       <c r="W225" s="53"/>
-      <c r="X225" s="55"/>
-      <c r="Y225" s="55"/>
-      <c r="Z225" s="53"/>
-      <c r="AA225" s="56"/>
+      <c r="X225" s="55">
+        <v>32.67196589343657</v>
+      </c>
+      <c r="Y225" s="55">
+        <v>43.91570973337064</v>
+      </c>
+      <c r="Z225" s="53">
+        <v>0.1635</v>
+      </c>
+      <c r="AA225" s="56">
+        <v>0.257</v>
+      </c>
       <c r="AB225" s="57"/>
       <c r="AD225" s="35"/>
       <c r="AE225" s="35"/>
@@ -23987,30 +24999,74 @@
       <c r="C232" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D232" s="52"/>
-      <c r="E232" s="52"/>
-      <c r="F232" s="52"/>
-      <c r="G232" s="53"/>
-      <c r="H232" s="52"/>
-      <c r="I232" s="52"/>
-      <c r="J232" s="52"/>
-      <c r="K232" s="52"/>
-      <c r="L232" s="52"/>
-      <c r="M232" s="53"/>
+      <c r="D232" s="52">
+        <v>8795.02836582</v>
+      </c>
+      <c r="E232" s="52">
+        <v>0</v>
+      </c>
+      <c r="F232" s="52">
+        <v>8795.02836582</v>
+      </c>
+      <c r="G232" s="53">
+        <v>1</v>
+      </c>
+      <c r="H232" s="52">
+        <v>6369.1218</v>
+      </c>
+      <c r="I232" s="52">
+        <v>397</v>
+      </c>
+      <c r="J232" s="52">
+        <v>4527.894</v>
+      </c>
+      <c r="K232" s="52">
+        <v>397</v>
+      </c>
+      <c r="L232" s="52">
+        <v>4130.894</v>
+      </c>
+      <c r="M232" s="53">
+        <v>0.9123212690049723</v>
+      </c>
       <c r="N232" s="53"/>
-      <c r="O232" s="52"/>
-      <c r="P232" s="52"/>
-      <c r="Q232" s="52"/>
-      <c r="R232" s="53"/>
-      <c r="S232" s="54"/>
-      <c r="T232" s="54"/>
-      <c r="U232" s="54"/>
-      <c r="V232" s="53"/>
+      <c r="O232" s="52">
+        <v>1841.2278</v>
+      </c>
+      <c r="P232" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q232" s="52">
+        <v>1841.2278</v>
+      </c>
+      <c r="R232" s="53">
+        <v>1</v>
+      </c>
+      <c r="S232" s="54">
+        <v>36.92</v>
+      </c>
+      <c r="T232" s="54">
+        <v>0</v>
+      </c>
+      <c r="U232" s="54">
+        <v>36.92</v>
+      </c>
+      <c r="V232" s="53">
+        <v>1</v>
+      </c>
       <c r="W232" s="53"/>
-      <c r="X232" s="55"/>
-      <c r="Y232" s="55"/>
-      <c r="Z232" s="53"/>
-      <c r="AA232" s="56"/>
+      <c r="X232" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y232" s="55">
+        <v>65.70711175027087</v>
+      </c>
+      <c r="Z232" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA232" s="56">
+        <v>0.2758</v>
+      </c>
       <c r="AB232" s="57"/>
       <c r="AD232" s="35"/>
       <c r="AE232" s="35"/>
@@ -24372,30 +25428,74 @@
       <c r="C239" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D239" s="52"/>
-      <c r="E239" s="52"/>
-      <c r="F239" s="52"/>
-      <c r="G239" s="53"/>
-      <c r="H239" s="52"/>
-      <c r="I239" s="52"/>
-      <c r="J239" s="52"/>
-      <c r="K239" s="52"/>
-      <c r="L239" s="52"/>
-      <c r="M239" s="53"/>
+      <c r="D239" s="52">
+        <v>27503.13664251</v>
+      </c>
+      <c r="E239" s="52">
+        <v>0</v>
+      </c>
+      <c r="F239" s="52">
+        <v>27503.13664251</v>
+      </c>
+      <c r="G239" s="53">
+        <v>1</v>
+      </c>
+      <c r="H239" s="52">
+        <v>19683.280628</v>
+      </c>
+      <c r="I239" s="52">
+        <v>0</v>
+      </c>
+      <c r="J239" s="52">
+        <v>10693.531628</v>
+      </c>
+      <c r="K239" s="52">
+        <v>0</v>
+      </c>
+      <c r="L239" s="52">
+        <v>10693.531628</v>
+      </c>
+      <c r="M239" s="53">
+        <v>1</v>
+      </c>
       <c r="N239" s="53"/>
-      <c r="O239" s="52"/>
-      <c r="P239" s="52"/>
-      <c r="Q239" s="52"/>
-      <c r="R239" s="53"/>
-      <c r="S239" s="54"/>
-      <c r="T239" s="54"/>
-      <c r="U239" s="54"/>
-      <c r="V239" s="53"/>
+      <c r="O239" s="52">
+        <v>8989.749</v>
+      </c>
+      <c r="P239" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q239" s="52">
+        <v>8989.749</v>
+      </c>
+      <c r="R239" s="53">
+        <v>1</v>
+      </c>
+      <c r="S239" s="54">
+        <v>180.16</v>
+      </c>
+      <c r="T239" s="54">
+        <v>0</v>
+      </c>
+      <c r="U239" s="54">
+        <v>180.16</v>
+      </c>
+      <c r="V239" s="53">
+        <v>1</v>
+      </c>
       <c r="W239" s="53"/>
-      <c r="X239" s="55"/>
-      <c r="Y239" s="55"/>
-      <c r="Z239" s="53"/>
-      <c r="AA239" s="56"/>
+      <c r="X239" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y239" s="55">
+        <v>43.40506224750221</v>
+      </c>
+      <c r="Z239" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA239" s="56">
+        <v>0.2843</v>
+      </c>
       <c r="AB239" s="57"/>
       <c r="AD239" s="35"/>
       <c r="AE239" s="35"/>
@@ -24757,30 +25857,74 @@
       <c r="C246" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D246" s="52"/>
-      <c r="E246" s="52"/>
-      <c r="F246" s="52"/>
-      <c r="G246" s="53"/>
-      <c r="H246" s="52"/>
-      <c r="I246" s="52"/>
-      <c r="J246" s="52"/>
-      <c r="K246" s="52"/>
-      <c r="L246" s="52"/>
-      <c r="M246" s="53"/>
+      <c r="D246" s="52">
+        <v>40670.1518342</v>
+      </c>
+      <c r="E246" s="52">
+        <v>0</v>
+      </c>
+      <c r="F246" s="52">
+        <v>40670.1518342</v>
+      </c>
+      <c r="G246" s="53">
+        <v>1</v>
+      </c>
+      <c r="H246" s="52">
+        <v>29498.3116992</v>
+      </c>
+      <c r="I246" s="52">
+        <v>0</v>
+      </c>
+      <c r="J246" s="52">
+        <v>24964.3288992</v>
+      </c>
+      <c r="K246" s="52">
+        <v>0</v>
+      </c>
+      <c r="L246" s="52">
+        <v>24964.3288992</v>
+      </c>
+      <c r="M246" s="53">
+        <v>1</v>
+      </c>
       <c r="N246" s="53"/>
-      <c r="O246" s="52"/>
-      <c r="P246" s="52"/>
-      <c r="Q246" s="52"/>
-      <c r="R246" s="53"/>
-      <c r="S246" s="54"/>
-      <c r="T246" s="54"/>
-      <c r="U246" s="54"/>
-      <c r="V246" s="53"/>
+      <c r="O246" s="52">
+        <v>4533.9828</v>
+      </c>
+      <c r="P246" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q246" s="52">
+        <v>4533.9828</v>
+      </c>
+      <c r="R246" s="53">
+        <v>1</v>
+      </c>
+      <c r="S246" s="54">
+        <v>90.88</v>
+      </c>
+      <c r="T246" s="54">
+        <v>0</v>
+      </c>
+      <c r="U246" s="54">
+        <v>90.88</v>
+      </c>
+      <c r="V246" s="53">
+        <v>1</v>
+      </c>
       <c r="W246" s="53"/>
-      <c r="X246" s="55"/>
-      <c r="Y246" s="55"/>
-      <c r="Z246" s="53"/>
-      <c r="AA246" s="56"/>
+      <c r="X246" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y246" s="55">
+        <v>122.92957895026407</v>
+      </c>
+      <c r="Z246" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA246" s="56">
+        <v>0.2747</v>
+      </c>
       <c r="AB246" s="57"/>
       <c r="AD246" s="35"/>
       <c r="AE246" s="35"/>
@@ -25142,30 +26286,74 @@
       <c r="C253" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D253" s="52"/>
-      <c r="E253" s="52"/>
-      <c r="F253" s="52"/>
-      <c r="G253" s="53"/>
-      <c r="H253" s="52"/>
-      <c r="I253" s="52"/>
-      <c r="J253" s="52"/>
-      <c r="K253" s="52"/>
-      <c r="L253" s="52"/>
-      <c r="M253" s="53"/>
+      <c r="D253" s="52">
+        <v>21396.50036782</v>
+      </c>
+      <c r="E253" s="52">
+        <v>0</v>
+      </c>
+      <c r="F253" s="52">
+        <v>21396.50036782</v>
+      </c>
+      <c r="G253" s="53">
+        <v>1</v>
+      </c>
+      <c r="H253" s="52">
+        <v>15378.244372</v>
+      </c>
+      <c r="I253" s="52">
+        <v>0</v>
+      </c>
+      <c r="J253" s="52">
+        <v>8344.608772</v>
+      </c>
+      <c r="K253" s="52">
+        <v>0</v>
+      </c>
+      <c r="L253" s="52">
+        <v>8344.608772</v>
+      </c>
+      <c r="M253" s="53">
+        <v>1</v>
+      </c>
       <c r="N253" s="53"/>
-      <c r="O253" s="52"/>
-      <c r="P253" s="52"/>
-      <c r="Q253" s="52"/>
-      <c r="R253" s="53"/>
-      <c r="S253" s="54"/>
-      <c r="T253" s="54"/>
-      <c r="U253" s="54"/>
-      <c r="V253" s="53"/>
+      <c r="O253" s="52">
+        <v>7033.6356</v>
+      </c>
+      <c r="P253" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q253" s="52">
+        <v>7033.6356</v>
+      </c>
+      <c r="R253" s="53">
+        <v>1</v>
+      </c>
+      <c r="S253" s="54">
+        <v>140.9</v>
+      </c>
+      <c r="T253" s="54">
+        <v>0</v>
+      </c>
+      <c r="U253" s="54">
+        <v>140.9</v>
+      </c>
+      <c r="V253" s="53">
+        <v>1</v>
+      </c>
       <c r="W253" s="53"/>
-      <c r="X253" s="55"/>
-      <c r="Y253" s="55"/>
-      <c r="Z253" s="53"/>
-      <c r="AA253" s="56"/>
+      <c r="X253" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y253" s="55">
+        <v>42.71295951611073</v>
+      </c>
+      <c r="Z253" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA253" s="56">
+        <v>0.2813</v>
+      </c>
       <c r="AB253" s="57"/>
       <c r="AD253" s="35"/>
       <c r="AE253" s="35"/>
@@ -25527,30 +26715,74 @@
       <c r="C260" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="D260" s="52"/>
-      <c r="E260" s="52"/>
-      <c r="F260" s="52"/>
-      <c r="G260" s="53"/>
-      <c r="H260" s="52"/>
-      <c r="I260" s="52"/>
-      <c r="J260" s="52"/>
-      <c r="K260" s="52"/>
-      <c r="L260" s="52"/>
-      <c r="M260" s="53"/>
+      <c r="D260" s="52">
+        <v>239296.88379393</v>
+      </c>
+      <c r="E260" s="52">
+        <v>10598.48</v>
+      </c>
+      <c r="F260" s="52">
+        <v>228698.40379393</v>
+      </c>
+      <c r="G260" s="53">
+        <v>0.9557099121728352</v>
+      </c>
+      <c r="H260" s="52">
+        <v>203192.691868</v>
+      </c>
+      <c r="I260" s="52">
+        <v>18235.02</v>
+      </c>
+      <c r="J260" s="52">
+        <v>175849.529668</v>
+      </c>
+      <c r="K260" s="52">
+        <v>16839.61</v>
+      </c>
+      <c r="L260" s="52">
+        <v>159009.91966800002</v>
+      </c>
+      <c r="M260" s="53">
+        <v>0.9042385269281482</v>
+      </c>
       <c r="N260" s="53"/>
-      <c r="O260" s="52"/>
-      <c r="P260" s="52"/>
-      <c r="Q260" s="52"/>
-      <c r="R260" s="53"/>
-      <c r="S260" s="54"/>
-      <c r="T260" s="54"/>
-      <c r="U260" s="54"/>
-      <c r="V260" s="53"/>
+      <c r="O260" s="52">
+        <v>27343.1622</v>
+      </c>
+      <c r="P260" s="52">
+        <v>1395.41</v>
+      </c>
+      <c r="Q260" s="52">
+        <v>25947.7522</v>
+      </c>
+      <c r="R260" s="53">
+        <v>0.9489667658117465</v>
+      </c>
+      <c r="S260" s="54">
+        <v>547.57</v>
+      </c>
+      <c r="T260" s="54">
+        <v>27.84</v>
+      </c>
+      <c r="U260" s="54">
+        <v>519.73</v>
+      </c>
+      <c r="V260" s="53">
+        <v>0.9491571853826908</v>
+      </c>
       <c r="W260" s="53"/>
-      <c r="X260" s="55"/>
-      <c r="Y260" s="55"/>
-      <c r="Z260" s="53"/>
-      <c r="AA260" s="56"/>
+      <c r="X260" s="55">
+        <v>-274.30100574712645</v>
+      </c>
+      <c r="Y260" s="55">
+        <v>65.93529946112827</v>
+      </c>
+      <c r="Z260" s="53">
+        <v>-0.7204999999999999</v>
+      </c>
+      <c r="AA260" s="56">
+        <v>0.1509</v>
+      </c>
       <c r="AB260" s="57"/>
       <c r="AD260" s="35"/>
       <c r="AE260" s="35"/>
@@ -26274,10 +27506,10 @@
         <v>0</v>
       </c>
       <c r="D4" s="52">
-        <v>35.10000000000582</v>
+        <v>321.320000000007</v>
       </c>
       <c r="E4" s="52">
-        <v>-35.10000000000582</v>
+        <v>-321.320000000007</v>
       </c>
       <c r="F4" s="52">
         <v>0</v>
@@ -26301,13 +27533,13 @@
         <v>0</v>
       </c>
       <c r="M4" s="52">
-        <v>-7035.100000000006</v>
+        <v>-7321.320000000007</v>
       </c>
       <c r="N4" s="54">
         <v>20</v>
       </c>
       <c r="O4" s="58">
-        <v>-100.50142857142866</v>
+        <v>-104.59028571428581</v>
       </c>
     </row>
     <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -26338,10 +27570,10 @@
         <v>0</v>
       </c>
       <c r="D6" s="52">
-        <v>3846.6199999999953</v>
+        <v>16504.429999999993</v>
       </c>
       <c r="E6" s="52">
-        <v>-3846.6199999999953</v>
+        <v>-16504.429999999993</v>
       </c>
       <c r="F6" s="52">
         <v>7</v>
@@ -26365,13 +27597,13 @@
         <v>0</v>
       </c>
       <c r="M6" s="52">
-        <v>-24112.219999999994</v>
+        <v>-36770.02999999999</v>
       </c>
       <c r="N6" s="54">
         <v>-52.5</v>
       </c>
       <c r="O6" s="58">
-        <v>-53.88205586592177</v>
+        <v>-82.16766480446925</v>
       </c>
       <c r="Q6" s="35" t="s">
         <v>121</v>
@@ -26405,10 +27637,10 @@
         <v>0</v>
       </c>
       <c r="D8" s="52">
-        <v>300</v>
+        <v>462</v>
       </c>
       <c r="E8" s="52">
-        <v>-300</v>
+        <v>-462</v>
       </c>
       <c r="F8" s="52"/>
       <c r="G8" s="53">
@@ -26428,13 +27660,13 @@
         <v>0</v>
       </c>
       <c r="M8" s="52">
-        <v>-940</v>
+        <v>-1102</v>
       </c>
       <c r="N8" s="54">
         <v>-34.75</v>
       </c>
       <c r="O8" s="58">
-        <v>50.13333333333333</v>
+        <v>58.77333333333333</v>
       </c>
     </row>
     <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -26529,10 +27761,10 @@
         <v>0</v>
       </c>
       <c r="D12" s="52">
-        <v>11748.359999999986</v>
+        <v>60555.25999999998</v>
       </c>
       <c r="E12" s="52">
-        <v>-11748.359999999986</v>
+        <v>-60555.25999999998</v>
       </c>
       <c r="F12" s="52">
         <v>3</v>
@@ -26556,13 +27788,13 @@
         <v>0</v>
       </c>
       <c r="M12" s="52">
-        <v>-14385.359999999986</v>
+        <v>-63192.25999999998</v>
       </c>
       <c r="N12" s="54">
         <v>53</v>
       </c>
       <c r="O12" s="58">
-        <v>-208.48347826086936</v>
+        <v>-915.8298550724635</v>
       </c>
       <c r="Q12" s="35" t="s">
         <v>123</v>
@@ -26596,10 +27828,10 @@
         <v>0</v>
       </c>
       <c r="D14" s="52">
-        <v>9389.019999999997</v>
+        <v>13833.64</v>
       </c>
       <c r="E14" s="52">
-        <v>-9389.019999999997</v>
+        <v>-13833.64</v>
       </c>
       <c r="F14" s="52">
         <v>0</v>
@@ -26623,13 +27855,13 @@
         <v>0</v>
       </c>
       <c r="M14" s="52">
-        <v>-12389.019999999997</v>
+        <v>-16833.64</v>
       </c>
       <c r="N14" s="54">
         <v>-112</v>
       </c>
       <c r="O14" s="58">
-        <v>110.61624999999997</v>
+        <v>150.30035714285714</v>
       </c>
     </row>
     <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -26660,10 +27892,10 @@
         <v>0</v>
       </c>
       <c r="D16" s="52">
-        <v>552.5999999999985</v>
+        <v>4363.379999999997</v>
       </c>
       <c r="E16" s="52">
-        <v>-552.5999999999985</v>
+        <v>-4363.379999999997</v>
       </c>
       <c r="F16" s="52"/>
       <c r="G16" s="53">
@@ -26685,13 +27917,13 @@
         <v>0</v>
       </c>
       <c r="M16" s="52">
-        <v>-3552.5999999999985</v>
+        <v>-7363.379999999997</v>
       </c>
       <c r="N16" s="54">
         <v>-86.75</v>
       </c>
       <c r="O16" s="58">
-        <v>40.952161383285286</v>
+        <v>84.88046109510084</v>
       </c>
     </row>
     <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -26722,10 +27954,10 @@
         <v>0</v>
       </c>
       <c r="D18" s="52">
-        <v>5440.75</v>
+        <v>14297.850000000006</v>
       </c>
       <c r="E18" s="52">
-        <v>-5440.75</v>
+        <v>-14297.850000000006</v>
       </c>
       <c r="F18" s="52">
         <v>0</v>
@@ -26749,13 +27981,13 @@
         <v>0</v>
       </c>
       <c r="M18" s="52">
-        <v>-13640.75</v>
+        <v>-22497.850000000006</v>
       </c>
       <c r="N18" s="54">
         <v>-269</v>
       </c>
       <c r="O18" s="58">
-        <v>72.17328042328042</v>
+        <v>119.03624338624341</v>
       </c>
       <c r="Q18" s="35" t="s">
         <v>124</v>
@@ -26845,10 +28077,10 @@
         <v>0</v>
       </c>
       <c r="D22" s="52">
-        <v>7755.09</v>
+        <v>10950.11</v>
       </c>
       <c r="E22" s="52">
-        <v>-7755.09</v>
+        <v>-10950.11</v>
       </c>
       <c r="F22" s="52">
         <v>3</v>
@@ -26868,7 +28100,7 @@
         <v>0</v>
       </c>
       <c r="M22" s="52">
-        <v>-7752.09</v>
+        <v>-10947.11</v>
       </c>
       <c r="N22" s="54"/>
       <c r="O22" s="58">
@@ -26903,10 +28135,10 @@
         <v>0</v>
       </c>
       <c r="D24" s="52">
-        <v>499.0499999999993</v>
+        <v>9478.690000000002</v>
       </c>
       <c r="E24" s="52">
-        <v>-499.0499999999993</v>
+        <v>-9478.690000000002</v>
       </c>
       <c r="F24" s="52">
         <v>3</v>
@@ -26924,7 +28156,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="52">
-        <v>-496.0499999999993</v>
+        <v>-9475.690000000002</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="58">
@@ -26959,10 +28191,10 @@
         <v>0</v>
       </c>
       <c r="D26" s="52">
-        <v>-440.2600000000002</v>
+        <v>1159.83</v>
       </c>
       <c r="E26" s="52">
-        <v>440.2600000000002</v>
+        <v>-1159.83</v>
       </c>
       <c r="F26" s="52">
         <v>0</v>
@@ -26984,13 +28216,13 @@
         <v>0</v>
       </c>
       <c r="M26" s="52">
-        <v>440.2600000000002</v>
+        <v>-1159.83</v>
       </c>
       <c r="N26" s="54">
         <v>-143.25</v>
       </c>
       <c r="O26" s="58">
-        <v>-3.0733682373472964</v>
+        <v>8.096544502617801</v>
       </c>
     </row>
     <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -27021,10 +28253,10 @@
         <v>0</v>
       </c>
       <c r="D28" s="52">
-        <v>-945.4600000000028</v>
+        <v>-902.1700000000019</v>
       </c>
       <c r="E28" s="52">
-        <v>945.4600000000028</v>
+        <v>902.1700000000019</v>
       </c>
       <c r="F28" s="52">
         <v>0</v>
@@ -27044,13 +28276,13 @@
         <v>0</v>
       </c>
       <c r="M28" s="52">
-        <v>945.4600000000028</v>
+        <v>902.1700000000019</v>
       </c>
       <c r="N28" s="54">
         <v>-148.5</v>
       </c>
       <c r="O28" s="58">
-        <v>-6.366734006734025</v>
+        <v>-6.075218855218868</v>
       </c>
     </row>
     <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -27081,10 +28313,10 @@
         <v>0</v>
       </c>
       <c r="D30" s="52">
-        <v>0</v>
+        <v>93.54999999999927</v>
       </c>
       <c r="E30" s="52">
-        <v>0</v>
+        <v>-93.54999999999927</v>
       </c>
       <c r="F30" s="52">
         <v>0</v>
@@ -27104,13 +28336,13 @@
         <v>0</v>
       </c>
       <c r="M30" s="52">
-        <v>0</v>
+        <v>-93.54999999999927</v>
       </c>
       <c r="N30" s="54">
         <v>-5</v>
       </c>
       <c r="O30" s="58">
-        <v>0</v>
+        <v>18.709999999999855</v>
       </c>
     </row>
     <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -27327,16 +28559,16 @@
         <v>52040.560000000005</v>
       </c>
       <c r="D38" s="52">
-        <v>577.7200000000012</v>
+        <v>10303.779999999999</v>
       </c>
       <c r="E38" s="52">
-        <v>51462.840000000004</v>
+        <v>41736.780000000006</v>
       </c>
       <c r="F38" s="52">
         <v>0</v>
       </c>
       <c r="G38" s="53">
-        <v>0.9888986590459441</v>
+        <v>0.8020048208551177</v>
       </c>
       <c r="H38" s="53">
         <v>0.1750921737769</v>
@@ -27347,10 +28579,10 @@
         <v>0</v>
       </c>
       <c r="L38" s="53">
-        <v>0.9888986590459441</v>
+        <v>0.8020048208551177</v>
       </c>
       <c r="M38" s="52">
-        <v>51462.840000000004</v>
+        <v>41736.780000000006</v>
       </c>
       <c r="N38" s="54"/>
       <c r="O38" s="58">
@@ -27619,10 +28851,10 @@
         <v>0</v>
       </c>
       <c r="D48" s="99">
-        <v>1728.0999999999985</v>
+        <v>2218.25</v>
       </c>
       <c r="E48" s="99">
-        <v>-1728.0999999999985</v>
+        <v>-2218.25</v>
       </c>
       <c r="F48" s="99"/>
       <c r="G48" s="100">
@@ -27642,13 +28874,13 @@
         <v>0</v>
       </c>
       <c r="M48" s="99">
-        <v>-4258.0999999999985</v>
+        <v>-4748.25</v>
       </c>
       <c r="N48" s="98">
         <v>-44.75</v>
       </c>
       <c r="O48" s="60">
-        <v>95.15307262569829</v>
+        <v>106.10614525139665</v>
       </c>
     </row>
     <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -27738,10 +28970,10 @@
         <v>0</v>
       </c>
       <c r="D52" s="99">
-        <v>2775.6800000000076</v>
+        <v>2942.1800000000076</v>
       </c>
       <c r="E52" s="99">
-        <v>-2775.6800000000076</v>
+        <v>-2942.1800000000076</v>
       </c>
       <c r="F52" s="99"/>
       <c r="G52" s="100">
@@ -27763,13 +28995,13 @@
         <v>0</v>
       </c>
       <c r="M52" s="99">
-        <v>-4055.6800000000076</v>
+        <v>-4222.180000000008</v>
       </c>
       <c r="N52" s="98">
         <v>-304.75</v>
       </c>
       <c r="O52" s="60">
-        <v>14.869587534372164</v>
+        <v>15.480036663611394</v>
       </c>
     </row>
     <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -27800,10 +29032,10 @@
         <v>0</v>
       </c>
       <c r="D54" s="99">
-        <v>0</v>
+        <v>1024.2599999999998</v>
       </c>
       <c r="E54" s="99">
-        <v>0</v>
+        <v>-1024.2599999999998</v>
       </c>
       <c r="F54" s="99"/>
       <c r="G54" s="100">
@@ -27825,13 +29057,13 @@
         <v>0</v>
       </c>
       <c r="M54" s="99">
-        <v>-640</v>
+        <v>-1664.2599999999998</v>
       </c>
       <c r="N54" s="98">
         <v>-11.25</v>
       </c>
       <c r="O54" s="60">
-        <v>-134.73684210526315</v>
+        <v>-350.37052631578945</v>
       </c>
     </row>
     <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -28050,10 +29282,10 @@
         <v>0</v>
       </c>
       <c r="D64" s="99">
-        <v>4470.959999999999</v>
+        <v>11037.14</v>
       </c>
       <c r="E64" s="99">
-        <v>-4470.959999999999</v>
+        <v>-11037.14</v>
       </c>
       <c r="F64" s="99"/>
       <c r="G64" s="100">
@@ -28073,7 +29305,7 @@
         <v>0</v>
       </c>
       <c r="M64" s="99">
-        <v>-6220.959999999999</v>
+        <v>-12787.14</v>
       </c>
       <c r="N64" s="98"/>
       <c r="O64" s="60">
@@ -28108,14 +29340,14 @@
         <v>34650.399999999965</v>
       </c>
       <c r="D66" s="99">
-        <v>16579.28</v>
+        <v>21673.070000000007</v>
       </c>
       <c r="E66" s="99">
-        <v>18071.119999999966</v>
+        <v>12977.329999999958</v>
       </c>
       <c r="F66" s="99"/>
       <c r="G66" s="100">
-        <v>0.5215270242190562</v>
+        <v>0.37452179484219433</v>
       </c>
       <c r="H66" s="100">
         <v>0.256265521519856</v>
@@ -28130,16 +29362,16 @@
         <v>3200</v>
       </c>
       <c r="L66" s="100">
-        <v>0.4291759979682769</v>
+        <v>0.28217076859141504</v>
       </c>
       <c r="M66" s="99">
-        <v>14871.119999999966</v>
+        <v>9777.329999999958</v>
       </c>
       <c r="N66" s="98">
         <v>-1014.25</v>
       </c>
       <c r="O66" s="60">
-        <v>-15.917709392560841</v>
+        <v>-10.465432164838061</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -28153,14 +29385,14 @@
         <v>10598.48</v>
       </c>
       <c r="D67" s="99">
-        <v>18229.7</v>
+        <v>18235.02</v>
       </c>
       <c r="E67" s="99">
-        <v>-7631.220000000001</v>
+        <v>-7636.540000000001</v>
       </c>
       <c r="F67" s="99"/>
       <c r="G67" s="100">
-        <v>-0.7200296646311548</v>
+        <v>-0.7205316234026012</v>
       </c>
       <c r="H67" s="100">
         <f>'Deliverables Sheet'!AA256</f>
@@ -28171,10 +29403,10 @@
         <v>0</v>
       </c>
       <c r="L67" s="100">
-        <v>-0.7200296646311548</v>
+        <v>-0.7205316234026012</v>
       </c>
       <c r="M67" s="99">
-        <v>-7631.220000000001</v>
+        <v>-7636.540000000001</v>
       </c>
       <c r="N67" s="98"/>
       <c r="O67" s="60">
@@ -28309,10 +29541,10 @@
         <v>0</v>
       </c>
       <c r="D71" s="99">
-        <v>0</v>
+        <v>397</v>
       </c>
       <c r="E71" s="99">
-        <v>0</v>
+        <v>-397</v>
       </c>
       <c r="F71" s="99"/>
       <c r="G71" s="100">
@@ -28330,7 +29562,7 @@
         <v>0</v>
       </c>
       <c r="M71" s="99">
-        <v>0</v>
+        <v>-397</v>
       </c>
       <c r="N71" s="98"/>
       <c r="O71" s="60">
@@ -28382,22 +29614,22 @@
         <v>98702.24999999996</v>
       </c>
       <c r="D74" s="104">
-        <v>90534.78999999996</v>
+        <v>206941.06999999998</v>
       </c>
       <c r="E74" s="105">
-        <v>8167.459999999994</v>
+        <v>-108238.82000000004</v>
       </c>
       <c r="F74" s="106" t="s">
         <v>128</v>
       </c>
       <c r="G74" s="107">
-        <v>0.08274846824667115</v>
+        <v>-1.0966195806073324</v>
       </c>
       <c r="H74" s="108" t="s">
         <v>129</v>
       </c>
       <c r="I74" s="109">
-        <v>-0.6288118052020095</v>
+        <v>-1.8081798540560132</v>
       </c>
       <c r="J74" s="36"/>
       <c r="K74" s="36"/>
@@ -28952,10 +30184,10 @@
         <v>638.02</v>
       </c>
       <c r="D4" s="54">
-        <v>600.25</v>
+        <v>605.75</v>
       </c>
       <c r="E4" s="54">
-        <v>37.76999999999998</v>
+        <v>32.26999999999998</v>
       </c>
       <c r="F4" s="54">
         <v>0</v>
@@ -29011,10 +30243,10 @@
         <v>363.57</v>
       </c>
       <c r="D6" s="54">
-        <v>168.25</v>
+        <v>217</v>
       </c>
       <c r="E6" s="54">
-        <v>195.32</v>
+        <v>146.57</v>
       </c>
       <c r="F6" s="54"/>
       <c r="G6" s="54"/>
@@ -29178,10 +30410,10 @@
         <v>1124.47</v>
       </c>
       <c r="D12" s="54">
-        <v>667.75</v>
+        <v>750.5</v>
       </c>
       <c r="E12" s="54">
-        <v>456.72</v>
+        <v>373.97</v>
       </c>
       <c r="F12" s="54"/>
       <c r="G12" s="54"/>
@@ -29237,10 +30469,10 @@
         <v>501.83</v>
       </c>
       <c r="D14" s="54">
-        <v>354.75</v>
+        <v>358.75</v>
       </c>
       <c r="E14" s="54">
-        <v>147.07999999999998</v>
+        <v>143.07999999999998</v>
       </c>
       <c r="F14" s="54"/>
       <c r="G14" s="54"/>
@@ -29296,10 +30528,10 @@
         <v>223.22</v>
       </c>
       <c r="D16" s="54">
-        <v>129</v>
+        <v>216.5</v>
       </c>
       <c r="E16" s="54">
-        <v>94.22</v>
+        <v>6.719999999999999</v>
       </c>
       <c r="F16" s="54"/>
       <c r="G16" s="54"/>
@@ -29348,10 +30580,10 @@
         <v>685.48</v>
       </c>
       <c r="D18" s="54">
-        <v>610</v>
+        <v>660.25</v>
       </c>
       <c r="E18" s="54">
-        <v>75.48000000000002</v>
+        <v>25.230000000000018</v>
       </c>
       <c r="F18" s="54"/>
       <c r="G18" s="54"/>
@@ -29450,10 +30682,10 @@
         <v>193.32</v>
       </c>
       <c r="D22" s="54">
-        <v>2.75</v>
+        <v>27.25</v>
       </c>
       <c r="E22" s="54">
-        <v>190.57</v>
+        <v>166.07</v>
       </c>
       <c r="F22" s="54"/>
       <c r="G22" s="54"/>
@@ -29560,10 +30792,10 @@
         <v>139.07</v>
       </c>
       <c r="D26" s="54">
-        <v>147.75</v>
+        <v>167.75</v>
       </c>
       <c r="E26" s="54">
-        <v>-8.680000000000007</v>
+        <v>-28.680000000000007</v>
       </c>
       <c r="F26" s="54"/>
       <c r="G26" s="54"/>
@@ -29661,10 +30893,10 @@
         <v>147.9</v>
       </c>
       <c r="D30" s="54">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="E30" s="54">
-        <v>142.9</v>
+        <v>141.4</v>
       </c>
       <c r="F30" s="54"/>
       <c r="G30" s="54"/>
@@ -30143,10 +31375,10 @@
         <v>110.44</v>
       </c>
       <c r="D48" s="54">
-        <v>87</v>
+        <v>95.5</v>
       </c>
       <c r="E48" s="54">
-        <v>23.439999999999998</v>
+        <v>14.939999999999998</v>
       </c>
       <c r="F48" s="54"/>
       <c r="G48" s="54"/>
@@ -30306,10 +31538,10 @@
         <v>125.17</v>
       </c>
       <c r="D54" s="54">
-        <v>23.75</v>
+        <v>32.75</v>
       </c>
       <c r="E54" s="54">
-        <v>101.42</v>
+        <v>92.42</v>
       </c>
       <c r="F54" s="54"/>
       <c r="G54" s="54"/>
@@ -30608,10 +31840,10 @@
         <v>2412.45</v>
       </c>
       <c r="D66" s="54">
-        <v>1444.92</v>
+        <v>1531.67</v>
       </c>
       <c r="E66" s="54">
-        <v>967.5299999999997</v>
+        <v>880.7799999999997</v>
       </c>
       <c r="F66" s="54"/>
       <c r="G66" s="54"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-23T01:20:05Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -10342,66 +10342,66 @@
         <v>267886.84883856</v>
       </c>
       <c r="E8" s="52">
-        <v>216530.08</v>
+        <v>238732.97</v>
       </c>
       <c r="F8" s="52">
-        <v>51356.768838560005</v>
+        <v>29153.87883855999</v>
       </c>
       <c r="G8" s="53">
-        <v>0.19171067583653492</v>
+        <v>0.10882907826553799</v>
       </c>
       <c r="H8" s="52">
         <v>225410.5455298</v>
       </c>
       <c r="I8" s="52">
-        <v>168279</v>
+        <v>188603.61</v>
       </c>
       <c r="J8" s="52">
         <v>193787.2413298</v>
       </c>
       <c r="K8" s="52">
-        <v>138094.41999999998</v>
+        <v>158312.05</v>
       </c>
       <c r="L8" s="52">
-        <v>55692.821329800005</v>
+        <v>35475.1913298</v>
       </c>
       <c r="M8" s="53">
-        <v>0.2873915792785257</v>
+        <v>0.18306257463785228</v>
       </c>
       <c r="N8" s="53"/>
       <c r="O8" s="52">
         <v>31623.3042</v>
       </c>
       <c r="P8" s="52">
-        <v>30184.58</v>
+        <v>30291.56</v>
       </c>
       <c r="Q8" s="52">
-        <v>1438.724199999997</v>
+        <v>1331.7441999999974</v>
       </c>
       <c r="R8" s="53">
-        <v>0.045495694912234916</v>
+        <v>0.042112746712912985</v>
       </c>
       <c r="S8" s="54">
         <v>638.02</v>
       </c>
       <c r="T8" s="54">
-        <v>605.75</v>
+        <v>608.25</v>
       </c>
       <c r="U8" s="54">
-        <v>32.26999999999998</v>
+        <v>29.769999999999982</v>
       </c>
       <c r="V8" s="53">
-        <v>0.05057835177580637</v>
+        <v>0.04665997931099336</v>
       </c>
       <c r="W8" s="53"/>
       <c r="X8" s="55">
-        <v>79.65510524143625</v>
+        <v>82.4157172215372</v>
       </c>
       <c r="Y8" s="55">
         <v>66.57519091683645</v>
       </c>
       <c r="Z8" s="53">
-        <v>0.2228</v>
+        <v>0.21</v>
       </c>
       <c r="AA8" s="56">
         <v>0.1586</v>
@@ -10834,72 +10834,72 @@
         <v>103</v>
       </c>
       <c r="D15" s="52">
-        <v>129996.91589078</v>
+        <v>131888.19931324</v>
       </c>
       <c r="E15" s="62">
         <v>85864.08</v>
       </c>
       <c r="F15" s="52">
-        <v>44132.83589078</v>
+        <v>46024.11931324001</v>
       </c>
       <c r="G15" s="53">
-        <v>0.3394914070719897</v>
+        <v>0.34896313356990183</v>
       </c>
       <c r="H15" s="52">
-        <v>101885.523895</v>
+        <v>103653.873895</v>
       </c>
       <c r="I15" s="52">
-        <v>90641.75</v>
+        <v>91501.08</v>
       </c>
       <c r="J15" s="52">
-        <v>83735.424895</v>
+        <v>85503.774895</v>
       </c>
       <c r="K15" s="52">
-        <v>80523.92</v>
+        <v>80310.8</v>
       </c>
       <c r="L15" s="52">
-        <v>3211.5048950000055</v>
+        <v>5192.974894999992</v>
       </c>
       <c r="M15" s="53">
-        <v>0.03835300171972699</v>
+        <v>0.060733867029579086</v>
       </c>
       <c r="N15" s="53"/>
       <c r="O15" s="52">
         <v>18150.099</v>
       </c>
       <c r="P15" s="52">
-        <v>10117.83</v>
+        <v>11190.28</v>
       </c>
       <c r="Q15" s="52">
-        <v>8032.268999999998</v>
+        <v>6959.818999999998</v>
       </c>
       <c r="R15" s="53">
-        <v>0.44254684230647995</v>
+        <v>0.3834590103337727</v>
       </c>
       <c r="S15" s="54">
         <v>363.57</v>
       </c>
       <c r="T15" s="54">
-        <v>217</v>
+        <v>242.5</v>
       </c>
       <c r="U15" s="54">
-        <v>146.57</v>
+        <v>121.07</v>
       </c>
       <c r="V15" s="53">
-        <v>0.40314107324586734</v>
+        <v>0.33300327309734024</v>
       </c>
       <c r="W15" s="53"/>
       <c r="X15" s="55">
-        <v>-22.016912442396315</v>
+        <v>-23.245360824742267</v>
       </c>
       <c r="Y15" s="55">
-        <v>77.32043896850674</v>
+        <v>77.65856758874499</v>
       </c>
       <c r="Z15" s="53">
-        <v>-0.0556</v>
+        <v>-0.06570000000000001</v>
       </c>
       <c r="AA15" s="56">
-        <v>0.2162</v>
+        <v>0.2141</v>
       </c>
       <c r="AB15" s="57"/>
       <c r="AD15" s="35"/>
@@ -12248,54 +12248,54 @@
         <v>328046.93216</v>
       </c>
       <c r="I36" s="52">
-        <v>276899.86</v>
+        <v>276751.71</v>
       </c>
       <c r="J36" s="52">
         <v>271925.57216000004</v>
       </c>
       <c r="K36" s="52">
-        <v>244422.38999999998</v>
+        <v>243603.26</v>
       </c>
       <c r="L36" s="52">
-        <v>27503.182160000055</v>
+        <v>28322.31216000003</v>
       </c>
       <c r="M36" s="53">
-        <v>0.10114231604454355</v>
+        <v>0.10415464766710239</v>
       </c>
       <c r="N36" s="53"/>
       <c r="O36" s="52">
         <v>56121.36</v>
       </c>
       <c r="P36" s="52">
-        <v>32477.47</v>
+        <v>33148.45</v>
       </c>
       <c r="Q36" s="52">
-        <v>23643.89</v>
+        <v>22972.910000000003</v>
       </c>
       <c r="R36" s="53">
-        <v>0.4212993056476179</v>
+        <v>0.40934343002379137</v>
       </c>
       <c r="S36" s="54">
         <v>1124.47</v>
       </c>
       <c r="T36" s="54">
-        <v>750.5</v>
+        <v>766.5</v>
       </c>
       <c r="U36" s="54">
-        <v>373.97</v>
+        <v>357.97</v>
       </c>
       <c r="V36" s="53">
-        <v>0.3325744572998835</v>
+        <v>0.31834553167269913</v>
       </c>
       <c r="W36" s="53"/>
       <c r="X36" s="55">
-        <v>-23.38727514990007</v>
+        <v>-22.7058056099152</v>
       </c>
       <c r="Y36" s="55">
         <v>61.532703026350184</v>
       </c>
       <c r="Z36" s="53">
-        <v>-0.0677</v>
+        <v>-0.06709999999999999</v>
       </c>
       <c r="AA36" s="56">
         <v>0.1742</v>
@@ -12743,19 +12743,19 @@
         <v>94098.31685</v>
       </c>
       <c r="I43" s="52">
-        <v>56107.33</v>
+        <v>56767.07</v>
       </c>
       <c r="J43" s="52">
         <v>69042.08885</v>
       </c>
       <c r="K43" s="52">
-        <v>40219.090000000004</v>
+        <v>40878.83</v>
       </c>
       <c r="L43" s="52">
-        <v>28822.998849999996</v>
+        <v>28163.25885</v>
       </c>
       <c r="M43" s="53">
-        <v>0.41746997128983876</v>
+        <v>0.40791435078372484</v>
       </c>
       <c r="N43" s="53"/>
       <c r="O43" s="52">
@@ -12784,13 +12784,13 @@
       </c>
       <c r="W43" s="53"/>
       <c r="X43" s="55">
-        <v>-6.02787456445993</v>
+        <v>-7.866871080139372</v>
       </c>
       <c r="Y43" s="55">
         <v>68.07122423898531</v>
       </c>
       <c r="Z43" s="53">
-        <v>-0.0401</v>
+        <v>-0.052300000000000006</v>
       </c>
       <c r="AA43" s="56">
         <v>0.2663</v>
@@ -13240,19 +13240,19 @@
         <v>50582.36785</v>
       </c>
       <c r="I50" s="52">
-        <v>29574.96</v>
+        <v>29601.04</v>
       </c>
       <c r="J50" s="52">
         <v>39438.99025</v>
       </c>
       <c r="K50" s="52">
-        <v>20218.23</v>
+        <v>20244.31</v>
       </c>
       <c r="L50" s="52">
-        <v>19220.760250000003</v>
+        <v>19194.68025</v>
       </c>
       <c r="M50" s="53">
-        <v>0.48735426866056747</v>
+        <v>0.4866929941240065</v>
       </c>
       <c r="N50" s="53"/>
       <c r="O50" s="52">
@@ -13281,13 +13281,13 @@
       </c>
       <c r="W50" s="53"/>
       <c r="X50" s="55">
-        <v>17.3280831408776</v>
+        <v>17.207621247113163</v>
       </c>
       <c r="Y50" s="55">
         <v>67.69550512136009</v>
       </c>
       <c r="Z50" s="53">
-        <v>0.11259999999999999</v>
+        <v>0.1118</v>
       </c>
       <c r="AA50" s="56">
         <v>0.23</v>
@@ -13735,54 +13735,54 @@
         <v>109364.9721</v>
       </c>
       <c r="I57" s="52">
-        <v>109618.36</v>
+        <v>110172.19</v>
       </c>
       <c r="J57" s="52">
         <v>75135.0159</v>
       </c>
       <c r="K57" s="52">
-        <v>78027.66</v>
+        <v>78187.74</v>
       </c>
       <c r="L57" s="52">
-        <v>-2892.644100000005</v>
+        <v>-3052.7241000000067</v>
       </c>
       <c r="M57" s="53">
-        <v>-0.03849928113211466</v>
+        <v>-0.04062984566427711</v>
       </c>
       <c r="N57" s="53"/>
       <c r="O57" s="52">
         <v>34229.9562</v>
       </c>
       <c r="P57" s="52">
-        <v>31590.7</v>
+        <v>31984.45</v>
       </c>
       <c r="Q57" s="52">
-        <v>2639.2562</v>
+        <v>2245.5062</v>
       </c>
       <c r="R57" s="53">
-        <v>0.07710369784230106</v>
+        <v>0.06560061563853242</v>
       </c>
       <c r="S57" s="54">
         <v>685.48</v>
       </c>
       <c r="T57" s="54">
-        <v>660.25</v>
+        <v>669</v>
       </c>
       <c r="U57" s="54">
-        <v>25.230000000000018</v>
+        <v>16.480000000000018</v>
       </c>
       <c r="V57" s="53">
-        <v>0.036806325494544</v>
+        <v>0.02404154752873901</v>
       </c>
       <c r="W57" s="53"/>
       <c r="X57" s="55">
-        <v>27.559439606209768</v>
+        <v>26.371136023916293</v>
       </c>
       <c r="Y57" s="55">
         <v>67.00679527854935</v>
       </c>
       <c r="Z57" s="53">
-        <v>0.1424</v>
+        <v>0.138</v>
       </c>
       <c r="AA57" s="56">
         <v>0.2958</v>
@@ -14631,54 +14631,54 @@
         <v>39055.77825</v>
       </c>
       <c r="I71" s="52">
-        <v>20931.54</v>
+        <v>22176.82</v>
       </c>
       <c r="J71" s="52">
         <v>29537.289750000004</v>
       </c>
       <c r="K71" s="52">
-        <v>19627.920000000002</v>
+        <v>19672.02</v>
       </c>
       <c r="L71" s="52">
-        <v>9909.369750000002</v>
+        <v>9865.269750000003</v>
       </c>
       <c r="M71" s="53">
-        <v>0.3354867638118355</v>
+        <v>0.3339937358335323</v>
       </c>
       <c r="N71" s="53"/>
       <c r="O71" s="52">
         <v>9518.4885</v>
       </c>
       <c r="P71" s="52">
-        <v>1303.62</v>
+        <v>2504.8</v>
       </c>
       <c r="Q71" s="52">
-        <v>8214.8685</v>
+        <v>7013.688499999999</v>
       </c>
       <c r="R71" s="53">
-        <v>0.8630433813099634</v>
+        <v>0.7368489755490065</v>
       </c>
       <c r="S71" s="54">
         <v>193.32</v>
       </c>
       <c r="T71" s="54">
-        <v>27.25</v>
+        <v>52.75</v>
       </c>
       <c r="U71" s="54">
-        <v>166.07</v>
+        <v>140.57</v>
       </c>
       <c r="V71" s="53">
-        <v>0.8590420028967515</v>
+        <v>0.7271363542313263</v>
       </c>
       <c r="W71" s="53"/>
       <c r="X71" s="55">
-        <v>-377.2884403669725</v>
+        <v>-218.50976303317535</v>
       </c>
       <c r="Y71" s="55">
         <v>72.28396616733912</v>
       </c>
       <c r="Z71" s="53">
-        <v>-0.9653</v>
+        <v>-1.0822</v>
       </c>
       <c r="AA71" s="56">
         <v>0.2635</v>
@@ -15116,19 +15116,19 @@
         <v>55589.7822</v>
       </c>
       <c r="I78" s="52">
-        <v>41397.62</v>
+        <v>41600.05</v>
       </c>
       <c r="J78" s="52">
         <v>32594.7534</v>
       </c>
       <c r="K78" s="52">
-        <v>32996.44</v>
+        <v>33198.87</v>
       </c>
       <c r="L78" s="52">
-        <v>-401.6866000000009</v>
+        <v>-604.1166000000012</v>
       </c>
       <c r="M78" s="53">
-        <v>-0.01232365819954327</v>
+        <v>-0.018534166912887312</v>
       </c>
       <c r="N78" s="53"/>
       <c r="O78" s="52">
@@ -15157,13 +15157,13 @@
       </c>
       <c r="W78" s="53"/>
       <c r="X78" s="55">
-        <v>20.133751868460386</v>
+        <v>18.92340807174888</v>
       </c>
       <c r="Y78" s="55">
         <v>49.060202993773025</v>
       </c>
       <c r="Z78" s="53">
-        <v>0.07519999999999999</v>
+        <v>0.0707</v>
       </c>
       <c r="AA78" s="56">
         <v>0.2941</v>
@@ -17887,56 +17887,56 @@
         <v>103</v>
       </c>
       <c r="D120" s="52">
-        <v>21404.8192765</v>
+        <v>21978.65615186</v>
       </c>
       <c r="E120" s="52">
         <v>0</v>
       </c>
       <c r="F120" s="52">
-        <v>21404.8192765</v>
+        <v>21978.65615186</v>
       </c>
       <c r="G120" s="53">
         <v>1</v>
       </c>
       <c r="H120" s="52">
-        <v>17514.092529</v>
+        <v>17872.766891</v>
       </c>
       <c r="I120" s="52">
         <v>0</v>
       </c>
       <c r="J120" s="52">
-        <v>13318.886529000001</v>
+        <v>13579.636691</v>
       </c>
       <c r="K120" s="52">
         <v>0</v>
       </c>
       <c r="L120" s="52">
-        <v>13318.886529000001</v>
+        <v>13579.636691</v>
       </c>
       <c r="M120" s="53">
         <v>1</v>
       </c>
       <c r="N120" s="53"/>
       <c r="O120" s="52">
-        <v>4195.206</v>
+        <v>4293.1302</v>
       </c>
       <c r="P120" s="52">
         <v>0</v>
       </c>
       <c r="Q120" s="52">
-        <v>4195.206</v>
+        <v>4293.1302</v>
       </c>
       <c r="R120" s="53">
         <v>1</v>
       </c>
       <c r="S120" s="54">
-        <v>84.05</v>
+        <v>86.01</v>
       </c>
       <c r="T120" s="54">
         <v>0</v>
       </c>
       <c r="U120" s="54">
-        <v>84.05</v>
+        <v>86.01</v>
       </c>
       <c r="V120" s="53">
         <v>1</v>
@@ -17946,13 +17946,13 @@
         <v>0</v>
       </c>
       <c r="Y120" s="55">
-        <v>46.29062162403328</v>
+        <v>47.73734752772933</v>
       </c>
       <c r="Z120" s="53">
         <v>0</v>
       </c>
       <c r="AA120" s="56">
-        <v>0.1818</v>
+        <v>0.1868</v>
       </c>
       <c r="AB120" s="57"/>
       <c r="AD120" s="35"/>
@@ -22022,7 +22022,7 @@
         <v>9226.2731</v>
       </c>
       <c r="I183" s="52">
-        <v>4727.04</v>
+        <v>5421.03</v>
       </c>
       <c r="J183" s="52">
         <v>2977.1135000000004</v>
@@ -22041,35 +22041,35 @@
         <v>6249.1596</v>
       </c>
       <c r="P183" s="52">
-        <v>1884.76</v>
+        <v>2578.75</v>
       </c>
       <c r="Q183" s="52">
-        <v>4364.3996</v>
+        <v>3670.4096</v>
       </c>
       <c r="R183" s="53">
-        <v>0.6983978453678795</v>
+        <v>0.5873445126925547</v>
       </c>
       <c r="S183" s="54">
         <v>125.17</v>
       </c>
       <c r="T183" s="54">
-        <v>32.75</v>
+        <v>49.25</v>
       </c>
       <c r="U183" s="54">
-        <v>92.42</v>
+        <v>75.92</v>
       </c>
       <c r="V183" s="53">
-        <v>0.7383558360629544</v>
+        <v>0.6065351122473436</v>
       </c>
       <c r="W183" s="53"/>
       <c r="X183" s="55">
-        <v>23.348396946564886</v>
+        <v>1.4349238578680203</v>
       </c>
       <c r="Y183" s="55">
         <v>61.286703843093385</v>
       </c>
       <c r="Z183" s="53">
-        <v>0.1392</v>
+        <v>0.0129</v>
       </c>
       <c r="AA183" s="56">
         <v>0.454</v>
@@ -24540,19 +24540,19 @@
         <v>306356.278672</v>
       </c>
       <c r="I225" s="52">
-        <v>255995.88</v>
+        <v>256209</v>
       </c>
       <c r="J225" s="52">
         <v>186357.488872</v>
       </c>
       <c r="K225" s="52">
-        <v>184261.79</v>
+        <v>184474.91</v>
       </c>
       <c r="L225" s="52">
-        <v>2095.698871999979</v>
+        <v>1882.5788719999837</v>
       </c>
       <c r="M225" s="53">
-        <v>0.011245584412437613</v>
+        <v>0.010101975957043706</v>
       </c>
       <c r="N225" s="53"/>
       <c r="O225" s="52">
@@ -24581,13 +24581,13 @@
       </c>
       <c r="W225" s="53"/>
       <c r="X225" s="55">
-        <v>32.67196589343657</v>
+        <v>32.53282365000294</v>
       </c>
       <c r="Y225" s="55">
         <v>43.91570973337064</v>
       </c>
       <c r="Z225" s="53">
-        <v>0.1635</v>
+        <v>0.1628</v>
       </c>
       <c r="AA225" s="56">
         <v>0.257</v>
@@ -27503,19 +27503,19 @@
         <v>25</v>
       </c>
       <c r="C4" s="52">
-        <v>0</v>
+        <v>22202.890000000014</v>
       </c>
       <c r="D4" s="52">
-        <v>321.320000000007</v>
+        <v>20645.929999999993</v>
       </c>
       <c r="E4" s="52">
-        <v>-321.320000000007</v>
+        <v>1556.960000000021</v>
       </c>
       <c r="F4" s="52">
         <v>0</v>
       </c>
       <c r="G4" s="53">
-        <v>0</v>
+        <v>0.0701242045517507</v>
       </c>
       <c r="H4" s="53">
         <v>0.2149</v>
@@ -27530,16 +27530,16 @@
         <v>7000</v>
       </c>
       <c r="L4" s="53">
-        <v>0</v>
+        <v>-0.24515006830191816</v>
       </c>
       <c r="M4" s="52">
-        <v>-7321.320000000007</v>
+        <v>-5443.039999999979</v>
       </c>
       <c r="N4" s="54">
         <v>20</v>
       </c>
       <c r="O4" s="58">
-        <v>-104.59028571428581</v>
+        <v>-77.75771428571399</v>
       </c>
     </row>
     <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -27570,10 +27570,10 @@
         <v>0</v>
       </c>
       <c r="D6" s="52">
-        <v>16504.429999999993</v>
+        <v>17363.759999999995</v>
       </c>
       <c r="E6" s="52">
-        <v>-16504.429999999993</v>
+        <v>-17363.759999999995</v>
       </c>
       <c r="F6" s="52">
         <v>7</v>
@@ -27597,13 +27597,13 @@
         <v>0</v>
       </c>
       <c r="M6" s="52">
-        <v>-36770.02999999999</v>
+        <v>-37629.35999999999</v>
       </c>
       <c r="N6" s="54">
         <v>-52.5</v>
       </c>
       <c r="O6" s="58">
-        <v>-82.16766480446925</v>
+        <v>-84.08795530726256</v>
       </c>
       <c r="Q6" s="35" t="s">
         <v>121</v>
@@ -27761,10 +27761,10 @@
         <v>0</v>
       </c>
       <c r="D12" s="52">
-        <v>60555.25999999998</v>
+        <v>60407.110000000015</v>
       </c>
       <c r="E12" s="52">
-        <v>-60555.25999999998</v>
+        <v>-60407.110000000015</v>
       </c>
       <c r="F12" s="52">
         <v>3</v>
@@ -27788,13 +27788,13 @@
         <v>0</v>
       </c>
       <c r="M12" s="52">
-        <v>-63192.25999999998</v>
+        <v>-63044.110000000015</v>
       </c>
       <c r="N12" s="54">
         <v>53</v>
       </c>
       <c r="O12" s="58">
-        <v>-915.8298550724635</v>
+        <v>-913.6827536231887</v>
       </c>
       <c r="Q12" s="35" t="s">
         <v>123</v>
@@ -27828,10 +27828,10 @@
         <v>0</v>
       </c>
       <c r="D14" s="52">
-        <v>13833.64</v>
+        <v>14493.379999999997</v>
       </c>
       <c r="E14" s="52">
-        <v>-13833.64</v>
+        <v>-14493.379999999997</v>
       </c>
       <c r="F14" s="52">
         <v>0</v>
@@ -27855,13 +27855,13 @@
         <v>0</v>
       </c>
       <c r="M14" s="52">
-        <v>-16833.64</v>
+        <v>-17493.379999999997</v>
       </c>
       <c r="N14" s="54">
         <v>-112</v>
       </c>
       <c r="O14" s="58">
-        <v>150.30035714285714</v>
+        <v>156.19089285714284</v>
       </c>
     </row>
     <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -27892,10 +27892,10 @@
         <v>0</v>
       </c>
       <c r="D16" s="52">
-        <v>4363.379999999997</v>
+        <v>4389.459999999999</v>
       </c>
       <c r="E16" s="52">
-        <v>-4363.379999999997</v>
+        <v>-4389.459999999999</v>
       </c>
       <c r="F16" s="52"/>
       <c r="G16" s="53">
@@ -27917,13 +27917,13 @@
         <v>0</v>
       </c>
       <c r="M16" s="52">
-        <v>-7363.379999999997</v>
+        <v>-7389.459999999999</v>
       </c>
       <c r="N16" s="54">
         <v>-86.75</v>
       </c>
       <c r="O16" s="58">
-        <v>84.88046109510084</v>
+        <v>85.18109510086454</v>
       </c>
     </row>
     <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -27954,10 +27954,10 @@
         <v>0</v>
       </c>
       <c r="D18" s="52">
-        <v>14297.850000000006</v>
+        <v>14851.680000000008</v>
       </c>
       <c r="E18" s="52">
-        <v>-14297.850000000006</v>
+        <v>-14851.680000000008</v>
       </c>
       <c r="F18" s="52">
         <v>0</v>
@@ -27981,13 +27981,13 @@
         <v>0</v>
       </c>
       <c r="M18" s="52">
-        <v>-22497.850000000006</v>
+        <v>-23051.680000000008</v>
       </c>
       <c r="N18" s="54">
         <v>-269</v>
       </c>
       <c r="O18" s="58">
-        <v>119.03624338624341</v>
+        <v>121.96656084656088</v>
       </c>
       <c r="Q18" s="35" t="s">
         <v>124</v>
@@ -28077,10 +28077,10 @@
         <v>0</v>
       </c>
       <c r="D22" s="52">
-        <v>10950.11</v>
+        <v>12195.39</v>
       </c>
       <c r="E22" s="52">
-        <v>-10950.11</v>
+        <v>-12195.39</v>
       </c>
       <c r="F22" s="52">
         <v>3</v>
@@ -28100,7 +28100,7 @@
         <v>0</v>
       </c>
       <c r="M22" s="52">
-        <v>-10947.11</v>
+        <v>-12192.39</v>
       </c>
       <c r="N22" s="54"/>
       <c r="O22" s="58">
@@ -28135,10 +28135,10 @@
         <v>0</v>
       </c>
       <c r="D24" s="52">
-        <v>9478.690000000002</v>
+        <v>9681.120000000003</v>
       </c>
       <c r="E24" s="52">
-        <v>-9478.690000000002</v>
+        <v>-9681.120000000003</v>
       </c>
       <c r="F24" s="52">
         <v>3</v>
@@ -28156,7 +28156,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="52">
-        <v>-9475.690000000002</v>
+        <v>-9678.120000000003</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="58">
@@ -29032,10 +29032,10 @@
         <v>0</v>
       </c>
       <c r="D54" s="99">
-        <v>1024.2599999999998</v>
+        <v>1718.2499999999995</v>
       </c>
       <c r="E54" s="99">
-        <v>-1024.2599999999998</v>
+        <v>-1718.2499999999995</v>
       </c>
       <c r="F54" s="99"/>
       <c r="G54" s="100">
@@ -29057,13 +29057,13 @@
         <v>0</v>
       </c>
       <c r="M54" s="99">
-        <v>-1664.2599999999998</v>
+        <v>-2358.2499999999995</v>
       </c>
       <c r="N54" s="98">
         <v>-11.25</v>
       </c>
       <c r="O54" s="60">
-        <v>-350.37052631578945</v>
+        <v>-496.47368421052624</v>
       </c>
     </row>
     <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -29340,14 +29340,14 @@
         <v>34650.399999999965</v>
       </c>
       <c r="D66" s="99">
-        <v>21673.070000000007</v>
+        <v>21886.190000000002</v>
       </c>
       <c r="E66" s="99">
-        <v>12977.329999999958</v>
+        <v>12764.209999999963</v>
       </c>
       <c r="F66" s="99"/>
       <c r="G66" s="100">
-        <v>0.37452179484219433</v>
+        <v>0.3683712164938926</v>
       </c>
       <c r="H66" s="100">
         <v>0.256265521519856</v>
@@ -29362,16 +29362,16 @@
         <v>3200</v>
       </c>
       <c r="L66" s="100">
-        <v>0.28217076859141504</v>
+        <v>0.2760201902431133</v>
       </c>
       <c r="M66" s="99">
-        <v>9777.329999999958</v>
+        <v>9564.209999999963</v>
       </c>
       <c r="N66" s="98">
         <v>-1014.25</v>
       </c>
       <c r="O66" s="60">
-        <v>-10.465432164838061</v>
+        <v>-10.237313352956878</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -29611,25 +29611,25 @@
         <v>127</v>
       </c>
       <c r="C74" s="104">
-        <v>98702.24999999996</v>
+        <v>120905.13999999997</v>
       </c>
       <c r="D74" s="104">
-        <v>206941.06999999998</v>
+        <v>231571.33</v>
       </c>
       <c r="E74" s="105">
-        <v>-108238.82000000004</v>
+        <v>-110666.19000000003</v>
       </c>
       <c r="F74" s="106" t="s">
         <v>128</v>
       </c>
       <c r="G74" s="107">
-        <v>-1.0966195806073324</v>
+        <v>-0.915314187635034</v>
       </c>
       <c r="H74" s="108" t="s">
         <v>129</v>
       </c>
       <c r="I74" s="109">
-        <v>-1.8081798540560132</v>
+        <v>-1.496204297021616</v>
       </c>
       <c r="J74" s="36"/>
       <c r="K74" s="36"/>
@@ -30184,10 +30184,10 @@
         <v>638.02</v>
       </c>
       <c r="D4" s="54">
-        <v>605.75</v>
+        <v>608.25</v>
       </c>
       <c r="E4" s="54">
-        <v>32.26999999999998</v>
+        <v>29.769999999999982</v>
       </c>
       <c r="F4" s="54">
         <v>0</v>
@@ -30243,10 +30243,10 @@
         <v>363.57</v>
       </c>
       <c r="D6" s="54">
-        <v>217</v>
+        <v>242.5</v>
       </c>
       <c r="E6" s="54">
-        <v>146.57</v>
+        <v>121.07</v>
       </c>
       <c r="F6" s="54"/>
       <c r="G6" s="54"/>
@@ -30410,10 +30410,10 @@
         <v>1124.47</v>
       </c>
       <c r="D12" s="54">
-        <v>750.5</v>
+        <v>766.5</v>
       </c>
       <c r="E12" s="54">
-        <v>373.97</v>
+        <v>357.97</v>
       </c>
       <c r="F12" s="54"/>
       <c r="G12" s="54"/>
@@ -30580,10 +30580,10 @@
         <v>685.48</v>
       </c>
       <c r="D18" s="54">
-        <v>660.25</v>
+        <v>669</v>
       </c>
       <c r="E18" s="54">
-        <v>25.230000000000018</v>
+        <v>16.480000000000018</v>
       </c>
       <c r="F18" s="54"/>
       <c r="G18" s="54"/>
@@ -30682,10 +30682,10 @@
         <v>193.32</v>
       </c>
       <c r="D22" s="54">
-        <v>27.25</v>
+        <v>52.75</v>
       </c>
       <c r="E22" s="54">
-        <v>166.07</v>
+        <v>140.57</v>
       </c>
       <c r="F22" s="54"/>
       <c r="G22" s="54"/>
@@ -31045,13 +31045,13 @@
         <v>48</v>
       </c>
       <c r="C36" s="54">
-        <v>84.05</v>
+        <v>86.01</v>
       </c>
       <c r="D36" s="54">
         <v>0</v>
       </c>
       <c r="E36" s="54">
-        <v>84.05</v>
+        <v>86.01</v>
       </c>
       <c r="F36" s="54"/>
       <c r="G36" s="54"/>
@@ -31538,10 +31538,10 @@
         <v>125.17</v>
       </c>
       <c r="D54" s="54">
-        <v>32.75</v>
+        <v>49.25</v>
       </c>
       <c r="E54" s="54">
-        <v>92.42</v>
+        <v>75.92</v>
       </c>
       <c r="F54" s="54"/>
       <c r="G54" s="54"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-24T01:37:33Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -10354,7 +10354,7 @@
         <v>225410.5455298</v>
       </c>
       <c r="I8" s="52">
-        <v>188603.61</v>
+        <v>188979.91</v>
       </c>
       <c r="J8" s="52">
         <v>193787.2413298</v>
@@ -10373,35 +10373,35 @@
         <v>31623.3042</v>
       </c>
       <c r="P8" s="52">
-        <v>30291.56</v>
+        <v>30667.86</v>
       </c>
       <c r="Q8" s="52">
-        <v>1331.7441999999974</v>
+        <v>955.4441999999981</v>
       </c>
       <c r="R8" s="53">
-        <v>0.042112746712912985</v>
+        <v>0.030213294409633454</v>
       </c>
       <c r="S8" s="54">
         <v>638.02</v>
       </c>
       <c r="T8" s="54">
-        <v>608.25</v>
+        <v>616.75</v>
       </c>
       <c r="U8" s="54">
-        <v>29.769999999999982</v>
+        <v>21.269999999999982</v>
       </c>
       <c r="V8" s="53">
-        <v>0.04665997931099336</v>
+        <v>0.03333751293062911</v>
       </c>
       <c r="W8" s="53"/>
       <c r="X8" s="55">
-        <v>82.4157172215372</v>
+        <v>80.66973652209161</v>
       </c>
       <c r="Y8" s="55">
         <v>66.57519091683645</v>
       </c>
       <c r="Z8" s="53">
-        <v>0.21</v>
+        <v>0.2084</v>
       </c>
       <c r="AA8" s="56">
         <v>0.1586</v>
@@ -10834,72 +10834,72 @@
         <v>103</v>
       </c>
       <c r="D15" s="52">
-        <v>131888.19931324</v>
+        <v>132076.08820213</v>
       </c>
       <c r="E15" s="62">
-        <v>85864.08</v>
+        <v>127883.98</v>
       </c>
       <c r="F15" s="52">
-        <v>46024.11931324001</v>
+        <v>4192.108202129995</v>
       </c>
       <c r="G15" s="53">
-        <v>0.34896313356990183</v>
+        <v>0.031740099659178046</v>
       </c>
       <c r="H15" s="52">
-        <v>103653.873895</v>
+        <v>103822.973895</v>
       </c>
       <c r="I15" s="52">
-        <v>91501.08</v>
+        <v>92794.34</v>
       </c>
       <c r="J15" s="52">
-        <v>85503.774895</v>
+        <v>85672.874895</v>
       </c>
       <c r="K15" s="52">
-        <v>80310.8</v>
+        <v>80310.79999999999</v>
       </c>
       <c r="L15" s="52">
-        <v>5192.974894999992</v>
+        <v>5362.0748950000125</v>
       </c>
       <c r="M15" s="53">
-        <v>0.060733867029579086</v>
+        <v>0.0625877782386984</v>
       </c>
       <c r="N15" s="53"/>
       <c r="O15" s="52">
         <v>18150.099</v>
       </c>
       <c r="P15" s="52">
-        <v>11190.28</v>
+        <v>12483.54</v>
       </c>
       <c r="Q15" s="52">
-        <v>6959.818999999998</v>
+        <v>5666.5589999999975</v>
       </c>
       <c r="R15" s="53">
-        <v>0.3834590103337727</v>
+        <v>0.31220540449944645</v>
       </c>
       <c r="S15" s="54">
         <v>363.57</v>
       </c>
       <c r="T15" s="54">
-        <v>242.5</v>
+        <v>272.5</v>
       </c>
       <c r="U15" s="54">
-        <v>121.07</v>
+        <v>91.07</v>
       </c>
       <c r="V15" s="53">
-        <v>0.33300327309734024</v>
+        <v>0.25048821409907307</v>
       </c>
       <c r="W15" s="53"/>
       <c r="X15" s="55">
-        <v>-23.245360824742267</v>
+        <v>128.76932110091744</v>
       </c>
       <c r="Y15" s="55">
-        <v>77.65856758874499</v>
+        <v>77.71024646458726</v>
       </c>
       <c r="Z15" s="53">
-        <v>-0.06570000000000001</v>
+        <v>0.27440000000000003</v>
       </c>
       <c r="AA15" s="56">
-        <v>0.2141</v>
+        <v>0.2139</v>
       </c>
       <c r="AB15" s="57"/>
       <c r="AD15" s="35"/>
@@ -12236,66 +12236,66 @@
         <v>397238.61073204</v>
       </c>
       <c r="E36" s="52">
-        <v>259347.71</v>
+        <v>352623.79</v>
       </c>
       <c r="F36" s="52">
-        <v>137890.90073204003</v>
+        <v>44614.82073204004</v>
       </c>
       <c r="G36" s="53">
-        <v>0.3471236103608651</v>
+        <v>0.112312397452561</v>
       </c>
       <c r="H36" s="52">
         <v>328046.93216</v>
       </c>
       <c r="I36" s="52">
-        <v>276751.71</v>
+        <v>277449.99</v>
       </c>
       <c r="J36" s="52">
         <v>271925.57216000004</v>
       </c>
       <c r="K36" s="52">
-        <v>243603.26</v>
+        <v>243603.25999999998</v>
       </c>
       <c r="L36" s="52">
-        <v>28322.31216000003</v>
+        <v>28322.31216000006</v>
       </c>
       <c r="M36" s="53">
-        <v>0.10415464766710239</v>
+        <v>0.1041546476671025</v>
       </c>
       <c r="N36" s="53"/>
       <c r="O36" s="52">
         <v>56121.36</v>
       </c>
       <c r="P36" s="52">
-        <v>33148.45</v>
+        <v>33846.73</v>
       </c>
       <c r="Q36" s="52">
-        <v>22972.910000000003</v>
+        <v>22274.629999999997</v>
       </c>
       <c r="R36" s="53">
-        <v>0.40934343002379137</v>
+        <v>0.39690110859751077</v>
       </c>
       <c r="S36" s="54">
         <v>1124.47</v>
       </c>
       <c r="T36" s="54">
-        <v>766.5</v>
+        <v>783</v>
       </c>
       <c r="U36" s="54">
-        <v>357.97</v>
+        <v>341.47</v>
       </c>
       <c r="V36" s="53">
-        <v>0.31834553167269913</v>
+        <v>0.3036719521196653</v>
       </c>
       <c r="W36" s="53"/>
       <c r="X36" s="55">
-        <v>-22.7058056099152</v>
+        <v>96.00740740740741</v>
       </c>
       <c r="Y36" s="55">
         <v>61.532703026350184</v>
       </c>
       <c r="Z36" s="53">
-        <v>-0.06709999999999999</v>
+        <v>0.2132</v>
       </c>
       <c r="AA36" s="56">
         <v>0.1742</v>
@@ -12731,13 +12731,13 @@
         <v>128258.49930985</v>
       </c>
       <c r="E43" s="52">
-        <v>53944.83</v>
+        <v>115314.55</v>
       </c>
       <c r="F43" s="52">
-        <v>74313.66930985</v>
+        <v>12943.949309849995</v>
       </c>
       <c r="G43" s="53">
-        <v>0.5794054172606622</v>
+        <v>0.10092079183446305</v>
       </c>
       <c r="H43" s="52">
         <v>94098.31685</v>
@@ -12784,13 +12784,13 @@
       </c>
       <c r="W43" s="53"/>
       <c r="X43" s="55">
-        <v>-7.866871080139372</v>
+        <v>163.1985505226481</v>
       </c>
       <c r="Y43" s="55">
         <v>68.07122423898531</v>
       </c>
       <c r="Z43" s="53">
-        <v>-0.052300000000000006</v>
+        <v>0.5077</v>
       </c>
       <c r="AA43" s="56">
         <v>0.2663</v>
@@ -13723,31 +13723,31 @@
         <v>155296.79012754</v>
       </c>
       <c r="E57" s="52">
-        <v>127814.48</v>
+        <v>155296.8</v>
       </c>
       <c r="F57" s="52">
-        <v>27482.31012754001</v>
+        <v>-0.009872459981124848</v>
       </c>
       <c r="G57" s="53">
-        <v>0.17696637583410268</v>
+        <v>-6.357156495647419e-8</v>
       </c>
       <c r="H57" s="52">
         <v>109364.9721</v>
       </c>
       <c r="I57" s="52">
-        <v>110172.19</v>
+        <v>110254.03</v>
       </c>
       <c r="J57" s="52">
         <v>75135.0159</v>
       </c>
       <c r="K57" s="52">
-        <v>78187.74</v>
+        <v>78269.58</v>
       </c>
       <c r="L57" s="52">
-        <v>-3052.7241000000067</v>
+        <v>-3134.5641000000032</v>
       </c>
       <c r="M57" s="53">
-        <v>-0.04062984566427711</v>
+        <v>-0.04171908480290883</v>
       </c>
       <c r="N57" s="53"/>
       <c r="O57" s="52">
@@ -13776,13 +13776,13 @@
       </c>
       <c r="W57" s="53"/>
       <c r="X57" s="55">
-        <v>26.371136023916293</v>
+        <v>67.32850523168908</v>
       </c>
       <c r="Y57" s="55">
         <v>67.00679527854935</v>
       </c>
       <c r="Z57" s="53">
-        <v>0.138</v>
+        <v>0.29</v>
       </c>
       <c r="AA57" s="56">
         <v>0.2958</v>
@@ -18375,13 +18375,13 @@
         <v>105896.9567712</v>
       </c>
       <c r="E127" s="52">
-        <v>67407.3</v>
+        <v>79457.73</v>
       </c>
       <c r="F127" s="52">
-        <v>38489.656771199996</v>
+        <v>26439.226771200003</v>
       </c>
       <c r="G127" s="53">
-        <v>0.3634632943641657</v>
+        <v>0.2496693727311197</v>
       </c>
       <c r="H127" s="52">
         <v>85934.2000148</v>
@@ -18428,13 +18428,13 @@
       </c>
       <c r="W127" s="53"/>
       <c r="X127" s="55">
-        <v>8.172358490566037</v>
+        <v>121.8556603773585</v>
       </c>
       <c r="Y127" s="55">
         <v>62.79176131227983</v>
       </c>
       <c r="Z127" s="53">
-        <v>0.0129</v>
+        <v>0.16260000000000002</v>
       </c>
       <c r="AA127" s="56">
         <v>0.1885</v>
@@ -24528,66 +24528,66 @@
         <v>412300.73261827</v>
       </c>
       <c r="E225" s="52">
-        <v>306038.55</v>
+        <v>353667.87</v>
       </c>
       <c r="F225" s="52">
-        <v>106262.18261826999</v>
+        <v>58632.86261826998</v>
       </c>
       <c r="G225" s="53">
-        <v>0.257729793356087</v>
+        <v>0.1422089702483149</v>
       </c>
       <c r="H225" s="52">
         <v>306356.278672</v>
       </c>
       <c r="I225" s="52">
-        <v>256209</v>
+        <v>256729.4</v>
       </c>
       <c r="J225" s="52">
         <v>186357.488872</v>
       </c>
       <c r="K225" s="52">
-        <v>184474.91</v>
+        <v>184765.38</v>
       </c>
       <c r="L225" s="52">
-        <v>1882.5788719999837</v>
+        <v>1592.1088719999825</v>
       </c>
       <c r="M225" s="53">
-        <v>0.010101975957043706</v>
+        <v>0.008543305029686924</v>
       </c>
       <c r="N225" s="53"/>
       <c r="O225" s="52">
         <v>119998.7898</v>
       </c>
       <c r="P225" s="52">
-        <v>71734.09</v>
+        <v>71964.02</v>
       </c>
       <c r="Q225" s="52">
-        <v>48264.6998</v>
+        <v>48034.769799999995</v>
       </c>
       <c r="R225" s="53">
-        <v>0.4022098879533867</v>
+        <v>0.400293785296158</v>
       </c>
       <c r="S225" s="54">
         <v>2412.45</v>
       </c>
       <c r="T225" s="54">
-        <v>1531.67</v>
+        <v>1535.92</v>
       </c>
       <c r="U225" s="54">
-        <v>880.7799999999997</v>
+        <v>876.5299999999997</v>
       </c>
       <c r="V225" s="53">
-        <v>0.3650977222325851</v>
+        <v>0.363336027689693</v>
       </c>
       <c r="W225" s="53"/>
       <c r="X225" s="55">
-        <v>32.53282365000294</v>
+        <v>63.114270274493464</v>
       </c>
       <c r="Y225" s="55">
         <v>43.91570973337064</v>
       </c>
       <c r="Z225" s="53">
-        <v>0.1628</v>
+        <v>0.2741</v>
       </c>
       <c r="AA225" s="56">
         <v>0.257</v>
@@ -27506,16 +27506,16 @@
         <v>22202.890000000014</v>
       </c>
       <c r="D4" s="52">
-        <v>20645.929999999993</v>
+        <v>21022.23000000001</v>
       </c>
       <c r="E4" s="52">
-        <v>1556.960000000021</v>
+        <v>1180.6600000000035</v>
       </c>
       <c r="F4" s="52">
         <v>0</v>
       </c>
       <c r="G4" s="53">
-        <v>0.0701242045517507</v>
+        <v>0.053175960426773396</v>
       </c>
       <c r="H4" s="53">
         <v>0.2149</v>
@@ -27530,16 +27530,16 @@
         <v>7000</v>
       </c>
       <c r="L4" s="53">
-        <v>-0.24515006830191816</v>
+        <v>-0.26209831242689546</v>
       </c>
       <c r="M4" s="52">
-        <v>-5443.039999999979</v>
+        <v>-5819.3399999999965</v>
       </c>
       <c r="N4" s="54">
         <v>20</v>
       </c>
       <c r="O4" s="58">
-        <v>-77.75771428571399</v>
+        <v>-83.13342857142852</v>
       </c>
     </row>
     <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -27567,19 +27567,19 @@
         <v>29</v>
       </c>
       <c r="C6" s="52">
-        <v>0</v>
+        <v>42019.899999999994</v>
       </c>
       <c r="D6" s="52">
-        <v>17363.759999999995</v>
+        <v>18657.01999999999</v>
       </c>
       <c r="E6" s="52">
-        <v>-17363.759999999995</v>
+        <v>23362.880000000005</v>
       </c>
       <c r="F6" s="52">
         <v>7</v>
       </c>
       <c r="G6" s="53">
-        <v>0</v>
+        <v>0.5561621993388849</v>
       </c>
       <c r="H6" s="53">
         <v>0.239214585617637</v>
@@ -27594,16 +27594,16 @@
         <v>20272.6</v>
       </c>
       <c r="L6" s="53">
-        <v>0</v>
+        <v>0.07370983748176475</v>
       </c>
       <c r="M6" s="52">
-        <v>-37629.35999999999</v>
+        <v>3097.280000000006</v>
       </c>
       <c r="N6" s="54">
         <v>-52.5</v>
       </c>
       <c r="O6" s="58">
-        <v>-84.08795530726256</v>
+        <v>6.921296089385488</v>
       </c>
       <c r="Q6" s="35" t="s">
         <v>121</v>
@@ -27758,19 +27758,19 @@
         <v>122</v>
       </c>
       <c r="C12" s="52">
-        <v>0</v>
+        <v>93276.07999999999</v>
       </c>
       <c r="D12" s="52">
-        <v>60407.110000000015</v>
+        <v>61105.389999999985</v>
       </c>
       <c r="E12" s="52">
-        <v>-60407.110000000015</v>
+        <v>32170.690000000002</v>
       </c>
       <c r="F12" s="52">
         <v>3</v>
       </c>
       <c r="G12" s="53">
-        <v>0</v>
+        <v>0.34492969687405395</v>
       </c>
       <c r="H12" s="53">
         <v>0.176316261575212</v>
@@ -27785,16 +27785,16 @@
         <v>2640</v>
       </c>
       <c r="L12" s="53">
-        <v>0</v>
+        <v>0.31662662067273845</v>
       </c>
       <c r="M12" s="52">
-        <v>-63044.110000000015</v>
+        <v>29533.690000000002</v>
       </c>
       <c r="N12" s="54">
         <v>53</v>
       </c>
       <c r="O12" s="58">
-        <v>-913.6827536231887</v>
+        <v>428.02449275362324</v>
       </c>
       <c r="Q12" s="35" t="s">
         <v>123</v>
@@ -27825,19 +27825,19 @@
         <v>35</v>
       </c>
       <c r="C14" s="52">
-        <v>0</v>
+        <v>61369.72</v>
       </c>
       <c r="D14" s="52">
         <v>14493.379999999997</v>
       </c>
       <c r="E14" s="52">
-        <v>-14493.379999999997</v>
+        <v>46876.340000000004</v>
       </c>
       <c r="F14" s="52">
         <v>0</v>
       </c>
       <c r="G14" s="53">
-        <v>0</v>
+        <v>0.7638349987583454</v>
       </c>
       <c r="H14" s="53">
         <v>0.266338527271097</v>
@@ -27852,16 +27852,16 @@
         <v>3000</v>
       </c>
       <c r="L14" s="53">
-        <v>0</v>
+        <v>0.7149509562696392</v>
       </c>
       <c r="M14" s="52">
-        <v>-17493.379999999997</v>
+        <v>43876.340000000004</v>
       </c>
       <c r="N14" s="54">
         <v>-112</v>
       </c>
       <c r="O14" s="58">
-        <v>156.19089285714284</v>
+        <v>-391.7530357142858</v>
       </c>
     </row>
     <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -27951,19 +27951,19 @@
         <v>37</v>
       </c>
       <c r="C18" s="52">
-        <v>0</v>
+        <v>27482.319999999992</v>
       </c>
       <c r="D18" s="52">
-        <v>14851.680000000008</v>
+        <v>14933.520000000004</v>
       </c>
       <c r="E18" s="52">
-        <v>-14851.680000000008</v>
+        <v>12548.799999999988</v>
       </c>
       <c r="F18" s="52">
         <v>0</v>
       </c>
       <c r="G18" s="53">
-        <v>0</v>
+        <v>0.45661356100940503</v>
       </c>
       <c r="H18" s="53">
         <v>0.296537658865514</v>
@@ -27978,16 +27978,16 @@
         <v>8200</v>
       </c>
       <c r="L18" s="53">
-        <v>0</v>
+        <v>0.15823991569852872</v>
       </c>
       <c r="M18" s="52">
-        <v>-23051.680000000008</v>
+        <v>4348.799999999988</v>
       </c>
       <c r="N18" s="54">
         <v>-269</v>
       </c>
       <c r="O18" s="58">
-        <v>121.96656084656088</v>
+        <v>-23.00952380952375</v>
       </c>
       <c r="Q18" s="35" t="s">
         <v>124</v>
@@ -28556,19 +28556,19 @@
         <v>49</v>
       </c>
       <c r="C38" s="52">
-        <v>52040.560000000005</v>
+        <v>64090.99</v>
       </c>
       <c r="D38" s="52">
         <v>10303.779999999999</v>
       </c>
       <c r="E38" s="52">
-        <v>41736.780000000006</v>
+        <v>53787.21</v>
       </c>
       <c r="F38" s="52">
         <v>0</v>
       </c>
       <c r="G38" s="53">
-        <v>0.8020048208551177</v>
+        <v>0.8392320043737818</v>
       </c>
       <c r="H38" s="53">
         <v>0.1750921737769</v>
@@ -28579,10 +28579,10 @@
         <v>0</v>
       </c>
       <c r="L38" s="53">
-        <v>0.8020048208551177</v>
+        <v>0.8392320043737818</v>
       </c>
       <c r="M38" s="52">
-        <v>41736.780000000006</v>
+        <v>53787.21</v>
       </c>
       <c r="N38" s="54"/>
       <c r="O38" s="58">
@@ -29337,17 +29337,17 @@
         <v>62</v>
       </c>
       <c r="C66" s="99">
-        <v>34650.399999999965</v>
+        <v>82279.71999999997</v>
       </c>
       <c r="D66" s="99">
-        <v>21886.190000000002</v>
+        <v>22406.589999999997</v>
       </c>
       <c r="E66" s="99">
-        <v>12764.209999999963</v>
+        <v>59873.129999999976</v>
       </c>
       <c r="F66" s="99"/>
       <c r="G66" s="100">
-        <v>0.3683712164938926</v>
+        <v>0.727677853060268</v>
       </c>
       <c r="H66" s="100">
         <v>0.256265521519856</v>
@@ -29362,16 +29362,16 @@
         <v>3200</v>
       </c>
       <c r="L66" s="100">
-        <v>0.2760201902431133</v>
+        <v>0.6887861310174609</v>
       </c>
       <c r="M66" s="99">
-        <v>9564.209999999963</v>
+        <v>56673.129999999976</v>
       </c>
       <c r="N66" s="98">
         <v>-1014.25</v>
       </c>
       <c r="O66" s="60">
-        <v>-10.237313352956878</v>
+        <v>-60.66163232539468</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -29611,25 +29611,25 @@
         <v>127</v>
       </c>
       <c r="C74" s="104">
-        <v>120905.13999999997</v>
+        <v>404732.9099999999</v>
       </c>
       <c r="D74" s="104">
-        <v>231571.33</v>
+        <v>234541.40999999992</v>
       </c>
       <c r="E74" s="105">
-        <v>-110666.19000000003</v>
+        <v>170191.49999999997</v>
       </c>
       <c r="F74" s="106" t="s">
         <v>128</v>
       </c>
       <c r="G74" s="107">
-        <v>-0.915314187635034</v>
+        <v>0.4205032400256258</v>
       </c>
       <c r="H74" s="108" t="s">
         <v>129</v>
       </c>
       <c r="I74" s="109">
-        <v>-1.496204297021616</v>
+        <v>0.24697497418729794</v>
       </c>
       <c r="J74" s="36"/>
       <c r="K74" s="36"/>
@@ -30184,10 +30184,10 @@
         <v>638.02</v>
       </c>
       <c r="D4" s="54">
-        <v>608.25</v>
+        <v>616.75</v>
       </c>
       <c r="E4" s="54">
-        <v>29.769999999999982</v>
+        <v>21.269999999999982</v>
       </c>
       <c r="F4" s="54">
         <v>0</v>
@@ -30243,10 +30243,10 @@
         <v>363.57</v>
       </c>
       <c r="D6" s="54">
-        <v>242.5</v>
+        <v>272.5</v>
       </c>
       <c r="E6" s="54">
-        <v>121.07</v>
+        <v>91.07</v>
       </c>
       <c r="F6" s="54"/>
       <c r="G6" s="54"/>
@@ -30410,10 +30410,10 @@
         <v>1124.47</v>
       </c>
       <c r="D12" s="54">
-        <v>766.5</v>
+        <v>783</v>
       </c>
       <c r="E12" s="54">
-        <v>357.97</v>
+        <v>341.47</v>
       </c>
       <c r="F12" s="54"/>
       <c r="G12" s="54"/>
@@ -31840,10 +31840,10 @@
         <v>2412.45</v>
       </c>
       <c r="D66" s="54">
-        <v>1531.67</v>
+        <v>1535.92</v>
       </c>
       <c r="E66" s="54">
-        <v>880.7799999999997</v>
+        <v>876.5299999999997</v>
       </c>
       <c r="F66" s="54"/>
       <c r="G66" s="54"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-24T01:41:23Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -13228,13 +13228,13 @@
         <v>65693.35850319</v>
       </c>
       <c r="E50" s="52">
-        <v>33326.49</v>
+        <v>61277.97</v>
       </c>
       <c r="F50" s="52">
-        <v>32366.868503190002</v>
+        <v>4415.388503189999</v>
       </c>
       <c r="G50" s="53">
-        <v>0.49269620614111703</v>
+        <v>0.06721209881476212</v>
       </c>
       <c r="H50" s="52">
         <v>50582.36785</v>
@@ -13281,13 +13281,13 @@
       </c>
       <c r="W50" s="53"/>
       <c r="X50" s="55">
-        <v>17.207621247113163</v>
+        <v>146.31376443418014</v>
       </c>
       <c r="Y50" s="55">
         <v>67.69550512136009</v>
       </c>
       <c r="Z50" s="53">
-        <v>0.1118</v>
+        <v>0.5169</v>
       </c>
       <c r="AA50" s="56">
         <v>0.23</v>
@@ -27889,17 +27889,17 @@
         <v>36</v>
       </c>
       <c r="C16" s="52">
-        <v>0</v>
+        <v>27951.480000000003</v>
       </c>
       <c r="D16" s="52">
         <v>4389.459999999999</v>
       </c>
       <c r="E16" s="52">
-        <v>-4389.459999999999</v>
+        <v>23562.020000000004</v>
       </c>
       <c r="F16" s="52"/>
       <c r="G16" s="53">
-        <v>0</v>
+        <v>0.842961446048653</v>
       </c>
       <c r="H16" s="53">
         <v>0.226353821097855</v>
@@ -27914,16 +27914,16 @@
         <v>3000</v>
       </c>
       <c r="L16" s="53">
-        <v>0</v>
+        <v>0.735632603354098</v>
       </c>
       <c r="M16" s="52">
-        <v>-7389.459999999999</v>
+        <v>20562.020000000004</v>
       </c>
       <c r="N16" s="54">
         <v>-86.75</v>
       </c>
       <c r="O16" s="58">
-        <v>85.18109510086454</v>
+        <v>-237.0261671469741</v>
       </c>
     </row>
     <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -29611,25 +29611,25 @@
         <v>127</v>
       </c>
       <c r="C74" s="104">
-        <v>404732.9099999999</v>
+        <v>432684.38999999996</v>
       </c>
       <c r="D74" s="104">
         <v>234541.40999999992</v>
       </c>
       <c r="E74" s="105">
-        <v>170191.49999999997</v>
+        <v>198142.97999999998</v>
       </c>
       <c r="F74" s="106" t="s">
         <v>128</v>
       </c>
       <c r="G74" s="107">
-        <v>0.4205032400256258</v>
+        <v>0.4579388223365303</v>
       </c>
       <c r="H74" s="108" t="s">
         <v>129</v>
       </c>
       <c r="I74" s="109">
-        <v>0.24697497418729794</v>
+        <v>0.295620509905615</v>
       </c>
       <c r="J74" s="36"/>
       <c r="K74" s="36"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-28T19:04:15Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -10418,30 +10418,74 @@
       <c r="C9" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D9" s="52"/>
-      <c r="E9" s="52"/>
-      <c r="F9" s="52"/>
-      <c r="G9" s="53"/>
-      <c r="H9" s="52"/>
-      <c r="I9" s="52"/>
-      <c r="J9" s="52"/>
-      <c r="K9" s="52"/>
-      <c r="L9" s="52"/>
-      <c r="M9" s="53"/>
+      <c r="D9" s="52">
+        <v>267886.84883856</v>
+      </c>
+      <c r="E9" s="52">
+        <v>238732.97</v>
+      </c>
+      <c r="F9" s="52">
+        <v>29153.87883855999</v>
+      </c>
+      <c r="G9" s="53">
+        <v>0.10882907826553799</v>
+      </c>
+      <c r="H9" s="52">
+        <v>225410.5455298</v>
+      </c>
+      <c r="I9" s="52">
+        <v>189481.67</v>
+      </c>
+      <c r="J9" s="52">
+        <v>193787.2413298</v>
+      </c>
+      <c r="K9" s="52">
+        <v>158312.05000000002</v>
+      </c>
+      <c r="L9" s="52">
+        <v>35475.19132979997</v>
+      </c>
+      <c r="M9" s="53">
+        <v>0.1830625746378521</v>
+      </c>
       <c r="N9" s="53"/>
-      <c r="O9" s="52"/>
-      <c r="P9" s="52"/>
-      <c r="Q9" s="52"/>
-      <c r="R9" s="53"/>
-      <c r="S9" s="54"/>
-      <c r="T9" s="54"/>
-      <c r="U9" s="54"/>
-      <c r="V9" s="53"/>
+      <c r="O9" s="52">
+        <v>31623.3042</v>
+      </c>
+      <c r="P9" s="52">
+        <v>31169.62</v>
+      </c>
+      <c r="Q9" s="52">
+        <v>453.6841999999997</v>
+      </c>
+      <c r="R9" s="53">
+        <v>0.014346514745287108</v>
+      </c>
+      <c r="S9" s="54">
+        <v>638.02</v>
+      </c>
+      <c r="T9" s="54">
+        <v>625.25</v>
+      </c>
+      <c r="U9" s="54">
+        <v>12.769999999999982</v>
+      </c>
+      <c r="V9" s="53">
+        <v>0.020015046550264853</v>
+      </c>
       <c r="W9" s="53"/>
-      <c r="X9" s="55"/>
-      <c r="Y9" s="55"/>
-      <c r="Z9" s="53"/>
-      <c r="AA9" s="56"/>
+      <c r="X9" s="55">
+        <v>78.77057177129149</v>
+      </c>
+      <c r="Y9" s="55">
+        <v>66.57519091683645</v>
+      </c>
+      <c r="Z9" s="53">
+        <v>0.20629999999999998</v>
+      </c>
+      <c r="AA9" s="56">
+        <v>0.1586</v>
+      </c>
       <c r="AB9" s="57"/>
       <c r="AD9" s="35"/>
       <c r="AE9" s="35"/>
@@ -10913,30 +10957,74 @@
       <c r="C16" s="63" t="s">
         <v>104</v>
       </c>
-      <c r="D16" s="52"/>
-      <c r="E16" s="62"/>
-      <c r="F16" s="52"/>
-      <c r="G16" s="53"/>
-      <c r="H16" s="52"/>
-      <c r="I16" s="52"/>
-      <c r="J16" s="52"/>
-      <c r="K16" s="52"/>
-      <c r="L16" s="52"/>
-      <c r="M16" s="53"/>
+      <c r="D16" s="52">
+        <v>132076.08820213</v>
+      </c>
+      <c r="E16" s="62">
+        <v>127883.98</v>
+      </c>
+      <c r="F16" s="52">
+        <v>4192.108202129995</v>
+      </c>
+      <c r="G16" s="53">
+        <v>0.031740099659178046</v>
+      </c>
+      <c r="H16" s="52">
+        <v>103822.973895</v>
+      </c>
+      <c r="I16" s="52">
+        <v>94249.74</v>
+      </c>
+      <c r="J16" s="52">
+        <v>85672.874895</v>
+      </c>
+      <c r="K16" s="52">
+        <v>80502.31</v>
+      </c>
+      <c r="L16" s="52">
+        <v>5170.564895000003</v>
+      </c>
+      <c r="M16" s="53">
+        <v>0.060352414942734287</v>
+      </c>
       <c r="N16" s="53"/>
-      <c r="O16" s="52"/>
-      <c r="P16" s="52"/>
-      <c r="Q16" s="52"/>
-      <c r="R16" s="53"/>
-      <c r="S16" s="54"/>
-      <c r="T16" s="54"/>
-      <c r="U16" s="54"/>
-      <c r="V16" s="53"/>
+      <c r="O16" s="52">
+        <v>18150.099</v>
+      </c>
+      <c r="P16" s="52">
+        <v>13747.43</v>
+      </c>
+      <c r="Q16" s="52">
+        <v>4402.668999999998</v>
+      </c>
+      <c r="R16" s="53">
+        <v>0.24256997165690383</v>
+      </c>
+      <c r="S16" s="54">
+        <v>363.57</v>
+      </c>
+      <c r="T16" s="54">
+        <v>304.75</v>
+      </c>
+      <c r="U16" s="54">
+        <v>58.81999999999999</v>
+      </c>
+      <c r="V16" s="53">
+        <v>0.16178452567593585</v>
+      </c>
       <c r="W16" s="53"/>
-      <c r="X16" s="55"/>
-      <c r="Y16" s="55"/>
-      <c r="Z16" s="53"/>
-      <c r="AA16" s="56"/>
+      <c r="X16" s="55">
+        <v>110.36666119770302</v>
+      </c>
+      <c r="Y16" s="55">
+        <v>77.71024646458726</v>
+      </c>
+      <c r="Z16" s="53">
+        <v>0.263</v>
+      </c>
+      <c r="AA16" s="56">
+        <v>0.2139</v>
+      </c>
       <c r="AB16" s="57"/>
       <c r="AD16" s="35"/>
       <c r="AE16" s="35"/>
@@ -11408,30 +11496,74 @@
       <c r="C23" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D23" s="52"/>
-      <c r="E23" s="52"/>
-      <c r="F23" s="52"/>
-      <c r="G23" s="53"/>
-      <c r="H23" s="52"/>
-      <c r="I23" s="52"/>
-      <c r="J23" s="52"/>
-      <c r="K23" s="52"/>
-      <c r="L23" s="52"/>
-      <c r="M23" s="53"/>
+      <c r="D23" s="52">
+        <v>27500.3157</v>
+      </c>
+      <c r="E23" s="52">
+        <v>11999.08</v>
+      </c>
+      <c r="F23" s="52">
+        <v>15501.2357</v>
+      </c>
+      <c r="G23" s="53">
+        <v>0.563674827194802</v>
+      </c>
+      <c r="H23" s="52">
+        <v>19565.829</v>
+      </c>
+      <c r="I23" s="52">
+        <v>8083.92</v>
+      </c>
+      <c r="J23" s="52">
+        <v>13767.337200000002</v>
+      </c>
+      <c r="K23" s="52">
+        <v>6373.24</v>
+      </c>
+      <c r="L23" s="52">
+        <v>7394.097200000002</v>
+      </c>
+      <c r="M23" s="53">
+        <v>0.5370753321855152</v>
+      </c>
       <c r="N23" s="53"/>
-      <c r="O23" s="52"/>
-      <c r="P23" s="52"/>
-      <c r="Q23" s="52"/>
-      <c r="R23" s="53"/>
-      <c r="S23" s="54"/>
-      <c r="T23" s="54"/>
-      <c r="U23" s="54"/>
-      <c r="V23" s="53"/>
+      <c r="O23" s="52">
+        <v>5798.4918</v>
+      </c>
+      <c r="P23" s="52">
+        <v>1710.68</v>
+      </c>
+      <c r="Q23" s="52">
+        <v>4087.8117999999995</v>
+      </c>
+      <c r="R23" s="53">
+        <v>0.7049784566393626</v>
+      </c>
+      <c r="S23" s="54">
+        <v>125.39</v>
+      </c>
+      <c r="T23" s="54">
+        <v>34.75</v>
+      </c>
+      <c r="U23" s="54">
+        <v>90.64</v>
+      </c>
+      <c r="V23" s="53">
+        <v>0.7228646622537682</v>
+      </c>
       <c r="W23" s="53"/>
-      <c r="X23" s="55"/>
-      <c r="Y23" s="55"/>
-      <c r="Z23" s="53"/>
-      <c r="AA23" s="56"/>
+      <c r="X23" s="55">
+        <v>112.66647482014388</v>
+      </c>
+      <c r="Y23" s="55">
+        <v>63.27846478985563</v>
+      </c>
+      <c r="Z23" s="53">
+        <v>0.32630000000000003</v>
+      </c>
+      <c r="AA23" s="56">
+        <v>0.2885</v>
+      </c>
       <c r="AB23" s="57"/>
       <c r="AD23" s="35"/>
       <c r="AE23" s="35"/>
@@ -12312,30 +12444,74 @@
       <c r="C37" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D37" s="52"/>
-      <c r="E37" s="52"/>
-      <c r="F37" s="52"/>
-      <c r="G37" s="53"/>
-      <c r="H37" s="52"/>
-      <c r="I37" s="52"/>
-      <c r="J37" s="52"/>
-      <c r="K37" s="52"/>
-      <c r="L37" s="52"/>
-      <c r="M37" s="53"/>
+      <c r="D37" s="52">
+        <v>397238.61073204</v>
+      </c>
+      <c r="E37" s="52">
+        <v>352623.79</v>
+      </c>
+      <c r="F37" s="52">
+        <v>44614.82073204004</v>
+      </c>
+      <c r="G37" s="53">
+        <v>0.112312397452561</v>
+      </c>
+      <c r="H37" s="52">
+        <v>328046.93216</v>
+      </c>
+      <c r="I37" s="52">
+        <v>278838.99</v>
+      </c>
+      <c r="J37" s="52">
+        <v>271925.57216000004</v>
+      </c>
+      <c r="K37" s="52">
+        <v>243603.25999999998</v>
+      </c>
+      <c r="L37" s="52">
+        <v>28322.31216000006</v>
+      </c>
+      <c r="M37" s="53">
+        <v>0.1041546476671025</v>
+      </c>
       <c r="N37" s="53"/>
-      <c r="O37" s="52"/>
-      <c r="P37" s="52"/>
-      <c r="Q37" s="52"/>
-      <c r="R37" s="53"/>
-      <c r="S37" s="54"/>
-      <c r="T37" s="54"/>
-      <c r="U37" s="54"/>
-      <c r="V37" s="53"/>
+      <c r="O37" s="52">
+        <v>56121.36</v>
+      </c>
+      <c r="P37" s="52">
+        <v>35235.73</v>
+      </c>
+      <c r="Q37" s="52">
+        <v>20885.629999999997</v>
+      </c>
+      <c r="R37" s="53">
+        <v>0.37215117381332163</v>
+      </c>
+      <c r="S37" s="54">
+        <v>1124.47</v>
+      </c>
+      <c r="T37" s="54">
+        <v>813.5</v>
+      </c>
+      <c r="U37" s="54">
+        <v>310.97</v>
+      </c>
+      <c r="V37" s="53">
+        <v>0.2765480626428451</v>
+      </c>
       <c r="W37" s="53"/>
-      <c r="X37" s="55"/>
-      <c r="Y37" s="55"/>
-      <c r="Z37" s="53"/>
-      <c r="AA37" s="56"/>
+      <c r="X37" s="55">
+        <v>90.70043023970499</v>
+      </c>
+      <c r="Y37" s="55">
+        <v>61.532703026350184</v>
+      </c>
+      <c r="Z37" s="53">
+        <v>0.20920000000000002</v>
+      </c>
+      <c r="AA37" s="56">
+        <v>0.1742</v>
+      </c>
       <c r="AB37" s="57"/>
       <c r="AD37" s="35"/>
       <c r="AE37" s="35"/>
@@ -12807,30 +12983,74 @@
       <c r="C44" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D44" s="52"/>
-      <c r="E44" s="52"/>
-      <c r="F44" s="52"/>
-      <c r="G44" s="53"/>
-      <c r="H44" s="52"/>
-      <c r="I44" s="52"/>
-      <c r="J44" s="52"/>
-      <c r="K44" s="52"/>
-      <c r="L44" s="52"/>
-      <c r="M44" s="53"/>
+      <c r="D44" s="52">
+        <v>128258.49930985</v>
+      </c>
+      <c r="E44" s="52">
+        <v>115314.55</v>
+      </c>
+      <c r="F44" s="52">
+        <v>12943.949309849995</v>
+      </c>
+      <c r="G44" s="53">
+        <v>0.10092079183446305</v>
+      </c>
+      <c r="H44" s="52">
+        <v>94098.31685</v>
+      </c>
+      <c r="I44" s="52">
+        <v>57104.57</v>
+      </c>
+      <c r="J44" s="52">
+        <v>69042.08885</v>
+      </c>
+      <c r="K44" s="52">
+        <v>40878.83</v>
+      </c>
+      <c r="L44" s="52">
+        <v>28163.25885</v>
+      </c>
+      <c r="M44" s="53">
+        <v>0.40791435078372484</v>
+      </c>
       <c r="N44" s="53"/>
-      <c r="O44" s="52"/>
-      <c r="P44" s="52"/>
-      <c r="Q44" s="52"/>
-      <c r="R44" s="53"/>
-      <c r="S44" s="54"/>
-      <c r="T44" s="54"/>
-      <c r="U44" s="54"/>
-      <c r="V44" s="53"/>
+      <c r="O44" s="52">
+        <v>25056.228</v>
+      </c>
+      <c r="P44" s="52">
+        <v>16225.74</v>
+      </c>
+      <c r="Q44" s="52">
+        <v>8830.488</v>
+      </c>
+      <c r="R44" s="53">
+        <v>0.3524268696788678</v>
+      </c>
+      <c r="S44" s="54">
+        <v>501.83</v>
+      </c>
+      <c r="T44" s="54">
+        <v>366.25</v>
+      </c>
+      <c r="U44" s="54">
+        <v>135.57999999999998</v>
+      </c>
+      <c r="V44" s="53">
+        <v>0.2701711735049718</v>
+      </c>
       <c r="W44" s="53"/>
-      <c r="X44" s="55"/>
-      <c r="Y44" s="55"/>
-      <c r="Z44" s="53"/>
-      <c r="AA44" s="56"/>
+      <c r="X44" s="55">
+        <v>158.93509897610923</v>
+      </c>
+      <c r="Y44" s="55">
+        <v>68.07122423898531</v>
+      </c>
+      <c r="Z44" s="53">
+        <v>0.5047999999999999</v>
+      </c>
+      <c r="AA44" s="56">
+        <v>0.2663</v>
+      </c>
       <c r="AB44" s="57"/>
       <c r="AD44" s="35"/>
       <c r="AE44" s="35"/>
@@ -13304,30 +13524,74 @@
       <c r="C51" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D51" s="52"/>
-      <c r="E51" s="52"/>
-      <c r="F51" s="52"/>
-      <c r="G51" s="53"/>
-      <c r="H51" s="52"/>
-      <c r="I51" s="52"/>
-      <c r="J51" s="52"/>
-      <c r="K51" s="52"/>
-      <c r="L51" s="52"/>
-      <c r="M51" s="53"/>
+      <c r="D51" s="52">
+        <v>65693.35850319</v>
+      </c>
+      <c r="E51" s="52">
+        <v>61277.97</v>
+      </c>
+      <c r="F51" s="52">
+        <v>4415.388503189999</v>
+      </c>
+      <c r="G51" s="53">
+        <v>0.06721209881476212</v>
+      </c>
+      <c r="H51" s="52">
+        <v>50582.36785</v>
+      </c>
+      <c r="I51" s="52">
+        <v>29601.04</v>
+      </c>
+      <c r="J51" s="52">
+        <v>39438.99025</v>
+      </c>
+      <c r="K51" s="52">
+        <v>20244.31</v>
+      </c>
+      <c r="L51" s="52">
+        <v>19194.68025</v>
+      </c>
+      <c r="M51" s="53">
+        <v>0.4866929941240065</v>
+      </c>
       <c r="N51" s="53"/>
-      <c r="O51" s="52"/>
-      <c r="P51" s="52"/>
-      <c r="Q51" s="52"/>
-      <c r="R51" s="53"/>
-      <c r="S51" s="54"/>
-      <c r="T51" s="54"/>
-      <c r="U51" s="54"/>
-      <c r="V51" s="53"/>
+      <c r="O51" s="52">
+        <v>11143.3776</v>
+      </c>
+      <c r="P51" s="52">
+        <v>9356.73</v>
+      </c>
+      <c r="Q51" s="52">
+        <v>1786.6476000000002</v>
+      </c>
+      <c r="R51" s="53">
+        <v>0.1603326804612634</v>
+      </c>
+      <c r="S51" s="54">
+        <v>223.22</v>
+      </c>
+      <c r="T51" s="54">
+        <v>216.5</v>
+      </c>
+      <c r="U51" s="54">
+        <v>6.719999999999999</v>
+      </c>
+      <c r="V51" s="53">
+        <v>0.030104829316369496</v>
+      </c>
       <c r="W51" s="53"/>
-      <c r="X51" s="55"/>
-      <c r="Y51" s="55"/>
-      <c r="Z51" s="53"/>
-      <c r="AA51" s="56"/>
+      <c r="X51" s="55">
+        <v>146.31376443418014</v>
+      </c>
+      <c r="Y51" s="55">
+        <v>67.69550512136009</v>
+      </c>
+      <c r="Z51" s="53">
+        <v>0.5169</v>
+      </c>
+      <c r="AA51" s="56">
+        <v>0.23</v>
+      </c>
       <c r="AB51" s="57"/>
       <c r="AD51" s="35"/>
       <c r="AE51" s="35"/>
@@ -13799,30 +14063,74 @@
       <c r="C58" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D58" s="52"/>
-      <c r="E58" s="52"/>
-      <c r="F58" s="52"/>
-      <c r="G58" s="53"/>
-      <c r="H58" s="52"/>
-      <c r="I58" s="52"/>
-      <c r="J58" s="52"/>
-      <c r="K58" s="52"/>
-      <c r="L58" s="52"/>
-      <c r="M58" s="53"/>
+      <c r="D58" s="52">
+        <v>155296.79012754</v>
+      </c>
+      <c r="E58" s="52">
+        <v>155296.8</v>
+      </c>
+      <c r="F58" s="52">
+        <v>-0.009872459981124848</v>
+      </c>
+      <c r="G58" s="53">
+        <v>-6.357156495647419e-8</v>
+      </c>
+      <c r="H58" s="52">
+        <v>109364.9721</v>
+      </c>
+      <c r="I58" s="52">
+        <v>113859.52</v>
+      </c>
+      <c r="J58" s="52">
+        <v>75135.0159</v>
+      </c>
+      <c r="K58" s="52">
+        <v>80491.32</v>
+      </c>
+      <c r="L58" s="52">
+        <v>-5356.3041000000085</v>
+      </c>
+      <c r="M58" s="53">
+        <v>-0.07128905259205527</v>
+      </c>
       <c r="N58" s="53"/>
-      <c r="O58" s="52"/>
-      <c r="P58" s="52"/>
-      <c r="Q58" s="52"/>
-      <c r="R58" s="53"/>
-      <c r="S58" s="54"/>
-      <c r="T58" s="54"/>
-      <c r="U58" s="54"/>
-      <c r="V58" s="53"/>
+      <c r="O58" s="52">
+        <v>34229.9562</v>
+      </c>
+      <c r="P58" s="52">
+        <v>33368.2</v>
+      </c>
+      <c r="Q58" s="52">
+        <v>861.7562000000034</v>
+      </c>
+      <c r="R58" s="53">
+        <v>0.025175498179574166</v>
+      </c>
+      <c r="S58" s="54">
+        <v>685.48</v>
+      </c>
+      <c r="T58" s="54">
+        <v>699.75</v>
+      </c>
+      <c r="U58" s="54">
+        <v>-14.269999999999982</v>
+      </c>
+      <c r="V58" s="53">
+        <v>-0.0208175293225185</v>
+      </c>
       <c r="W58" s="53"/>
-      <c r="X58" s="55"/>
-      <c r="Y58" s="55"/>
-      <c r="Z58" s="53"/>
-      <c r="AA58" s="56"/>
+      <c r="X58" s="55">
+        <v>59.2172633083244</v>
+      </c>
+      <c r="Y58" s="55">
+        <v>67.00679527854935</v>
+      </c>
+      <c r="Z58" s="53">
+        <v>0.2668</v>
+      </c>
+      <c r="AA58" s="56">
+        <v>0.2958</v>
+      </c>
       <c r="AB58" s="57"/>
       <c r="AD58" s="35"/>
       <c r="AE58" s="35"/>
@@ -14695,30 +15003,74 @@
       <c r="C72" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D72" s="52"/>
-      <c r="E72" s="52"/>
-      <c r="F72" s="52"/>
-      <c r="G72" s="53"/>
-      <c r="H72" s="52"/>
-      <c r="I72" s="52"/>
-      <c r="J72" s="52"/>
-      <c r="K72" s="52"/>
-      <c r="L72" s="52"/>
-      <c r="M72" s="53"/>
+      <c r="D72" s="52">
+        <v>53029.71458947</v>
+      </c>
+      <c r="E72" s="52">
+        <v>29715.67</v>
+      </c>
+      <c r="F72" s="52">
+        <v>23314.044589470002</v>
+      </c>
+      <c r="G72" s="53">
+        <v>0.43964114779715263</v>
+      </c>
+      <c r="H72" s="52">
+        <v>39055.77825</v>
+      </c>
+      <c r="I72" s="52">
+        <v>24880.27</v>
+      </c>
+      <c r="J72" s="52">
+        <v>29537.289750000004</v>
+      </c>
+      <c r="K72" s="52">
+        <v>20998.84</v>
+      </c>
+      <c r="L72" s="52">
+        <v>8538.449750000003</v>
+      </c>
+      <c r="M72" s="53">
+        <v>0.28907356843733445</v>
+      </c>
       <c r="N72" s="53"/>
-      <c r="O72" s="52"/>
-      <c r="P72" s="52"/>
-      <c r="Q72" s="52"/>
-      <c r="R72" s="53"/>
-      <c r="S72" s="54"/>
-      <c r="T72" s="54"/>
-      <c r="U72" s="54"/>
-      <c r="V72" s="53"/>
+      <c r="O72" s="52">
+        <v>9518.4885</v>
+      </c>
+      <c r="P72" s="52">
+        <v>3881.43</v>
+      </c>
+      <c r="Q72" s="52">
+        <v>5637.058499999999</v>
+      </c>
+      <c r="R72" s="53">
+        <v>0.5922220213850129</v>
+      </c>
+      <c r="S72" s="54">
+        <v>193.32</v>
+      </c>
+      <c r="T72" s="54">
+        <v>83.5</v>
+      </c>
+      <c r="U72" s="54">
+        <v>109.82</v>
+      </c>
+      <c r="V72" s="53">
+        <v>0.5680736602524312</v>
+      </c>
       <c r="W72" s="53"/>
-      <c r="X72" s="55"/>
-      <c r="Y72" s="55"/>
-      <c r="Z72" s="53"/>
-      <c r="AA72" s="56"/>
+      <c r="X72" s="55">
+        <v>57.90898203592814</v>
+      </c>
+      <c r="Y72" s="55">
+        <v>72.28396616733912</v>
+      </c>
+      <c r="Z72" s="53">
+        <v>0.16269999999999998</v>
+      </c>
+      <c r="AA72" s="56">
+        <v>0.2635</v>
+      </c>
       <c r="AB72" s="57"/>
       <c r="AD72" s="35"/>
       <c r="AE72" s="35"/>
@@ -15180,30 +15532,74 @@
       <c r="C79" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D79" s="52"/>
-      <c r="E79" s="52"/>
-      <c r="F79" s="52"/>
-      <c r="G79" s="53"/>
-      <c r="H79" s="52"/>
-      <c r="I79" s="52"/>
-      <c r="J79" s="52"/>
-      <c r="K79" s="52"/>
-      <c r="L79" s="52"/>
-      <c r="M79" s="53"/>
+      <c r="D79" s="52">
+        <v>78753.06644148</v>
+      </c>
+      <c r="E79" s="52">
+        <v>61764.82</v>
+      </c>
+      <c r="F79" s="52">
+        <v>16988.246441479998</v>
+      </c>
+      <c r="G79" s="53">
+        <v>0.21571536460873764</v>
+      </c>
+      <c r="H79" s="52">
+        <v>55589.7822</v>
+      </c>
+      <c r="I79" s="52">
+        <v>44814.24</v>
+      </c>
+      <c r="J79" s="52">
+        <v>32594.7534</v>
+      </c>
+      <c r="K79" s="52">
+        <v>34770.899999999994</v>
+      </c>
+      <c r="L79" s="52">
+        <v>-2176.1465999999928</v>
+      </c>
+      <c r="M79" s="53">
+        <v>-0.06676370805124707</v>
+      </c>
       <c r="N79" s="53"/>
-      <c r="O79" s="52"/>
-      <c r="P79" s="52"/>
-      <c r="Q79" s="52"/>
-      <c r="R79" s="53"/>
-      <c r="S79" s="54"/>
-      <c r="T79" s="54"/>
-      <c r="U79" s="54"/>
-      <c r="V79" s="53"/>
+      <c r="O79" s="52">
+        <v>22995.0288</v>
+      </c>
+      <c r="P79" s="52">
+        <v>10043.34</v>
+      </c>
+      <c r="Q79" s="52">
+        <v>12951.6888</v>
+      </c>
+      <c r="R79" s="53">
+        <v>0.563238642258191</v>
+      </c>
+      <c r="S79" s="54">
+        <v>472.14</v>
+      </c>
+      <c r="T79" s="54">
+        <v>202</v>
+      </c>
+      <c r="U79" s="54">
+        <v>270.14</v>
+      </c>
+      <c r="V79" s="53">
+        <v>0.5721607997627822</v>
+      </c>
       <c r="W79" s="53"/>
-      <c r="X79" s="55"/>
-      <c r="Y79" s="55"/>
-      <c r="Z79" s="53"/>
-      <c r="AA79" s="56"/>
+      <c r="X79" s="55">
+        <v>83.91376237623763</v>
+      </c>
+      <c r="Y79" s="55">
+        <v>49.060202993773025</v>
+      </c>
+      <c r="Z79" s="53">
+        <v>0.27440000000000003</v>
+      </c>
+      <c r="AA79" s="56">
+        <v>0.2941</v>
+      </c>
       <c r="AB79" s="57"/>
       <c r="AD79" s="35"/>
       <c r="AE79" s="35"/>
@@ -15671,30 +16067,74 @@
       <c r="C86" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D86" s="52"/>
-      <c r="E86" s="52"/>
-      <c r="F86" s="52"/>
-      <c r="G86" s="53"/>
-      <c r="H86" s="52"/>
-      <c r="I86" s="52"/>
-      <c r="J86" s="52"/>
-      <c r="K86" s="52"/>
-      <c r="L86" s="52"/>
-      <c r="M86" s="53"/>
+      <c r="D86" s="52">
+        <v>25467.8441072</v>
+      </c>
+      <c r="E86" s="52">
+        <v>19598.41</v>
+      </c>
+      <c r="F86" s="52">
+        <v>5869.434107199999</v>
+      </c>
+      <c r="G86" s="53">
+        <v>0.23046450584879521</v>
+      </c>
+      <c r="H86" s="52">
+        <v>16606.829916</v>
+      </c>
+      <c r="I86" s="52">
+        <v>14118.07</v>
+      </c>
+      <c r="J86" s="52">
+        <v>9659.986716</v>
+      </c>
+      <c r="K86" s="52">
+        <v>5298.48</v>
+      </c>
+      <c r="L86" s="52">
+        <v>4361.506716</v>
+      </c>
+      <c r="M86" s="53">
+        <v>0.4515023513206248</v>
+      </c>
       <c r="N86" s="53"/>
-      <c r="O86" s="52"/>
-      <c r="P86" s="52"/>
-      <c r="Q86" s="52"/>
-      <c r="R86" s="53"/>
-      <c r="S86" s="54"/>
-      <c r="T86" s="54"/>
-      <c r="U86" s="54"/>
-      <c r="V86" s="53"/>
+      <c r="O86" s="52">
+        <v>6946.8432</v>
+      </c>
+      <c r="P86" s="52">
+        <v>8819.59</v>
+      </c>
+      <c r="Q86" s="52">
+        <v>-1872.7468</v>
+      </c>
+      <c r="R86" s="53">
+        <v>-0.26958241982487813</v>
+      </c>
+      <c r="S86" s="54">
+        <v>139.07</v>
+      </c>
+      <c r="T86" s="54">
+        <v>167.75</v>
+      </c>
+      <c r="U86" s="54">
+        <v>-28.680000000000007</v>
+      </c>
+      <c r="V86" s="53">
+        <v>-0.20622707988782632</v>
+      </c>
       <c r="W86" s="53"/>
-      <c r="X86" s="55"/>
-      <c r="Y86" s="55"/>
-      <c r="Z86" s="53"/>
-      <c r="AA86" s="56"/>
+      <c r="X86" s="55">
+        <v>32.669687034277196</v>
+      </c>
+      <c r="Y86" s="55">
+        <v>63.7162162306752</v>
+      </c>
+      <c r="Z86" s="53">
+        <v>0.2796</v>
+      </c>
+      <c r="AA86" s="56">
+        <v>0.3479</v>
+      </c>
       <c r="AB86" s="57"/>
       <c r="AD86" s="35"/>
       <c r="AE86" s="35"/>
@@ -16166,30 +16606,74 @@
       <c r="C93" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D93" s="67"/>
-      <c r="E93" s="67"/>
-      <c r="F93" s="52"/>
-      <c r="G93" s="53"/>
-      <c r="H93" s="52"/>
-      <c r="I93" s="52"/>
-      <c r="J93" s="52"/>
-      <c r="K93" s="52"/>
-      <c r="L93" s="52"/>
-      <c r="M93" s="53"/>
+      <c r="D93" s="67">
+        <v>37083.0313712</v>
+      </c>
+      <c r="E93" s="67">
+        <v>36381.33</v>
+      </c>
+      <c r="F93" s="52">
+        <v>701.7013711999971</v>
+      </c>
+      <c r="G93" s="53">
+        <v>0.018922438248804095</v>
+      </c>
+      <c r="H93" s="52">
+        <v>27002.93286</v>
+      </c>
+      <c r="I93" s="52">
+        <v>25103.82</v>
+      </c>
+      <c r="J93" s="52">
+        <v>15440.324460000002</v>
+      </c>
+      <c r="K93" s="52">
+        <v>13974.73</v>
+      </c>
+      <c r="L93" s="52">
+        <v>1465.594460000002</v>
+      </c>
+      <c r="M93" s="53">
+        <v>0.0949199263135175</v>
+      </c>
       <c r="N93" s="53"/>
-      <c r="O93" s="52"/>
-      <c r="P93" s="52"/>
-      <c r="Q93" s="52"/>
-      <c r="R93" s="53"/>
-      <c r="S93" s="68"/>
-      <c r="T93" s="68"/>
-      <c r="U93" s="54"/>
-      <c r="V93" s="53"/>
+      <c r="O93" s="52">
+        <v>11562.6084</v>
+      </c>
+      <c r="P93" s="52">
+        <v>11129.09</v>
+      </c>
+      <c r="Q93" s="52">
+        <v>433.518399999999</v>
+      </c>
+      <c r="R93" s="53">
+        <v>0.03749313174006646</v>
+      </c>
+      <c r="S93" s="68">
+        <v>231.75</v>
+      </c>
+      <c r="T93" s="68">
+        <v>225.5</v>
+      </c>
+      <c r="U93" s="54">
+        <v>6.25</v>
+      </c>
+      <c r="V93" s="53">
+        <v>0.02696871628910464</v>
+      </c>
       <c r="W93" s="53"/>
-      <c r="X93" s="55"/>
-      <c r="Y93" s="55"/>
-      <c r="Z93" s="53"/>
-      <c r="AA93" s="56"/>
+      <c r="X93" s="55">
+        <v>50.01113082039912</v>
+      </c>
+      <c r="Y93" s="55">
+        <v>43.49557070636461</v>
+      </c>
+      <c r="Z93" s="53">
+        <v>0.31</v>
+      </c>
+      <c r="AA93" s="56">
+        <v>0.2718</v>
+      </c>
       <c r="AB93" s="57"/>
       <c r="AD93" s="35"/>
       <c r="AE93" s="35"/>
@@ -16661,30 +17145,74 @@
       <c r="C100" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D100" s="52"/>
-      <c r="E100" s="52"/>
-      <c r="F100" s="52"/>
-      <c r="G100" s="53"/>
-      <c r="H100" s="52"/>
-      <c r="I100" s="52"/>
-      <c r="J100" s="52"/>
-      <c r="K100" s="52"/>
-      <c r="L100" s="52"/>
-      <c r="M100" s="53"/>
+      <c r="D100" s="52">
+        <v>26186.1354</v>
+      </c>
+      <c r="E100" s="52">
+        <v>5762.27</v>
+      </c>
+      <c r="F100" s="52">
+        <v>20423.8654</v>
+      </c>
+      <c r="G100" s="53">
+        <v>0.7799495835494686</v>
+      </c>
+      <c r="H100" s="52">
+        <v>19428.9760178</v>
+      </c>
+      <c r="I100" s="52">
+        <v>8019.36</v>
+      </c>
+      <c r="J100" s="52">
+        <v>12051.3142178</v>
+      </c>
+      <c r="K100" s="52">
+        <v>7687.129999999999</v>
+      </c>
+      <c r="L100" s="52">
+        <v>4364.184217800001</v>
+      </c>
+      <c r="M100" s="53">
+        <v>0.3621334685103493</v>
+      </c>
       <c r="N100" s="53"/>
-      <c r="O100" s="52"/>
-      <c r="P100" s="52"/>
-      <c r="Q100" s="52"/>
-      <c r="R100" s="53"/>
-      <c r="S100" s="54"/>
-      <c r="T100" s="54"/>
-      <c r="U100" s="54"/>
-      <c r="V100" s="53"/>
+      <c r="O100" s="52">
+        <v>7377.6618</v>
+      </c>
+      <c r="P100" s="52">
+        <v>332.23</v>
+      </c>
+      <c r="Q100" s="52">
+        <v>7045.4318</v>
+      </c>
+      <c r="R100" s="53">
+        <v>0.954968117405436</v>
+      </c>
+      <c r="S100" s="54">
+        <v>147.9</v>
+      </c>
+      <c r="T100" s="54">
+        <v>6.5</v>
+      </c>
+      <c r="U100" s="54">
+        <v>141.4</v>
+      </c>
+      <c r="V100" s="53">
+        <v>0.9560513860716701</v>
+      </c>
       <c r="W100" s="53"/>
-      <c r="X100" s="55"/>
-      <c r="Y100" s="55"/>
-      <c r="Z100" s="53"/>
-      <c r="AA100" s="56"/>
+      <c r="X100" s="55">
+        <v>-347.24461538461543</v>
+      </c>
+      <c r="Y100" s="55">
+        <v>45.687352144692355</v>
+      </c>
+      <c r="Z100" s="53">
+        <v>-0.3917</v>
+      </c>
+      <c r="AA100" s="56">
+        <v>0.258</v>
+      </c>
       <c r="AB100" s="57"/>
       <c r="AD100" s="35"/>
       <c r="AE100" s="35"/>
@@ -17966,30 +18494,74 @@
       <c r="C121" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D121" s="52"/>
-      <c r="E121" s="52"/>
-      <c r="F121" s="52"/>
-      <c r="G121" s="53"/>
-      <c r="H121" s="52"/>
-      <c r="I121" s="52"/>
-      <c r="J121" s="52"/>
-      <c r="K121" s="52"/>
-      <c r="L121" s="52"/>
-      <c r="M121" s="53"/>
+      <c r="D121" s="52">
+        <v>20278.45679756</v>
+      </c>
+      <c r="E121" s="52">
+        <v>0</v>
+      </c>
+      <c r="F121" s="52">
+        <v>20278.45679756</v>
+      </c>
+      <c r="G121" s="53">
+        <v>1</v>
+      </c>
+      <c r="H121" s="52">
+        <v>16648.056795</v>
+      </c>
+      <c r="I121" s="52">
+        <v>58.32</v>
+      </c>
+      <c r="J121" s="52">
+        <v>12536.982795</v>
+      </c>
+      <c r="K121" s="52">
+        <v>58.32</v>
+      </c>
+      <c r="L121" s="52">
+        <v>12478.662795</v>
+      </c>
+      <c r="M121" s="53">
+        <v>0.9953481630346291</v>
+      </c>
       <c r="N121" s="53"/>
-      <c r="O121" s="52"/>
-      <c r="P121" s="52"/>
-      <c r="Q121" s="52"/>
-      <c r="R121" s="53"/>
-      <c r="S121" s="54"/>
-      <c r="T121" s="54"/>
-      <c r="U121" s="54"/>
-      <c r="V121" s="53"/>
+      <c r="O121" s="52">
+        <v>4111.074</v>
+      </c>
+      <c r="P121" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q121" s="52">
+        <v>4111.074</v>
+      </c>
+      <c r="R121" s="53">
+        <v>1</v>
+      </c>
+      <c r="S121" s="54">
+        <v>82.37</v>
+      </c>
+      <c r="T121" s="54">
+        <v>0</v>
+      </c>
+      <c r="U121" s="54">
+        <v>82.37</v>
+      </c>
+      <c r="V121" s="53">
+        <v>1</v>
+      </c>
       <c r="W121" s="53"/>
-      <c r="X121" s="55"/>
-      <c r="Y121" s="55"/>
-      <c r="Z121" s="53"/>
-      <c r="AA121" s="56"/>
+      <c r="X121" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y121" s="55">
+        <v>44.07429892630812</v>
+      </c>
+      <c r="Z121" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA121" s="56">
+        <v>0.179</v>
+      </c>
       <c r="AB121" s="57"/>
       <c r="AD121" s="35"/>
       <c r="AE121" s="35"/>
@@ -18451,30 +19023,74 @@
       <c r="C128" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D128" s="52"/>
-      <c r="E128" s="52"/>
-      <c r="F128" s="52"/>
-      <c r="G128" s="53"/>
-      <c r="H128" s="52"/>
-      <c r="I128" s="52"/>
-      <c r="J128" s="52"/>
-      <c r="K128" s="52"/>
-      <c r="L128" s="52"/>
-      <c r="M128" s="53"/>
+      <c r="D128" s="52">
+        <v>105896.9567712</v>
+      </c>
+      <c r="E128" s="52">
+        <v>79457.73</v>
+      </c>
+      <c r="F128" s="52">
+        <v>26439.226771200003</v>
+      </c>
+      <c r="G128" s="53">
+        <v>0.2496693727311197</v>
+      </c>
+      <c r="H128" s="52">
+        <v>85934.2000148</v>
+      </c>
+      <c r="I128" s="52">
+        <v>66541.03</v>
+      </c>
+      <c r="J128" s="52">
+        <v>70065.71561479999</v>
+      </c>
+      <c r="K128" s="52">
+        <v>61659.44</v>
+      </c>
+      <c r="L128" s="52">
+        <v>8406.27561479999</v>
+      </c>
+      <c r="M128" s="53">
+        <v>0.11997701787583442</v>
+      </c>
       <c r="N128" s="53"/>
-      <c r="O128" s="52"/>
-      <c r="P128" s="52"/>
-      <c r="Q128" s="52"/>
-      <c r="R128" s="53"/>
-      <c r="S128" s="54"/>
-      <c r="T128" s="54"/>
-      <c r="U128" s="54"/>
-      <c r="V128" s="53"/>
+      <c r="O128" s="52">
+        <v>15868.4844</v>
+      </c>
+      <c r="P128" s="52">
+        <v>4881.59</v>
+      </c>
+      <c r="Q128" s="52">
+        <v>10986.8944</v>
+      </c>
+      <c r="R128" s="53">
+        <v>0.6923720074993425</v>
+      </c>
+      <c r="S128" s="54">
+        <v>317.92</v>
+      </c>
+      <c r="T128" s="54">
+        <v>106</v>
+      </c>
+      <c r="U128" s="54">
+        <v>211.92000000000002</v>
+      </c>
+      <c r="V128" s="53">
+        <v>0.6665827881227983</v>
+      </c>
       <c r="W128" s="53"/>
-      <c r="X128" s="55"/>
-      <c r="Y128" s="55"/>
-      <c r="Z128" s="53"/>
-      <c r="AA128" s="56"/>
+      <c r="X128" s="55">
+        <v>121.8556603773585</v>
+      </c>
+      <c r="Y128" s="55">
+        <v>62.79176131227983</v>
+      </c>
+      <c r="Z128" s="53">
+        <v>0.16260000000000002</v>
+      </c>
+      <c r="AA128" s="56">
+        <v>0.1885</v>
+      </c>
       <c r="AB128" s="57"/>
       <c r="AD128" s="35"/>
       <c r="AE128" s="35"/>
@@ -18943,30 +19559,74 @@
       <c r="C135" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D135" s="52"/>
-      <c r="E135" s="52"/>
-      <c r="F135" s="52"/>
-      <c r="G135" s="53"/>
-      <c r="H135" s="52"/>
-      <c r="I135" s="52"/>
-      <c r="J135" s="52"/>
-      <c r="K135" s="52"/>
-      <c r="L135" s="52"/>
-      <c r="M135" s="53"/>
+      <c r="D135" s="52">
+        <v>31802.4136956</v>
+      </c>
+      <c r="E135" s="52">
+        <v>16498.64</v>
+      </c>
+      <c r="F135" s="52">
+        <v>15303.7736956</v>
+      </c>
+      <c r="G135" s="53">
+        <v>0.48121421984134943</v>
+      </c>
+      <c r="H135" s="52">
+        <v>23448.14263</v>
+      </c>
+      <c r="I135" s="52">
+        <v>12360.83</v>
+      </c>
+      <c r="J135" s="52">
+        <v>15632.028429999998</v>
+      </c>
+      <c r="K135" s="52">
+        <v>11772.08</v>
+      </c>
+      <c r="L135" s="52">
+        <v>3859.9484299999986</v>
+      </c>
+      <c r="M135" s="53">
+        <v>0.24692562755273845</v>
+      </c>
       <c r="N135" s="53"/>
-      <c r="O135" s="52"/>
-      <c r="P135" s="52"/>
-      <c r="Q135" s="52"/>
-      <c r="R135" s="53"/>
-      <c r="S135" s="54"/>
-      <c r="T135" s="54"/>
-      <c r="U135" s="54"/>
-      <c r="V135" s="53"/>
+      <c r="O135" s="52">
+        <v>7816.1142</v>
+      </c>
+      <c r="P135" s="52">
+        <v>588.75</v>
+      </c>
+      <c r="Q135" s="52">
+        <v>7227.3642</v>
+      </c>
+      <c r="R135" s="53">
+        <v>0.92467484674162</v>
+      </c>
+      <c r="S135" s="54">
+        <v>156.69</v>
+      </c>
+      <c r="T135" s="54">
+        <v>11.5</v>
+      </c>
+      <c r="U135" s="54">
+        <v>145.19</v>
+      </c>
+      <c r="V135" s="53">
+        <v>0.9266066756015061</v>
+      </c>
       <c r="W135" s="53"/>
-      <c r="X135" s="55"/>
-      <c r="Y135" s="55"/>
-      <c r="Z135" s="53"/>
-      <c r="AA135" s="56"/>
+      <c r="X135" s="55">
+        <v>359.80956521739137</v>
+      </c>
+      <c r="Y135" s="55">
+        <v>53.31719360265494</v>
+      </c>
+      <c r="Z135" s="53">
+        <v>0.25079999999999997</v>
+      </c>
+      <c r="AA135" s="56">
+        <v>0.2627</v>
+      </c>
       <c r="AB135" s="57"/>
       <c r="AD135" s="35"/>
       <c r="AE135" s="35"/>
@@ -20637,30 +21297,74 @@
       <c r="C163" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D163" s="52"/>
-      <c r="E163" s="52"/>
-      <c r="F163" s="52"/>
-      <c r="G163" s="53"/>
-      <c r="H163" s="52"/>
-      <c r="I163" s="52"/>
-      <c r="J163" s="52"/>
-      <c r="K163" s="52"/>
-      <c r="L163" s="52"/>
-      <c r="M163" s="53"/>
+      <c r="D163" s="52">
+        <v>17899.333054</v>
+      </c>
+      <c r="E163" s="52">
+        <v>13424.5</v>
+      </c>
+      <c r="F163" s="52">
+        <v>4474.833053999999</v>
+      </c>
+      <c r="G163" s="53">
+        <v>0.24999998829565323</v>
+      </c>
+      <c r="H163" s="52">
+        <v>13919.4012884</v>
+      </c>
+      <c r="I163" s="52">
+        <v>14052.73</v>
+      </c>
+      <c r="J163" s="52">
+        <v>8410.9272884</v>
+      </c>
+      <c r="K163" s="52">
+        <v>8190.78</v>
+      </c>
+      <c r="L163" s="52">
+        <v>220.14728840000043</v>
+      </c>
+      <c r="M163" s="53">
+        <v>0.02617396166337312</v>
+      </c>
       <c r="N163" s="53"/>
-      <c r="O163" s="52"/>
-      <c r="P163" s="52"/>
-      <c r="Q163" s="52"/>
-      <c r="R163" s="53"/>
-      <c r="S163" s="54"/>
-      <c r="T163" s="54"/>
-      <c r="U163" s="54"/>
-      <c r="V163" s="53"/>
+      <c r="O163" s="52">
+        <v>5508.474</v>
+      </c>
+      <c r="P163" s="52">
+        <v>5861.95</v>
+      </c>
+      <c r="Q163" s="52">
+        <v>-353.47599999999966</v>
+      </c>
+      <c r="R163" s="53">
+        <v>-0.06416949594388567</v>
+      </c>
+      <c r="S163" s="54">
+        <v>110.44</v>
+      </c>
+      <c r="T163" s="54">
+        <v>116.25</v>
+      </c>
+      <c r="U163" s="54">
+        <v>-5.810000000000002</v>
+      </c>
+      <c r="V163" s="53">
+        <v>-0.05260775081492215</v>
+      </c>
       <c r="W163" s="53"/>
-      <c r="X163" s="55"/>
-      <c r="Y163" s="55"/>
-      <c r="Z163" s="53"/>
-      <c r="AA163" s="56"/>
+      <c r="X163" s="55">
+        <v>-5.404129032258065</v>
+      </c>
+      <c r="Y163" s="55">
+        <v>36.03704967040926</v>
+      </c>
+      <c r="Z163" s="53">
+        <v>-0.046799999999999994</v>
+      </c>
+      <c r="AA163" s="56">
+        <v>0.2224</v>
+      </c>
       <c r="AB163" s="57"/>
       <c r="AD163" s="35"/>
       <c r="AE163" s="35"/>
@@ -21108,30 +21812,74 @@
       <c r="C170" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D170" s="52"/>
-      <c r="E170" s="52"/>
-      <c r="F170" s="52"/>
-      <c r="G170" s="53"/>
-      <c r="H170" s="52"/>
-      <c r="I170" s="52"/>
-      <c r="J170" s="52"/>
-      <c r="K170" s="52"/>
-      <c r="L170" s="52"/>
-      <c r="M170" s="53"/>
+      <c r="D170" s="52">
+        <v>10827.20261235</v>
+      </c>
+      <c r="E170" s="52">
+        <v>0</v>
+      </c>
+      <c r="F170" s="52">
+        <v>10827.20261235</v>
+      </c>
+      <c r="G170" s="53">
+        <v>1</v>
+      </c>
+      <c r="H170" s="52">
+        <v>7687.765097</v>
+      </c>
+      <c r="I170" s="52">
+        <v>2116.21</v>
+      </c>
+      <c r="J170" s="52">
+        <v>4437.133697</v>
+      </c>
+      <c r="K170" s="52">
+        <v>1029.51</v>
+      </c>
+      <c r="L170" s="52">
+        <v>3407.623697</v>
+      </c>
+      <c r="M170" s="53">
+        <v>0.7679785937719064</v>
+      </c>
       <c r="N170" s="53"/>
-      <c r="O170" s="52"/>
-      <c r="P170" s="52"/>
-      <c r="Q170" s="52"/>
-      <c r="R170" s="53"/>
-      <c r="S170" s="54"/>
-      <c r="T170" s="54"/>
-      <c r="U170" s="54"/>
-      <c r="V170" s="53"/>
+      <c r="O170" s="52">
+        <v>3250.6314</v>
+      </c>
+      <c r="P170" s="52">
+        <v>1086.7</v>
+      </c>
+      <c r="Q170" s="52">
+        <v>2163.9314000000004</v>
+      </c>
+      <c r="R170" s="53">
+        <v>0.6656957168382734</v>
+      </c>
+      <c r="S170" s="54">
+        <v>65.13</v>
+      </c>
+      <c r="T170" s="54">
+        <v>24.33</v>
+      </c>
+      <c r="U170" s="54">
+        <v>40.8</v>
+      </c>
+      <c r="V170" s="53">
+        <v>0.6264394288346384</v>
+      </c>
       <c r="W170" s="53"/>
-      <c r="X170" s="55"/>
-      <c r="Y170" s="55"/>
-      <c r="Z170" s="53"/>
-      <c r="AA170" s="56"/>
+      <c r="X170" s="55">
+        <v>-86.97944923962187</v>
+      </c>
+      <c r="Y170" s="55">
+        <v>48.202633430830645</v>
+      </c>
+      <c r="Z170" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA170" s="56">
+        <v>0.29</v>
+      </c>
       <c r="AB170" s="57"/>
       <c r="AD170" s="35"/>
       <c r="AE170" s="35"/>
@@ -21593,30 +22341,74 @@
       <c r="C177" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D177" s="52"/>
-      <c r="E177" s="52"/>
-      <c r="F177" s="52"/>
-      <c r="G177" s="53"/>
-      <c r="H177" s="52"/>
-      <c r="I177" s="52"/>
-      <c r="J177" s="52"/>
-      <c r="K177" s="52"/>
-      <c r="L177" s="52"/>
-      <c r="M177" s="53"/>
+      <c r="D177" s="52">
+        <v>146237.1072</v>
+      </c>
+      <c r="E177" s="52">
+        <v>125386.21</v>
+      </c>
+      <c r="F177" s="52">
+        <v>20850.897199999992</v>
+      </c>
+      <c r="G177" s="53">
+        <v>0.14258280678024784</v>
+      </c>
+      <c r="H177" s="52">
+        <v>114651.8653946</v>
+      </c>
+      <c r="I177" s="52">
+        <v>105944.62</v>
+      </c>
+      <c r="J177" s="52">
+        <v>82888.0783946</v>
+      </c>
+      <c r="K177" s="52">
+        <v>78318.72</v>
+      </c>
+      <c r="L177" s="52">
+        <v>4569.3583946</v>
+      </c>
+      <c r="M177" s="53">
+        <v>0.055126846744437075</v>
+      </c>
       <c r="N177" s="53"/>
-      <c r="O177" s="52"/>
-      <c r="P177" s="52"/>
-      <c r="Q177" s="52"/>
-      <c r="R177" s="53"/>
-      <c r="S177" s="54"/>
-      <c r="T177" s="54"/>
-      <c r="U177" s="54"/>
-      <c r="V177" s="53"/>
+      <c r="O177" s="52">
+        <v>31763.787</v>
+      </c>
+      <c r="P177" s="52">
+        <v>27625.9</v>
+      </c>
+      <c r="Q177" s="52">
+        <v>4137.886999999999</v>
+      </c>
+      <c r="R177" s="53">
+        <v>0.1302705814013927</v>
+      </c>
+      <c r="S177" s="54">
+        <v>659.73</v>
+      </c>
+      <c r="T177" s="54">
+        <v>550.75</v>
+      </c>
+      <c r="U177" s="54">
+        <v>108.98000000000002</v>
+      </c>
+      <c r="V177" s="53">
+        <v>0.1651887893532203</v>
+      </c>
       <c r="W177" s="53"/>
-      <c r="X177" s="55"/>
-      <c r="Y177" s="55"/>
-      <c r="Z177" s="53"/>
-      <c r="AA177" s="56"/>
+      <c r="X177" s="55">
+        <v>35.3002088061734</v>
+      </c>
+      <c r="Y177" s="55">
+        <v>47.87601261940491</v>
+      </c>
+      <c r="Z177" s="53">
+        <v>0.1551</v>
+      </c>
+      <c r="AA177" s="56">
+        <v>0.216</v>
+      </c>
       <c r="AB177" s="57"/>
       <c r="AD177" s="35"/>
       <c r="AE177" s="35"/>
@@ -22086,30 +22878,74 @@
       <c r="C184" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D184" s="52"/>
-      <c r="E184" s="52"/>
-      <c r="F184" s="52"/>
-      <c r="G184" s="53"/>
-      <c r="H184" s="52"/>
-      <c r="I184" s="52"/>
-      <c r="J184" s="52"/>
-      <c r="K184" s="52"/>
-      <c r="L184" s="52"/>
-      <c r="M184" s="53"/>
+      <c r="D184" s="52">
+        <v>16897.52982004</v>
+      </c>
+      <c r="E184" s="52">
+        <v>5491.7</v>
+      </c>
+      <c r="F184" s="52">
+        <v>11405.829820039999</v>
+      </c>
+      <c r="G184" s="53">
+        <v>0.6749998337930436</v>
+      </c>
+      <c r="H184" s="52">
+        <v>9226.2731</v>
+      </c>
+      <c r="I184" s="52">
+        <v>5812.29</v>
+      </c>
+      <c r="J184" s="52">
+        <v>2977.1135000000004</v>
+      </c>
+      <c r="K184" s="52">
+        <v>2773.14</v>
+      </c>
+      <c r="L184" s="52">
+        <v>203.9735000000005</v>
+      </c>
+      <c r="M184" s="53">
+        <v>0.0685138473894262</v>
+      </c>
       <c r="N184" s="53"/>
-      <c r="O184" s="52"/>
-      <c r="P184" s="52"/>
-      <c r="Q184" s="52"/>
-      <c r="R184" s="53"/>
-      <c r="S184" s="54"/>
-      <c r="T184" s="54"/>
-      <c r="U184" s="54"/>
-      <c r="V184" s="53"/>
+      <c r="O184" s="52">
+        <v>6249.1596</v>
+      </c>
+      <c r="P184" s="52">
+        <v>3039.15</v>
+      </c>
+      <c r="Q184" s="52">
+        <v>3210.0096</v>
+      </c>
+      <c r="R184" s="53">
+        <v>0.5136706062043926</v>
+      </c>
+      <c r="S184" s="54">
+        <v>125.17</v>
+      </c>
+      <c r="T184" s="54">
+        <v>57.25</v>
+      </c>
+      <c r="U184" s="54">
+        <v>67.92</v>
+      </c>
+      <c r="V184" s="53">
+        <v>0.5426220340337141</v>
+      </c>
       <c r="W184" s="53"/>
-      <c r="X184" s="55"/>
-      <c r="Y184" s="55"/>
-      <c r="Z184" s="53"/>
-      <c r="AA184" s="56"/>
+      <c r="X184" s="55">
+        <v>-5.599825327510916</v>
+      </c>
+      <c r="Y184" s="55">
+        <v>61.286703843093385</v>
+      </c>
+      <c r="Z184" s="53">
+        <v>-0.0584</v>
+      </c>
+      <c r="AA184" s="56">
+        <v>0.454</v>
+      </c>
       <c r="AB184" s="57"/>
       <c r="AD184" s="35"/>
       <c r="AE184" s="35"/>
@@ -22575,30 +23411,74 @@
       <c r="C191" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D191" s="52"/>
-      <c r="E191" s="52"/>
-      <c r="F191" s="52"/>
-      <c r="G191" s="53"/>
-      <c r="H191" s="52"/>
-      <c r="I191" s="52"/>
-      <c r="J191" s="52"/>
-      <c r="K191" s="52"/>
-      <c r="L191" s="52"/>
-      <c r="M191" s="53"/>
+      <c r="D191" s="52">
+        <v>20992.11525559</v>
+      </c>
+      <c r="E191" s="52">
+        <v>14169.68</v>
+      </c>
+      <c r="F191" s="52">
+        <v>6822.43525559</v>
+      </c>
+      <c r="G191" s="53">
+        <v>0.3249998950807614</v>
+      </c>
+      <c r="H191" s="52">
+        <v>16299.085174</v>
+      </c>
+      <c r="I191" s="52">
+        <v>9699.51</v>
+      </c>
+      <c r="J191" s="52">
+        <v>9784.324774</v>
+      </c>
+      <c r="K191" s="52">
+        <v>8137.88</v>
+      </c>
+      <c r="L191" s="52">
+        <v>1646.4447740000005</v>
+      </c>
+      <c r="M191" s="53">
+        <v>0.16827372476178604</v>
+      </c>
       <c r="N191" s="53"/>
-      <c r="O191" s="52"/>
-      <c r="P191" s="52"/>
-      <c r="Q191" s="52"/>
-      <c r="R191" s="53"/>
-      <c r="S191" s="54"/>
-      <c r="T191" s="54"/>
-      <c r="U191" s="54"/>
-      <c r="V191" s="53"/>
+      <c r="O191" s="52">
+        <v>6514.7604</v>
+      </c>
+      <c r="P191" s="52">
+        <v>1561.63</v>
+      </c>
+      <c r="Q191" s="52">
+        <v>4953.1304</v>
+      </c>
+      <c r="R191" s="53">
+        <v>0.7602935635207705</v>
+      </c>
+      <c r="S191" s="54">
+        <v>130.62</v>
+      </c>
+      <c r="T191" s="54">
+        <v>34.75</v>
+      </c>
+      <c r="U191" s="54">
+        <v>95.87</v>
+      </c>
+      <c r="V191" s="53">
+        <v>0.7339611085591793</v>
+      </c>
       <c r="W191" s="53"/>
-      <c r="X191" s="55"/>
-      <c r="Y191" s="55"/>
-      <c r="Z191" s="53"/>
-      <c r="AA191" s="56"/>
+      <c r="X191" s="55">
+        <v>128.6379856115108</v>
+      </c>
+      <c r="Y191" s="55">
+        <v>35.92887828502527</v>
+      </c>
+      <c r="Z191" s="53">
+        <v>0.3155</v>
+      </c>
+      <c r="AA191" s="56">
+        <v>0.2236</v>
+      </c>
       <c r="AB191" s="57"/>
       <c r="AD191" s="35"/>
       <c r="AE191" s="35"/>
@@ -23058,30 +23938,74 @@
       <c r="C198" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D198" s="52"/>
-      <c r="E198" s="52"/>
-      <c r="F198" s="52"/>
-      <c r="G198" s="53"/>
-      <c r="H198" s="52"/>
-      <c r="I198" s="52"/>
-      <c r="J198" s="52"/>
-      <c r="K198" s="52"/>
-      <c r="L198" s="52"/>
-      <c r="M198" s="53"/>
+      <c r="D198" s="52">
+        <v>23770.94615247</v>
+      </c>
+      <c r="E198" s="52">
+        <v>10204.54</v>
+      </c>
+      <c r="F198" s="52">
+        <v>13566.406152469997</v>
+      </c>
+      <c r="G198" s="53">
+        <v>0.5707137639980029</v>
+      </c>
+      <c r="H198" s="52">
+        <v>14310.9577</v>
+      </c>
+      <c r="I198" s="52">
+        <v>7116.73</v>
+      </c>
+      <c r="J198" s="52">
+        <v>7389.335500000001</v>
+      </c>
+      <c r="K198" s="52">
+        <v>6605.049999999999</v>
+      </c>
+      <c r="L198" s="52">
+        <v>784.2855000000018</v>
+      </c>
+      <c r="M198" s="53">
+        <v>0.10613748692287713</v>
+      </c>
       <c r="N198" s="53"/>
-      <c r="O198" s="52"/>
-      <c r="P198" s="52"/>
-      <c r="Q198" s="52"/>
-      <c r="R198" s="53"/>
-      <c r="S198" s="54"/>
-      <c r="T198" s="54"/>
-      <c r="U198" s="54"/>
-      <c r="V198" s="53"/>
+      <c r="O198" s="52">
+        <v>6921.6222</v>
+      </c>
+      <c r="P198" s="52">
+        <v>511.68</v>
+      </c>
+      <c r="Q198" s="52">
+        <v>6409.9421999999995</v>
+      </c>
+      <c r="R198" s="53">
+        <v>0.9260751330807971</v>
+      </c>
+      <c r="S198" s="54">
+        <v>140.15</v>
+      </c>
+      <c r="T198" s="54">
+        <v>9.25</v>
+      </c>
+      <c r="U198" s="54">
+        <v>130.9</v>
+      </c>
+      <c r="V198" s="53">
+        <v>0.9339992864787727</v>
+      </c>
       <c r="W198" s="53"/>
-      <c r="X198" s="55"/>
-      <c r="Y198" s="55"/>
-      <c r="Z198" s="53"/>
-      <c r="AA198" s="56"/>
+      <c r="X198" s="55">
+        <v>333.8172972972973</v>
+      </c>
+      <c r="Y198" s="55">
+        <v>67.49902570438813</v>
+      </c>
+      <c r="Z198" s="53">
+        <v>0.30260000000000004</v>
+      </c>
+      <c r="AA198" s="56">
+        <v>0.398</v>
+      </c>
       <c r="AB198" s="57"/>
       <c r="AD198" s="35"/>
       <c r="AE198" s="35"/>
@@ -24119,30 +25043,74 @@
       <c r="C219" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D219" s="52"/>
-      <c r="E219" s="52"/>
-      <c r="F219" s="52"/>
-      <c r="G219" s="53"/>
-      <c r="H219" s="52"/>
-      <c r="I219" s="52"/>
-      <c r="J219" s="52"/>
-      <c r="K219" s="52"/>
-      <c r="L219" s="52"/>
-      <c r="M219" s="53"/>
+      <c r="D219" s="52">
+        <v>137109.56054889</v>
+      </c>
+      <c r="E219" s="52">
+        <v>42368.33</v>
+      </c>
+      <c r="F219" s="52">
+        <v>94741.23054889</v>
+      </c>
+      <c r="G219" s="53">
+        <v>0.6909892364151188</v>
+      </c>
+      <c r="H219" s="52">
+        <v>117394.569232</v>
+      </c>
+      <c r="I219" s="52">
+        <v>37161.14</v>
+      </c>
+      <c r="J219" s="52">
+        <v>99479.615032</v>
+      </c>
+      <c r="K219" s="52">
+        <v>37161.14</v>
+      </c>
+      <c r="L219" s="52">
+        <v>62318.475032</v>
+      </c>
+      <c r="M219" s="53">
+        <v>0.6264446742375689</v>
+      </c>
       <c r="N219" s="53"/>
-      <c r="O219" s="52"/>
-      <c r="P219" s="52"/>
-      <c r="Q219" s="52"/>
-      <c r="R219" s="53"/>
-      <c r="S219" s="54"/>
-      <c r="T219" s="54"/>
-      <c r="U219" s="54"/>
-      <c r="V219" s="53"/>
+      <c r="O219" s="52">
+        <v>17914.9542</v>
+      </c>
+      <c r="P219" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q219" s="52">
+        <v>17914.9542</v>
+      </c>
+      <c r="R219" s="53">
+        <v>1</v>
+      </c>
+      <c r="S219" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="T219" s="54">
+        <v>0</v>
+      </c>
+      <c r="U219" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="V219" s="53">
+        <v>1</v>
+      </c>
       <c r="W219" s="53"/>
-      <c r="X219" s="55"/>
-      <c r="Y219" s="55"/>
-      <c r="Z219" s="53"/>
-      <c r="AA219" s="56"/>
+      <c r="X219" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y219" s="55">
+        <v>54.93783457863793</v>
+      </c>
+      <c r="Z219" s="53">
+        <v>0.1229</v>
+      </c>
+      <c r="AA219" s="56">
+        <v>0.1438</v>
+      </c>
       <c r="AB219" s="57"/>
       <c r="AD219" s="35"/>
       <c r="AE219" s="35"/>
@@ -24604,30 +25572,74 @@
       <c r="C226" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D226" s="52"/>
-      <c r="E226" s="52"/>
-      <c r="F226" s="52"/>
-      <c r="G226" s="53"/>
-      <c r="H226" s="52"/>
-      <c r="I226" s="52"/>
-      <c r="J226" s="52"/>
-      <c r="K226" s="52"/>
-      <c r="L226" s="52"/>
-      <c r="M226" s="53"/>
+      <c r="D226" s="52">
+        <v>412300.73261827</v>
+      </c>
+      <c r="E226" s="52">
+        <v>353667.87</v>
+      </c>
+      <c r="F226" s="52">
+        <v>58632.86261826998</v>
+      </c>
+      <c r="G226" s="53">
+        <v>0.1422089702483149</v>
+      </c>
+      <c r="H226" s="52">
+        <v>306356.278672</v>
+      </c>
+      <c r="I226" s="52">
+        <v>253305.89</v>
+      </c>
+      <c r="J226" s="52">
+        <v>186357.488872</v>
+      </c>
+      <c r="K226" s="52">
+        <v>181341.87</v>
+      </c>
+      <c r="L226" s="52">
+        <v>5015.618871999992</v>
+      </c>
+      <c r="M226" s="53">
+        <v>0.026913964672731664</v>
+      </c>
       <c r="N226" s="53"/>
-      <c r="O226" s="52"/>
-      <c r="P226" s="52"/>
-      <c r="Q226" s="52"/>
-      <c r="R226" s="53"/>
-      <c r="S226" s="54"/>
-      <c r="T226" s="54"/>
-      <c r="U226" s="54"/>
-      <c r="V226" s="53"/>
+      <c r="O226" s="52">
+        <v>119998.7898</v>
+      </c>
+      <c r="P226" s="52">
+        <v>71964.02</v>
+      </c>
+      <c r="Q226" s="52">
+        <v>48034.769799999995</v>
+      </c>
+      <c r="R226" s="53">
+        <v>0.400293785296158</v>
+      </c>
+      <c r="S226" s="54">
+        <v>2412.45</v>
+      </c>
+      <c r="T226" s="54">
+        <v>1535.92</v>
+      </c>
+      <c r="U226" s="54">
+        <v>876.5299999999997</v>
+      </c>
+      <c r="V226" s="53">
+        <v>0.363336027689693</v>
+      </c>
       <c r="W226" s="53"/>
-      <c r="X226" s="55"/>
-      <c r="Y226" s="55"/>
-      <c r="Z226" s="53"/>
-      <c r="AA226" s="56"/>
+      <c r="X226" s="55">
+        <v>65.34323402260534</v>
+      </c>
+      <c r="Y226" s="55">
+        <v>43.91570973337064</v>
+      </c>
+      <c r="Z226" s="53">
+        <v>0.2838</v>
+      </c>
+      <c r="AA226" s="56">
+        <v>0.257</v>
+      </c>
       <c r="AB226" s="57"/>
       <c r="AD226" s="35"/>
       <c r="AE226" s="35"/>
@@ -25079,30 +26091,74 @@
       <c r="C233" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D233" s="52"/>
-      <c r="E233" s="52"/>
-      <c r="F233" s="52"/>
-      <c r="G233" s="53"/>
-      <c r="H233" s="52"/>
-      <c r="I233" s="52"/>
-      <c r="J233" s="52"/>
-      <c r="K233" s="52"/>
-      <c r="L233" s="52"/>
-      <c r="M233" s="53"/>
+      <c r="D233" s="52">
+        <v>8795.02836582</v>
+      </c>
+      <c r="E233" s="52">
+        <v>1740.2</v>
+      </c>
+      <c r="F233" s="52">
+        <v>7054.828365820001</v>
+      </c>
+      <c r="G233" s="53">
+        <v>0.8021382163174237</v>
+      </c>
+      <c r="H233" s="52">
+        <v>6369.1218</v>
+      </c>
+      <c r="I233" s="52">
+        <v>239.55</v>
+      </c>
+      <c r="J233" s="52">
+        <v>4527.894</v>
+      </c>
+      <c r="K233" s="52">
+        <v>239.55</v>
+      </c>
+      <c r="L233" s="52">
+        <v>4288.344</v>
+      </c>
+      <c r="M233" s="53">
+        <v>0.9470946095469549</v>
+      </c>
       <c r="N233" s="53"/>
-      <c r="O233" s="52"/>
-      <c r="P233" s="52"/>
-      <c r="Q233" s="52"/>
-      <c r="R233" s="53"/>
-      <c r="S233" s="54"/>
-      <c r="T233" s="54"/>
-      <c r="U233" s="54"/>
-      <c r="V233" s="53"/>
+      <c r="O233" s="52">
+        <v>1841.2278</v>
+      </c>
+      <c r="P233" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q233" s="52">
+        <v>1841.2278</v>
+      </c>
+      <c r="R233" s="53">
+        <v>1</v>
+      </c>
+      <c r="S233" s="54">
+        <v>36.92</v>
+      </c>
+      <c r="T233" s="54">
+        <v>0</v>
+      </c>
+      <c r="U233" s="54">
+        <v>36.92</v>
+      </c>
+      <c r="V233" s="53">
+        <v>1</v>
+      </c>
       <c r="W233" s="53"/>
-      <c r="X233" s="55"/>
-      <c r="Y233" s="55"/>
-      <c r="Z233" s="53"/>
-      <c r="AA233" s="56"/>
+      <c r="X233" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y233" s="55">
+        <v>65.70711175027087</v>
+      </c>
+      <c r="Z233" s="53">
+        <v>0.8623000000000001</v>
+      </c>
+      <c r="AA233" s="56">
+        <v>0.2758</v>
+      </c>
       <c r="AB233" s="57"/>
       <c r="AD233" s="35"/>
       <c r="AE233" s="35"/>
@@ -25508,30 +26564,74 @@
       <c r="C240" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D240" s="52"/>
-      <c r="E240" s="52"/>
-      <c r="F240" s="52"/>
-      <c r="G240" s="53"/>
-      <c r="H240" s="52"/>
-      <c r="I240" s="52"/>
-      <c r="J240" s="52"/>
-      <c r="K240" s="52"/>
-      <c r="L240" s="52"/>
-      <c r="M240" s="53"/>
+      <c r="D240" s="52">
+        <v>27503.13664251</v>
+      </c>
+      <c r="E240" s="52">
+        <v>0</v>
+      </c>
+      <c r="F240" s="52">
+        <v>27503.13664251</v>
+      </c>
+      <c r="G240" s="53">
+        <v>1</v>
+      </c>
+      <c r="H240" s="52">
+        <v>19683.280628</v>
+      </c>
+      <c r="I240" s="52">
+        <v>0</v>
+      </c>
+      <c r="J240" s="52">
+        <v>10693.531628</v>
+      </c>
+      <c r="K240" s="52">
+        <v>0</v>
+      </c>
+      <c r="L240" s="52">
+        <v>10693.531628</v>
+      </c>
+      <c r="M240" s="53">
+        <v>1</v>
+      </c>
       <c r="N240" s="53"/>
-      <c r="O240" s="52"/>
-      <c r="P240" s="52"/>
-      <c r="Q240" s="52"/>
-      <c r="R240" s="53"/>
-      <c r="S240" s="54"/>
-      <c r="T240" s="54"/>
-      <c r="U240" s="54"/>
-      <c r="V240" s="53"/>
+      <c r="O240" s="52">
+        <v>8989.749</v>
+      </c>
+      <c r="P240" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q240" s="52">
+        <v>8989.749</v>
+      </c>
+      <c r="R240" s="53">
+        <v>1</v>
+      </c>
+      <c r="S240" s="54">
+        <v>180.16</v>
+      </c>
+      <c r="T240" s="54">
+        <v>0</v>
+      </c>
+      <c r="U240" s="54">
+        <v>180.16</v>
+      </c>
+      <c r="V240" s="53">
+        <v>1</v>
+      </c>
       <c r="W240" s="53"/>
-      <c r="X240" s="55"/>
-      <c r="Y240" s="55"/>
-      <c r="Z240" s="53"/>
-      <c r="AA240" s="56"/>
+      <c r="X240" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y240" s="55">
+        <v>43.40506224750221</v>
+      </c>
+      <c r="Z240" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA240" s="56">
+        <v>0.2843</v>
+      </c>
       <c r="AB240" s="57"/>
       <c r="AD240" s="35"/>
       <c r="AE240" s="35"/>
@@ -25937,30 +27037,74 @@
       <c r="C247" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D247" s="52"/>
-      <c r="E247" s="52"/>
-      <c r="F247" s="52"/>
-      <c r="G247" s="53"/>
-      <c r="H247" s="52"/>
-      <c r="I247" s="52"/>
-      <c r="J247" s="52"/>
-      <c r="K247" s="52"/>
-      <c r="L247" s="52"/>
-      <c r="M247" s="53"/>
+      <c r="D247" s="52">
+        <v>40670.1518342</v>
+      </c>
+      <c r="E247" s="52">
+        <v>0</v>
+      </c>
+      <c r="F247" s="52">
+        <v>40670.1518342</v>
+      </c>
+      <c r="G247" s="53">
+        <v>1</v>
+      </c>
+      <c r="H247" s="52">
+        <v>29498.3116992</v>
+      </c>
+      <c r="I247" s="52">
+        <v>0</v>
+      </c>
+      <c r="J247" s="52">
+        <v>24964.3288992</v>
+      </c>
+      <c r="K247" s="52">
+        <v>0</v>
+      </c>
+      <c r="L247" s="52">
+        <v>24964.3288992</v>
+      </c>
+      <c r="M247" s="53">
+        <v>1</v>
+      </c>
       <c r="N247" s="53"/>
-      <c r="O247" s="52"/>
-      <c r="P247" s="52"/>
-      <c r="Q247" s="52"/>
-      <c r="R247" s="53"/>
-      <c r="S247" s="54"/>
-      <c r="T247" s="54"/>
-      <c r="U247" s="54"/>
-      <c r="V247" s="53"/>
+      <c r="O247" s="52">
+        <v>4533.9828</v>
+      </c>
+      <c r="P247" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q247" s="52">
+        <v>4533.9828</v>
+      </c>
+      <c r="R247" s="53">
+        <v>1</v>
+      </c>
+      <c r="S247" s="54">
+        <v>90.88</v>
+      </c>
+      <c r="T247" s="54">
+        <v>0</v>
+      </c>
+      <c r="U247" s="54">
+        <v>90.88</v>
+      </c>
+      <c r="V247" s="53">
+        <v>1</v>
+      </c>
       <c r="W247" s="53"/>
-      <c r="X247" s="55"/>
-      <c r="Y247" s="55"/>
-      <c r="Z247" s="53"/>
-      <c r="AA247" s="56"/>
+      <c r="X247" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y247" s="55">
+        <v>122.92957895026407</v>
+      </c>
+      <c r="Z247" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA247" s="56">
+        <v>0.2747</v>
+      </c>
       <c r="AB247" s="57"/>
       <c r="AD247" s="35"/>
       <c r="AE247" s="35"/>
@@ -26366,30 +27510,74 @@
       <c r="C254" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D254" s="52"/>
-      <c r="E254" s="52"/>
-      <c r="F254" s="52"/>
-      <c r="G254" s="53"/>
-      <c r="H254" s="52"/>
-      <c r="I254" s="52"/>
-      <c r="J254" s="52"/>
-      <c r="K254" s="52"/>
-      <c r="L254" s="52"/>
-      <c r="M254" s="53"/>
+      <c r="D254" s="52">
+        <v>21396.50036782</v>
+      </c>
+      <c r="E254" s="52">
+        <v>0</v>
+      </c>
+      <c r="F254" s="52">
+        <v>21396.50036782</v>
+      </c>
+      <c r="G254" s="53">
+        <v>1</v>
+      </c>
+      <c r="H254" s="52">
+        <v>15378.244372</v>
+      </c>
+      <c r="I254" s="52">
+        <v>0</v>
+      </c>
+      <c r="J254" s="52">
+        <v>8344.608772</v>
+      </c>
+      <c r="K254" s="52">
+        <v>0</v>
+      </c>
+      <c r="L254" s="52">
+        <v>8344.608772</v>
+      </c>
+      <c r="M254" s="53">
+        <v>1</v>
+      </c>
       <c r="N254" s="53"/>
-      <c r="O254" s="52"/>
-      <c r="P254" s="52"/>
-      <c r="Q254" s="52"/>
-      <c r="R254" s="53"/>
-      <c r="S254" s="54"/>
-      <c r="T254" s="54"/>
-      <c r="U254" s="54"/>
-      <c r="V254" s="53"/>
+      <c r="O254" s="52">
+        <v>7033.6356</v>
+      </c>
+      <c r="P254" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q254" s="52">
+        <v>7033.6356</v>
+      </c>
+      <c r="R254" s="53">
+        <v>1</v>
+      </c>
+      <c r="S254" s="54">
+        <v>140.9</v>
+      </c>
+      <c r="T254" s="54">
+        <v>0</v>
+      </c>
+      <c r="U254" s="54">
+        <v>140.9</v>
+      </c>
+      <c r="V254" s="53">
+        <v>1</v>
+      </c>
       <c r="W254" s="53"/>
-      <c r="X254" s="55"/>
-      <c r="Y254" s="55"/>
-      <c r="Z254" s="53"/>
-      <c r="AA254" s="56"/>
+      <c r="X254" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y254" s="55">
+        <v>42.71295951611073</v>
+      </c>
+      <c r="Z254" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA254" s="56">
+        <v>0.2813</v>
+      </c>
       <c r="AB254" s="57"/>
       <c r="AD254" s="35"/>
       <c r="AE254" s="35"/>
@@ -26795,30 +27983,74 @@
       <c r="C261" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D261" s="52"/>
-      <c r="E261" s="52"/>
-      <c r="F261" s="52"/>
-      <c r="G261" s="53"/>
-      <c r="H261" s="52"/>
-      <c r="I261" s="52"/>
-      <c r="J261" s="52"/>
-      <c r="K261" s="52"/>
-      <c r="L261" s="52"/>
-      <c r="M261" s="53"/>
+      <c r="D261" s="52">
+        <v>239296.88379393</v>
+      </c>
+      <c r="E261" s="52">
+        <v>19872.16</v>
+      </c>
+      <c r="F261" s="52">
+        <v>219424.72379393</v>
+      </c>
+      <c r="G261" s="53">
+        <v>0.916956043534972</v>
+      </c>
+      <c r="H261" s="52">
+        <v>203192.691868</v>
+      </c>
+      <c r="I261" s="52">
+        <v>18292.87</v>
+      </c>
+      <c r="J261" s="52">
+        <v>175849.529668</v>
+      </c>
+      <c r="K261" s="52">
+        <v>16897.46</v>
+      </c>
+      <c r="L261" s="52">
+        <v>158952.069668</v>
+      </c>
+      <c r="M261" s="53">
+        <v>0.9039095524912576</v>
+      </c>
       <c r="N261" s="53"/>
-      <c r="O261" s="52"/>
-      <c r="P261" s="52"/>
-      <c r="Q261" s="52"/>
-      <c r="R261" s="53"/>
-      <c r="S261" s="54"/>
-      <c r="T261" s="54"/>
-      <c r="U261" s="54"/>
-      <c r="V261" s="53"/>
+      <c r="O261" s="52">
+        <v>27343.1622</v>
+      </c>
+      <c r="P261" s="52">
+        <v>1395.41</v>
+      </c>
+      <c r="Q261" s="52">
+        <v>25947.7522</v>
+      </c>
+      <c r="R261" s="53">
+        <v>0.9489667658117465</v>
+      </c>
+      <c r="S261" s="54">
+        <v>547.57</v>
+      </c>
+      <c r="T261" s="54">
+        <v>27.84</v>
+      </c>
+      <c r="U261" s="54">
+        <v>519.73</v>
+      </c>
+      <c r="V261" s="53">
+        <v>0.9491571853826908</v>
+      </c>
       <c r="W261" s="53"/>
-      <c r="X261" s="55"/>
-      <c r="Y261" s="55"/>
-      <c r="Z261" s="53"/>
-      <c r="AA261" s="56"/>
+      <c r="X261" s="55">
+        <v>56.727370689655174</v>
+      </c>
+      <c r="Y261" s="55">
+        <v>65.93529946112827</v>
+      </c>
+      <c r="Z261" s="53">
+        <v>0.0795</v>
+      </c>
+      <c r="AA261" s="56">
+        <v>0.1509</v>
+      </c>
       <c r="AB261" s="57"/>
       <c r="AD261" s="35"/>
       <c r="AE261" s="35"/>
@@ -27506,16 +28738,16 @@
         <v>22202.890000000014</v>
       </c>
       <c r="D4" s="52">
-        <v>21022.23000000001</v>
+        <v>21523.99000000002</v>
       </c>
       <c r="E4" s="52">
-        <v>1180.6600000000035</v>
+        <v>678.8999999999942</v>
       </c>
       <c r="F4" s="52">
         <v>0</v>
       </c>
       <c r="G4" s="53">
-        <v>0.053175960426773396</v>
+        <v>0.03057710054862199</v>
       </c>
       <c r="H4" s="53">
         <v>0.2149</v>
@@ -27530,16 +28762,16 @@
         <v>7000</v>
       </c>
       <c r="L4" s="53">
-        <v>-0.26209831242689546</v>
+        <v>-0.2846971723050469</v>
       </c>
       <c r="M4" s="52">
-        <v>-5819.3399999999965</v>
+        <v>-6321.100000000006</v>
       </c>
       <c r="N4" s="54">
         <v>20</v>
       </c>
       <c r="O4" s="58">
-        <v>-83.13342857142852</v>
+        <v>-90.30142857142866</v>
       </c>
     </row>
     <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -27570,16 +28802,16 @@
         <v>42019.899999999994</v>
       </c>
       <c r="D6" s="52">
-        <v>18657.01999999999</v>
+        <v>20112.42</v>
       </c>
       <c r="E6" s="52">
-        <v>23362.880000000005</v>
+        <v>21907.479999999996</v>
       </c>
       <c r="F6" s="52">
         <v>7</v>
       </c>
       <c r="G6" s="53">
-        <v>0.5561621993388849</v>
+        <v>0.5215262292390034</v>
       </c>
       <c r="H6" s="53">
         <v>0.239214585617637</v>
@@ -27594,16 +28826,16 @@
         <v>20272.6</v>
       </c>
       <c r="L6" s="53">
-        <v>0.07370983748176475</v>
+        <v>0.03907386738188329</v>
       </c>
       <c r="M6" s="52">
-        <v>3097.280000000006</v>
+        <v>1641.8799999999974</v>
       </c>
       <c r="N6" s="54">
         <v>-52.5</v>
       </c>
       <c r="O6" s="58">
-        <v>6.921296089385488</v>
+        <v>3.669005586592173</v>
       </c>
       <c r="Q6" s="35" t="s">
         <v>121</v>
@@ -27761,16 +28993,16 @@
         <v>93276.07999999999</v>
       </c>
       <c r="D12" s="52">
-        <v>61105.389999999985</v>
+        <v>62494.389999999985</v>
       </c>
       <c r="E12" s="52">
-        <v>32170.690000000002</v>
+        <v>30781.690000000002</v>
       </c>
       <c r="F12" s="52">
         <v>3</v>
       </c>
       <c r="G12" s="53">
-        <v>0.34492969687405395</v>
+        <v>0.3300384192817709</v>
       </c>
       <c r="H12" s="53">
         <v>0.176316261575212</v>
@@ -27785,16 +29017,16 @@
         <v>2640</v>
       </c>
       <c r="L12" s="53">
-        <v>0.31662662067273845</v>
+        <v>0.3017353430804554</v>
       </c>
       <c r="M12" s="52">
-        <v>29533.690000000002</v>
+        <v>28144.690000000002</v>
       </c>
       <c r="N12" s="54">
         <v>53</v>
       </c>
       <c r="O12" s="58">
-        <v>428.02449275362324</v>
+        <v>407.89405797101455</v>
       </c>
       <c r="Q12" s="35" t="s">
         <v>123</v>
@@ -27828,16 +29060,16 @@
         <v>61369.72</v>
       </c>
       <c r="D14" s="52">
-        <v>14493.379999999997</v>
+        <v>14830.879999999997</v>
       </c>
       <c r="E14" s="52">
-        <v>46876.340000000004</v>
+        <v>46538.840000000004</v>
       </c>
       <c r="F14" s="52">
         <v>0</v>
       </c>
       <c r="G14" s="53">
-        <v>0.7638349987583454</v>
+        <v>0.7583355439783659</v>
       </c>
       <c r="H14" s="53">
         <v>0.266338527271097</v>
@@ -27852,16 +29084,16 @@
         <v>3000</v>
       </c>
       <c r="L14" s="53">
-        <v>0.7149509562696392</v>
+        <v>0.7094515014896597</v>
       </c>
       <c r="M14" s="52">
-        <v>43876.340000000004</v>
+        <v>43538.840000000004</v>
       </c>
       <c r="N14" s="54">
         <v>-112</v>
       </c>
       <c r="O14" s="58">
-        <v>-391.7530357142858</v>
+        <v>-388.7396428571429</v>
       </c>
     </row>
     <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -27954,16 +29186,16 @@
         <v>27482.319999999992</v>
       </c>
       <c r="D18" s="52">
-        <v>14933.520000000004</v>
+        <v>18539.01000000001</v>
       </c>
       <c r="E18" s="52">
-        <v>12548.799999999988</v>
+        <v>8943.309999999983</v>
       </c>
       <c r="F18" s="52">
         <v>0</v>
       </c>
       <c r="G18" s="53">
-        <v>0.45661356100940503</v>
+        <v>0.32542048851770833</v>
       </c>
       <c r="H18" s="53">
         <v>0.296537658865514</v>
@@ -27978,16 +29210,16 @@
         <v>8200</v>
       </c>
       <c r="L18" s="53">
-        <v>0.15823991569852872</v>
+        <v>0.027046843206832004</v>
       </c>
       <c r="M18" s="52">
-        <v>4348.799999999988</v>
+        <v>743.3099999999831</v>
       </c>
       <c r="N18" s="54">
         <v>-269</v>
       </c>
       <c r="O18" s="58">
-        <v>-23.00952380952375</v>
+        <v>-3.9328571428570536</v>
       </c>
       <c r="Q18" s="35" t="s">
         <v>124</v>
@@ -28074,19 +29306,19 @@
         <v>39</v>
       </c>
       <c r="C22" s="52">
-        <v>0</v>
+        <v>19065.239999999998</v>
       </c>
       <c r="D22" s="52">
-        <v>12195.39</v>
+        <v>14898.84</v>
       </c>
       <c r="E22" s="52">
-        <v>-12195.39</v>
+        <v>4166.399999999998</v>
       </c>
       <c r="F22" s="52">
         <v>3</v>
       </c>
       <c r="G22" s="53">
-        <v>0</v>
+        <v>0.21869118878125837</v>
       </c>
       <c r="H22" s="53">
         <v>0.252488256827238</v>
@@ -28097,10 +29329,10 @@
         <v>0</v>
       </c>
       <c r="L22" s="53">
-        <v>0</v>
+        <v>0.21869118878125837</v>
       </c>
       <c r="M22" s="52">
-        <v>-12192.39</v>
+        <v>4169.399999999998</v>
       </c>
       <c r="N22" s="54"/>
       <c r="O22" s="58">
@@ -28132,19 +29364,19 @@
         <v>40</v>
       </c>
       <c r="C24" s="52">
-        <v>0</v>
+        <v>16999.83</v>
       </c>
       <c r="D24" s="52">
-        <v>9681.120000000003</v>
+        <v>12895.309999999998</v>
       </c>
       <c r="E24" s="52">
-        <v>-9681.120000000003</v>
+        <v>4104.520000000004</v>
       </c>
       <c r="F24" s="52">
         <v>3</v>
       </c>
       <c r="G24" s="53">
-        <v>0</v>
+        <v>0.2416212397418094</v>
       </c>
       <c r="H24" s="53"/>
       <c r="I24" s="54"/>
@@ -28153,10 +29385,10 @@
         <v>0</v>
       </c>
       <c r="L24" s="53">
-        <v>0</v>
+        <v>0.2416212397418094</v>
       </c>
       <c r="M24" s="52">
-        <v>-9678.120000000003</v>
+        <v>4107.520000000004</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="58">
@@ -28499,10 +29731,10 @@
         <v>0</v>
       </c>
       <c r="D36" s="52">
-        <v>0</v>
+        <v>58.32</v>
       </c>
       <c r="E36" s="52">
-        <v>0</v>
+        <v>-58.32</v>
       </c>
       <c r="F36" s="52">
         <v>0</v>
@@ -28524,11 +29756,11 @@
         <v>0</v>
       </c>
       <c r="M36" s="52">
-        <v>-3200</v>
+        <v>-3258.32</v>
       </c>
       <c r="N36" s="54"/>
       <c r="O36" s="58">
-        <v>-40</v>
+        <v>-40.729</v>
       </c>
     </row>
     <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -28851,10 +30083,10 @@
         <v>0</v>
       </c>
       <c r="D48" s="99">
-        <v>2218.25</v>
+        <v>3650.3599999999988</v>
       </c>
       <c r="E48" s="99">
-        <v>-2218.25</v>
+        <v>-3650.3599999999988</v>
       </c>
       <c r="F48" s="99"/>
       <c r="G48" s="100">
@@ -28874,13 +30106,13 @@
         <v>0</v>
       </c>
       <c r="M48" s="99">
-        <v>-4748.25</v>
+        <v>-6180.359999999999</v>
       </c>
       <c r="N48" s="98">
         <v>-44.75</v>
       </c>
       <c r="O48" s="60">
-        <v>106.10614525139665</v>
+        <v>138.10860335195528</v>
       </c>
     </row>
     <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -28970,10 +30202,10 @@
         <v>0</v>
       </c>
       <c r="D52" s="99">
-        <v>2942.1800000000076</v>
+        <v>3062.5</v>
       </c>
       <c r="E52" s="99">
-        <v>-2942.1800000000076</v>
+        <v>-3062.5</v>
       </c>
       <c r="F52" s="99"/>
       <c r="G52" s="100">
@@ -28995,13 +30227,13 @@
         <v>0</v>
       </c>
       <c r="M52" s="99">
-        <v>-4222.180000000008</v>
+        <v>-4342.5</v>
       </c>
       <c r="N52" s="98">
         <v>-304.75</v>
       </c>
       <c r="O52" s="60">
-        <v>15.480036663611394</v>
+        <v>15.921173235563703</v>
       </c>
     </row>
     <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -29032,10 +30264,10 @@
         <v>0</v>
       </c>
       <c r="D54" s="99">
-        <v>1718.2499999999995</v>
+        <v>2109.5099999999998</v>
       </c>
       <c r="E54" s="99">
-        <v>-1718.2499999999995</v>
+        <v>-2109.5099999999998</v>
       </c>
       <c r="F54" s="99"/>
       <c r="G54" s="100">
@@ -29057,13 +30289,13 @@
         <v>0</v>
       </c>
       <c r="M54" s="99">
-        <v>-2358.2499999999995</v>
+        <v>-2749.5099999999998</v>
       </c>
       <c r="N54" s="98">
         <v>-11.25</v>
       </c>
       <c r="O54" s="60">
-        <v>-496.47368421052624</v>
+        <v>-578.8442105263157</v>
       </c>
     </row>
     <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -29279,17 +30511,17 @@
         <v>61</v>
       </c>
       <c r="C64" s="99">
-        <v>0</v>
+        <v>12193.580000000002</v>
       </c>
       <c r="D64" s="99">
         <v>11037.14</v>
       </c>
       <c r="E64" s="99">
-        <v>-11037.14</v>
+        <v>1156.4400000000023</v>
       </c>
       <c r="F64" s="99"/>
       <c r="G64" s="100">
-        <v>0</v>
+        <v>0.09484007157865058</v>
       </c>
       <c r="H64" s="100">
         <v>0.143790046441692</v>
@@ -29302,10 +30534,10 @@
         <v>1750</v>
       </c>
       <c r="L64" s="100">
-        <v>0</v>
+        <v>-0.04867807485578457</v>
       </c>
       <c r="M64" s="99">
-        <v>-12787.14</v>
+        <v>-593.5599999999977</v>
       </c>
       <c r="N64" s="98"/>
       <c r="O64" s="60">
@@ -29340,14 +30572,14 @@
         <v>82279.71999999997</v>
       </c>
       <c r="D66" s="99">
-        <v>22406.589999999997</v>
+        <v>18983.080000000016</v>
       </c>
       <c r="E66" s="99">
-        <v>59873.129999999976</v>
+        <v>63296.639999999956</v>
       </c>
       <c r="F66" s="99"/>
       <c r="G66" s="100">
-        <v>0.727677853060268</v>
+        <v>0.7692860403511337</v>
       </c>
       <c r="H66" s="100">
         <v>0.256265521519856</v>
@@ -29362,16 +30594,16 @@
         <v>3200</v>
       </c>
       <c r="L66" s="100">
-        <v>0.6887861310174609</v>
+        <v>0.7303943183083265</v>
       </c>
       <c r="M66" s="99">
-        <v>56673.129999999976</v>
+        <v>60096.639999999956</v>
       </c>
       <c r="N66" s="98">
         <v>-1014.25</v>
       </c>
       <c r="O66" s="60">
-        <v>-60.66163232539468</v>
+        <v>-64.3260797431094</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -29382,17 +30614,17 @@
         <v>68</v>
       </c>
       <c r="C67" s="99">
-        <v>10598.48</v>
+        <v>19872.16</v>
       </c>
       <c r="D67" s="99">
-        <v>18235.02</v>
+        <v>18292.87</v>
       </c>
       <c r="E67" s="99">
-        <v>-7636.540000000001</v>
+        <v>1579.2900000000009</v>
       </c>
       <c r="F67" s="99"/>
       <c r="G67" s="100">
-        <v>-0.7205316234026012</v>
+        <v>0.07947248814421788</v>
       </c>
       <c r="H67" s="100">
         <f>'Deliverables Sheet'!AA256</f>
@@ -29403,10 +30635,10 @@
         <v>0</v>
       </c>
       <c r="L67" s="100">
-        <v>-0.7205316234026012</v>
+        <v>0.07947248814421788</v>
       </c>
       <c r="M67" s="99">
-        <v>-7636.540000000001</v>
+        <v>1579.2900000000009</v>
       </c>
       <c r="N67" s="98"/>
       <c r="O67" s="60">
@@ -29538,17 +30770,17 @@
         <v>63</v>
       </c>
       <c r="C71" s="99">
-        <v>0</v>
+        <v>1740.2</v>
       </c>
       <c r="D71" s="99">
-        <v>397</v>
+        <v>239.55</v>
       </c>
       <c r="E71" s="99">
-        <v>-397</v>
+        <v>1500.65</v>
       </c>
       <c r="F71" s="99"/>
       <c r="G71" s="100">
-        <v>0</v>
+        <v>0.8623434088035858</v>
       </c>
       <c r="H71" s="100">
         <f>'Deliverables Sheet'!AA228</f>
@@ -29559,10 +30791,10 @@
         <v>0</v>
       </c>
       <c r="L71" s="100">
-        <v>0</v>
+        <v>0.8623434088035858</v>
       </c>
       <c r="M71" s="99">
-        <v>-397</v>
+        <v>1500.65</v>
       </c>
       <c r="N71" s="98"/>
       <c r="O71" s="60">
@@ -29611,25 +30843,25 @@
         <v>127</v>
       </c>
       <c r="C74" s="104">
-        <v>432684.38999999996</v>
+        <v>491956.92</v>
       </c>
       <c r="D74" s="104">
-        <v>234541.40999999992</v>
+        <v>246227.09999999998</v>
       </c>
       <c r="E74" s="105">
-        <v>198142.97999999998</v>
+        <v>245729.81999999995</v>
       </c>
       <c r="F74" s="106" t="s">
         <v>128</v>
       </c>
       <c r="G74" s="107">
-        <v>0.4579388223365303</v>
+        <v>0.49949458989213924</v>
       </c>
       <c r="H74" s="108" t="s">
         <v>129</v>
       </c>
       <c r="I74" s="109">
-        <v>0.295620509905615</v>
+        <v>0.3567329025476457</v>
       </c>
       <c r="J74" s="36"/>
       <c r="K74" s="36"/>
@@ -30184,10 +31416,10 @@
         <v>638.02</v>
       </c>
       <c r="D4" s="54">
-        <v>616.75</v>
+        <v>625.25</v>
       </c>
       <c r="E4" s="54">
-        <v>21.269999999999982</v>
+        <v>12.769999999999982</v>
       </c>
       <c r="F4" s="54">
         <v>0</v>
@@ -30243,10 +31475,10 @@
         <v>363.57</v>
       </c>
       <c r="D6" s="54">
-        <v>272.5</v>
+        <v>304.75</v>
       </c>
       <c r="E6" s="54">
-        <v>91.07</v>
+        <v>58.81999999999999</v>
       </c>
       <c r="F6" s="54"/>
       <c r="G6" s="54"/>
@@ -30410,10 +31642,10 @@
         <v>1124.47</v>
       </c>
       <c r="D12" s="54">
-        <v>783</v>
+        <v>813.5</v>
       </c>
       <c r="E12" s="54">
-        <v>341.47</v>
+        <v>310.97</v>
       </c>
       <c r="F12" s="54"/>
       <c r="G12" s="54"/>
@@ -30469,10 +31701,10 @@
         <v>501.83</v>
       </c>
       <c r="D14" s="54">
-        <v>358.75</v>
+        <v>366.25</v>
       </c>
       <c r="E14" s="54">
-        <v>143.07999999999998</v>
+        <v>135.57999999999998</v>
       </c>
       <c r="F14" s="54"/>
       <c r="G14" s="54"/>
@@ -30580,10 +31812,10 @@
         <v>685.48</v>
       </c>
       <c r="D18" s="54">
-        <v>669</v>
+        <v>699.75</v>
       </c>
       <c r="E18" s="54">
-        <v>16.480000000000018</v>
+        <v>-14.269999999999982</v>
       </c>
       <c r="F18" s="54"/>
       <c r="G18" s="54"/>
@@ -30682,10 +31914,10 @@
         <v>193.32</v>
       </c>
       <c r="D22" s="54">
-        <v>52.75</v>
+        <v>83.5</v>
       </c>
       <c r="E22" s="54">
-        <v>140.57</v>
+        <v>109.82</v>
       </c>
       <c r="F22" s="54"/>
       <c r="G22" s="54"/>
@@ -30738,10 +31970,10 @@
         <v>472.14</v>
       </c>
       <c r="D24" s="54">
-        <v>167.25</v>
+        <v>202</v>
       </c>
       <c r="E24" s="54">
-        <v>304.89</v>
+        <v>270.14</v>
       </c>
       <c r="F24" s="54"/>
       <c r="G24" s="54"/>
@@ -31045,13 +32277,13 @@
         <v>48</v>
       </c>
       <c r="C36" s="54">
-        <v>86.01</v>
+        <v>82.37</v>
       </c>
       <c r="D36" s="54">
         <v>0</v>
       </c>
       <c r="E36" s="54">
-        <v>86.01</v>
+        <v>82.37</v>
       </c>
       <c r="F36" s="54"/>
       <c r="G36" s="54"/>
@@ -31375,10 +32607,10 @@
         <v>110.44</v>
       </c>
       <c r="D48" s="54">
-        <v>95.5</v>
+        <v>116.25</v>
       </c>
       <c r="E48" s="54">
-        <v>14.939999999999998</v>
+        <v>-5.810000000000002</v>
       </c>
       <c r="F48" s="54"/>
       <c r="G48" s="54"/>
@@ -31483,10 +32715,10 @@
         <v>659.73</v>
       </c>
       <c r="D52" s="54">
-        <v>548.75</v>
+        <v>550.75</v>
       </c>
       <c r="E52" s="54">
-        <v>110.98000000000002</v>
+        <v>108.98000000000002</v>
       </c>
       <c r="F52" s="54"/>
       <c r="G52" s="54"/>
@@ -31538,10 +32770,10 @@
         <v>125.17</v>
       </c>
       <c r="D54" s="54">
-        <v>49.25</v>
+        <v>57.25</v>
       </c>
       <c r="E54" s="54">
-        <v>75.92</v>
+        <v>67.92</v>
       </c>
       <c r="F54" s="54"/>
       <c r="G54" s="54"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-28T19:05:07Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -10418,30 +10418,74 @@
       <c r="C9" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D9" s="52"/>
-      <c r="E9" s="52"/>
-      <c r="F9" s="52"/>
-      <c r="G9" s="53"/>
-      <c r="H9" s="52"/>
-      <c r="I9" s="52"/>
-      <c r="J9" s="52"/>
-      <c r="K9" s="52"/>
-      <c r="L9" s="52"/>
-      <c r="M9" s="53"/>
+      <c r="D9" s="52">
+        <v>267886.84883856</v>
+      </c>
+      <c r="E9" s="52">
+        <v>238732.97</v>
+      </c>
+      <c r="F9" s="52">
+        <v>29153.87883855999</v>
+      </c>
+      <c r="G9" s="53">
+        <v>0.10882907826553799</v>
+      </c>
+      <c r="H9" s="52">
+        <v>225410.5455298</v>
+      </c>
+      <c r="I9" s="52">
+        <v>189481.67</v>
+      </c>
+      <c r="J9" s="52">
+        <v>193787.2413298</v>
+      </c>
+      <c r="K9" s="52">
+        <v>158312.05000000002</v>
+      </c>
+      <c r="L9" s="52">
+        <v>35475.19132979997</v>
+      </c>
+      <c r="M9" s="53">
+        <v>0.1830625746378521</v>
+      </c>
       <c r="N9" s="53"/>
-      <c r="O9" s="52"/>
-      <c r="P9" s="52"/>
-      <c r="Q9" s="52"/>
-      <c r="R9" s="53"/>
-      <c r="S9" s="54"/>
-      <c r="T9" s="54"/>
-      <c r="U9" s="54"/>
-      <c r="V9" s="53"/>
+      <c r="O9" s="52">
+        <v>31623.3042</v>
+      </c>
+      <c r="P9" s="52">
+        <v>31169.62</v>
+      </c>
+      <c r="Q9" s="52">
+        <v>453.6841999999997</v>
+      </c>
+      <c r="R9" s="53">
+        <v>0.014346514745287108</v>
+      </c>
+      <c r="S9" s="54">
+        <v>638.02</v>
+      </c>
+      <c r="T9" s="54">
+        <v>625.25</v>
+      </c>
+      <c r="U9" s="54">
+        <v>12.769999999999982</v>
+      </c>
+      <c r="V9" s="53">
+        <v>0.020015046550264853</v>
+      </c>
       <c r="W9" s="53"/>
-      <c r="X9" s="55"/>
-      <c r="Y9" s="55"/>
-      <c r="Z9" s="53"/>
-      <c r="AA9" s="56"/>
+      <c r="X9" s="55">
+        <v>78.77057177129149</v>
+      </c>
+      <c r="Y9" s="55">
+        <v>66.57519091683645</v>
+      </c>
+      <c r="Z9" s="53">
+        <v>0.20629999999999998</v>
+      </c>
+      <c r="AA9" s="56">
+        <v>0.1586</v>
+      </c>
       <c r="AB9" s="57"/>
       <c r="AD9" s="35"/>
       <c r="AE9" s="35"/>
@@ -10913,30 +10957,74 @@
       <c r="C16" s="63" t="s">
         <v>104</v>
       </c>
-      <c r="D16" s="52"/>
-      <c r="E16" s="62"/>
-      <c r="F16" s="52"/>
-      <c r="G16" s="53"/>
-      <c r="H16" s="52"/>
-      <c r="I16" s="52"/>
-      <c r="J16" s="52"/>
-      <c r="K16" s="52"/>
-      <c r="L16" s="52"/>
-      <c r="M16" s="53"/>
+      <c r="D16" s="52">
+        <v>132076.08820213</v>
+      </c>
+      <c r="E16" s="62">
+        <v>127883.98</v>
+      </c>
+      <c r="F16" s="52">
+        <v>4192.108202129995</v>
+      </c>
+      <c r="G16" s="53">
+        <v>0.031740099659178046</v>
+      </c>
+      <c r="H16" s="52">
+        <v>103822.973895</v>
+      </c>
+      <c r="I16" s="52">
+        <v>94249.74</v>
+      </c>
+      <c r="J16" s="52">
+        <v>85672.874895</v>
+      </c>
+      <c r="K16" s="52">
+        <v>80502.31</v>
+      </c>
+      <c r="L16" s="52">
+        <v>5170.564895000003</v>
+      </c>
+      <c r="M16" s="53">
+        <v>0.060352414942734287</v>
+      </c>
       <c r="N16" s="53"/>
-      <c r="O16" s="52"/>
-      <c r="P16" s="52"/>
-      <c r="Q16" s="52"/>
-      <c r="R16" s="53"/>
-      <c r="S16" s="54"/>
-      <c r="T16" s="54"/>
-      <c r="U16" s="54"/>
-      <c r="V16" s="53"/>
+      <c r="O16" s="52">
+        <v>18150.099</v>
+      </c>
+      <c r="P16" s="52">
+        <v>13747.43</v>
+      </c>
+      <c r="Q16" s="52">
+        <v>4402.668999999998</v>
+      </c>
+      <c r="R16" s="53">
+        <v>0.24256997165690383</v>
+      </c>
+      <c r="S16" s="54">
+        <v>363.57</v>
+      </c>
+      <c r="T16" s="54">
+        <v>304.75</v>
+      </c>
+      <c r="U16" s="54">
+        <v>58.81999999999999</v>
+      </c>
+      <c r="V16" s="53">
+        <v>0.16178452567593585</v>
+      </c>
       <c r="W16" s="53"/>
-      <c r="X16" s="55"/>
-      <c r="Y16" s="55"/>
-      <c r="Z16" s="53"/>
-      <c r="AA16" s="56"/>
+      <c r="X16" s="55">
+        <v>110.36666119770302</v>
+      </c>
+      <c r="Y16" s="55">
+        <v>77.71024646458726</v>
+      </c>
+      <c r="Z16" s="53">
+        <v>0.263</v>
+      </c>
+      <c r="AA16" s="56">
+        <v>0.2139</v>
+      </c>
       <c r="AB16" s="57"/>
       <c r="AD16" s="35"/>
       <c r="AE16" s="35"/>
@@ -11408,30 +11496,74 @@
       <c r="C23" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D23" s="52"/>
-      <c r="E23" s="52"/>
-      <c r="F23" s="52"/>
-      <c r="G23" s="53"/>
-      <c r="H23" s="52"/>
-      <c r="I23" s="52"/>
-      <c r="J23" s="52"/>
-      <c r="K23" s="52"/>
-      <c r="L23" s="52"/>
-      <c r="M23" s="53"/>
+      <c r="D23" s="52">
+        <v>27500.3157</v>
+      </c>
+      <c r="E23" s="52">
+        <v>11999.08</v>
+      </c>
+      <c r="F23" s="52">
+        <v>15501.2357</v>
+      </c>
+      <c r="G23" s="53">
+        <v>0.563674827194802</v>
+      </c>
+      <c r="H23" s="52">
+        <v>19565.829</v>
+      </c>
+      <c r="I23" s="52">
+        <v>8083.92</v>
+      </c>
+      <c r="J23" s="52">
+        <v>13767.337200000002</v>
+      </c>
+      <c r="K23" s="52">
+        <v>6373.24</v>
+      </c>
+      <c r="L23" s="52">
+        <v>7394.097200000002</v>
+      </c>
+      <c r="M23" s="53">
+        <v>0.5370753321855152</v>
+      </c>
       <c r="N23" s="53"/>
-      <c r="O23" s="52"/>
-      <c r="P23" s="52"/>
-      <c r="Q23" s="52"/>
-      <c r="R23" s="53"/>
-      <c r="S23" s="54"/>
-      <c r="T23" s="54"/>
-      <c r="U23" s="54"/>
-      <c r="V23" s="53"/>
+      <c r="O23" s="52">
+        <v>5798.4918</v>
+      </c>
+      <c r="P23" s="52">
+        <v>1710.68</v>
+      </c>
+      <c r="Q23" s="52">
+        <v>4087.8117999999995</v>
+      </c>
+      <c r="R23" s="53">
+        <v>0.7049784566393626</v>
+      </c>
+      <c r="S23" s="54">
+        <v>125.39</v>
+      </c>
+      <c r="T23" s="54">
+        <v>34.75</v>
+      </c>
+      <c r="U23" s="54">
+        <v>90.64</v>
+      </c>
+      <c r="V23" s="53">
+        <v>0.7228646622537682</v>
+      </c>
       <c r="W23" s="53"/>
-      <c r="X23" s="55"/>
-      <c r="Y23" s="55"/>
-      <c r="Z23" s="53"/>
-      <c r="AA23" s="56"/>
+      <c r="X23" s="55">
+        <v>112.66647482014388</v>
+      </c>
+      <c r="Y23" s="55">
+        <v>63.27846478985563</v>
+      </c>
+      <c r="Z23" s="53">
+        <v>0.32630000000000003</v>
+      </c>
+      <c r="AA23" s="56">
+        <v>0.2885</v>
+      </c>
       <c r="AB23" s="57"/>
       <c r="AD23" s="35"/>
       <c r="AE23" s="35"/>
@@ -12312,30 +12444,74 @@
       <c r="C37" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D37" s="52"/>
-      <c r="E37" s="52"/>
-      <c r="F37" s="52"/>
-      <c r="G37" s="53"/>
-      <c r="H37" s="52"/>
-      <c r="I37" s="52"/>
-      <c r="J37" s="52"/>
-      <c r="K37" s="52"/>
-      <c r="L37" s="52"/>
-      <c r="M37" s="53"/>
+      <c r="D37" s="52">
+        <v>397238.61073204</v>
+      </c>
+      <c r="E37" s="52">
+        <v>352623.79</v>
+      </c>
+      <c r="F37" s="52">
+        <v>44614.82073204004</v>
+      </c>
+      <c r="G37" s="53">
+        <v>0.112312397452561</v>
+      </c>
+      <c r="H37" s="52">
+        <v>328046.93216</v>
+      </c>
+      <c r="I37" s="52">
+        <v>278838.99</v>
+      </c>
+      <c r="J37" s="52">
+        <v>271925.57216000004</v>
+      </c>
+      <c r="K37" s="52">
+        <v>243603.25999999998</v>
+      </c>
+      <c r="L37" s="52">
+        <v>28322.31216000006</v>
+      </c>
+      <c r="M37" s="53">
+        <v>0.1041546476671025</v>
+      </c>
       <c r="N37" s="53"/>
-      <c r="O37" s="52"/>
-      <c r="P37" s="52"/>
-      <c r="Q37" s="52"/>
-      <c r="R37" s="53"/>
-      <c r="S37" s="54"/>
-      <c r="T37" s="54"/>
-      <c r="U37" s="54"/>
-      <c r="V37" s="53"/>
+      <c r="O37" s="52">
+        <v>56121.36</v>
+      </c>
+      <c r="P37" s="52">
+        <v>35235.73</v>
+      </c>
+      <c r="Q37" s="52">
+        <v>20885.629999999997</v>
+      </c>
+      <c r="R37" s="53">
+        <v>0.37215117381332163</v>
+      </c>
+      <c r="S37" s="54">
+        <v>1124.47</v>
+      </c>
+      <c r="T37" s="54">
+        <v>813.5</v>
+      </c>
+      <c r="U37" s="54">
+        <v>310.97</v>
+      </c>
+      <c r="V37" s="53">
+        <v>0.2765480626428451</v>
+      </c>
       <c r="W37" s="53"/>
-      <c r="X37" s="55"/>
-      <c r="Y37" s="55"/>
-      <c r="Z37" s="53"/>
-      <c r="AA37" s="56"/>
+      <c r="X37" s="55">
+        <v>90.70043023970499</v>
+      </c>
+      <c r="Y37" s="55">
+        <v>61.532703026350184</v>
+      </c>
+      <c r="Z37" s="53">
+        <v>0.20920000000000002</v>
+      </c>
+      <c r="AA37" s="56">
+        <v>0.1742</v>
+      </c>
       <c r="AB37" s="57"/>
       <c r="AD37" s="35"/>
       <c r="AE37" s="35"/>
@@ -12807,30 +12983,74 @@
       <c r="C44" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D44" s="52"/>
-      <c r="E44" s="52"/>
-      <c r="F44" s="52"/>
-      <c r="G44" s="53"/>
-      <c r="H44" s="52"/>
-      <c r="I44" s="52"/>
-      <c r="J44" s="52"/>
-      <c r="K44" s="52"/>
-      <c r="L44" s="52"/>
-      <c r="M44" s="53"/>
+      <c r="D44" s="52">
+        <v>128258.49930985</v>
+      </c>
+      <c r="E44" s="52">
+        <v>115314.55</v>
+      </c>
+      <c r="F44" s="52">
+        <v>12943.949309849995</v>
+      </c>
+      <c r="G44" s="53">
+        <v>0.10092079183446305</v>
+      </c>
+      <c r="H44" s="52">
+        <v>94098.31685</v>
+      </c>
+      <c r="I44" s="52">
+        <v>57104.57</v>
+      </c>
+      <c r="J44" s="52">
+        <v>69042.08885</v>
+      </c>
+      <c r="K44" s="52">
+        <v>40878.83</v>
+      </c>
+      <c r="L44" s="52">
+        <v>28163.25885</v>
+      </c>
+      <c r="M44" s="53">
+        <v>0.40791435078372484</v>
+      </c>
       <c r="N44" s="53"/>
-      <c r="O44" s="52"/>
-      <c r="P44" s="52"/>
-      <c r="Q44" s="52"/>
-      <c r="R44" s="53"/>
-      <c r="S44" s="54"/>
-      <c r="T44" s="54"/>
-      <c r="U44" s="54"/>
-      <c r="V44" s="53"/>
+      <c r="O44" s="52">
+        <v>25056.228</v>
+      </c>
+      <c r="P44" s="52">
+        <v>16225.74</v>
+      </c>
+      <c r="Q44" s="52">
+        <v>8830.488</v>
+      </c>
+      <c r="R44" s="53">
+        <v>0.3524268696788678</v>
+      </c>
+      <c r="S44" s="54">
+        <v>501.83</v>
+      </c>
+      <c r="T44" s="54">
+        <v>366.25</v>
+      </c>
+      <c r="U44" s="54">
+        <v>135.57999999999998</v>
+      </c>
+      <c r="V44" s="53">
+        <v>0.2701711735049718</v>
+      </c>
       <c r="W44" s="53"/>
-      <c r="X44" s="55"/>
-      <c r="Y44" s="55"/>
-      <c r="Z44" s="53"/>
-      <c r="AA44" s="56"/>
+      <c r="X44" s="55">
+        <v>158.93509897610923</v>
+      </c>
+      <c r="Y44" s="55">
+        <v>68.07122423898531</v>
+      </c>
+      <c r="Z44" s="53">
+        <v>0.5047999999999999</v>
+      </c>
+      <c r="AA44" s="56">
+        <v>0.2663</v>
+      </c>
       <c r="AB44" s="57"/>
       <c r="AD44" s="35"/>
       <c r="AE44" s="35"/>
@@ -13304,30 +13524,74 @@
       <c r="C51" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D51" s="52"/>
-      <c r="E51" s="52"/>
-      <c r="F51" s="52"/>
-      <c r="G51" s="53"/>
-      <c r="H51" s="52"/>
-      <c r="I51" s="52"/>
-      <c r="J51" s="52"/>
-      <c r="K51" s="52"/>
-      <c r="L51" s="52"/>
-      <c r="M51" s="53"/>
+      <c r="D51" s="52">
+        <v>65693.35850319</v>
+      </c>
+      <c r="E51" s="52">
+        <v>61277.97</v>
+      </c>
+      <c r="F51" s="52">
+        <v>4415.388503189999</v>
+      </c>
+      <c r="G51" s="53">
+        <v>0.06721209881476212</v>
+      </c>
+      <c r="H51" s="52">
+        <v>50582.36785</v>
+      </c>
+      <c r="I51" s="52">
+        <v>29601.04</v>
+      </c>
+      <c r="J51" s="52">
+        <v>39438.99025</v>
+      </c>
+      <c r="K51" s="52">
+        <v>20244.31</v>
+      </c>
+      <c r="L51" s="52">
+        <v>19194.68025</v>
+      </c>
+      <c r="M51" s="53">
+        <v>0.4866929941240065</v>
+      </c>
       <c r="N51" s="53"/>
-      <c r="O51" s="52"/>
-      <c r="P51" s="52"/>
-      <c r="Q51" s="52"/>
-      <c r="R51" s="53"/>
-      <c r="S51" s="54"/>
-      <c r="T51" s="54"/>
-      <c r="U51" s="54"/>
-      <c r="V51" s="53"/>
+      <c r="O51" s="52">
+        <v>11143.3776</v>
+      </c>
+      <c r="P51" s="52">
+        <v>9356.73</v>
+      </c>
+      <c r="Q51" s="52">
+        <v>1786.6476000000002</v>
+      </c>
+      <c r="R51" s="53">
+        <v>0.1603326804612634</v>
+      </c>
+      <c r="S51" s="54">
+        <v>223.22</v>
+      </c>
+      <c r="T51" s="54">
+        <v>216.5</v>
+      </c>
+      <c r="U51" s="54">
+        <v>6.719999999999999</v>
+      </c>
+      <c r="V51" s="53">
+        <v>0.030104829316369496</v>
+      </c>
       <c r="W51" s="53"/>
-      <c r="X51" s="55"/>
-      <c r="Y51" s="55"/>
-      <c r="Z51" s="53"/>
-      <c r="AA51" s="56"/>
+      <c r="X51" s="55">
+        <v>146.31376443418014</v>
+      </c>
+      <c r="Y51" s="55">
+        <v>67.69550512136009</v>
+      </c>
+      <c r="Z51" s="53">
+        <v>0.5169</v>
+      </c>
+      <c r="AA51" s="56">
+        <v>0.23</v>
+      </c>
       <c r="AB51" s="57"/>
       <c r="AD51" s="35"/>
       <c r="AE51" s="35"/>
@@ -13799,30 +14063,74 @@
       <c r="C58" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D58" s="52"/>
-      <c r="E58" s="52"/>
-      <c r="F58" s="52"/>
-      <c r="G58" s="53"/>
-      <c r="H58" s="52"/>
-      <c r="I58" s="52"/>
-      <c r="J58" s="52"/>
-      <c r="K58" s="52"/>
-      <c r="L58" s="52"/>
-      <c r="M58" s="53"/>
+      <c r="D58" s="52">
+        <v>155296.79012754</v>
+      </c>
+      <c r="E58" s="52">
+        <v>155296.8</v>
+      </c>
+      <c r="F58" s="52">
+        <v>-0.009872459981124848</v>
+      </c>
+      <c r="G58" s="53">
+        <v>-6.357156495647419e-8</v>
+      </c>
+      <c r="H58" s="52">
+        <v>109364.9721</v>
+      </c>
+      <c r="I58" s="52">
+        <v>113859.52</v>
+      </c>
+      <c r="J58" s="52">
+        <v>75135.0159</v>
+      </c>
+      <c r="K58" s="52">
+        <v>80491.32</v>
+      </c>
+      <c r="L58" s="52">
+        <v>-5356.3041000000085</v>
+      </c>
+      <c r="M58" s="53">
+        <v>-0.07128905259205527</v>
+      </c>
       <c r="N58" s="53"/>
-      <c r="O58" s="52"/>
-      <c r="P58" s="52"/>
-      <c r="Q58" s="52"/>
-      <c r="R58" s="53"/>
-      <c r="S58" s="54"/>
-      <c r="T58" s="54"/>
-      <c r="U58" s="54"/>
-      <c r="V58" s="53"/>
+      <c r="O58" s="52">
+        <v>34229.9562</v>
+      </c>
+      <c r="P58" s="52">
+        <v>33368.2</v>
+      </c>
+      <c r="Q58" s="52">
+        <v>861.7562000000034</v>
+      </c>
+      <c r="R58" s="53">
+        <v>0.025175498179574166</v>
+      </c>
+      <c r="S58" s="54">
+        <v>685.48</v>
+      </c>
+      <c r="T58" s="54">
+        <v>699.75</v>
+      </c>
+      <c r="U58" s="54">
+        <v>-14.269999999999982</v>
+      </c>
+      <c r="V58" s="53">
+        <v>-0.0208175293225185</v>
+      </c>
       <c r="W58" s="53"/>
-      <c r="X58" s="55"/>
-      <c r="Y58" s="55"/>
-      <c r="Z58" s="53"/>
-      <c r="AA58" s="56"/>
+      <c r="X58" s="55">
+        <v>59.2172633083244</v>
+      </c>
+      <c r="Y58" s="55">
+        <v>67.00679527854935</v>
+      </c>
+      <c r="Z58" s="53">
+        <v>0.2668</v>
+      </c>
+      <c r="AA58" s="56">
+        <v>0.2958</v>
+      </c>
       <c r="AB58" s="57"/>
       <c r="AD58" s="35"/>
       <c r="AE58" s="35"/>
@@ -14695,30 +15003,74 @@
       <c r="C72" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D72" s="52"/>
-      <c r="E72" s="52"/>
-      <c r="F72" s="52"/>
-      <c r="G72" s="53"/>
-      <c r="H72" s="52"/>
-      <c r="I72" s="52"/>
-      <c r="J72" s="52"/>
-      <c r="K72" s="52"/>
-      <c r="L72" s="52"/>
-      <c r="M72" s="53"/>
+      <c r="D72" s="52">
+        <v>53029.71458947</v>
+      </c>
+      <c r="E72" s="52">
+        <v>29715.67</v>
+      </c>
+      <c r="F72" s="52">
+        <v>23314.044589470002</v>
+      </c>
+      <c r="G72" s="53">
+        <v>0.43964114779715263</v>
+      </c>
+      <c r="H72" s="52">
+        <v>39055.77825</v>
+      </c>
+      <c r="I72" s="52">
+        <v>24880.27</v>
+      </c>
+      <c r="J72" s="52">
+        <v>29537.289750000004</v>
+      </c>
+      <c r="K72" s="52">
+        <v>20998.84</v>
+      </c>
+      <c r="L72" s="52">
+        <v>8538.449750000003</v>
+      </c>
+      <c r="M72" s="53">
+        <v>0.28907356843733445</v>
+      </c>
       <c r="N72" s="53"/>
-      <c r="O72" s="52"/>
-      <c r="P72" s="52"/>
-      <c r="Q72" s="52"/>
-      <c r="R72" s="53"/>
-      <c r="S72" s="54"/>
-      <c r="T72" s="54"/>
-      <c r="U72" s="54"/>
-      <c r="V72" s="53"/>
+      <c r="O72" s="52">
+        <v>9518.4885</v>
+      </c>
+      <c r="P72" s="52">
+        <v>3881.43</v>
+      </c>
+      <c r="Q72" s="52">
+        <v>5637.058499999999</v>
+      </c>
+      <c r="R72" s="53">
+        <v>0.5922220213850129</v>
+      </c>
+      <c r="S72" s="54">
+        <v>193.32</v>
+      </c>
+      <c r="T72" s="54">
+        <v>83.5</v>
+      </c>
+      <c r="U72" s="54">
+        <v>109.82</v>
+      </c>
+      <c r="V72" s="53">
+        <v>0.5680736602524312</v>
+      </c>
       <c r="W72" s="53"/>
-      <c r="X72" s="55"/>
-      <c r="Y72" s="55"/>
-      <c r="Z72" s="53"/>
-      <c r="AA72" s="56"/>
+      <c r="X72" s="55">
+        <v>57.90898203592814</v>
+      </c>
+      <c r="Y72" s="55">
+        <v>72.28396616733912</v>
+      </c>
+      <c r="Z72" s="53">
+        <v>0.16269999999999998</v>
+      </c>
+      <c r="AA72" s="56">
+        <v>0.2635</v>
+      </c>
       <c r="AB72" s="57"/>
       <c r="AD72" s="35"/>
       <c r="AE72" s="35"/>
@@ -15180,30 +15532,74 @@
       <c r="C79" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D79" s="52"/>
-      <c r="E79" s="52"/>
-      <c r="F79" s="52"/>
-      <c r="G79" s="53"/>
-      <c r="H79" s="52"/>
-      <c r="I79" s="52"/>
-      <c r="J79" s="52"/>
-      <c r="K79" s="52"/>
-      <c r="L79" s="52"/>
-      <c r="M79" s="53"/>
+      <c r="D79" s="52">
+        <v>78753.06644148</v>
+      </c>
+      <c r="E79" s="52">
+        <v>61764.82</v>
+      </c>
+      <c r="F79" s="52">
+        <v>16988.246441479998</v>
+      </c>
+      <c r="G79" s="53">
+        <v>0.21571536460873764</v>
+      </c>
+      <c r="H79" s="52">
+        <v>55589.7822</v>
+      </c>
+      <c r="I79" s="52">
+        <v>44814.24</v>
+      </c>
+      <c r="J79" s="52">
+        <v>32594.7534</v>
+      </c>
+      <c r="K79" s="52">
+        <v>34770.899999999994</v>
+      </c>
+      <c r="L79" s="52">
+        <v>-2176.1465999999928</v>
+      </c>
+      <c r="M79" s="53">
+        <v>-0.06676370805124707</v>
+      </c>
       <c r="N79" s="53"/>
-      <c r="O79" s="52"/>
-      <c r="P79" s="52"/>
-      <c r="Q79" s="52"/>
-      <c r="R79" s="53"/>
-      <c r="S79" s="54"/>
-      <c r="T79" s="54"/>
-      <c r="U79" s="54"/>
-      <c r="V79" s="53"/>
+      <c r="O79" s="52">
+        <v>22995.0288</v>
+      </c>
+      <c r="P79" s="52">
+        <v>10043.34</v>
+      </c>
+      <c r="Q79" s="52">
+        <v>12951.6888</v>
+      </c>
+      <c r="R79" s="53">
+        <v>0.563238642258191</v>
+      </c>
+      <c r="S79" s="54">
+        <v>472.14</v>
+      </c>
+      <c r="T79" s="54">
+        <v>202</v>
+      </c>
+      <c r="U79" s="54">
+        <v>270.14</v>
+      </c>
+      <c r="V79" s="53">
+        <v>0.5721607997627822</v>
+      </c>
       <c r="W79" s="53"/>
-      <c r="X79" s="55"/>
-      <c r="Y79" s="55"/>
-      <c r="Z79" s="53"/>
-      <c r="AA79" s="56"/>
+      <c r="X79" s="55">
+        <v>83.91376237623763</v>
+      </c>
+      <c r="Y79" s="55">
+        <v>49.060202993773025</v>
+      </c>
+      <c r="Z79" s="53">
+        <v>0.27440000000000003</v>
+      </c>
+      <c r="AA79" s="56">
+        <v>0.2941</v>
+      </c>
       <c r="AB79" s="57"/>
       <c r="AD79" s="35"/>
       <c r="AE79" s="35"/>
@@ -15671,30 +16067,74 @@
       <c r="C86" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D86" s="52"/>
-      <c r="E86" s="52"/>
-      <c r="F86" s="52"/>
-      <c r="G86" s="53"/>
-      <c r="H86" s="52"/>
-      <c r="I86" s="52"/>
-      <c r="J86" s="52"/>
-      <c r="K86" s="52"/>
-      <c r="L86" s="52"/>
-      <c r="M86" s="53"/>
+      <c r="D86" s="52">
+        <v>25467.8441072</v>
+      </c>
+      <c r="E86" s="52">
+        <v>19598.41</v>
+      </c>
+      <c r="F86" s="52">
+        <v>5869.434107199999</v>
+      </c>
+      <c r="G86" s="53">
+        <v>0.23046450584879521</v>
+      </c>
+      <c r="H86" s="52">
+        <v>16606.829916</v>
+      </c>
+      <c r="I86" s="52">
+        <v>14118.07</v>
+      </c>
+      <c r="J86" s="52">
+        <v>9659.986716</v>
+      </c>
+      <c r="K86" s="52">
+        <v>5298.48</v>
+      </c>
+      <c r="L86" s="52">
+        <v>4361.506716</v>
+      </c>
+      <c r="M86" s="53">
+        <v>0.4515023513206248</v>
+      </c>
       <c r="N86" s="53"/>
-      <c r="O86" s="52"/>
-      <c r="P86" s="52"/>
-      <c r="Q86" s="52"/>
-      <c r="R86" s="53"/>
-      <c r="S86" s="54"/>
-      <c r="T86" s="54"/>
-      <c r="U86" s="54"/>
-      <c r="V86" s="53"/>
+      <c r="O86" s="52">
+        <v>6946.8432</v>
+      </c>
+      <c r="P86" s="52">
+        <v>8819.59</v>
+      </c>
+      <c r="Q86" s="52">
+        <v>-1872.7468</v>
+      </c>
+      <c r="R86" s="53">
+        <v>-0.26958241982487813</v>
+      </c>
+      <c r="S86" s="54">
+        <v>139.07</v>
+      </c>
+      <c r="T86" s="54">
+        <v>167.75</v>
+      </c>
+      <c r="U86" s="54">
+        <v>-28.680000000000007</v>
+      </c>
+      <c r="V86" s="53">
+        <v>-0.20622707988782632</v>
+      </c>
       <c r="W86" s="53"/>
-      <c r="X86" s="55"/>
-      <c r="Y86" s="55"/>
-      <c r="Z86" s="53"/>
-      <c r="AA86" s="56"/>
+      <c r="X86" s="55">
+        <v>32.669687034277196</v>
+      </c>
+      <c r="Y86" s="55">
+        <v>63.7162162306752</v>
+      </c>
+      <c r="Z86" s="53">
+        <v>0.2796</v>
+      </c>
+      <c r="AA86" s="56">
+        <v>0.3479</v>
+      </c>
       <c r="AB86" s="57"/>
       <c r="AD86" s="35"/>
       <c r="AE86" s="35"/>
@@ -16166,30 +16606,74 @@
       <c r="C93" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D93" s="67"/>
-      <c r="E93" s="67"/>
-      <c r="F93" s="52"/>
-      <c r="G93" s="53"/>
-      <c r="H93" s="52"/>
-      <c r="I93" s="52"/>
-      <c r="J93" s="52"/>
-      <c r="K93" s="52"/>
-      <c r="L93" s="52"/>
-      <c r="M93" s="53"/>
+      <c r="D93" s="67">
+        <v>37083.0313712</v>
+      </c>
+      <c r="E93" s="67">
+        <v>36381.33</v>
+      </c>
+      <c r="F93" s="52">
+        <v>701.7013711999971</v>
+      </c>
+      <c r="G93" s="53">
+        <v>0.018922438248804095</v>
+      </c>
+      <c r="H93" s="52">
+        <v>27002.93286</v>
+      </c>
+      <c r="I93" s="52">
+        <v>25103.82</v>
+      </c>
+      <c r="J93" s="52">
+        <v>15440.324460000002</v>
+      </c>
+      <c r="K93" s="52">
+        <v>13974.73</v>
+      </c>
+      <c r="L93" s="52">
+        <v>1465.594460000002</v>
+      </c>
+      <c r="M93" s="53">
+        <v>0.0949199263135175</v>
+      </c>
       <c r="N93" s="53"/>
-      <c r="O93" s="52"/>
-      <c r="P93" s="52"/>
-      <c r="Q93" s="52"/>
-      <c r="R93" s="53"/>
-      <c r="S93" s="68"/>
-      <c r="T93" s="68"/>
-      <c r="U93" s="54"/>
-      <c r="V93" s="53"/>
+      <c r="O93" s="52">
+        <v>11562.6084</v>
+      </c>
+      <c r="P93" s="52">
+        <v>11129.09</v>
+      </c>
+      <c r="Q93" s="52">
+        <v>433.518399999999</v>
+      </c>
+      <c r="R93" s="53">
+        <v>0.03749313174006646</v>
+      </c>
+      <c r="S93" s="68">
+        <v>231.75</v>
+      </c>
+      <c r="T93" s="68">
+        <v>225.5</v>
+      </c>
+      <c r="U93" s="54">
+        <v>6.25</v>
+      </c>
+      <c r="V93" s="53">
+        <v>0.02696871628910464</v>
+      </c>
       <c r="W93" s="53"/>
-      <c r="X93" s="55"/>
-      <c r="Y93" s="55"/>
-      <c r="Z93" s="53"/>
-      <c r="AA93" s="56"/>
+      <c r="X93" s="55">
+        <v>50.01113082039912</v>
+      </c>
+      <c r="Y93" s="55">
+        <v>43.49557070636461</v>
+      </c>
+      <c r="Z93" s="53">
+        <v>0.31</v>
+      </c>
+      <c r="AA93" s="56">
+        <v>0.2718</v>
+      </c>
       <c r="AB93" s="57"/>
       <c r="AD93" s="35"/>
       <c r="AE93" s="35"/>
@@ -16661,30 +17145,74 @@
       <c r="C100" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D100" s="52"/>
-      <c r="E100" s="52"/>
-      <c r="F100" s="52"/>
-      <c r="G100" s="53"/>
-      <c r="H100" s="52"/>
-      <c r="I100" s="52"/>
-      <c r="J100" s="52"/>
-      <c r="K100" s="52"/>
-      <c r="L100" s="52"/>
-      <c r="M100" s="53"/>
+      <c r="D100" s="52">
+        <v>26186.1354</v>
+      </c>
+      <c r="E100" s="52">
+        <v>5762.27</v>
+      </c>
+      <c r="F100" s="52">
+        <v>20423.8654</v>
+      </c>
+      <c r="G100" s="53">
+        <v>0.7799495835494686</v>
+      </c>
+      <c r="H100" s="52">
+        <v>19428.9760178</v>
+      </c>
+      <c r="I100" s="52">
+        <v>8019.36</v>
+      </c>
+      <c r="J100" s="52">
+        <v>12051.3142178</v>
+      </c>
+      <c r="K100" s="52">
+        <v>7687.129999999999</v>
+      </c>
+      <c r="L100" s="52">
+        <v>4364.184217800001</v>
+      </c>
+      <c r="M100" s="53">
+        <v>0.3621334685103493</v>
+      </c>
       <c r="N100" s="53"/>
-      <c r="O100" s="52"/>
-      <c r="P100" s="52"/>
-      <c r="Q100" s="52"/>
-      <c r="R100" s="53"/>
-      <c r="S100" s="54"/>
-      <c r="T100" s="54"/>
-      <c r="U100" s="54"/>
-      <c r="V100" s="53"/>
+      <c r="O100" s="52">
+        <v>7377.6618</v>
+      </c>
+      <c r="P100" s="52">
+        <v>332.23</v>
+      </c>
+      <c r="Q100" s="52">
+        <v>7045.4318</v>
+      </c>
+      <c r="R100" s="53">
+        <v>0.954968117405436</v>
+      </c>
+      <c r="S100" s="54">
+        <v>147.9</v>
+      </c>
+      <c r="T100" s="54">
+        <v>6.5</v>
+      </c>
+      <c r="U100" s="54">
+        <v>141.4</v>
+      </c>
+      <c r="V100" s="53">
+        <v>0.9560513860716701</v>
+      </c>
       <c r="W100" s="53"/>
-      <c r="X100" s="55"/>
-      <c r="Y100" s="55"/>
-      <c r="Z100" s="53"/>
-      <c r="AA100" s="56"/>
+      <c r="X100" s="55">
+        <v>-347.24461538461543</v>
+      </c>
+      <c r="Y100" s="55">
+        <v>45.687352144692355</v>
+      </c>
+      <c r="Z100" s="53">
+        <v>-0.3917</v>
+      </c>
+      <c r="AA100" s="56">
+        <v>0.258</v>
+      </c>
       <c r="AB100" s="57"/>
       <c r="AD100" s="35"/>
       <c r="AE100" s="35"/>
@@ -17966,30 +18494,74 @@
       <c r="C121" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D121" s="52"/>
-      <c r="E121" s="52"/>
-      <c r="F121" s="52"/>
-      <c r="G121" s="53"/>
-      <c r="H121" s="52"/>
-      <c r="I121" s="52"/>
-      <c r="J121" s="52"/>
-      <c r="K121" s="52"/>
-      <c r="L121" s="52"/>
-      <c r="M121" s="53"/>
+      <c r="D121" s="52">
+        <v>20278.45679756</v>
+      </c>
+      <c r="E121" s="52">
+        <v>0</v>
+      </c>
+      <c r="F121" s="52">
+        <v>20278.45679756</v>
+      </c>
+      <c r="G121" s="53">
+        <v>1</v>
+      </c>
+      <c r="H121" s="52">
+        <v>16648.056795</v>
+      </c>
+      <c r="I121" s="52">
+        <v>58.32</v>
+      </c>
+      <c r="J121" s="52">
+        <v>12536.982795</v>
+      </c>
+      <c r="K121" s="52">
+        <v>58.32</v>
+      </c>
+      <c r="L121" s="52">
+        <v>12478.662795</v>
+      </c>
+      <c r="M121" s="53">
+        <v>0.9953481630346291</v>
+      </c>
       <c r="N121" s="53"/>
-      <c r="O121" s="52"/>
-      <c r="P121" s="52"/>
-      <c r="Q121" s="52"/>
-      <c r="R121" s="53"/>
-      <c r="S121" s="54"/>
-      <c r="T121" s="54"/>
-      <c r="U121" s="54"/>
-      <c r="V121" s="53"/>
+      <c r="O121" s="52">
+        <v>4111.074</v>
+      </c>
+      <c r="P121" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q121" s="52">
+        <v>4111.074</v>
+      </c>
+      <c r="R121" s="53">
+        <v>1</v>
+      </c>
+      <c r="S121" s="54">
+        <v>82.37</v>
+      </c>
+      <c r="T121" s="54">
+        <v>0</v>
+      </c>
+      <c r="U121" s="54">
+        <v>82.37</v>
+      </c>
+      <c r="V121" s="53">
+        <v>1</v>
+      </c>
       <c r="W121" s="53"/>
-      <c r="X121" s="55"/>
-      <c r="Y121" s="55"/>
-      <c r="Z121" s="53"/>
-      <c r="AA121" s="56"/>
+      <c r="X121" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y121" s="55">
+        <v>44.07429892630812</v>
+      </c>
+      <c r="Z121" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA121" s="56">
+        <v>0.179</v>
+      </c>
       <c r="AB121" s="57"/>
       <c r="AD121" s="35"/>
       <c r="AE121" s="35"/>
@@ -18451,30 +19023,74 @@
       <c r="C128" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D128" s="52"/>
-      <c r="E128" s="52"/>
-      <c r="F128" s="52"/>
-      <c r="G128" s="53"/>
-      <c r="H128" s="52"/>
-      <c r="I128" s="52"/>
-      <c r="J128" s="52"/>
-      <c r="K128" s="52"/>
-      <c r="L128" s="52"/>
-      <c r="M128" s="53"/>
+      <c r="D128" s="52">
+        <v>105896.9567712</v>
+      </c>
+      <c r="E128" s="52">
+        <v>79457.73</v>
+      </c>
+      <c r="F128" s="52">
+        <v>26439.226771200003</v>
+      </c>
+      <c r="G128" s="53">
+        <v>0.2496693727311197</v>
+      </c>
+      <c r="H128" s="52">
+        <v>85934.2000148</v>
+      </c>
+      <c r="I128" s="52">
+        <v>66541.03</v>
+      </c>
+      <c r="J128" s="52">
+        <v>70065.71561479999</v>
+      </c>
+      <c r="K128" s="52">
+        <v>61659.44</v>
+      </c>
+      <c r="L128" s="52">
+        <v>8406.27561479999</v>
+      </c>
+      <c r="M128" s="53">
+        <v>0.11997701787583442</v>
+      </c>
       <c r="N128" s="53"/>
-      <c r="O128" s="52"/>
-      <c r="P128" s="52"/>
-      <c r="Q128" s="52"/>
-      <c r="R128" s="53"/>
-      <c r="S128" s="54"/>
-      <c r="T128" s="54"/>
-      <c r="U128" s="54"/>
-      <c r="V128" s="53"/>
+      <c r="O128" s="52">
+        <v>15868.4844</v>
+      </c>
+      <c r="P128" s="52">
+        <v>4881.59</v>
+      </c>
+      <c r="Q128" s="52">
+        <v>10986.8944</v>
+      </c>
+      <c r="R128" s="53">
+        <v>0.6923720074993425</v>
+      </c>
+      <c r="S128" s="54">
+        <v>317.92</v>
+      </c>
+      <c r="T128" s="54">
+        <v>106</v>
+      </c>
+      <c r="U128" s="54">
+        <v>211.92000000000002</v>
+      </c>
+      <c r="V128" s="53">
+        <v>0.6665827881227983</v>
+      </c>
       <c r="W128" s="53"/>
-      <c r="X128" s="55"/>
-      <c r="Y128" s="55"/>
-      <c r="Z128" s="53"/>
-      <c r="AA128" s="56"/>
+      <c r="X128" s="55">
+        <v>121.8556603773585</v>
+      </c>
+      <c r="Y128" s="55">
+        <v>62.79176131227983</v>
+      </c>
+      <c r="Z128" s="53">
+        <v>0.16260000000000002</v>
+      </c>
+      <c r="AA128" s="56">
+        <v>0.1885</v>
+      </c>
       <c r="AB128" s="57"/>
       <c r="AD128" s="35"/>
       <c r="AE128" s="35"/>
@@ -18943,30 +19559,74 @@
       <c r="C135" s="51" t="s">
         <v>104</v>
       </c>
-      <c r="D135" s="52"/>
-      <c r="E135" s="52"/>
-      <c r="F135" s="52"/>
-      <c r="G135" s="53"/>
-      <c r="H135" s="52"/>
-      <c r="I135" s="52"/>
-      <c r="J135" s="52"/>
-      <c r="K135" s="52"/>
-      <c r="L135" s="52"/>
-      <c r="M135" s="53"/>
+      <c r="D135" s="52">
+        <v>31802.4136956</v>
+      </c>
+      <c r="E135" s="52">
+        <v>16498.64</v>
+      </c>
+      <c r="F135" s="52">
+        <v>15303.7736956</v>
+      </c>
+      <c r="G135" s="53">
+        <v>0.48121421984134943</v>
+      </c>
+      <c r="H135" s="52">
+        <v>23448.14263</v>
+      </c>
+      <c r="I135" s="52">
+        <v>12360.83</v>
+      </c>
+      <c r="J135" s="52">
+        <v>15632.028429999998</v>
+      </c>
+      <c r="K135" s="52">
+        <v>11772.08</v>
+      </c>
+      <c r="L135" s="52">
+        <v>3859.9484299999986</v>
+      </c>
+      <c r="M135" s="53">
+        <v>0.24692562755273845</v>
+      </c>
       <c r="N135" s="53"/>
-      <c r="O135" s="52"/>
-      <c r="P135" s="52"/>
-      <c r="Q135" s="52"/>
-      <c r="R135" s="53"/>
-      <c r="S135" s="54"/>
-      <c r="T135" s="54"/>
-      <c r="U135" s="54"/>
-      <c r="V135" s="53"/>
+      <c r="O135" s="52">
+        <v>7816.1142</v>
+      </c>
+      <c r="P135" s="52">
+        <v>588.75</v>
+      </c>
+      <c r="Q135" s="52">
+        <v>7227.3642</v>
+      </c>
+      <c r="R135" s="53">
+        <v>0.92467484674162</v>
+      </c>
+      <c r="S135" s="54">
+        <v>156.69</v>
+      </c>
+      <c r="T135" s="54">
+        <v>11.5</v>
+      </c>
+      <c r="U135" s="54">
+        <v>145.19</v>
+      </c>
+      <c r="V135" s="53">
+        <v>0.9266066756015061</v>
+      </c>
       <c r="W135" s="53"/>
-      <c r="X135" s="55"/>
-      <c r="Y135" s="55"/>
-      <c r="Z135" s="53"/>
-      <c r="AA135" s="56"/>
+      <c r="X135" s="55">
+        <v>359.80956521739137</v>
+      </c>
+      <c r="Y135" s="55">
+        <v>53.31719360265494</v>
+      </c>
+      <c r="Z135" s="53">
+        <v>0.25079999999999997</v>
+      </c>
+      <c r="AA135" s="56">
+        <v>0.2627</v>
+      </c>
       <c r="AB135" s="57"/>
       <c r="AD135" s="35"/>
       <c r="AE135" s="35"/>
@@ -20637,30 +21297,74 @@
       <c r="C163" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D163" s="52"/>
-      <c r="E163" s="52"/>
-      <c r="F163" s="52"/>
-      <c r="G163" s="53"/>
-      <c r="H163" s="52"/>
-      <c r="I163" s="52"/>
-      <c r="J163" s="52"/>
-      <c r="K163" s="52"/>
-      <c r="L163" s="52"/>
-      <c r="M163" s="53"/>
+      <c r="D163" s="52">
+        <v>17899.333054</v>
+      </c>
+      <c r="E163" s="52">
+        <v>13424.5</v>
+      </c>
+      <c r="F163" s="52">
+        <v>4474.833053999999</v>
+      </c>
+      <c r="G163" s="53">
+        <v>0.24999998829565323</v>
+      </c>
+      <c r="H163" s="52">
+        <v>13919.4012884</v>
+      </c>
+      <c r="I163" s="52">
+        <v>14052.73</v>
+      </c>
+      <c r="J163" s="52">
+        <v>8410.9272884</v>
+      </c>
+      <c r="K163" s="52">
+        <v>8190.78</v>
+      </c>
+      <c r="L163" s="52">
+        <v>220.14728840000043</v>
+      </c>
+      <c r="M163" s="53">
+        <v>0.02617396166337312</v>
+      </c>
       <c r="N163" s="53"/>
-      <c r="O163" s="52"/>
-      <c r="P163" s="52"/>
-      <c r="Q163" s="52"/>
-      <c r="R163" s="53"/>
-      <c r="S163" s="54"/>
-      <c r="T163" s="54"/>
-      <c r="U163" s="54"/>
-      <c r="V163" s="53"/>
+      <c r="O163" s="52">
+        <v>5508.474</v>
+      </c>
+      <c r="P163" s="52">
+        <v>5861.95</v>
+      </c>
+      <c r="Q163" s="52">
+        <v>-353.47599999999966</v>
+      </c>
+      <c r="R163" s="53">
+        <v>-0.06416949594388567</v>
+      </c>
+      <c r="S163" s="54">
+        <v>110.44</v>
+      </c>
+      <c r="T163" s="54">
+        <v>116.25</v>
+      </c>
+      <c r="U163" s="54">
+        <v>-5.810000000000002</v>
+      </c>
+      <c r="V163" s="53">
+        <v>-0.05260775081492215</v>
+      </c>
       <c r="W163" s="53"/>
-      <c r="X163" s="55"/>
-      <c r="Y163" s="55"/>
-      <c r="Z163" s="53"/>
-      <c r="AA163" s="56"/>
+      <c r="X163" s="55">
+        <v>-5.404129032258065</v>
+      </c>
+      <c r="Y163" s="55">
+        <v>36.03704967040926</v>
+      </c>
+      <c r="Z163" s="53">
+        <v>-0.046799999999999994</v>
+      </c>
+      <c r="AA163" s="56">
+        <v>0.2224</v>
+      </c>
       <c r="AB163" s="57"/>
       <c r="AD163" s="35"/>
       <c r="AE163" s="35"/>
@@ -21108,30 +21812,74 @@
       <c r="C170" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D170" s="52"/>
-      <c r="E170" s="52"/>
-      <c r="F170" s="52"/>
-      <c r="G170" s="53"/>
-      <c r="H170" s="52"/>
-      <c r="I170" s="52"/>
-      <c r="J170" s="52"/>
-      <c r="K170" s="52"/>
-      <c r="L170" s="52"/>
-      <c r="M170" s="53"/>
+      <c r="D170" s="52">
+        <v>10827.20261235</v>
+      </c>
+      <c r="E170" s="52">
+        <v>0</v>
+      </c>
+      <c r="F170" s="52">
+        <v>10827.20261235</v>
+      </c>
+      <c r="G170" s="53">
+        <v>1</v>
+      </c>
+      <c r="H170" s="52">
+        <v>7687.765097</v>
+      </c>
+      <c r="I170" s="52">
+        <v>2116.21</v>
+      </c>
+      <c r="J170" s="52">
+        <v>4437.133697</v>
+      </c>
+      <c r="K170" s="52">
+        <v>1029.51</v>
+      </c>
+      <c r="L170" s="52">
+        <v>3407.623697</v>
+      </c>
+      <c r="M170" s="53">
+        <v>0.7679785937719064</v>
+      </c>
       <c r="N170" s="53"/>
-      <c r="O170" s="52"/>
-      <c r="P170" s="52"/>
-      <c r="Q170" s="52"/>
-      <c r="R170" s="53"/>
-      <c r="S170" s="54"/>
-      <c r="T170" s="54"/>
-      <c r="U170" s="54"/>
-      <c r="V170" s="53"/>
+      <c r="O170" s="52">
+        <v>3250.6314</v>
+      </c>
+      <c r="P170" s="52">
+        <v>1086.7</v>
+      </c>
+      <c r="Q170" s="52">
+        <v>2163.9314000000004</v>
+      </c>
+      <c r="R170" s="53">
+        <v>0.6656957168382734</v>
+      </c>
+      <c r="S170" s="54">
+        <v>65.13</v>
+      </c>
+      <c r="T170" s="54">
+        <v>24.33</v>
+      </c>
+      <c r="U170" s="54">
+        <v>40.8</v>
+      </c>
+      <c r="V170" s="53">
+        <v>0.6264394288346384</v>
+      </c>
       <c r="W170" s="53"/>
-      <c r="X170" s="55"/>
-      <c r="Y170" s="55"/>
-      <c r="Z170" s="53"/>
-      <c r="AA170" s="56"/>
+      <c r="X170" s="55">
+        <v>-86.97944923962187</v>
+      </c>
+      <c r="Y170" s="55">
+        <v>48.202633430830645</v>
+      </c>
+      <c r="Z170" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA170" s="56">
+        <v>0.29</v>
+      </c>
       <c r="AB170" s="57"/>
       <c r="AD170" s="35"/>
       <c r="AE170" s="35"/>
@@ -21593,30 +22341,74 @@
       <c r="C177" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D177" s="52"/>
-      <c r="E177" s="52"/>
-      <c r="F177" s="52"/>
-      <c r="G177" s="53"/>
-      <c r="H177" s="52"/>
-      <c r="I177" s="52"/>
-      <c r="J177" s="52"/>
-      <c r="K177" s="52"/>
-      <c r="L177" s="52"/>
-      <c r="M177" s="53"/>
+      <c r="D177" s="52">
+        <v>146237.1072</v>
+      </c>
+      <c r="E177" s="52">
+        <v>125386.21</v>
+      </c>
+      <c r="F177" s="52">
+        <v>20850.897199999992</v>
+      </c>
+      <c r="G177" s="53">
+        <v>0.14258280678024784</v>
+      </c>
+      <c r="H177" s="52">
+        <v>114651.8653946</v>
+      </c>
+      <c r="I177" s="52">
+        <v>105944.62</v>
+      </c>
+      <c r="J177" s="52">
+        <v>82888.0783946</v>
+      </c>
+      <c r="K177" s="52">
+        <v>78318.72</v>
+      </c>
+      <c r="L177" s="52">
+        <v>4569.3583946</v>
+      </c>
+      <c r="M177" s="53">
+        <v>0.055126846744437075</v>
+      </c>
       <c r="N177" s="53"/>
-      <c r="O177" s="52"/>
-      <c r="P177" s="52"/>
-      <c r="Q177" s="52"/>
-      <c r="R177" s="53"/>
-      <c r="S177" s="54"/>
-      <c r="T177" s="54"/>
-      <c r="U177" s="54"/>
-      <c r="V177" s="53"/>
+      <c r="O177" s="52">
+        <v>31763.787</v>
+      </c>
+      <c r="P177" s="52">
+        <v>27625.9</v>
+      </c>
+      <c r="Q177" s="52">
+        <v>4137.886999999999</v>
+      </c>
+      <c r="R177" s="53">
+        <v>0.1302705814013927</v>
+      </c>
+      <c r="S177" s="54">
+        <v>659.73</v>
+      </c>
+      <c r="T177" s="54">
+        <v>550.75</v>
+      </c>
+      <c r="U177" s="54">
+        <v>108.98000000000002</v>
+      </c>
+      <c r="V177" s="53">
+        <v>0.1651887893532203</v>
+      </c>
       <c r="W177" s="53"/>
-      <c r="X177" s="55"/>
-      <c r="Y177" s="55"/>
-      <c r="Z177" s="53"/>
-      <c r="AA177" s="56"/>
+      <c r="X177" s="55">
+        <v>35.3002088061734</v>
+      </c>
+      <c r="Y177" s="55">
+        <v>47.87601261940491</v>
+      </c>
+      <c r="Z177" s="53">
+        <v>0.1551</v>
+      </c>
+      <c r="AA177" s="56">
+        <v>0.216</v>
+      </c>
       <c r="AB177" s="57"/>
       <c r="AD177" s="35"/>
       <c r="AE177" s="35"/>
@@ -22086,30 +22878,74 @@
       <c r="C184" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D184" s="52"/>
-      <c r="E184" s="52"/>
-      <c r="F184" s="52"/>
-      <c r="G184" s="53"/>
-      <c r="H184" s="52"/>
-      <c r="I184" s="52"/>
-      <c r="J184" s="52"/>
-      <c r="K184" s="52"/>
-      <c r="L184" s="52"/>
-      <c r="M184" s="53"/>
+      <c r="D184" s="52">
+        <v>16897.52982004</v>
+      </c>
+      <c r="E184" s="52">
+        <v>5491.7</v>
+      </c>
+      <c r="F184" s="52">
+        <v>11405.829820039999</v>
+      </c>
+      <c r="G184" s="53">
+        <v>0.6749998337930436</v>
+      </c>
+      <c r="H184" s="52">
+        <v>9226.2731</v>
+      </c>
+      <c r="I184" s="52">
+        <v>5812.29</v>
+      </c>
+      <c r="J184" s="52">
+        <v>2977.1135000000004</v>
+      </c>
+      <c r="K184" s="52">
+        <v>2773.14</v>
+      </c>
+      <c r="L184" s="52">
+        <v>203.9735000000005</v>
+      </c>
+      <c r="M184" s="53">
+        <v>0.0685138473894262</v>
+      </c>
       <c r="N184" s="53"/>
-      <c r="O184" s="52"/>
-      <c r="P184" s="52"/>
-      <c r="Q184" s="52"/>
-      <c r="R184" s="53"/>
-      <c r="S184" s="54"/>
-      <c r="T184" s="54"/>
-      <c r="U184" s="54"/>
-      <c r="V184" s="53"/>
+      <c r="O184" s="52">
+        <v>6249.1596</v>
+      </c>
+      <c r="P184" s="52">
+        <v>3039.15</v>
+      </c>
+      <c r="Q184" s="52">
+        <v>3210.0096</v>
+      </c>
+      <c r="R184" s="53">
+        <v>0.5136706062043926</v>
+      </c>
+      <c r="S184" s="54">
+        <v>125.17</v>
+      </c>
+      <c r="T184" s="54">
+        <v>57.25</v>
+      </c>
+      <c r="U184" s="54">
+        <v>67.92</v>
+      </c>
+      <c r="V184" s="53">
+        <v>0.5426220340337141</v>
+      </c>
       <c r="W184" s="53"/>
-      <c r="X184" s="55"/>
-      <c r="Y184" s="55"/>
-      <c r="Z184" s="53"/>
-      <c r="AA184" s="56"/>
+      <c r="X184" s="55">
+        <v>-5.599825327510916</v>
+      </c>
+      <c r="Y184" s="55">
+        <v>61.286703843093385</v>
+      </c>
+      <c r="Z184" s="53">
+        <v>-0.0584</v>
+      </c>
+      <c r="AA184" s="56">
+        <v>0.454</v>
+      </c>
       <c r="AB184" s="57"/>
       <c r="AD184" s="35"/>
       <c r="AE184" s="35"/>
@@ -22575,30 +23411,74 @@
       <c r="C191" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D191" s="52"/>
-      <c r="E191" s="52"/>
-      <c r="F191" s="52"/>
-      <c r="G191" s="53"/>
-      <c r="H191" s="52"/>
-      <c r="I191" s="52"/>
-      <c r="J191" s="52"/>
-      <c r="K191" s="52"/>
-      <c r="L191" s="52"/>
-      <c r="M191" s="53"/>
+      <c r="D191" s="52">
+        <v>20992.11525559</v>
+      </c>
+      <c r="E191" s="52">
+        <v>14169.68</v>
+      </c>
+      <c r="F191" s="52">
+        <v>6822.43525559</v>
+      </c>
+      <c r="G191" s="53">
+        <v>0.3249998950807614</v>
+      </c>
+      <c r="H191" s="52">
+        <v>16299.085174</v>
+      </c>
+      <c r="I191" s="52">
+        <v>9699.51</v>
+      </c>
+      <c r="J191" s="52">
+        <v>9784.324774</v>
+      </c>
+      <c r="K191" s="52">
+        <v>8137.88</v>
+      </c>
+      <c r="L191" s="52">
+        <v>1646.4447740000005</v>
+      </c>
+      <c r="M191" s="53">
+        <v>0.16827372476178604</v>
+      </c>
       <c r="N191" s="53"/>
-      <c r="O191" s="52"/>
-      <c r="P191" s="52"/>
-      <c r="Q191" s="52"/>
-      <c r="R191" s="53"/>
-      <c r="S191" s="54"/>
-      <c r="T191" s="54"/>
-      <c r="U191" s="54"/>
-      <c r="V191" s="53"/>
+      <c r="O191" s="52">
+        <v>6514.7604</v>
+      </c>
+      <c r="P191" s="52">
+        <v>1561.63</v>
+      </c>
+      <c r="Q191" s="52">
+        <v>4953.1304</v>
+      </c>
+      <c r="R191" s="53">
+        <v>0.7602935635207705</v>
+      </c>
+      <c r="S191" s="54">
+        <v>130.62</v>
+      </c>
+      <c r="T191" s="54">
+        <v>34.75</v>
+      </c>
+      <c r="U191" s="54">
+        <v>95.87</v>
+      </c>
+      <c r="V191" s="53">
+        <v>0.7339611085591793</v>
+      </c>
       <c r="W191" s="53"/>
-      <c r="X191" s="55"/>
-      <c r="Y191" s="55"/>
-      <c r="Z191" s="53"/>
-      <c r="AA191" s="56"/>
+      <c r="X191" s="55">
+        <v>128.6379856115108</v>
+      </c>
+      <c r="Y191" s="55">
+        <v>35.92887828502527</v>
+      </c>
+      <c r="Z191" s="53">
+        <v>0.3155</v>
+      </c>
+      <c r="AA191" s="56">
+        <v>0.2236</v>
+      </c>
       <c r="AB191" s="57"/>
       <c r="AD191" s="35"/>
       <c r="AE191" s="35"/>
@@ -23058,30 +23938,74 @@
       <c r="C198" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D198" s="52"/>
-      <c r="E198" s="52"/>
-      <c r="F198" s="52"/>
-      <c r="G198" s="53"/>
-      <c r="H198" s="52"/>
-      <c r="I198" s="52"/>
-      <c r="J198" s="52"/>
-      <c r="K198" s="52"/>
-      <c r="L198" s="52"/>
-      <c r="M198" s="53"/>
+      <c r="D198" s="52">
+        <v>23770.94615247</v>
+      </c>
+      <c r="E198" s="52">
+        <v>10204.54</v>
+      </c>
+      <c r="F198" s="52">
+        <v>13566.406152469997</v>
+      </c>
+      <c r="G198" s="53">
+        <v>0.5707137639980029</v>
+      </c>
+      <c r="H198" s="52">
+        <v>14310.9577</v>
+      </c>
+      <c r="I198" s="52">
+        <v>7116.73</v>
+      </c>
+      <c r="J198" s="52">
+        <v>7389.335500000001</v>
+      </c>
+      <c r="K198" s="52">
+        <v>6605.049999999999</v>
+      </c>
+      <c r="L198" s="52">
+        <v>784.2855000000018</v>
+      </c>
+      <c r="M198" s="53">
+        <v>0.10613748692287713</v>
+      </c>
       <c r="N198" s="53"/>
-      <c r="O198" s="52"/>
-      <c r="P198" s="52"/>
-      <c r="Q198" s="52"/>
-      <c r="R198" s="53"/>
-      <c r="S198" s="54"/>
-      <c r="T198" s="54"/>
-      <c r="U198" s="54"/>
-      <c r="V198" s="53"/>
+      <c r="O198" s="52">
+        <v>6921.6222</v>
+      </c>
+      <c r="P198" s="52">
+        <v>511.68</v>
+      </c>
+      <c r="Q198" s="52">
+        <v>6409.9421999999995</v>
+      </c>
+      <c r="R198" s="53">
+        <v>0.9260751330807971</v>
+      </c>
+      <c r="S198" s="54">
+        <v>140.15</v>
+      </c>
+      <c r="T198" s="54">
+        <v>9.25</v>
+      </c>
+      <c r="U198" s="54">
+        <v>130.9</v>
+      </c>
+      <c r="V198" s="53">
+        <v>0.9339992864787727</v>
+      </c>
       <c r="W198" s="53"/>
-      <c r="X198" s="55"/>
-      <c r="Y198" s="55"/>
-      <c r="Z198" s="53"/>
-      <c r="AA198" s="56"/>
+      <c r="X198" s="55">
+        <v>333.8172972972973</v>
+      </c>
+      <c r="Y198" s="55">
+        <v>67.49902570438813</v>
+      </c>
+      <c r="Z198" s="53">
+        <v>0.30260000000000004</v>
+      </c>
+      <c r="AA198" s="56">
+        <v>0.398</v>
+      </c>
       <c r="AB198" s="57"/>
       <c r="AD198" s="35"/>
       <c r="AE198" s="35"/>
@@ -24119,30 +25043,74 @@
       <c r="C219" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D219" s="52"/>
-      <c r="E219" s="52"/>
-      <c r="F219" s="52"/>
-      <c r="G219" s="53"/>
-      <c r="H219" s="52"/>
-      <c r="I219" s="52"/>
-      <c r="J219" s="52"/>
-      <c r="K219" s="52"/>
-      <c r="L219" s="52"/>
-      <c r="M219" s="53"/>
+      <c r="D219" s="52">
+        <v>137109.56054889</v>
+      </c>
+      <c r="E219" s="52">
+        <v>42368.33</v>
+      </c>
+      <c r="F219" s="52">
+        <v>94741.23054889</v>
+      </c>
+      <c r="G219" s="53">
+        <v>0.6909892364151188</v>
+      </c>
+      <c r="H219" s="52">
+        <v>117394.569232</v>
+      </c>
+      <c r="I219" s="52">
+        <v>37161.14</v>
+      </c>
+      <c r="J219" s="52">
+        <v>99479.615032</v>
+      </c>
+      <c r="K219" s="52">
+        <v>37161.14</v>
+      </c>
+      <c r="L219" s="52">
+        <v>62318.475032</v>
+      </c>
+      <c r="M219" s="53">
+        <v>0.6264446742375689</v>
+      </c>
       <c r="N219" s="53"/>
-      <c r="O219" s="52"/>
-      <c r="P219" s="52"/>
-      <c r="Q219" s="52"/>
-      <c r="R219" s="53"/>
-      <c r="S219" s="54"/>
-      <c r="T219" s="54"/>
-      <c r="U219" s="54"/>
-      <c r="V219" s="53"/>
+      <c r="O219" s="52">
+        <v>17914.9542</v>
+      </c>
+      <c r="P219" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q219" s="52">
+        <v>17914.9542</v>
+      </c>
+      <c r="R219" s="53">
+        <v>1</v>
+      </c>
+      <c r="S219" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="T219" s="54">
+        <v>0</v>
+      </c>
+      <c r="U219" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="V219" s="53">
+        <v>1</v>
+      </c>
       <c r="W219" s="53"/>
-      <c r="X219" s="55"/>
-      <c r="Y219" s="55"/>
-      <c r="Z219" s="53"/>
-      <c r="AA219" s="56"/>
+      <c r="X219" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y219" s="55">
+        <v>54.93783457863793</v>
+      </c>
+      <c r="Z219" s="53">
+        <v>0.1229</v>
+      </c>
+      <c r="AA219" s="56">
+        <v>0.1438</v>
+      </c>
       <c r="AB219" s="57"/>
       <c r="AD219" s="35"/>
       <c r="AE219" s="35"/>
@@ -24604,30 +25572,74 @@
       <c r="C226" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D226" s="52"/>
-      <c r="E226" s="52"/>
-      <c r="F226" s="52"/>
-      <c r="G226" s="53"/>
-      <c r="H226" s="52"/>
-      <c r="I226" s="52"/>
-      <c r="J226" s="52"/>
-      <c r="K226" s="52"/>
-      <c r="L226" s="52"/>
-      <c r="M226" s="53"/>
+      <c r="D226" s="52">
+        <v>412300.73261827</v>
+      </c>
+      <c r="E226" s="52">
+        <v>353667.87</v>
+      </c>
+      <c r="F226" s="52">
+        <v>58632.86261826998</v>
+      </c>
+      <c r="G226" s="53">
+        <v>0.1422089702483149</v>
+      </c>
+      <c r="H226" s="52">
+        <v>306356.278672</v>
+      </c>
+      <c r="I226" s="52">
+        <v>253305.89</v>
+      </c>
+      <c r="J226" s="52">
+        <v>186357.488872</v>
+      </c>
+      <c r="K226" s="52">
+        <v>181341.87</v>
+      </c>
+      <c r="L226" s="52">
+        <v>5015.618871999992</v>
+      </c>
+      <c r="M226" s="53">
+        <v>0.026913964672731664</v>
+      </c>
       <c r="N226" s="53"/>
-      <c r="O226" s="52"/>
-      <c r="P226" s="52"/>
-      <c r="Q226" s="52"/>
-      <c r="R226" s="53"/>
-      <c r="S226" s="54"/>
-      <c r="T226" s="54"/>
-      <c r="U226" s="54"/>
-      <c r="V226" s="53"/>
+      <c r="O226" s="52">
+        <v>119998.7898</v>
+      </c>
+      <c r="P226" s="52">
+        <v>71964.02</v>
+      </c>
+      <c r="Q226" s="52">
+        <v>48034.769799999995</v>
+      </c>
+      <c r="R226" s="53">
+        <v>0.400293785296158</v>
+      </c>
+      <c r="S226" s="54">
+        <v>2412.45</v>
+      </c>
+      <c r="T226" s="54">
+        <v>1535.92</v>
+      </c>
+      <c r="U226" s="54">
+        <v>876.5299999999997</v>
+      </c>
+      <c r="V226" s="53">
+        <v>0.363336027689693</v>
+      </c>
       <c r="W226" s="53"/>
-      <c r="X226" s="55"/>
-      <c r="Y226" s="55"/>
-      <c r="Z226" s="53"/>
-      <c r="AA226" s="56"/>
+      <c r="X226" s="55">
+        <v>65.34323402260534</v>
+      </c>
+      <c r="Y226" s="55">
+        <v>43.91570973337064</v>
+      </c>
+      <c r="Z226" s="53">
+        <v>0.2838</v>
+      </c>
+      <c r="AA226" s="56">
+        <v>0.257</v>
+      </c>
       <c r="AB226" s="57"/>
       <c r="AD226" s="35"/>
       <c r="AE226" s="35"/>
@@ -25079,30 +26091,74 @@
       <c r="C233" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D233" s="52"/>
-      <c r="E233" s="52"/>
-      <c r="F233" s="52"/>
-      <c r="G233" s="53"/>
-      <c r="H233" s="52"/>
-      <c r="I233" s="52"/>
-      <c r="J233" s="52"/>
-      <c r="K233" s="52"/>
-      <c r="L233" s="52"/>
-      <c r="M233" s="53"/>
+      <c r="D233" s="52">
+        <v>8795.02836582</v>
+      </c>
+      <c r="E233" s="52">
+        <v>1740.2</v>
+      </c>
+      <c r="F233" s="52">
+        <v>7054.828365820001</v>
+      </c>
+      <c r="G233" s="53">
+        <v>0.8021382163174237</v>
+      </c>
+      <c r="H233" s="52">
+        <v>6369.1218</v>
+      </c>
+      <c r="I233" s="52">
+        <v>239.55</v>
+      </c>
+      <c r="J233" s="52">
+        <v>4527.894</v>
+      </c>
+      <c r="K233" s="52">
+        <v>239.55</v>
+      </c>
+      <c r="L233" s="52">
+        <v>4288.344</v>
+      </c>
+      <c r="M233" s="53">
+        <v>0.9470946095469549</v>
+      </c>
       <c r="N233" s="53"/>
-      <c r="O233" s="52"/>
-      <c r="P233" s="52"/>
-      <c r="Q233" s="52"/>
-      <c r="R233" s="53"/>
-      <c r="S233" s="54"/>
-      <c r="T233" s="54"/>
-      <c r="U233" s="54"/>
-      <c r="V233" s="53"/>
+      <c r="O233" s="52">
+        <v>1841.2278</v>
+      </c>
+      <c r="P233" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q233" s="52">
+        <v>1841.2278</v>
+      </c>
+      <c r="R233" s="53">
+        <v>1</v>
+      </c>
+      <c r="S233" s="54">
+        <v>36.92</v>
+      </c>
+      <c r="T233" s="54">
+        <v>0</v>
+      </c>
+      <c r="U233" s="54">
+        <v>36.92</v>
+      </c>
+      <c r="V233" s="53">
+        <v>1</v>
+      </c>
       <c r="W233" s="53"/>
-      <c r="X233" s="55"/>
-      <c r="Y233" s="55"/>
-      <c r="Z233" s="53"/>
-      <c r="AA233" s="56"/>
+      <c r="X233" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y233" s="55">
+        <v>65.70711175027087</v>
+      </c>
+      <c r="Z233" s="53">
+        <v>0.8623000000000001</v>
+      </c>
+      <c r="AA233" s="56">
+        <v>0.2758</v>
+      </c>
       <c r="AB233" s="57"/>
       <c r="AD233" s="35"/>
       <c r="AE233" s="35"/>
@@ -25508,30 +26564,74 @@
       <c r="C240" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D240" s="52"/>
-      <c r="E240" s="52"/>
-      <c r="F240" s="52"/>
-      <c r="G240" s="53"/>
-      <c r="H240" s="52"/>
-      <c r="I240" s="52"/>
-      <c r="J240" s="52"/>
-      <c r="K240" s="52"/>
-      <c r="L240" s="52"/>
-      <c r="M240" s="53"/>
+      <c r="D240" s="52">
+        <v>27503.13664251</v>
+      </c>
+      <c r="E240" s="52">
+        <v>0</v>
+      </c>
+      <c r="F240" s="52">
+        <v>27503.13664251</v>
+      </c>
+      <c r="G240" s="53">
+        <v>1</v>
+      </c>
+      <c r="H240" s="52">
+        <v>19683.280628</v>
+      </c>
+      <c r="I240" s="52">
+        <v>0</v>
+      </c>
+      <c r="J240" s="52">
+        <v>10693.531628</v>
+      </c>
+      <c r="K240" s="52">
+        <v>0</v>
+      </c>
+      <c r="L240" s="52">
+        <v>10693.531628</v>
+      </c>
+      <c r="M240" s="53">
+        <v>1</v>
+      </c>
       <c r="N240" s="53"/>
-      <c r="O240" s="52"/>
-      <c r="P240" s="52"/>
-      <c r="Q240" s="52"/>
-      <c r="R240" s="53"/>
-      <c r="S240" s="54"/>
-      <c r="T240" s="54"/>
-      <c r="U240" s="54"/>
-      <c r="V240" s="53"/>
+      <c r="O240" s="52">
+        <v>8989.749</v>
+      </c>
+      <c r="P240" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q240" s="52">
+        <v>8989.749</v>
+      </c>
+      <c r="R240" s="53">
+        <v>1</v>
+      </c>
+      <c r="S240" s="54">
+        <v>180.16</v>
+      </c>
+      <c r="T240" s="54">
+        <v>0</v>
+      </c>
+      <c r="U240" s="54">
+        <v>180.16</v>
+      </c>
+      <c r="V240" s="53">
+        <v>1</v>
+      </c>
       <c r="W240" s="53"/>
-      <c r="X240" s="55"/>
-      <c r="Y240" s="55"/>
-      <c r="Z240" s="53"/>
-      <c r="AA240" s="56"/>
+      <c r="X240" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y240" s="55">
+        <v>43.40506224750221</v>
+      </c>
+      <c r="Z240" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA240" s="56">
+        <v>0.2843</v>
+      </c>
       <c r="AB240" s="57"/>
       <c r="AD240" s="35"/>
       <c r="AE240" s="35"/>
@@ -25937,30 +27037,74 @@
       <c r="C247" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D247" s="52"/>
-      <c r="E247" s="52"/>
-      <c r="F247" s="52"/>
-      <c r="G247" s="53"/>
-      <c r="H247" s="52"/>
-      <c r="I247" s="52"/>
-      <c r="J247" s="52"/>
-      <c r="K247" s="52"/>
-      <c r="L247" s="52"/>
-      <c r="M247" s="53"/>
+      <c r="D247" s="52">
+        <v>40670.1518342</v>
+      </c>
+      <c r="E247" s="52">
+        <v>0</v>
+      </c>
+      <c r="F247" s="52">
+        <v>40670.1518342</v>
+      </c>
+      <c r="G247" s="53">
+        <v>1</v>
+      </c>
+      <c r="H247" s="52">
+        <v>29498.3116992</v>
+      </c>
+      <c r="I247" s="52">
+        <v>0</v>
+      </c>
+      <c r="J247" s="52">
+        <v>24964.3288992</v>
+      </c>
+      <c r="K247" s="52">
+        <v>0</v>
+      </c>
+      <c r="L247" s="52">
+        <v>24964.3288992</v>
+      </c>
+      <c r="M247" s="53">
+        <v>1</v>
+      </c>
       <c r="N247" s="53"/>
-      <c r="O247" s="52"/>
-      <c r="P247" s="52"/>
-      <c r="Q247" s="52"/>
-      <c r="R247" s="53"/>
-      <c r="S247" s="54"/>
-      <c r="T247" s="54"/>
-      <c r="U247" s="54"/>
-      <c r="V247" s="53"/>
+      <c r="O247" s="52">
+        <v>4533.9828</v>
+      </c>
+      <c r="P247" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q247" s="52">
+        <v>4533.9828</v>
+      </c>
+      <c r="R247" s="53">
+        <v>1</v>
+      </c>
+      <c r="S247" s="54">
+        <v>90.88</v>
+      </c>
+      <c r="T247" s="54">
+        <v>0</v>
+      </c>
+      <c r="U247" s="54">
+        <v>90.88</v>
+      </c>
+      <c r="V247" s="53">
+        <v>1</v>
+      </c>
       <c r="W247" s="53"/>
-      <c r="X247" s="55"/>
-      <c r="Y247" s="55"/>
-      <c r="Z247" s="53"/>
-      <c r="AA247" s="56"/>
+      <c r="X247" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y247" s="55">
+        <v>122.92957895026407</v>
+      </c>
+      <c r="Z247" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA247" s="56">
+        <v>0.2747</v>
+      </c>
       <c r="AB247" s="57"/>
       <c r="AD247" s="35"/>
       <c r="AE247" s="35"/>
@@ -26366,30 +27510,74 @@
       <c r="C254" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D254" s="52"/>
-      <c r="E254" s="52"/>
-      <c r="F254" s="52"/>
-      <c r="G254" s="53"/>
-      <c r="H254" s="52"/>
-      <c r="I254" s="52"/>
-      <c r="J254" s="52"/>
-      <c r="K254" s="52"/>
-      <c r="L254" s="52"/>
-      <c r="M254" s="53"/>
+      <c r="D254" s="52">
+        <v>21396.50036782</v>
+      </c>
+      <c r="E254" s="52">
+        <v>0</v>
+      </c>
+      <c r="F254" s="52">
+        <v>21396.50036782</v>
+      </c>
+      <c r="G254" s="53">
+        <v>1</v>
+      </c>
+      <c r="H254" s="52">
+        <v>15378.244372</v>
+      </c>
+      <c r="I254" s="52">
+        <v>0</v>
+      </c>
+      <c r="J254" s="52">
+        <v>8344.608772</v>
+      </c>
+      <c r="K254" s="52">
+        <v>0</v>
+      </c>
+      <c r="L254" s="52">
+        <v>8344.608772</v>
+      </c>
+      <c r="M254" s="53">
+        <v>1</v>
+      </c>
       <c r="N254" s="53"/>
-      <c r="O254" s="52"/>
-      <c r="P254" s="52"/>
-      <c r="Q254" s="52"/>
-      <c r="R254" s="53"/>
-      <c r="S254" s="54"/>
-      <c r="T254" s="54"/>
-      <c r="U254" s="54"/>
-      <c r="V254" s="53"/>
+      <c r="O254" s="52">
+        <v>7033.6356</v>
+      </c>
+      <c r="P254" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q254" s="52">
+        <v>7033.6356</v>
+      </c>
+      <c r="R254" s="53">
+        <v>1</v>
+      </c>
+      <c r="S254" s="54">
+        <v>140.9</v>
+      </c>
+      <c r="T254" s="54">
+        <v>0</v>
+      </c>
+      <c r="U254" s="54">
+        <v>140.9</v>
+      </c>
+      <c r="V254" s="53">
+        <v>1</v>
+      </c>
       <c r="W254" s="53"/>
-      <c r="X254" s="55"/>
-      <c r="Y254" s="55"/>
-      <c r="Z254" s="53"/>
-      <c r="AA254" s="56"/>
+      <c r="X254" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y254" s="55">
+        <v>42.71295951611073</v>
+      </c>
+      <c r="Z254" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA254" s="56">
+        <v>0.2813</v>
+      </c>
       <c r="AB254" s="57"/>
       <c r="AD254" s="35"/>
       <c r="AE254" s="35"/>
@@ -26795,30 +27983,74 @@
       <c r="C261" s="76" t="s">
         <v>104</v>
       </c>
-      <c r="D261" s="52"/>
-      <c r="E261" s="52"/>
-      <c r="F261" s="52"/>
-      <c r="G261" s="53"/>
-      <c r="H261" s="52"/>
-      <c r="I261" s="52"/>
-      <c r="J261" s="52"/>
-      <c r="K261" s="52"/>
-      <c r="L261" s="52"/>
-      <c r="M261" s="53"/>
+      <c r="D261" s="52">
+        <v>239296.88379393</v>
+      </c>
+      <c r="E261" s="52">
+        <v>19872.16</v>
+      </c>
+      <c r="F261" s="52">
+        <v>219424.72379393</v>
+      </c>
+      <c r="G261" s="53">
+        <v>0.916956043534972</v>
+      </c>
+      <c r="H261" s="52">
+        <v>203192.691868</v>
+      </c>
+      <c r="I261" s="52">
+        <v>18292.87</v>
+      </c>
+      <c r="J261" s="52">
+        <v>175849.529668</v>
+      </c>
+      <c r="K261" s="52">
+        <v>16897.46</v>
+      </c>
+      <c r="L261" s="52">
+        <v>158952.069668</v>
+      </c>
+      <c r="M261" s="53">
+        <v>0.9039095524912576</v>
+      </c>
       <c r="N261" s="53"/>
-      <c r="O261" s="52"/>
-      <c r="P261" s="52"/>
-      <c r="Q261" s="52"/>
-      <c r="R261" s="53"/>
-      <c r="S261" s="54"/>
-      <c r="T261" s="54"/>
-      <c r="U261" s="54"/>
-      <c r="V261" s="53"/>
+      <c r="O261" s="52">
+        <v>27343.1622</v>
+      </c>
+      <c r="P261" s="52">
+        <v>1395.41</v>
+      </c>
+      <c r="Q261" s="52">
+        <v>25947.7522</v>
+      </c>
+      <c r="R261" s="53">
+        <v>0.9489667658117465</v>
+      </c>
+      <c r="S261" s="54">
+        <v>547.57</v>
+      </c>
+      <c r="T261" s="54">
+        <v>27.84</v>
+      </c>
+      <c r="U261" s="54">
+        <v>519.73</v>
+      </c>
+      <c r="V261" s="53">
+        <v>0.9491571853826908</v>
+      </c>
       <c r="W261" s="53"/>
-      <c r="X261" s="55"/>
-      <c r="Y261" s="55"/>
-      <c r="Z261" s="53"/>
-      <c r="AA261" s="56"/>
+      <c r="X261" s="55">
+        <v>56.727370689655174</v>
+      </c>
+      <c r="Y261" s="55">
+        <v>65.93529946112827</v>
+      </c>
+      <c r="Z261" s="53">
+        <v>0.0795</v>
+      </c>
+      <c r="AA261" s="56">
+        <v>0.1509</v>
+      </c>
       <c r="AB261" s="57"/>
       <c r="AD261" s="35"/>
       <c r="AE261" s="35"/>
@@ -27506,16 +28738,16 @@
         <v>22202.890000000014</v>
       </c>
       <c r="D4" s="52">
-        <v>21022.23000000001</v>
+        <v>21523.99000000002</v>
       </c>
       <c r="E4" s="52">
-        <v>1180.6600000000035</v>
+        <v>678.8999999999942</v>
       </c>
       <c r="F4" s="52">
         <v>0</v>
       </c>
       <c r="G4" s="53">
-        <v>0.053175960426773396</v>
+        <v>0.03057710054862199</v>
       </c>
       <c r="H4" s="53">
         <v>0.2149</v>
@@ -27530,16 +28762,16 @@
         <v>7000</v>
       </c>
       <c r="L4" s="53">
-        <v>-0.26209831242689546</v>
+        <v>-0.2846971723050469</v>
       </c>
       <c r="M4" s="52">
-        <v>-5819.3399999999965</v>
+        <v>-6321.100000000006</v>
       </c>
       <c r="N4" s="54">
         <v>20</v>
       </c>
       <c r="O4" s="58">
-        <v>-83.13342857142852</v>
+        <v>-90.30142857142866</v>
       </c>
     </row>
     <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -27570,16 +28802,16 @@
         <v>42019.899999999994</v>
       </c>
       <c r="D6" s="52">
-        <v>18657.01999999999</v>
+        <v>20112.42</v>
       </c>
       <c r="E6" s="52">
-        <v>23362.880000000005</v>
+        <v>21907.479999999996</v>
       </c>
       <c r="F6" s="52">
         <v>7</v>
       </c>
       <c r="G6" s="53">
-        <v>0.5561621993388849</v>
+        <v>0.5215262292390034</v>
       </c>
       <c r="H6" s="53">
         <v>0.239214585617637</v>
@@ -27594,16 +28826,16 @@
         <v>20272.6</v>
       </c>
       <c r="L6" s="53">
-        <v>0.07370983748176475</v>
+        <v>0.03907386738188329</v>
       </c>
       <c r="M6" s="52">
-        <v>3097.280000000006</v>
+        <v>1641.8799999999974</v>
       </c>
       <c r="N6" s="54">
         <v>-52.5</v>
       </c>
       <c r="O6" s="58">
-        <v>6.921296089385488</v>
+        <v>3.669005586592173</v>
       </c>
       <c r="Q6" s="35" t="s">
         <v>121</v>
@@ -27761,16 +28993,16 @@
         <v>93276.07999999999</v>
       </c>
       <c r="D12" s="52">
-        <v>61105.389999999985</v>
+        <v>62494.389999999985</v>
       </c>
       <c r="E12" s="52">
-        <v>32170.690000000002</v>
+        <v>30781.690000000002</v>
       </c>
       <c r="F12" s="52">
         <v>3</v>
       </c>
       <c r="G12" s="53">
-        <v>0.34492969687405395</v>
+        <v>0.3300384192817709</v>
       </c>
       <c r="H12" s="53">
         <v>0.176316261575212</v>
@@ -27785,16 +29017,16 @@
         <v>2640</v>
       </c>
       <c r="L12" s="53">
-        <v>0.31662662067273845</v>
+        <v>0.3017353430804554</v>
       </c>
       <c r="M12" s="52">
-        <v>29533.690000000002</v>
+        <v>28144.690000000002</v>
       </c>
       <c r="N12" s="54">
         <v>53</v>
       </c>
       <c r="O12" s="58">
-        <v>428.02449275362324</v>
+        <v>407.89405797101455</v>
       </c>
       <c r="Q12" s="35" t="s">
         <v>123</v>
@@ -27828,16 +29060,16 @@
         <v>61369.72</v>
       </c>
       <c r="D14" s="52">
-        <v>14493.379999999997</v>
+        <v>14830.879999999997</v>
       </c>
       <c r="E14" s="52">
-        <v>46876.340000000004</v>
+        <v>46538.840000000004</v>
       </c>
       <c r="F14" s="52">
         <v>0</v>
       </c>
       <c r="G14" s="53">
-        <v>0.7638349987583454</v>
+        <v>0.7583355439783659</v>
       </c>
       <c r="H14" s="53">
         <v>0.266338527271097</v>
@@ -27852,16 +29084,16 @@
         <v>3000</v>
       </c>
       <c r="L14" s="53">
-        <v>0.7149509562696392</v>
+        <v>0.7094515014896597</v>
       </c>
       <c r="M14" s="52">
-        <v>43876.340000000004</v>
+        <v>43538.840000000004</v>
       </c>
       <c r="N14" s="54">
         <v>-112</v>
       </c>
       <c r="O14" s="58">
-        <v>-391.7530357142858</v>
+        <v>-388.7396428571429</v>
       </c>
     </row>
     <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -27954,16 +29186,16 @@
         <v>27482.319999999992</v>
       </c>
       <c r="D18" s="52">
-        <v>14933.520000000004</v>
+        <v>18539.01000000001</v>
       </c>
       <c r="E18" s="52">
-        <v>12548.799999999988</v>
+        <v>8943.309999999983</v>
       </c>
       <c r="F18" s="52">
         <v>0</v>
       </c>
       <c r="G18" s="53">
-        <v>0.45661356100940503</v>
+        <v>0.32542048851770833</v>
       </c>
       <c r="H18" s="53">
         <v>0.296537658865514</v>
@@ -27978,16 +29210,16 @@
         <v>8200</v>
       </c>
       <c r="L18" s="53">
-        <v>0.15823991569852872</v>
+        <v>0.027046843206832004</v>
       </c>
       <c r="M18" s="52">
-        <v>4348.799999999988</v>
+        <v>743.3099999999831</v>
       </c>
       <c r="N18" s="54">
         <v>-269</v>
       </c>
       <c r="O18" s="58">
-        <v>-23.00952380952375</v>
+        <v>-3.9328571428570536</v>
       </c>
       <c r="Q18" s="35" t="s">
         <v>124</v>
@@ -28074,19 +29306,19 @@
         <v>39</v>
       </c>
       <c r="C22" s="52">
-        <v>0</v>
+        <v>19065.239999999998</v>
       </c>
       <c r="D22" s="52">
-        <v>12195.39</v>
+        <v>14898.84</v>
       </c>
       <c r="E22" s="52">
-        <v>-12195.39</v>
+        <v>4166.399999999998</v>
       </c>
       <c r="F22" s="52">
         <v>3</v>
       </c>
       <c r="G22" s="53">
-        <v>0</v>
+        <v>0.21869118878125837</v>
       </c>
       <c r="H22" s="53">
         <v>0.252488256827238</v>
@@ -28097,10 +29329,10 @@
         <v>0</v>
       </c>
       <c r="L22" s="53">
-        <v>0</v>
+        <v>0.21869118878125837</v>
       </c>
       <c r="M22" s="52">
-        <v>-12192.39</v>
+        <v>4169.399999999998</v>
       </c>
       <c r="N22" s="54"/>
       <c r="O22" s="58">
@@ -28132,19 +29364,19 @@
         <v>40</v>
       </c>
       <c r="C24" s="52">
-        <v>0</v>
+        <v>16999.83</v>
       </c>
       <c r="D24" s="52">
-        <v>9681.120000000003</v>
+        <v>12895.309999999998</v>
       </c>
       <c r="E24" s="52">
-        <v>-9681.120000000003</v>
+        <v>4104.520000000004</v>
       </c>
       <c r="F24" s="52">
         <v>3</v>
       </c>
       <c r="G24" s="53">
-        <v>0</v>
+        <v>0.2416212397418094</v>
       </c>
       <c r="H24" s="53"/>
       <c r="I24" s="54"/>
@@ -28153,10 +29385,10 @@
         <v>0</v>
       </c>
       <c r="L24" s="53">
-        <v>0</v>
+        <v>0.2416212397418094</v>
       </c>
       <c r="M24" s="52">
-        <v>-9678.120000000003</v>
+        <v>4107.520000000004</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="58">
@@ -28499,10 +29731,10 @@
         <v>0</v>
       </c>
       <c r="D36" s="52">
-        <v>0</v>
+        <v>58.32</v>
       </c>
       <c r="E36" s="52">
-        <v>0</v>
+        <v>-58.32</v>
       </c>
       <c r="F36" s="52">
         <v>0</v>
@@ -28524,11 +29756,11 @@
         <v>0</v>
       </c>
       <c r="M36" s="52">
-        <v>-3200</v>
+        <v>-3258.32</v>
       </c>
       <c r="N36" s="54"/>
       <c r="O36" s="58">
-        <v>-40</v>
+        <v>-40.729</v>
       </c>
     </row>
     <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -28851,10 +30083,10 @@
         <v>0</v>
       </c>
       <c r="D48" s="99">
-        <v>2218.25</v>
+        <v>3650.3599999999988</v>
       </c>
       <c r="E48" s="99">
-        <v>-2218.25</v>
+        <v>-3650.3599999999988</v>
       </c>
       <c r="F48" s="99"/>
       <c r="G48" s="100">
@@ -28874,13 +30106,13 @@
         <v>0</v>
       </c>
       <c r="M48" s="99">
-        <v>-4748.25</v>
+        <v>-6180.359999999999</v>
       </c>
       <c r="N48" s="98">
         <v>-44.75</v>
       </c>
       <c r="O48" s="60">
-        <v>106.10614525139665</v>
+        <v>138.10860335195528</v>
       </c>
     </row>
     <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -28970,10 +30202,10 @@
         <v>0</v>
       </c>
       <c r="D52" s="99">
-        <v>2942.1800000000076</v>
+        <v>3062.5</v>
       </c>
       <c r="E52" s="99">
-        <v>-2942.1800000000076</v>
+        <v>-3062.5</v>
       </c>
       <c r="F52" s="99"/>
       <c r="G52" s="100">
@@ -28995,13 +30227,13 @@
         <v>0</v>
       </c>
       <c r="M52" s="99">
-        <v>-4222.180000000008</v>
+        <v>-4342.5</v>
       </c>
       <c r="N52" s="98">
         <v>-304.75</v>
       </c>
       <c r="O52" s="60">
-        <v>15.480036663611394</v>
+        <v>15.921173235563703</v>
       </c>
     </row>
     <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -29032,10 +30264,10 @@
         <v>0</v>
       </c>
       <c r="D54" s="99">
-        <v>1718.2499999999995</v>
+        <v>2109.5099999999998</v>
       </c>
       <c r="E54" s="99">
-        <v>-1718.2499999999995</v>
+        <v>-2109.5099999999998</v>
       </c>
       <c r="F54" s="99"/>
       <c r="G54" s="100">
@@ -29057,13 +30289,13 @@
         <v>0</v>
       </c>
       <c r="M54" s="99">
-        <v>-2358.2499999999995</v>
+        <v>-2749.5099999999998</v>
       </c>
       <c r="N54" s="98">
         <v>-11.25</v>
       </c>
       <c r="O54" s="60">
-        <v>-496.47368421052624</v>
+        <v>-578.8442105263157</v>
       </c>
     </row>
     <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -29279,17 +30511,17 @@
         <v>61</v>
       </c>
       <c r="C64" s="99">
-        <v>0</v>
+        <v>12193.580000000002</v>
       </c>
       <c r="D64" s="99">
         <v>11037.14</v>
       </c>
       <c r="E64" s="99">
-        <v>-11037.14</v>
+        <v>1156.4400000000023</v>
       </c>
       <c r="F64" s="99"/>
       <c r="G64" s="100">
-        <v>0</v>
+        <v>0.09484007157865058</v>
       </c>
       <c r="H64" s="100">
         <v>0.143790046441692</v>
@@ -29302,10 +30534,10 @@
         <v>1750</v>
       </c>
       <c r="L64" s="100">
-        <v>0</v>
+        <v>-0.04867807485578457</v>
       </c>
       <c r="M64" s="99">
-        <v>-12787.14</v>
+        <v>-593.5599999999977</v>
       </c>
       <c r="N64" s="98"/>
       <c r="O64" s="60">
@@ -29340,14 +30572,14 @@
         <v>82279.71999999997</v>
       </c>
       <c r="D66" s="99">
-        <v>22406.589999999997</v>
+        <v>18983.080000000016</v>
       </c>
       <c r="E66" s="99">
-        <v>59873.129999999976</v>
+        <v>63296.639999999956</v>
       </c>
       <c r="F66" s="99"/>
       <c r="G66" s="100">
-        <v>0.727677853060268</v>
+        <v>0.7692860403511337</v>
       </c>
       <c r="H66" s="100">
         <v>0.256265521519856</v>
@@ -29362,16 +30594,16 @@
         <v>3200</v>
       </c>
       <c r="L66" s="100">
-        <v>0.6887861310174609</v>
+        <v>0.7303943183083265</v>
       </c>
       <c r="M66" s="99">
-        <v>56673.129999999976</v>
+        <v>60096.639999999956</v>
       </c>
       <c r="N66" s="98">
         <v>-1014.25</v>
       </c>
       <c r="O66" s="60">
-        <v>-60.66163232539468</v>
+        <v>-64.3260797431094</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -29382,17 +30614,17 @@
         <v>68</v>
       </c>
       <c r="C67" s="99">
-        <v>10598.48</v>
+        <v>19872.16</v>
       </c>
       <c r="D67" s="99">
-        <v>18235.02</v>
+        <v>18292.87</v>
       </c>
       <c r="E67" s="99">
-        <v>-7636.540000000001</v>
+        <v>1579.2900000000009</v>
       </c>
       <c r="F67" s="99"/>
       <c r="G67" s="100">
-        <v>-0.7205316234026012</v>
+        <v>0.07947248814421788</v>
       </c>
       <c r="H67" s="100">
         <f>'Deliverables Sheet'!AA256</f>
@@ -29403,10 +30635,10 @@
         <v>0</v>
       </c>
       <c r="L67" s="100">
-        <v>-0.7205316234026012</v>
+        <v>0.07947248814421788</v>
       </c>
       <c r="M67" s="99">
-        <v>-7636.540000000001</v>
+        <v>1579.2900000000009</v>
       </c>
       <c r="N67" s="98"/>
       <c r="O67" s="60">
@@ -29538,17 +30770,17 @@
         <v>63</v>
       </c>
       <c r="C71" s="99">
-        <v>0</v>
+        <v>1740.2</v>
       </c>
       <c r="D71" s="99">
-        <v>397</v>
+        <v>239.55</v>
       </c>
       <c r="E71" s="99">
-        <v>-397</v>
+        <v>1500.65</v>
       </c>
       <c r="F71" s="99"/>
       <c r="G71" s="100">
-        <v>0</v>
+        <v>0.8623434088035858</v>
       </c>
       <c r="H71" s="100">
         <f>'Deliverables Sheet'!AA228</f>
@@ -29559,10 +30791,10 @@
         <v>0</v>
       </c>
       <c r="L71" s="100">
-        <v>0</v>
+        <v>0.8623434088035858</v>
       </c>
       <c r="M71" s="99">
-        <v>-397</v>
+        <v>1500.65</v>
       </c>
       <c r="N71" s="98"/>
       <c r="O71" s="60">
@@ -29611,25 +30843,25 @@
         <v>127</v>
       </c>
       <c r="C74" s="104">
-        <v>432684.38999999996</v>
+        <v>491956.92</v>
       </c>
       <c r="D74" s="104">
-        <v>234541.40999999992</v>
+        <v>246227.09999999998</v>
       </c>
       <c r="E74" s="105">
-        <v>198142.97999999998</v>
+        <v>245729.81999999995</v>
       </c>
       <c r="F74" s="106" t="s">
         <v>128</v>
       </c>
       <c r="G74" s="107">
-        <v>0.4579388223365303</v>
+        <v>0.49949458989213924</v>
       </c>
       <c r="H74" s="108" t="s">
         <v>129</v>
       </c>
       <c r="I74" s="109">
-        <v>0.295620509905615</v>
+        <v>0.3567329025476457</v>
       </c>
       <c r="J74" s="36"/>
       <c r="K74" s="36"/>
@@ -30184,10 +31416,10 @@
         <v>638.02</v>
       </c>
       <c r="D4" s="54">
-        <v>616.75</v>
+        <v>625.25</v>
       </c>
       <c r="E4" s="54">
-        <v>21.269999999999982</v>
+        <v>12.769999999999982</v>
       </c>
       <c r="F4" s="54">
         <v>0</v>
@@ -30243,10 +31475,10 @@
         <v>363.57</v>
       </c>
       <c r="D6" s="54">
-        <v>272.5</v>
+        <v>304.75</v>
       </c>
       <c r="E6" s="54">
-        <v>91.07</v>
+        <v>58.81999999999999</v>
       </c>
       <c r="F6" s="54"/>
       <c r="G6" s="54"/>
@@ -30410,10 +31642,10 @@
         <v>1124.47</v>
       </c>
       <c r="D12" s="54">
-        <v>783</v>
+        <v>813.5</v>
       </c>
       <c r="E12" s="54">
-        <v>341.47</v>
+        <v>310.97</v>
       </c>
       <c r="F12" s="54"/>
       <c r="G12" s="54"/>
@@ -30469,10 +31701,10 @@
         <v>501.83</v>
       </c>
       <c r="D14" s="54">
-        <v>358.75</v>
+        <v>366.25</v>
       </c>
       <c r="E14" s="54">
-        <v>143.07999999999998</v>
+        <v>135.57999999999998</v>
       </c>
       <c r="F14" s="54"/>
       <c r="G14" s="54"/>
@@ -30580,10 +31812,10 @@
         <v>685.48</v>
       </c>
       <c r="D18" s="54">
-        <v>669</v>
+        <v>699.75</v>
       </c>
       <c r="E18" s="54">
-        <v>16.480000000000018</v>
+        <v>-14.269999999999982</v>
       </c>
       <c r="F18" s="54"/>
       <c r="G18" s="54"/>
@@ -30682,10 +31914,10 @@
         <v>193.32</v>
       </c>
       <c r="D22" s="54">
-        <v>52.75</v>
+        <v>83.5</v>
       </c>
       <c r="E22" s="54">
-        <v>140.57</v>
+        <v>109.82</v>
       </c>
       <c r="F22" s="54"/>
       <c r="G22" s="54"/>
@@ -30738,10 +31970,10 @@
         <v>472.14</v>
       </c>
       <c r="D24" s="54">
-        <v>167.25</v>
+        <v>202</v>
       </c>
       <c r="E24" s="54">
-        <v>304.89</v>
+        <v>270.14</v>
       </c>
       <c r="F24" s="54"/>
       <c r="G24" s="54"/>
@@ -31045,13 +32277,13 @@
         <v>48</v>
       </c>
       <c r="C36" s="54">
-        <v>86.01</v>
+        <v>82.37</v>
       </c>
       <c r="D36" s="54">
         <v>0</v>
       </c>
       <c r="E36" s="54">
-        <v>86.01</v>
+        <v>82.37</v>
       </c>
       <c r="F36" s="54"/>
       <c r="G36" s="54"/>
@@ -31375,10 +32607,10 @@
         <v>110.44</v>
       </c>
       <c r="D48" s="54">
-        <v>95.5</v>
+        <v>116.25</v>
       </c>
       <c r="E48" s="54">
-        <v>14.939999999999998</v>
+        <v>-5.810000000000002</v>
       </c>
       <c r="F48" s="54"/>
       <c r="G48" s="54"/>
@@ -31483,10 +32715,10 @@
         <v>659.73</v>
       </c>
       <c r="D52" s="54">
-        <v>548.75</v>
+        <v>550.75</v>
       </c>
       <c r="E52" s="54">
-        <v>110.98000000000002</v>
+        <v>108.98000000000002</v>
       </c>
       <c r="F52" s="54"/>
       <c r="G52" s="54"/>
@@ -31538,10 +32770,10 @@
         <v>125.17</v>
       </c>
       <c r="D54" s="54">
-        <v>49.25</v>
+        <v>57.25</v>
       </c>
       <c r="E54" s="54">
-        <v>75.92</v>
+        <v>67.92</v>
       </c>
       <c r="F54" s="54"/>
       <c r="G54" s="54"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-28T19:15:27Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -10973,7 +10973,7 @@
         <v>103822.973895</v>
       </c>
       <c r="I16" s="52">
-        <v>94249.74</v>
+        <v>95219.95</v>
       </c>
       <c r="J16" s="52">
         <v>85672.874895</v>
@@ -10992,35 +10992,35 @@
         <v>18150.099</v>
       </c>
       <c r="P16" s="52">
-        <v>13747.43</v>
+        <v>14717.64</v>
       </c>
       <c r="Q16" s="52">
-        <v>4402.668999999998</v>
+        <v>3432.458999999999</v>
       </c>
       <c r="R16" s="53">
-        <v>0.24256997165690383</v>
+        <v>0.1891151668098339</v>
       </c>
       <c r="S16" s="54">
         <v>363.57</v>
       </c>
       <c r="T16" s="54">
-        <v>304.75</v>
+        <v>331.25</v>
       </c>
       <c r="U16" s="54">
-        <v>58.81999999999999</v>
+        <v>32.31999999999999</v>
       </c>
       <c r="V16" s="53">
-        <v>0.16178452567593585</v>
+        <v>0.08889622356079983</v>
       </c>
       <c r="W16" s="53"/>
       <c r="X16" s="55">
-        <v>110.36666119770302</v>
+        <v>98.60839245283019</v>
       </c>
       <c r="Y16" s="55">
         <v>77.71024646458726</v>
       </c>
       <c r="Z16" s="53">
-        <v>0.263</v>
+        <v>0.2554</v>
       </c>
       <c r="AA16" s="56">
         <v>0.2139</v>
@@ -19039,19 +19039,19 @@
         <v>85934.2000148</v>
       </c>
       <c r="I128" s="52">
-        <v>66541.03</v>
+        <v>64275.8</v>
       </c>
       <c r="J128" s="52">
         <v>70065.71561479999</v>
       </c>
       <c r="K128" s="52">
-        <v>61659.44</v>
+        <v>59394.21000000001</v>
       </c>
       <c r="L128" s="52">
-        <v>8406.27561479999</v>
+        <v>10671.505614799986</v>
       </c>
       <c r="M128" s="53">
-        <v>0.11997701787583442</v>
+        <v>0.15230709514862703</v>
       </c>
       <c r="N128" s="53"/>
       <c r="O128" s="52">
@@ -19080,13 +19080,13 @@
       </c>
       <c r="W128" s="53"/>
       <c r="X128" s="55">
-        <v>121.8556603773585</v>
+        <v>143.22575471698113</v>
       </c>
       <c r="Y128" s="55">
         <v>62.79176131227983</v>
       </c>
       <c r="Z128" s="53">
-        <v>0.16260000000000002</v>
+        <v>0.1911</v>
       </c>
       <c r="AA128" s="56">
         <v>0.1885</v>
@@ -28802,16 +28802,16 @@
         <v>42019.899999999994</v>
       </c>
       <c r="D6" s="52">
-        <v>20112.42</v>
+        <v>21082.62999999999</v>
       </c>
       <c r="E6" s="52">
-        <v>21907.479999999996</v>
+        <v>20937.270000000004</v>
       </c>
       <c r="F6" s="52">
         <v>7</v>
       </c>
       <c r="G6" s="53">
-        <v>0.5215262292390034</v>
+        <v>0.4984369310731346</v>
       </c>
       <c r="H6" s="53">
         <v>0.239214585617637</v>
@@ -28826,16 +28826,16 @@
         <v>20272.6</v>
       </c>
       <c r="L6" s="53">
-        <v>0.03907386738188329</v>
+        <v>0.01598456921601445</v>
       </c>
       <c r="M6" s="52">
-        <v>1641.8799999999974</v>
+        <v>671.6700000000055</v>
       </c>
       <c r="N6" s="54">
         <v>-52.5</v>
       </c>
       <c r="O6" s="58">
-        <v>3.669005586592173</v>
+        <v>1.500938547486046</v>
       </c>
       <c r="Q6" s="35" t="s">
         <v>121</v>
@@ -29791,16 +29791,16 @@
         <v>64090.99</v>
       </c>
       <c r="D38" s="52">
-        <v>10303.779999999999</v>
+        <v>8038.550000000003</v>
       </c>
       <c r="E38" s="52">
-        <v>53787.21</v>
+        <v>56052.439999999995</v>
       </c>
       <c r="F38" s="52">
         <v>0</v>
       </c>
       <c r="G38" s="53">
-        <v>0.8392320043737818</v>
+        <v>0.8745759739395506</v>
       </c>
       <c r="H38" s="53">
         <v>0.1750921737769</v>
@@ -29811,10 +29811,10 @@
         <v>0</v>
       </c>
       <c r="L38" s="53">
-        <v>0.8392320043737818</v>
+        <v>0.8745759739395506</v>
       </c>
       <c r="M38" s="52">
-        <v>53787.21</v>
+        <v>56052.439999999995</v>
       </c>
       <c r="N38" s="54"/>
       <c r="O38" s="58">
@@ -30846,22 +30846,22 @@
         <v>491956.92</v>
       </c>
       <c r="D74" s="104">
-        <v>245764.33999999997</v>
+        <v>244469.31999999995</v>
       </c>
       <c r="E74" s="105">
-        <v>246192.57999999996</v>
+        <v>247487.6</v>
       </c>
       <c r="F74" s="106" t="s">
         <v>128</v>
       </c>
       <c r="G74" s="107">
-        <v>0.5004352413621908</v>
+        <v>0.5030676263279313</v>
       </c>
       <c r="H74" s="108" t="s">
         <v>129</v>
       </c>
       <c r="I74" s="109">
-        <v>0.35767355401769724</v>
+        <v>0.3603059389834378</v>
       </c>
       <c r="J74" s="36"/>
       <c r="K74" s="36"/>
@@ -31475,10 +31475,10 @@
         <v>363.57</v>
       </c>
       <c r="D6" s="54">
-        <v>304.75</v>
+        <v>331.25</v>
       </c>
       <c r="E6" s="54">
-        <v>58.81999999999999</v>
+        <v>32.31999999999999</v>
       </c>
       <c r="F6" s="54"/>
       <c r="G6" s="54"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-28T19:16:17Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -12460,54 +12460,54 @@
         <v>328046.93216</v>
       </c>
       <c r="I37" s="52">
-        <v>278838.99</v>
+        <v>279095.37</v>
       </c>
       <c r="J37" s="52">
         <v>271925.57216000004</v>
       </c>
       <c r="K37" s="52">
-        <v>243603.25999999998</v>
+        <v>243619.32</v>
       </c>
       <c r="L37" s="52">
-        <v>28322.31216000006</v>
+        <v>28306.252160000033</v>
       </c>
       <c r="M37" s="53">
-        <v>0.1041546476671025</v>
+        <v>0.10409558738868713</v>
       </c>
       <c r="N37" s="53"/>
       <c r="O37" s="52">
         <v>56121.36</v>
       </c>
       <c r="P37" s="52">
-        <v>35235.73</v>
+        <v>35476.05</v>
       </c>
       <c r="Q37" s="52">
-        <v>20885.629999999997</v>
+        <v>20645.309999999998</v>
       </c>
       <c r="R37" s="53">
-        <v>0.37215117381332163</v>
+        <v>0.367869025269523</v>
       </c>
       <c r="S37" s="54">
         <v>1124.47</v>
       </c>
       <c r="T37" s="54">
-        <v>813.5</v>
+        <v>821.5</v>
       </c>
       <c r="U37" s="54">
-        <v>310.97</v>
+        <v>302.97</v>
       </c>
       <c r="V37" s="53">
-        <v>0.2765480626428451</v>
+        <v>0.2694335998292529</v>
       </c>
       <c r="W37" s="53"/>
       <c r="X37" s="55">
-        <v>90.70043023970499</v>
+        <v>89.50507608034084</v>
       </c>
       <c r="Y37" s="55">
         <v>61.532703026350184</v>
       </c>
       <c r="Z37" s="53">
-        <v>0.20920000000000002</v>
+        <v>0.20850000000000002</v>
       </c>
       <c r="AA37" s="56">
         <v>0.1742</v>
@@ -28993,16 +28993,16 @@
         <v>93276.07999999999</v>
       </c>
       <c r="D12" s="52">
-        <v>62494.389999999985</v>
+        <v>62750.76999999999</v>
       </c>
       <c r="E12" s="52">
-        <v>30781.690000000002</v>
+        <v>30525.309999999998</v>
       </c>
       <c r="F12" s="52">
         <v>3</v>
       </c>
       <c r="G12" s="53">
-        <v>0.3300384192817709</v>
+        <v>0.327289804631584</v>
       </c>
       <c r="H12" s="53">
         <v>0.176316261575212</v>
@@ -29017,16 +29017,16 @@
         <v>2640</v>
       </c>
       <c r="L12" s="53">
-        <v>0.3017353430804554</v>
+        <v>0.2989867284302685</v>
       </c>
       <c r="M12" s="52">
-        <v>28144.690000000002</v>
+        <v>27888.309999999998</v>
       </c>
       <c r="N12" s="54">
         <v>53</v>
       </c>
       <c r="O12" s="58">
-        <v>407.89405797101455</v>
+        <v>404.1784057971014</v>
       </c>
       <c r="Q12" s="35" t="s">
         <v>123</v>
@@ -30846,22 +30846,22 @@
         <v>491956.92</v>
       </c>
       <c r="D74" s="104">
-        <v>244469.31999999995</v>
+        <v>244725.69999999995</v>
       </c>
       <c r="E74" s="105">
-        <v>247487.6</v>
+        <v>247231.22</v>
       </c>
       <c r="F74" s="106" t="s">
         <v>128</v>
       </c>
       <c r="G74" s="107">
-        <v>0.5030676263279313</v>
+        <v>0.5025464831351494</v>
       </c>
       <c r="H74" s="108" t="s">
         <v>129</v>
       </c>
       <c r="I74" s="109">
-        <v>0.3603059389834378</v>
+        <v>0.3597847957906558</v>
       </c>
       <c r="J74" s="36"/>
       <c r="K74" s="36"/>
@@ -31642,10 +31642,10 @@
         <v>1124.47</v>
       </c>
       <c r="D12" s="54">
-        <v>813.5</v>
+        <v>821.5</v>
       </c>
       <c r="E12" s="54">
-        <v>310.97</v>
+        <v>302.97</v>
       </c>
       <c r="F12" s="54"/>
       <c r="G12" s="54"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-28T19:22:55Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21298,72 +21298,72 @@
         <v>104</v>
       </c>
       <c r="D163" s="52">
-        <v>17899.333054</v>
+        <v>19505.5188968</v>
       </c>
       <c r="E163" s="52">
-        <v>13424.5</v>
+        <v>19505.52</v>
       </c>
       <c r="F163" s="52">
-        <v>4474.833053999999</v>
+        <v>-0.0011032000002160203</v>
       </c>
       <c r="G163" s="53">
-        <v>0.24999998829565323</v>
+        <v>-5.655835182098165e-8</v>
       </c>
       <c r="H163" s="52">
-        <v>13919.4012884</v>
+        <v>14923.5903884</v>
       </c>
       <c r="I163" s="52">
         <v>14052.73</v>
       </c>
       <c r="J163" s="52">
-        <v>8410.9272884</v>
+        <v>8915.0763884</v>
       </c>
       <c r="K163" s="52">
         <v>8190.78</v>
       </c>
       <c r="L163" s="52">
-        <v>220.14728840000043</v>
+        <v>724.296388400001</v>
       </c>
       <c r="M163" s="53">
-        <v>0.02617396166337312</v>
+        <v>0.08124399128452015</v>
       </c>
       <c r="N163" s="53"/>
       <c r="O163" s="52">
-        <v>5508.474</v>
+        <v>6008.514</v>
       </c>
       <c r="P163" s="52">
         <v>5861.95</v>
       </c>
       <c r="Q163" s="52">
-        <v>-353.47599999999966</v>
+        <v>146.5640000000003</v>
       </c>
       <c r="R163" s="53">
-        <v>-0.06416949594388567</v>
+        <v>0.02439272006356319</v>
       </c>
       <c r="S163" s="54">
-        <v>110.44</v>
+        <v>120.44</v>
       </c>
       <c r="T163" s="54">
         <v>116.25</v>
       </c>
       <c r="U163" s="54">
-        <v>-5.810000000000002</v>
+        <v>4.189999999999998</v>
       </c>
       <c r="V163" s="53">
-        <v>-0.05260775081492215</v>
+        <v>0.03478910660909995</v>
       </c>
       <c r="W163" s="53"/>
       <c r="X163" s="55">
-        <v>-5.404129032258065</v>
+        <v>46.90572043010753</v>
       </c>
       <c r="Y163" s="55">
-        <v>36.03704967040926</v>
+        <v>38.04324566921289</v>
       </c>
       <c r="Z163" s="53">
-        <v>-0.046799999999999994</v>
+        <v>0.2796</v>
       </c>
       <c r="AA163" s="56">
-        <v>0.2224</v>
+        <v>0.2349</v>
       </c>
       <c r="AB163" s="57"/>
       <c r="AD163" s="35"/>
@@ -25588,19 +25588,19 @@
         <v>306356.278672</v>
       </c>
       <c r="I226" s="52">
-        <v>253305.89</v>
+        <v>252680.7</v>
       </c>
       <c r="J226" s="52">
         <v>186357.488872</v>
       </c>
       <c r="K226" s="52">
-        <v>181341.87</v>
+        <v>180716.68</v>
       </c>
       <c r="L226" s="52">
-        <v>5015.618871999992</v>
+        <v>5640.808871999994</v>
       </c>
       <c r="M226" s="53">
-        <v>0.026913964672731664</v>
+        <v>0.03026875338438583</v>
       </c>
       <c r="N226" s="53"/>
       <c r="O226" s="52">
@@ -25629,13 +25629,13 @@
       </c>
       <c r="W226" s="53"/>
       <c r="X226" s="55">
-        <v>65.34323402260534</v>
+        <v>65.75027996249804</v>
       </c>
       <c r="Y226" s="55">
         <v>43.91570973337064</v>
       </c>
       <c r="Z226" s="53">
-        <v>0.2838</v>
+        <v>0.28550000000000003</v>
       </c>
       <c r="AA226" s="56">
         <v>0.257</v>
@@ -30080,17 +30080,17 @@
         <v>54</v>
       </c>
       <c r="C48" s="99">
-        <v>0</v>
+        <v>6081.02</v>
       </c>
       <c r="D48" s="99">
         <v>3650.3599999999988</v>
       </c>
       <c r="E48" s="99">
-        <v>-3650.3599999999988</v>
+        <v>2430.6600000000017</v>
       </c>
       <c r="F48" s="99"/>
       <c r="G48" s="100">
-        <v>0</v>
+        <v>0.39971254822381797</v>
       </c>
       <c r="H48" s="100">
         <v>0.222350780727547</v>
@@ -30103,16 +30103,16 @@
         <v>2530</v>
       </c>
       <c r="L48" s="100">
-        <v>0</v>
+        <v>-0.0163360751979106</v>
       </c>
       <c r="M48" s="99">
-        <v>-6180.359999999999</v>
+        <v>-99.33999999999833</v>
       </c>
       <c r="N48" s="98">
         <v>-44.75</v>
       </c>
       <c r="O48" s="60">
-        <v>138.10860335195528</v>
+        <v>2.2198882681563874</v>
       </c>
     </row>
     <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -30572,14 +30572,14 @@
         <v>82279.71999999997</v>
       </c>
       <c r="D66" s="99">
-        <v>18983.080000000016</v>
+        <v>18357.890000000014</v>
       </c>
       <c r="E66" s="99">
-        <v>63296.639999999956</v>
+        <v>63921.82999999996</v>
       </c>
       <c r="F66" s="99"/>
       <c r="G66" s="100">
-        <v>0.7692860403511337</v>
+        <v>0.7768843890086158</v>
       </c>
       <c r="H66" s="100">
         <v>0.256265521519856</v>
@@ -30594,16 +30594,16 @@
         <v>3200</v>
       </c>
       <c r="L66" s="100">
-        <v>0.7303943183083265</v>
+        <v>0.7379926669658086</v>
       </c>
       <c r="M66" s="99">
-        <v>60096.639999999956</v>
+        <v>60721.82999999996</v>
       </c>
       <c r="N66" s="98">
         <v>-1014.25</v>
       </c>
       <c r="O66" s="60">
-        <v>-64.3260797431094</v>
+        <v>-64.99526893229859</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -30843,25 +30843,25 @@
         <v>127</v>
       </c>
       <c r="C74" s="104">
-        <v>491956.92</v>
+        <v>498037.94</v>
       </c>
       <c r="D74" s="104">
-        <v>244725.69999999995</v>
+        <v>244100.50999999995</v>
       </c>
       <c r="E74" s="105">
-        <v>247231.22</v>
+        <v>253937.43</v>
       </c>
       <c r="F74" s="106" t="s">
         <v>128</v>
       </c>
       <c r="G74" s="107">
-        <v>0.5025464831351494</v>
+        <v>0.5098756733272167</v>
       </c>
       <c r="H74" s="108" t="s">
         <v>129</v>
       </c>
       <c r="I74" s="109">
-        <v>0.3597847957906558</v>
+        <v>0.3688570995213738</v>
       </c>
       <c r="J74" s="36"/>
       <c r="K74" s="36"/>
@@ -32604,13 +32604,13 @@
         <v>54</v>
       </c>
       <c r="C48" s="54">
-        <v>110.44</v>
+        <v>120.44</v>
       </c>
       <c r="D48" s="54">
         <v>116.25</v>
       </c>
       <c r="E48" s="54">
-        <v>-5.810000000000002</v>
+        <v>4.189999999999998</v>
       </c>
       <c r="F48" s="54"/>
       <c r="G48" s="54"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-28T19:42:31Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -12999,19 +12999,19 @@
         <v>94098.31685</v>
       </c>
       <c r="I44" s="52">
-        <v>57104.57</v>
+        <v>58294.37</v>
       </c>
       <c r="J44" s="52">
         <v>69042.08885</v>
       </c>
       <c r="K44" s="52">
-        <v>40878.83</v>
+        <v>42068.630000000005</v>
       </c>
       <c r="L44" s="52">
-        <v>28163.25885</v>
+        <v>26973.458849999995</v>
       </c>
       <c r="M44" s="53">
-        <v>0.40791435078372484</v>
+        <v>0.39068138434516664</v>
       </c>
       <c r="N44" s="53"/>
       <c r="O44" s="52">
@@ -13040,13 +13040,13 @@
       </c>
       <c r="W44" s="53"/>
       <c r="X44" s="55">
-        <v>158.93509897610923</v>
+        <v>155.68649829351537</v>
       </c>
       <c r="Y44" s="55">
         <v>68.07122423898531</v>
       </c>
       <c r="Z44" s="53">
-        <v>0.5047999999999999</v>
+        <v>0.49450000000000005</v>
       </c>
       <c r="AA44" s="56">
         <v>0.2663</v>
@@ -14079,19 +14079,19 @@
         <v>109364.9721</v>
       </c>
       <c r="I58" s="52">
-        <v>113859.52</v>
+        <v>114553.44</v>
       </c>
       <c r="J58" s="52">
         <v>75135.0159</v>
       </c>
       <c r="K58" s="52">
-        <v>80491.32</v>
+        <v>81185.24</v>
       </c>
       <c r="L58" s="52">
-        <v>-5356.3041000000085</v>
+        <v>-6050.224100000007</v>
       </c>
       <c r="M58" s="53">
-        <v>-0.07128905259205527</v>
+        <v>-0.08052469314776584</v>
       </c>
       <c r="N58" s="53"/>
       <c r="O58" s="52">
@@ -14120,13 +14120,13 @@
       </c>
       <c r="W58" s="53"/>
       <c r="X58" s="55">
-        <v>59.2172633083244</v>
+        <v>58.22559485530547</v>
       </c>
       <c r="Y58" s="55">
         <v>67.00679527854935</v>
       </c>
       <c r="Z58" s="53">
-        <v>0.2668</v>
+        <v>0.26239999999999997</v>
       </c>
       <c r="AA58" s="56">
         <v>0.2958</v>
@@ -15019,54 +15019,54 @@
         <v>39055.77825</v>
       </c>
       <c r="I72" s="52">
-        <v>24880.27</v>
+        <v>30684.03</v>
       </c>
       <c r="J72" s="52">
         <v>29537.289750000004</v>
       </c>
       <c r="K72" s="52">
-        <v>20998.84</v>
+        <v>26364.309999999998</v>
       </c>
       <c r="L72" s="52">
-        <v>8538.449750000003</v>
+        <v>3172.979750000006</v>
       </c>
       <c r="M72" s="53">
-        <v>0.28907356843733445</v>
+        <v>0.10742284674239638</v>
       </c>
       <c r="N72" s="53"/>
       <c r="O72" s="52">
         <v>9518.4885</v>
       </c>
       <c r="P72" s="52">
-        <v>3881.43</v>
+        <v>4319.72</v>
       </c>
       <c r="Q72" s="52">
-        <v>5637.058499999999</v>
+        <v>5198.768499999999</v>
       </c>
       <c r="R72" s="53">
-        <v>0.5922220213850129</v>
+        <v>0.5461758450409432</v>
       </c>
       <c r="S72" s="54">
         <v>193.32</v>
       </c>
       <c r="T72" s="54">
-        <v>83.5</v>
+        <v>90.75</v>
       </c>
       <c r="U72" s="54">
-        <v>109.82</v>
+        <v>102.57</v>
       </c>
       <c r="V72" s="53">
-        <v>0.5680736602524312</v>
+        <v>0.5305710738671633</v>
       </c>
       <c r="W72" s="53"/>
       <c r="X72" s="55">
-        <v>57.90898203592814</v>
+        <v>-10.670633608815427</v>
       </c>
       <c r="Y72" s="55">
         <v>72.28396616733912</v>
       </c>
       <c r="Z72" s="53">
-        <v>0.16269999999999998</v>
+        <v>-0.0326</v>
       </c>
       <c r="AA72" s="56">
         <v>0.2635</v>
@@ -15548,54 +15548,54 @@
         <v>55589.7822</v>
       </c>
       <c r="I79" s="52">
-        <v>44814.24</v>
+        <v>47207.1</v>
       </c>
       <c r="J79" s="52">
         <v>32594.7534</v>
       </c>
       <c r="K79" s="52">
-        <v>34770.899999999994</v>
+        <v>35050.6</v>
       </c>
       <c r="L79" s="52">
-        <v>-2176.1465999999928</v>
+        <v>-2455.846599999997</v>
       </c>
       <c r="M79" s="53">
-        <v>-0.06676370805124707</v>
+        <v>-0.07534484368886181</v>
       </c>
       <c r="N79" s="53"/>
       <c r="O79" s="52">
         <v>22995.0288</v>
       </c>
       <c r="P79" s="52">
-        <v>10043.34</v>
+        <v>12156.5</v>
       </c>
       <c r="Q79" s="52">
-        <v>12951.6888</v>
+        <v>10838.5288</v>
       </c>
       <c r="R79" s="53">
-        <v>0.563238642258191</v>
+        <v>0.4713422581145017</v>
       </c>
       <c r="S79" s="54">
         <v>472.14</v>
       </c>
       <c r="T79" s="54">
-        <v>202</v>
+        <v>237.25</v>
       </c>
       <c r="U79" s="54">
-        <v>270.14</v>
+        <v>234.89</v>
       </c>
       <c r="V79" s="53">
-        <v>0.5721607997627822</v>
+        <v>0.49750074130554495</v>
       </c>
       <c r="W79" s="53"/>
       <c r="X79" s="55">
-        <v>83.91376237623763</v>
+        <v>61.36025289778714</v>
       </c>
       <c r="Y79" s="55">
         <v>49.060202993773025</v>
       </c>
       <c r="Z79" s="53">
-        <v>0.27440000000000003</v>
+        <v>0.2357</v>
       </c>
       <c r="AA79" s="56">
         <v>0.2941</v>
@@ -21828,19 +21828,19 @@
         <v>7687.765097</v>
       </c>
       <c r="I170" s="52">
-        <v>2116.21</v>
+        <v>2097.39</v>
       </c>
       <c r="J170" s="52">
         <v>4437.133697</v>
       </c>
       <c r="K170" s="52">
-        <v>1029.51</v>
+        <v>1010.6899999999998</v>
       </c>
       <c r="L170" s="52">
-        <v>3407.623697</v>
+        <v>3426.4436970000006</v>
       </c>
       <c r="M170" s="53">
-        <v>0.7679785937719064</v>
+        <v>0.7722200706543192</v>
       </c>
       <c r="N170" s="53"/>
       <c r="O170" s="52">
@@ -21869,13 +21869,13 @@
       </c>
       <c r="W170" s="53"/>
       <c r="X170" s="55">
-        <v>-86.97944923962187</v>
+        <v>53.18249075215784</v>
       </c>
       <c r="Y170" s="55">
         <v>48.202633430830645</v>
       </c>
       <c r="Z170" s="53">
-        <v>0</v>
+        <v>0.3815</v>
       </c>
       <c r="AA170" s="56">
         <v>0.29</v>
@@ -22882,66 +22882,66 @@
         <v>16897.52982004</v>
       </c>
       <c r="E184" s="52">
-        <v>5491.7</v>
+        <v>9293.64</v>
       </c>
       <c r="F184" s="52">
-        <v>11405.829820039999</v>
+        <v>7603.88982004</v>
       </c>
       <c r="G184" s="53">
-        <v>0.6749998337930436</v>
+        <v>0.450000082912829</v>
       </c>
       <c r="H184" s="52">
         <v>9226.2731</v>
       </c>
       <c r="I184" s="52">
-        <v>5812.29</v>
+        <v>6976.46</v>
       </c>
       <c r="J184" s="52">
         <v>2977.1135000000004</v>
       </c>
       <c r="K184" s="52">
-        <v>2773.14</v>
+        <v>3448.13</v>
       </c>
       <c r="L184" s="52">
-        <v>203.9735000000005</v>
+        <v>-471.0164999999997</v>
       </c>
       <c r="M184" s="53">
-        <v>0.0685138473894262</v>
+        <v>-0.15821247661535232</v>
       </c>
       <c r="N184" s="53"/>
       <c r="O184" s="52">
         <v>6249.1596</v>
       </c>
       <c r="P184" s="52">
-        <v>3039.15</v>
+        <v>3528.33</v>
       </c>
       <c r="Q184" s="52">
-        <v>3210.0096</v>
+        <v>2720.8296</v>
       </c>
       <c r="R184" s="53">
-        <v>0.5136706062043926</v>
+        <v>0.43539128045313485</v>
       </c>
       <c r="S184" s="54">
         <v>125.17</v>
       </c>
       <c r="T184" s="54">
-        <v>57.25</v>
+        <v>65.75</v>
       </c>
       <c r="U184" s="54">
-        <v>67.92</v>
+        <v>59.42</v>
       </c>
       <c r="V184" s="53">
-        <v>0.5426220340337141</v>
+        <v>0.47471438843173286</v>
       </c>
       <c r="W184" s="53"/>
       <c r="X184" s="55">
-        <v>-5.599825327510916</v>
+        <v>35.24228136882129</v>
       </c>
       <c r="Y184" s="55">
         <v>61.286703843093385</v>
       </c>
       <c r="Z184" s="53">
-        <v>-0.0584</v>
+        <v>0.2493</v>
       </c>
       <c r="AA184" s="56">
         <v>0.454</v>
@@ -26107,7 +26107,7 @@
         <v>6369.1218</v>
       </c>
       <c r="I233" s="52">
-        <v>239.55</v>
+        <v>584.85</v>
       </c>
       <c r="J233" s="52">
         <v>4527.894</v>
@@ -26126,35 +26126,35 @@
         <v>1841.2278</v>
       </c>
       <c r="P233" s="52">
-        <v>0</v>
+        <v>345.3</v>
       </c>
       <c r="Q233" s="52">
-        <v>1841.2278</v>
+        <v>1495.9278</v>
       </c>
       <c r="R233" s="53">
-        <v>1</v>
+        <v>0.8124620973026804</v>
       </c>
       <c r="S233" s="54">
         <v>36.92</v>
       </c>
       <c r="T233" s="54">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U233" s="54">
-        <v>36.92</v>
+        <v>30.92</v>
       </c>
       <c r="V233" s="53">
-        <v>1</v>
+        <v>0.8374864572047671</v>
       </c>
       <c r="W233" s="53"/>
       <c r="X233" s="55">
-        <v>0</v>
+        <v>192.5583333333333</v>
       </c>
       <c r="Y233" s="55">
         <v>65.70711175027087</v>
       </c>
       <c r="Z233" s="53">
-        <v>0.8623000000000001</v>
+        <v>0.6639</v>
       </c>
       <c r="AA233" s="56">
         <v>0.2758</v>
@@ -29060,16 +29060,16 @@
         <v>61369.72</v>
       </c>
       <c r="D14" s="52">
-        <v>14830.879999999997</v>
+        <v>16020.68</v>
       </c>
       <c r="E14" s="52">
-        <v>46538.840000000004</v>
+        <v>45349.04</v>
       </c>
       <c r="F14" s="52">
         <v>0</v>
       </c>
       <c r="G14" s="53">
-        <v>0.7583355439783659</v>
+        <v>0.738948132727345</v>
       </c>
       <c r="H14" s="53">
         <v>0.266338527271097</v>
@@ -29084,16 +29084,16 @@
         <v>3000</v>
       </c>
       <c r="L14" s="53">
-        <v>0.7094515014896597</v>
+        <v>0.6900640902386389</v>
       </c>
       <c r="M14" s="52">
-        <v>43538.840000000004</v>
+        <v>42349.04</v>
       </c>
       <c r="N14" s="54">
         <v>-112</v>
       </c>
       <c r="O14" s="58">
-        <v>-388.7396428571429</v>
+        <v>-378.11642857142857</v>
       </c>
     </row>
     <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -29186,16 +29186,16 @@
         <v>27482.319999999992</v>
       </c>
       <c r="D18" s="52">
-        <v>18539.01000000001</v>
+        <v>19232.930000000008</v>
       </c>
       <c r="E18" s="52">
-        <v>8943.309999999983</v>
+        <v>8249.389999999985</v>
       </c>
       <c r="F18" s="52">
         <v>0</v>
       </c>
       <c r="G18" s="53">
-        <v>0.32542048851770833</v>
+        <v>0.30017080071842506</v>
       </c>
       <c r="H18" s="53">
         <v>0.296537658865514</v>
@@ -29210,16 +29210,16 @@
         <v>8200</v>
       </c>
       <c r="L18" s="53">
-        <v>0.027046843206832004</v>
+        <v>0.0017971554075487397</v>
       </c>
       <c r="M18" s="52">
-        <v>743.3099999999831</v>
+        <v>49.389999999984866</v>
       </c>
       <c r="N18" s="54">
         <v>-269</v>
       </c>
       <c r="O18" s="58">
-        <v>-3.9328571428570536</v>
+        <v>-0.26132275132267124</v>
       </c>
       <c r="Q18" s="35" t="s">
         <v>124</v>
@@ -29309,16 +29309,16 @@
         <v>19065.239999999998</v>
       </c>
       <c r="D22" s="52">
-        <v>14898.84</v>
+        <v>20702.6</v>
       </c>
       <c r="E22" s="52">
-        <v>4166.399999999998</v>
+        <v>-1637.3600000000006</v>
       </c>
       <c r="F22" s="52">
         <v>3</v>
       </c>
       <c r="G22" s="53">
-        <v>0.21869118878125837</v>
+        <v>-0.08572459617607756</v>
       </c>
       <c r="H22" s="53">
         <v>0.252488256827238</v>
@@ -29329,10 +29329,10 @@
         <v>0</v>
       </c>
       <c r="L22" s="53">
-        <v>0.21869118878125837</v>
+        <v>-0.08572459617607756</v>
       </c>
       <c r="M22" s="52">
-        <v>4169.399999999998</v>
+        <v>-1634.3600000000006</v>
       </c>
       <c r="N22" s="54"/>
       <c r="O22" s="58">
@@ -29367,16 +29367,16 @@
         <v>16999.83</v>
       </c>
       <c r="D24" s="52">
-        <v>12895.309999999998</v>
+        <v>15288.169999999998</v>
       </c>
       <c r="E24" s="52">
-        <v>4104.520000000004</v>
+        <v>1711.6600000000035</v>
       </c>
       <c r="F24" s="52">
         <v>3</v>
       </c>
       <c r="G24" s="53">
-        <v>0.2416212397418094</v>
+        <v>0.1008633615747924</v>
       </c>
       <c r="H24" s="53"/>
       <c r="I24" s="54"/>
@@ -29385,10 +29385,10 @@
         <v>0</v>
       </c>
       <c r="L24" s="53">
-        <v>0.2416212397418094</v>
+        <v>0.1008633615747924</v>
       </c>
       <c r="M24" s="52">
-        <v>4107.520000000004</v>
+        <v>1714.6600000000035</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="58">
@@ -30143,10 +30143,10 @@
         <v>0</v>
       </c>
       <c r="D50" s="99">
-        <v>2116.21</v>
+        <v>2097.39</v>
       </c>
       <c r="E50" s="99">
-        <v>-2116.21</v>
+        <v>-2097.39</v>
       </c>
       <c r="F50" s="99"/>
       <c r="G50" s="100">
@@ -30164,7 +30164,7 @@
         <v>0</v>
       </c>
       <c r="M50" s="99">
-        <v>-2116.21</v>
+        <v>-2097.39</v>
       </c>
       <c r="N50" s="98"/>
       <c r="O50" s="60">
@@ -30261,17 +30261,17 @@
         <v>57</v>
       </c>
       <c r="C54" s="99">
-        <v>0</v>
+        <v>3801.9399999999996</v>
       </c>
       <c r="D54" s="99">
-        <v>2109.5099999999998</v>
+        <v>3273.68</v>
       </c>
       <c r="E54" s="99">
-        <v>-2109.5099999999998</v>
+        <v>528.2599999999998</v>
       </c>
       <c r="F54" s="99"/>
       <c r="G54" s="100">
-        <v>0</v>
+        <v>0.13894485446903418</v>
       </c>
       <c r="H54" s="100">
         <v>0.453987062014389</v>
@@ -30286,16 +30286,16 @@
         <v>640</v>
       </c>
       <c r="L54" s="100">
-        <v>0</v>
+        <v>-0.029390258657422327</v>
       </c>
       <c r="M54" s="99">
-        <v>-2749.5099999999998</v>
+        <v>-111.74000000000024</v>
       </c>
       <c r="N54" s="98">
         <v>-11.25</v>
       </c>
       <c r="O54" s="60">
-        <v>-578.8442105263157</v>
+        <v>-23.52421052631584</v>
       </c>
     </row>
     <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -30773,14 +30773,14 @@
         <v>1740.2</v>
       </c>
       <c r="D71" s="99">
-        <v>239.55</v>
+        <v>584.85</v>
       </c>
       <c r="E71" s="99">
-        <v>1500.65</v>
+        <v>1155.35</v>
       </c>
       <c r="F71" s="99"/>
       <c r="G71" s="100">
-        <v>0.8623434088035858</v>
+        <v>0.663917940466613</v>
       </c>
       <c r="H71" s="100">
         <f>'Deliverables Sheet'!AA228</f>
@@ -30791,10 +30791,10 @@
         <v>0</v>
       </c>
       <c r="L71" s="100">
-        <v>0.8623434088035858</v>
+        <v>0.663917940466613</v>
       </c>
       <c r="M71" s="99">
-        <v>1500.65</v>
+        <v>1155.35</v>
       </c>
       <c r="N71" s="98"/>
       <c r="O71" s="60">
@@ -30843,25 +30843,25 @@
         <v>127</v>
       </c>
       <c r="C74" s="104">
-        <v>498037.94</v>
+        <v>501839.88</v>
       </c>
       <c r="D74" s="104">
-        <v>244100.50999999995</v>
+        <v>255671.49999999997</v>
       </c>
       <c r="E74" s="105">
-        <v>253937.43</v>
+        <v>246168.37999999998</v>
       </c>
       <c r="F74" s="106" t="s">
         <v>128</v>
       </c>
       <c r="G74" s="107">
-        <v>0.5098756733272167</v>
+        <v>0.49053172099435377</v>
       </c>
       <c r="H74" s="108" t="s">
         <v>129</v>
       </c>
       <c r="I74" s="109">
-        <v>0.3688570995213738</v>
+        <v>0.3505815042040899</v>
       </c>
       <c r="J74" s="36"/>
       <c r="K74" s="36"/>
@@ -31914,10 +31914,10 @@
         <v>193.32</v>
       </c>
       <c r="D22" s="54">
-        <v>83.5</v>
+        <v>90.75</v>
       </c>
       <c r="E22" s="54">
-        <v>109.82</v>
+        <v>102.57</v>
       </c>
       <c r="F22" s="54"/>
       <c r="G22" s="54"/>
@@ -31970,10 +31970,10 @@
         <v>472.14</v>
       </c>
       <c r="D24" s="54">
-        <v>202</v>
+        <v>237.25</v>
       </c>
       <c r="E24" s="54">
-        <v>270.14</v>
+        <v>234.89</v>
       </c>
       <c r="F24" s="54"/>
       <c r="G24" s="54"/>
@@ -32770,10 +32770,10 @@
         <v>125.17</v>
       </c>
       <c r="D54" s="54">
-        <v>57.25</v>
+        <v>65.75</v>
       </c>
       <c r="E54" s="54">
-        <v>67.92</v>
+        <v>59.42</v>
       </c>
       <c r="F54" s="54"/>
       <c r="G54" s="54"/>
@@ -33251,10 +33251,10 @@
         <v>36.92</v>
       </c>
       <c r="D71" s="54">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E71" s="54">
-        <v>36.92</v>
+        <v>30.92</v>
       </c>
       <c r="F71" s="54"/>
       <c r="G71" s="54"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-29T19:23:44Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -12460,19 +12460,19 @@
         <v>328046.93216</v>
       </c>
       <c r="I37" s="52">
-        <v>279095.37</v>
+        <v>278861.56</v>
       </c>
       <c r="J37" s="52">
         <v>271925.57216000004</v>
       </c>
       <c r="K37" s="52">
-        <v>243619.32</v>
+        <v>243385.51</v>
       </c>
       <c r="L37" s="52">
-        <v>28306.252160000033</v>
+        <v>28540.06216000003</v>
       </c>
       <c r="M37" s="53">
-        <v>0.10409558738868713</v>
+        <v>0.10495541825395943</v>
       </c>
       <c r="N37" s="53"/>
       <c r="O37" s="52">
@@ -12501,13 +12501,13 @@
       </c>
       <c r="W37" s="53"/>
       <c r="X37" s="55">
-        <v>89.50507608034084</v>
+        <v>89.78968959220937</v>
       </c>
       <c r="Y37" s="55">
         <v>61.532703026350184</v>
       </c>
       <c r="Z37" s="53">
-        <v>0.20850000000000002</v>
+        <v>0.20920000000000002</v>
       </c>
       <c r="AA37" s="56">
         <v>0.1742</v>
@@ -12999,7 +12999,7 @@
         <v>94098.31685</v>
       </c>
       <c r="I44" s="52">
-        <v>58294.37</v>
+        <v>58609.37</v>
       </c>
       <c r="J44" s="52">
         <v>69042.08885</v>
@@ -13018,35 +13018,35 @@
         <v>25056.228</v>
       </c>
       <c r="P44" s="52">
-        <v>16225.74</v>
+        <v>16540.74</v>
       </c>
       <c r="Q44" s="52">
-        <v>8830.488</v>
+        <v>8515.487999999998</v>
       </c>
       <c r="R44" s="53">
-        <v>0.3524268696788678</v>
+        <v>0.3398551449962859</v>
       </c>
       <c r="S44" s="54">
         <v>501.83</v>
       </c>
       <c r="T44" s="54">
-        <v>366.25</v>
+        <v>373.25</v>
       </c>
       <c r="U44" s="54">
-        <v>135.57999999999998</v>
+        <v>128.57999999999998</v>
       </c>
       <c r="V44" s="53">
-        <v>0.2701711735049718</v>
+        <v>0.2562222266504593</v>
       </c>
       <c r="W44" s="53"/>
       <c r="X44" s="55">
-        <v>155.68649829351537</v>
+        <v>151.92278633623576</v>
       </c>
       <c r="Y44" s="55">
         <v>68.07122423898531</v>
       </c>
       <c r="Z44" s="53">
-        <v>0.49450000000000005</v>
+        <v>0.4917</v>
       </c>
       <c r="AA44" s="56">
         <v>0.2663</v>
@@ -14079,54 +14079,54 @@
         <v>109364.9721</v>
       </c>
       <c r="I58" s="52">
-        <v>114553.44</v>
+        <v>115053.73</v>
       </c>
       <c r="J58" s="52">
         <v>75135.0159</v>
       </c>
       <c r="K58" s="52">
-        <v>81185.24</v>
+        <v>81019.67</v>
       </c>
       <c r="L58" s="52">
-        <v>-6050.224100000007</v>
+        <v>-5884.6541</v>
       </c>
       <c r="M58" s="53">
-        <v>-0.08052469314776584</v>
+        <v>-0.07832106015432413</v>
       </c>
       <c r="N58" s="53"/>
       <c r="O58" s="52">
         <v>34229.9562</v>
       </c>
       <c r="P58" s="52">
-        <v>33368.2</v>
+        <v>34034.06</v>
       </c>
       <c r="Q58" s="52">
-        <v>861.7562000000034</v>
+        <v>195.89620000000286</v>
       </c>
       <c r="R58" s="53">
-        <v>0.025175498179574166</v>
+        <v>0.005722946265411899</v>
       </c>
       <c r="S58" s="54">
         <v>685.48</v>
       </c>
       <c r="T58" s="54">
-        <v>699.75</v>
+        <v>718.75</v>
       </c>
       <c r="U58" s="54">
-        <v>-14.269999999999982</v>
+        <v>-33.26999999999998</v>
       </c>
       <c r="V58" s="53">
-        <v>-0.0208175293225185</v>
+        <v>-0.04853533290540932</v>
       </c>
       <c r="W58" s="53"/>
       <c r="X58" s="55">
-        <v>58.22559485530547</v>
+        <v>55.99035826086956</v>
       </c>
       <c r="Y58" s="55">
         <v>67.00679527854935</v>
       </c>
       <c r="Z58" s="53">
-        <v>0.26239999999999997</v>
+        <v>0.2591</v>
       </c>
       <c r="AA58" s="56">
         <v>0.2958</v>
@@ -15548,54 +15548,54 @@
         <v>55589.7822</v>
       </c>
       <c r="I79" s="52">
-        <v>47207.1</v>
+        <v>48815.57</v>
       </c>
       <c r="J79" s="52">
         <v>32594.7534</v>
       </c>
       <c r="K79" s="52">
-        <v>35050.6</v>
+        <v>35862.99</v>
       </c>
       <c r="L79" s="52">
-        <v>-2455.846599999997</v>
+        <v>-3268.2365999999965</v>
       </c>
       <c r="M79" s="53">
-        <v>-0.07534484368886181</v>
+        <v>-0.10026879356602209</v>
       </c>
       <c r="N79" s="53"/>
       <c r="O79" s="52">
         <v>22995.0288</v>
       </c>
       <c r="P79" s="52">
-        <v>12156.5</v>
+        <v>12952.58</v>
       </c>
       <c r="Q79" s="52">
-        <v>10838.5288</v>
+        <v>10042.4488</v>
       </c>
       <c r="R79" s="53">
-        <v>0.4713422581145017</v>
+        <v>0.43672260153899</v>
       </c>
       <c r="S79" s="54">
         <v>472.14</v>
       </c>
       <c r="T79" s="54">
-        <v>237.25</v>
+        <v>257.25</v>
       </c>
       <c r="U79" s="54">
-        <v>234.89</v>
+        <v>214.89</v>
       </c>
       <c r="V79" s="53">
-        <v>0.49750074130554495</v>
+        <v>0.4551404244503749</v>
       </c>
       <c r="W79" s="53"/>
       <c r="X79" s="55">
-        <v>61.36025289778714</v>
+        <v>50.33722060252673</v>
       </c>
       <c r="Y79" s="55">
         <v>49.060202993773025</v>
       </c>
       <c r="Z79" s="53">
-        <v>0.2357</v>
+        <v>0.2097</v>
       </c>
       <c r="AA79" s="56">
         <v>0.2941</v>
@@ -16068,34 +16068,34 @@
         <v>104</v>
       </c>
       <c r="D86" s="52">
-        <v>25467.8441072</v>
+        <v>26846.9041072</v>
       </c>
       <c r="E86" s="52">
-        <v>19598.41</v>
+        <v>20977.47</v>
       </c>
       <c r="F86" s="52">
         <v>5869.434107199999</v>
       </c>
       <c r="G86" s="53">
-        <v>0.23046450584879521</v>
+        <v>0.21862610615225056</v>
       </c>
       <c r="H86" s="52">
-        <v>16606.829916</v>
+        <v>17678.176816</v>
       </c>
       <c r="I86" s="52">
-        <v>14118.07</v>
+        <v>16373.33</v>
       </c>
       <c r="J86" s="52">
-        <v>9659.986716</v>
+        <v>10731.333616</v>
       </c>
       <c r="K86" s="52">
-        <v>5298.48</v>
+        <v>7553.74</v>
       </c>
       <c r="L86" s="52">
-        <v>4361.506716</v>
+        <v>3177.593616</v>
       </c>
       <c r="M86" s="53">
-        <v>0.4515023513206248</v>
+        <v>0.2961042615674842</v>
       </c>
       <c r="N86" s="53"/>
       <c r="O86" s="52">
@@ -16124,16 +16124,16 @@
       </c>
       <c r="W86" s="53"/>
       <c r="X86" s="55">
-        <v>32.669687034277196</v>
+        <v>27.446438152011925</v>
       </c>
       <c r="Y86" s="55">
-        <v>63.7162162306752</v>
+        <v>65.92886525634573</v>
       </c>
       <c r="Z86" s="53">
-        <v>0.2796</v>
+        <v>0.2195</v>
       </c>
       <c r="AA86" s="56">
-        <v>0.3479</v>
+        <v>0.3415</v>
       </c>
       <c r="AB86" s="57"/>
       <c r="AD86" s="35"/>
@@ -16607,72 +16607,72 @@
         <v>104</v>
       </c>
       <c r="D93" s="67">
-        <v>37083.0313712</v>
+        <v>37218.0313712</v>
       </c>
       <c r="E93" s="67">
         <v>36381.33</v>
       </c>
       <c r="F93" s="52">
-        <v>701.7013711999971</v>
+        <v>836.7013711999971</v>
       </c>
       <c r="G93" s="53">
-        <v>0.018922438248804095</v>
+        <v>0.022481075445797277</v>
       </c>
       <c r="H93" s="52">
-        <v>27002.93286</v>
+        <v>27090.14646</v>
       </c>
       <c r="I93" s="52">
         <v>25103.82</v>
       </c>
       <c r="J93" s="52">
-        <v>15440.324460000002</v>
+        <v>15515.12046</v>
       </c>
       <c r="K93" s="52">
         <v>13974.73</v>
       </c>
       <c r="L93" s="52">
-        <v>1465.594460000002</v>
+        <v>1540.3904600000005</v>
       </c>
       <c r="M93" s="53">
-        <v>0.0949199263135175</v>
+        <v>0.09928317759255094</v>
       </c>
       <c r="N93" s="53"/>
       <c r="O93" s="52">
-        <v>11562.6084</v>
+        <v>11575.026</v>
       </c>
       <c r="P93" s="52">
         <v>11129.09</v>
       </c>
       <c r="Q93" s="52">
-        <v>433.518399999999</v>
+        <v>445.9359999999997</v>
       </c>
       <c r="R93" s="53">
-        <v>0.03749313174006646</v>
+        <v>0.038525701799719474</v>
       </c>
       <c r="S93" s="68">
-        <v>231.75</v>
+        <v>232</v>
       </c>
       <c r="T93" s="68">
         <v>225.5</v>
       </c>
       <c r="U93" s="54">
-        <v>6.25</v>
+        <v>6.5</v>
       </c>
       <c r="V93" s="53">
-        <v>0.02696871628910464</v>
+        <v>0.028017241379310345</v>
       </c>
       <c r="W93" s="53"/>
       <c r="X93" s="55">
         <v>50.01113082039912</v>
       </c>
       <c r="Y93" s="55">
-        <v>43.49557070636461</v>
+        <v>43.65467634137931</v>
       </c>
       <c r="Z93" s="53">
         <v>0.31</v>
       </c>
       <c r="AA93" s="56">
-        <v>0.2718</v>
+        <v>0.2721</v>
       </c>
       <c r="AB93" s="57"/>
       <c r="AD93" s="35"/>
@@ -22357,19 +22357,19 @@
         <v>114651.8653946</v>
       </c>
       <c r="I177" s="52">
-        <v>105507.56</v>
+        <v>102580.79</v>
       </c>
       <c r="J177" s="52">
         <v>82888.0783946</v>
       </c>
       <c r="K177" s="52">
-        <v>77881.66</v>
+        <v>74954.88999999998</v>
       </c>
       <c r="L177" s="52">
-        <v>5006.418394599998</v>
+        <v>7933.188394600016</v>
       </c>
       <c r="M177" s="53">
-        <v>0.060399740126273166</v>
+        <v>0.095709643030123</v>
       </c>
       <c r="N177" s="53"/>
       <c r="O177" s="52">
@@ -22398,13 +22398,13 @@
       </c>
       <c r="W177" s="53"/>
       <c r="X177" s="55">
-        <v>36.093781207444394</v>
+        <v>41.407934634589196</v>
       </c>
       <c r="Y177" s="55">
         <v>47.87601261940491</v>
       </c>
       <c r="Z177" s="53">
-        <v>0.1585</v>
+        <v>0.1819</v>
       </c>
       <c r="AA177" s="56">
         <v>0.216</v>
@@ -28993,16 +28993,16 @@
         <v>93276.07999999999</v>
       </c>
       <c r="D12" s="52">
-        <v>62750.76999999999</v>
+        <v>62516.95999999999</v>
       </c>
       <c r="E12" s="52">
-        <v>30525.309999999998</v>
+        <v>30759.119999999995</v>
       </c>
       <c r="F12" s="52">
         <v>3</v>
       </c>
       <c r="G12" s="53">
-        <v>0.327289804631584</v>
+        <v>0.329796449421974</v>
       </c>
       <c r="H12" s="53">
         <v>0.176316261575212</v>
@@ -29017,16 +29017,16 @@
         <v>2640</v>
       </c>
       <c r="L12" s="53">
-        <v>0.2989867284302685</v>
+        <v>0.3014933732206585</v>
       </c>
       <c r="M12" s="52">
-        <v>27888.309999999998</v>
+        <v>28122.119999999995</v>
       </c>
       <c r="N12" s="54">
         <v>53</v>
       </c>
       <c r="O12" s="58">
-        <v>404.1784057971014</v>
+        <v>407.5669565217391</v>
       </c>
       <c r="Q12" s="35" t="s">
         <v>123</v>
@@ -29060,16 +29060,16 @@
         <v>61369.72</v>
       </c>
       <c r="D14" s="52">
-        <v>16020.68</v>
+        <v>16335.68</v>
       </c>
       <c r="E14" s="52">
-        <v>45349.04</v>
+        <v>45034.04</v>
       </c>
       <c r="F14" s="52">
         <v>0</v>
       </c>
       <c r="G14" s="53">
-        <v>0.738948132727345</v>
+        <v>0.7338153082660309</v>
       </c>
       <c r="H14" s="53">
         <v>0.266338527271097</v>
@@ -29084,16 +29084,16 @@
         <v>3000</v>
       </c>
       <c r="L14" s="53">
-        <v>0.6900640902386389</v>
+        <v>0.6849312657773247</v>
       </c>
       <c r="M14" s="52">
-        <v>42349.04</v>
+        <v>42034.04</v>
       </c>
       <c r="N14" s="54">
         <v>-112</v>
       </c>
       <c r="O14" s="58">
-        <v>-378.11642857142857</v>
+        <v>-375.30392857142857</v>
       </c>
     </row>
     <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -29186,16 +29186,16 @@
         <v>27482.319999999992</v>
       </c>
       <c r="D18" s="52">
-        <v>19232.930000000008</v>
+        <v>19733.22</v>
       </c>
       <c r="E18" s="52">
-        <v>8249.389999999985</v>
+        <v>7749.099999999991</v>
       </c>
       <c r="F18" s="52">
         <v>0</v>
       </c>
       <c r="G18" s="53">
-        <v>0.30017080071842506</v>
+        <v>0.2819667335217694</v>
       </c>
       <c r="H18" s="53">
         <v>0.296537658865514</v>
@@ -29210,16 +29210,16 @@
         <v>8200</v>
       </c>
       <c r="L18" s="53">
-        <v>0.0017971554075487397</v>
+        <v>-0.01640691178910692</v>
       </c>
       <c r="M18" s="52">
-        <v>49.389999999984866</v>
+        <v>-450.90000000000873</v>
       </c>
       <c r="N18" s="54">
         <v>-269</v>
       </c>
       <c r="O18" s="58">
-        <v>-0.26132275132267124</v>
+        <v>2.385714285714332</v>
       </c>
       <c r="Q18" s="35" t="s">
         <v>124</v>
@@ -29367,16 +29367,16 @@
         <v>16999.83</v>
       </c>
       <c r="D24" s="52">
-        <v>15288.169999999998</v>
+        <v>16896.64</v>
       </c>
       <c r="E24" s="52">
-        <v>1711.6600000000035</v>
+        <v>103.19000000000233</v>
       </c>
       <c r="F24" s="52">
         <v>3</v>
       </c>
       <c r="G24" s="53">
-        <v>0.1008633615747924</v>
+        <v>0.006246533053565966</v>
       </c>
       <c r="H24" s="53"/>
       <c r="I24" s="54"/>
@@ -29385,10 +29385,10 @@
         <v>0</v>
       </c>
       <c r="L24" s="53">
-        <v>0.1008633615747924</v>
+        <v>0.006246533053565966</v>
       </c>
       <c r="M24" s="52">
-        <v>1714.6600000000035</v>
+        <v>106.19000000000233</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="58">
@@ -29420,19 +29420,19 @@
         <v>41</v>
       </c>
       <c r="C26" s="52">
-        <v>0</v>
+        <v>1379.0600000000013</v>
       </c>
       <c r="D26" s="52">
-        <v>1159.83</v>
+        <v>3415.09</v>
       </c>
       <c r="E26" s="52">
-        <v>-1159.83</v>
+        <v>-2036.0299999999988</v>
       </c>
       <c r="F26" s="52">
         <v>0</v>
       </c>
       <c r="G26" s="53">
-        <v>0</v>
+        <v>-1.476389714733222</v>
       </c>
       <c r="H26" s="53">
         <v>0.347929388593615</v>
@@ -29445,16 +29445,16 @@
         <v>0</v>
       </c>
       <c r="L26" s="53">
-        <v>0</v>
+        <v>-1.476389714733222</v>
       </c>
       <c r="M26" s="52">
-        <v>-1159.83</v>
+        <v>-2036.0299999999988</v>
       </c>
       <c r="N26" s="54">
         <v>-143.25</v>
       </c>
       <c r="O26" s="58">
-        <v>8.096544502617801</v>
+        <v>14.213123909249555</v>
       </c>
     </row>
     <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -30202,10 +30202,10 @@
         <v>0</v>
       </c>
       <c r="D52" s="99">
-        <v>2625.4400000000023</v>
+        <v>-301.33000000000175</v>
       </c>
       <c r="E52" s="99">
-        <v>-2625.4400000000023</v>
+        <v>301.33000000000175</v>
       </c>
       <c r="F52" s="99"/>
       <c r="G52" s="100">
@@ -30227,13 +30227,13 @@
         <v>0</v>
       </c>
       <c r="M52" s="99">
-        <v>-3905.4400000000023</v>
+        <v>-978.6699999999983</v>
       </c>
       <c r="N52" s="98">
         <v>-304.75</v>
       </c>
       <c r="O52" s="60">
-        <v>14.318753437213575</v>
+        <v>3.5881576535288664</v>
       </c>
     </row>
     <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -30843,25 +30843,25 @@
         <v>127</v>
       </c>
       <c r="C74" s="104">
-        <v>501839.88</v>
+        <v>503218.94</v>
       </c>
       <c r="D74" s="104">
-        <v>255671.49999999997</v>
+        <v>257189.93999999997</v>
       </c>
       <c r="E74" s="105">
-        <v>246168.37999999998</v>
+        <v>246028.99999999997</v>
       </c>
       <c r="F74" s="106" t="s">
         <v>128</v>
       </c>
       <c r="G74" s="107">
-        <v>0.49053172099435377</v>
+        <v>0.4889104531717347</v>
       </c>
       <c r="H74" s="108" t="s">
         <v>129</v>
       </c>
       <c r="I74" s="109">
-        <v>0.3505815042040899</v>
+        <v>0.34934376675090956</v>
       </c>
       <c r="J74" s="36"/>
       <c r="K74" s="36"/>
@@ -31701,10 +31701,10 @@
         <v>501.83</v>
       </c>
       <c r="D14" s="54">
-        <v>366.25</v>
+        <v>373.25</v>
       </c>
       <c r="E14" s="54">
-        <v>135.57999999999998</v>
+        <v>128.57999999999998</v>
       </c>
       <c r="F14" s="54"/>
       <c r="G14" s="54"/>
@@ -31812,10 +31812,10 @@
         <v>685.48</v>
       </c>
       <c r="D18" s="54">
-        <v>699.75</v>
+        <v>718.75</v>
       </c>
       <c r="E18" s="54">
-        <v>-14.269999999999982</v>
+        <v>-33.26999999999998</v>
       </c>
       <c r="F18" s="54"/>
       <c r="G18" s="54"/>
@@ -31970,10 +31970,10 @@
         <v>472.14</v>
       </c>
       <c r="D24" s="54">
-        <v>237.25</v>
+        <v>257.25</v>
       </c>
       <c r="E24" s="54">
-        <v>234.89</v>
+        <v>214.89</v>
       </c>
       <c r="F24" s="54"/>
       <c r="G24" s="54"/>
@@ -32071,13 +32071,13 @@
         <v>43</v>
       </c>
       <c r="C28" s="54">
-        <v>231.75</v>
+        <v>232</v>
       </c>
       <c r="D28" s="54">
         <v>225.5</v>
       </c>
       <c r="E28" s="54">
-        <v>6.25</v>
+        <v>6.5</v>
       </c>
       <c r="F28" s="54"/>
       <c r="G28" s="54"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-30T22:49:08Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -10087,30 +10087,74 @@
       <c r="C5" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="53"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="52"/>
-      <c r="K5" s="52"/>
-      <c r="L5" s="52"/>
-      <c r="M5" s="53"/>
+      <c r="D5" s="52">
+        <v>267886.84883856</v>
+      </c>
+      <c r="E5" s="52">
+        <v>238732.97</v>
+      </c>
+      <c r="F5" s="52">
+        <v>29153.87883855999</v>
+      </c>
+      <c r="G5" s="53">
+        <v>0.10882907826553799</v>
+      </c>
+      <c r="H5" s="52">
+        <v>225410.5455298</v>
+      </c>
+      <c r="I5" s="52">
+        <v>189455.97</v>
+      </c>
+      <c r="J5" s="52">
+        <v>193787.2413298</v>
+      </c>
+      <c r="K5" s="52">
+        <v>158286.35</v>
+      </c>
+      <c r="L5" s="52">
+        <v>35500.89132979998</v>
+      </c>
+      <c r="M5" s="53">
+        <v>0.18319519430787606</v>
+      </c>
       <c r="N5" s="53"/>
-      <c r="O5" s="52"/>
-      <c r="P5" s="52"/>
-      <c r="Q5" s="52"/>
-      <c r="R5" s="53"/>
-      <c r="S5" s="54"/>
-      <c r="T5" s="54"/>
-      <c r="U5" s="54"/>
-      <c r="V5" s="53"/>
+      <c r="O5" s="52">
+        <v>31623.3042</v>
+      </c>
+      <c r="P5" s="52">
+        <v>31169.62</v>
+      </c>
+      <c r="Q5" s="52">
+        <v>453.6841999999997</v>
+      </c>
+      <c r="R5" s="53">
+        <v>0.014346514745287108</v>
+      </c>
+      <c r="S5" s="54">
+        <v>638.02</v>
+      </c>
+      <c r="T5" s="54">
+        <v>625.25</v>
+      </c>
+      <c r="U5" s="54">
+        <v>12.769999999999982</v>
+      </c>
+      <c r="V5" s="53">
+        <v>0.020015046550264853</v>
+      </c>
       <c r="W5" s="53"/>
-      <c r="X5" s="55"/>
-      <c r="Y5" s="55"/>
-      <c r="Z5" s="53"/>
-      <c r="AA5" s="56"/>
+      <c r="X5" s="55">
+        <v>78.81167532986805</v>
+      </c>
+      <c r="Y5" s="55">
+        <v>66.57519091683645</v>
+      </c>
+      <c r="Z5" s="53">
+        <v>0.2064</v>
+      </c>
+      <c r="AA5" s="56">
+        <v>0.1586</v>
+      </c>
       <c r="AB5" s="57"/>
       <c r="AD5" s="35" t="s">
         <v>99</v>
@@ -10406,30 +10450,74 @@
       <c r="C12" s="63" t="s">
         <v>98</v>
       </c>
-      <c r="D12" s="52"/>
-      <c r="E12" s="62"/>
-      <c r="F12" s="52"/>
-      <c r="G12" s="53"/>
-      <c r="H12" s="52"/>
-      <c r="I12" s="52"/>
-      <c r="J12" s="52"/>
-      <c r="K12" s="52"/>
-      <c r="L12" s="52"/>
-      <c r="M12" s="53"/>
+      <c r="D12" s="52">
+        <v>129798.36820213</v>
+      </c>
+      <c r="E12" s="62">
+        <v>127883.98</v>
+      </c>
+      <c r="F12" s="52">
+        <v>1914.3882021300087</v>
+      </c>
+      <c r="G12" s="53">
+        <v>0.014748938901518436</v>
+      </c>
+      <c r="H12" s="52">
+        <v>102331.503895</v>
+      </c>
+      <c r="I12" s="52">
+        <v>95264.02</v>
+      </c>
+      <c r="J12" s="52">
+        <v>84181.404895</v>
+      </c>
+      <c r="K12" s="52">
+        <v>80546.38</v>
+      </c>
+      <c r="L12" s="52">
+        <v>3635.024894999995</v>
+      </c>
+      <c r="M12" s="53">
+        <v>0.043180853295736565</v>
+      </c>
       <c r="N12" s="53"/>
-      <c r="O12" s="52"/>
-      <c r="P12" s="52"/>
-      <c r="Q12" s="52"/>
-      <c r="R12" s="53"/>
-      <c r="S12" s="54"/>
-      <c r="T12" s="54"/>
-      <c r="U12" s="54"/>
-      <c r="V12" s="53"/>
+      <c r="O12" s="52">
+        <v>18150.099</v>
+      </c>
+      <c r="P12" s="52">
+        <v>14717.64</v>
+      </c>
+      <c r="Q12" s="52">
+        <v>3432.458999999999</v>
+      </c>
+      <c r="R12" s="53">
+        <v>0.1891151668098339</v>
+      </c>
+      <c r="S12" s="54">
+        <v>363.57</v>
+      </c>
+      <c r="T12" s="54">
+        <v>331.25</v>
+      </c>
+      <c r="U12" s="54">
+        <v>32.31999999999999</v>
+      </c>
+      <c r="V12" s="53">
+        <v>0.08889622356079983</v>
+      </c>
       <c r="W12" s="53"/>
-      <c r="X12" s="55"/>
-      <c r="Y12" s="55"/>
-      <c r="Z12" s="53"/>
-      <c r="AA12" s="56"/>
+      <c r="X12" s="55">
+        <v>98.47535094339622</v>
+      </c>
+      <c r="Y12" s="55">
+        <v>75.54766429334104</v>
+      </c>
+      <c r="Z12" s="53">
+        <v>0.2551</v>
+      </c>
+      <c r="AA12" s="56">
+        <v>0.2116</v>
+      </c>
       <c r="AB12" s="57"/>
       <c r="AD12" s="35" t="s">
         <v>99</v>
@@ -10725,30 +10813,74 @@
       <c r="C19" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D19" s="52"/>
-      <c r="E19" s="52"/>
-      <c r="F19" s="52"/>
-      <c r="G19" s="53"/>
-      <c r="H19" s="52"/>
-      <c r="I19" s="52"/>
-      <c r="J19" s="52"/>
-      <c r="K19" s="52"/>
-      <c r="L19" s="52"/>
-      <c r="M19" s="53"/>
+      <c r="D19" s="52">
+        <v>27500.3157</v>
+      </c>
+      <c r="E19" s="52">
+        <v>11999.08</v>
+      </c>
+      <c r="F19" s="52">
+        <v>15501.2357</v>
+      </c>
+      <c r="G19" s="53">
+        <v>0.563674827194802</v>
+      </c>
+      <c r="H19" s="52">
+        <v>19565.829</v>
+      </c>
+      <c r="I19" s="52">
+        <v>8852.34</v>
+      </c>
+      <c r="J19" s="52">
+        <v>13767.337200000002</v>
+      </c>
+      <c r="K19" s="52">
+        <v>6787.5</v>
+      </c>
+      <c r="L19" s="52">
+        <v>6979.837200000002</v>
+      </c>
+      <c r="M19" s="53">
+        <v>0.506985272358986</v>
+      </c>
       <c r="N19" s="53"/>
-      <c r="O19" s="52"/>
-      <c r="P19" s="52"/>
-      <c r="Q19" s="52"/>
-      <c r="R19" s="53"/>
-      <c r="S19" s="54"/>
-      <c r="T19" s="54"/>
-      <c r="U19" s="54"/>
-      <c r="V19" s="53"/>
+      <c r="O19" s="52">
+        <v>5798.4918</v>
+      </c>
+      <c r="P19" s="52">
+        <v>2064.84</v>
+      </c>
+      <c r="Q19" s="52">
+        <v>3733.6517999999996</v>
+      </c>
+      <c r="R19" s="53">
+        <v>0.643900505300361</v>
+      </c>
+      <c r="S19" s="54">
+        <v>125.39</v>
+      </c>
+      <c r="T19" s="54">
+        <v>42.75</v>
+      </c>
+      <c r="U19" s="54">
+        <v>82.64</v>
+      </c>
+      <c r="V19" s="53">
+        <v>0.6590637211898875</v>
+      </c>
       <c r="W19" s="53"/>
-      <c r="X19" s="55"/>
-      <c r="Y19" s="55"/>
-      <c r="Z19" s="53"/>
-      <c r="AA19" s="56"/>
+      <c r="X19" s="55">
+        <v>73.60795321637427</v>
+      </c>
+      <c r="Y19" s="55">
+        <v>63.27846478985563</v>
+      </c>
+      <c r="Z19" s="53">
+        <v>0.2622</v>
+      </c>
+      <c r="AA19" s="56">
+        <v>0.2885</v>
+      </c>
       <c r="AB19" s="57"/>
       <c r="AD19" s="35" t="s">
         <v>99</v>
@@ -11365,30 +11497,74 @@
       <c r="C33" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D33" s="52"/>
-      <c r="E33" s="52"/>
-      <c r="F33" s="52"/>
-      <c r="G33" s="53"/>
-      <c r="H33" s="52"/>
-      <c r="I33" s="65"/>
-      <c r="J33" s="52"/>
-      <c r="K33" s="52"/>
-      <c r="L33" s="52"/>
-      <c r="M33" s="53"/>
+      <c r="D33" s="52">
+        <v>397238.61073204</v>
+      </c>
+      <c r="E33" s="52">
+        <v>352623.79</v>
+      </c>
+      <c r="F33" s="52">
+        <v>44614.82073204004</v>
+      </c>
+      <c r="G33" s="53">
+        <v>0.112312397452561</v>
+      </c>
+      <c r="H33" s="52">
+        <v>328046.93216</v>
+      </c>
+      <c r="I33" s="65">
+        <v>278861.56</v>
+      </c>
+      <c r="J33" s="52">
+        <v>271925.57216000004</v>
+      </c>
+      <c r="K33" s="52">
+        <v>243385.51</v>
+      </c>
+      <c r="L33" s="52">
+        <v>28540.06216000003</v>
+      </c>
+      <c r="M33" s="53">
+        <v>0.10495541825395943</v>
+      </c>
       <c r="N33" s="53"/>
-      <c r="O33" s="52"/>
-      <c r="P33" s="52"/>
-      <c r="Q33" s="52"/>
-      <c r="R33" s="53"/>
-      <c r="S33" s="54"/>
-      <c r="T33" s="54"/>
-      <c r="U33" s="54"/>
-      <c r="V33" s="53"/>
+      <c r="O33" s="52">
+        <v>56121.36</v>
+      </c>
+      <c r="P33" s="52">
+        <v>35476.05</v>
+      </c>
+      <c r="Q33" s="52">
+        <v>20645.309999999998</v>
+      </c>
+      <c r="R33" s="53">
+        <v>0.367869025269523</v>
+      </c>
+      <c r="S33" s="54">
+        <v>1124.47</v>
+      </c>
+      <c r="T33" s="54">
+        <v>821.5</v>
+      </c>
+      <c r="U33" s="54">
+        <v>302.97</v>
+      </c>
+      <c r="V33" s="53">
+        <v>0.2694335998292529</v>
+      </c>
       <c r="W33" s="53"/>
-      <c r="X33" s="55"/>
-      <c r="Y33" s="55"/>
-      <c r="Z33" s="53"/>
-      <c r="AA33" s="56"/>
+      <c r="X33" s="55">
+        <v>89.78968959220937</v>
+      </c>
+      <c r="Y33" s="55">
+        <v>61.532703026350184</v>
+      </c>
+      <c r="Z33" s="53">
+        <v>0.20920000000000002</v>
+      </c>
+      <c r="AA33" s="56">
+        <v>0.1742</v>
+      </c>
       <c r="AB33" s="57"/>
       <c r="AD33" s="35" t="s">
         <v>99</v>
@@ -11684,30 +11860,74 @@
       <c r="C40" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D40" s="52"/>
-      <c r="E40" s="52"/>
-      <c r="F40" s="52"/>
-      <c r="G40" s="53"/>
-      <c r="H40" s="52"/>
-      <c r="I40" s="52"/>
-      <c r="J40" s="52"/>
-      <c r="K40" s="52"/>
-      <c r="L40" s="52"/>
-      <c r="M40" s="53"/>
+      <c r="D40" s="52">
+        <v>128258.49930985</v>
+      </c>
+      <c r="E40" s="52">
+        <v>115314.55</v>
+      </c>
+      <c r="F40" s="52">
+        <v>12943.949309849995</v>
+      </c>
+      <c r="G40" s="53">
+        <v>0.10092079183446305</v>
+      </c>
+      <c r="H40" s="52">
+        <v>94098.31685</v>
+      </c>
+      <c r="I40" s="52">
+        <v>59765.09</v>
+      </c>
+      <c r="J40" s="52">
+        <v>69042.08885</v>
+      </c>
+      <c r="K40" s="52">
+        <v>42207.67</v>
+      </c>
+      <c r="L40" s="52">
+        <v>26834.418850000002</v>
+      </c>
+      <c r="M40" s="53">
+        <v>0.38866754029270656</v>
+      </c>
       <c r="N40" s="53"/>
-      <c r="O40" s="52"/>
-      <c r="P40" s="52"/>
-      <c r="Q40" s="52"/>
-      <c r="R40" s="53"/>
-      <c r="S40" s="54"/>
-      <c r="T40" s="54"/>
-      <c r="U40" s="54"/>
-      <c r="V40" s="53"/>
+      <c r="O40" s="52">
+        <v>25056.228</v>
+      </c>
+      <c r="P40" s="52">
+        <v>17557.42</v>
+      </c>
+      <c r="Q40" s="52">
+        <v>7498.808000000001</v>
+      </c>
+      <c r="R40" s="53">
+        <v>0.29927920515410383</v>
+      </c>
+      <c r="S40" s="54">
+        <v>501.83</v>
+      </c>
+      <c r="T40" s="54">
+        <v>393.75</v>
+      </c>
+      <c r="U40" s="54">
+        <v>108.07999999999998</v>
+      </c>
+      <c r="V40" s="53">
+        <v>0.21537173943367274</v>
+      </c>
       <c r="W40" s="53"/>
-      <c r="X40" s="55"/>
-      <c r="Y40" s="55"/>
-      <c r="Z40" s="53"/>
-      <c r="AA40" s="56"/>
+      <c r="X40" s="55">
+        <v>141.07799365079364</v>
+      </c>
+      <c r="Y40" s="55">
+        <v>68.07122423898531</v>
+      </c>
+      <c r="Z40" s="53">
+        <v>0.4817</v>
+      </c>
+      <c r="AA40" s="56">
+        <v>0.2663</v>
+      </c>
       <c r="AB40" s="57"/>
       <c r="AD40" s="35" t="s">
         <v>99</v>
@@ -12005,30 +12225,74 @@
       <c r="C47" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D47" s="52"/>
-      <c r="E47" s="52"/>
-      <c r="F47" s="52"/>
-      <c r="G47" s="53"/>
-      <c r="H47" s="52"/>
-      <c r="I47" s="52"/>
-      <c r="J47" s="52"/>
-      <c r="K47" s="52"/>
-      <c r="L47" s="52"/>
-      <c r="M47" s="53"/>
+      <c r="D47" s="52">
+        <v>65693.35850319</v>
+      </c>
+      <c r="E47" s="52">
+        <v>61277.97</v>
+      </c>
+      <c r="F47" s="52">
+        <v>4415.388503189999</v>
+      </c>
+      <c r="G47" s="53">
+        <v>0.06721209881476212</v>
+      </c>
+      <c r="H47" s="52">
+        <v>50582.36785</v>
+      </c>
+      <c r="I47" s="52">
+        <v>30176.95</v>
+      </c>
+      <c r="J47" s="52">
+        <v>39438.99025</v>
+      </c>
+      <c r="K47" s="52">
+        <v>20820.22</v>
+      </c>
+      <c r="L47" s="52">
+        <v>18618.77025</v>
+      </c>
+      <c r="M47" s="53">
+        <v>0.47209043973938963</v>
+      </c>
       <c r="N47" s="53"/>
-      <c r="O47" s="52"/>
-      <c r="P47" s="52"/>
-      <c r="Q47" s="52"/>
-      <c r="R47" s="53"/>
-      <c r="S47" s="54"/>
-      <c r="T47" s="54"/>
-      <c r="U47" s="54"/>
-      <c r="V47" s="53"/>
+      <c r="O47" s="52">
+        <v>11143.3776</v>
+      </c>
+      <c r="P47" s="52">
+        <v>9356.73</v>
+      </c>
+      <c r="Q47" s="52">
+        <v>1786.6476000000002</v>
+      </c>
+      <c r="R47" s="53">
+        <v>0.1603326804612634</v>
+      </c>
+      <c r="S47" s="54">
+        <v>223.22</v>
+      </c>
+      <c r="T47" s="54">
+        <v>216.5</v>
+      </c>
+      <c r="U47" s="54">
+        <v>6.719999999999999</v>
+      </c>
+      <c r="V47" s="53">
+        <v>0.030104829316369496</v>
+      </c>
       <c r="W47" s="53"/>
-      <c r="X47" s="55"/>
-      <c r="Y47" s="55"/>
-      <c r="Z47" s="53"/>
-      <c r="AA47" s="56"/>
+      <c r="X47" s="55">
+        <v>143.65367205542725</v>
+      </c>
+      <c r="Y47" s="55">
+        <v>67.69550512136009</v>
+      </c>
+      <c r="Z47" s="53">
+        <v>0.5075</v>
+      </c>
+      <c r="AA47" s="56">
+        <v>0.23</v>
+      </c>
       <c r="AB47" s="57"/>
       <c r="AD47" s="35" t="s">
         <v>99</v>
@@ -12324,30 +12588,74 @@
       <c r="C54" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D54" s="52"/>
-      <c r="E54" s="52"/>
-      <c r="F54" s="52"/>
-      <c r="G54" s="53"/>
-      <c r="H54" s="52"/>
-      <c r="I54" s="52"/>
-      <c r="J54" s="52"/>
-      <c r="K54" s="52"/>
-      <c r="L54" s="52"/>
-      <c r="M54" s="53"/>
+      <c r="D54" s="52">
+        <v>155296.79012754</v>
+      </c>
+      <c r="E54" s="52">
+        <v>155296.8</v>
+      </c>
+      <c r="F54" s="52">
+        <v>-0.009872459981124848</v>
+      </c>
+      <c r="G54" s="53">
+        <v>-6.357156495647419e-8</v>
+      </c>
+      <c r="H54" s="52">
+        <v>109364.9721</v>
+      </c>
+      <c r="I54" s="52">
+        <v>115851.63</v>
+      </c>
+      <c r="J54" s="52">
+        <v>75135.0159</v>
+      </c>
+      <c r="K54" s="52">
+        <v>81019.67000000001</v>
+      </c>
+      <c r="L54" s="52">
+        <v>-5884.654100000014</v>
+      </c>
+      <c r="M54" s="53">
+        <v>-0.07832106015432433</v>
+      </c>
       <c r="N54" s="53"/>
-      <c r="O54" s="52"/>
-      <c r="P54" s="52"/>
-      <c r="Q54" s="52"/>
-      <c r="R54" s="53"/>
-      <c r="S54" s="54"/>
-      <c r="T54" s="54"/>
-      <c r="U54" s="54"/>
-      <c r="V54" s="53"/>
+      <c r="O54" s="52">
+        <v>34229.9562</v>
+      </c>
+      <c r="P54" s="52">
+        <v>34831.96</v>
+      </c>
+      <c r="Q54" s="52">
+        <v>-602.0037999999986</v>
+      </c>
+      <c r="R54" s="53">
+        <v>-0.01758704558319004</v>
+      </c>
+      <c r="S54" s="54">
+        <v>685.48</v>
+      </c>
+      <c r="T54" s="54">
+        <v>740.5</v>
+      </c>
+      <c r="U54" s="54">
+        <v>-55.01999999999998</v>
+      </c>
+      <c r="V54" s="53">
+        <v>-0.0802649238489817</v>
+      </c>
       <c r="W54" s="53"/>
-      <c r="X54" s="55"/>
-      <c r="Y54" s="55"/>
-      <c r="Z54" s="53"/>
-      <c r="AA54" s="56"/>
+      <c r="X54" s="55">
+        <v>53.26829169480081</v>
+      </c>
+      <c r="Y54" s="55">
+        <v>67.00679527854935</v>
+      </c>
+      <c r="Z54" s="53">
+        <v>0.254</v>
+      </c>
+      <c r="AA54" s="56">
+        <v>0.2958</v>
+      </c>
       <c r="AB54" s="57"/>
       <c r="AD54" s="35" t="s">
         <v>99</v>
@@ -12956,30 +13264,74 @@
       <c r="C68" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D68" s="52"/>
-      <c r="E68" s="52"/>
-      <c r="F68" s="52"/>
-      <c r="G68" s="53"/>
-      <c r="H68" s="52"/>
-      <c r="I68" s="52"/>
-      <c r="J68" s="52"/>
-      <c r="K68" s="52"/>
-      <c r="L68" s="52"/>
-      <c r="M68" s="53"/>
+      <c r="D68" s="52">
+        <v>53029.71458947</v>
+      </c>
+      <c r="E68" s="52">
+        <v>29715.67</v>
+      </c>
+      <c r="F68" s="52">
+        <v>23314.044589470002</v>
+      </c>
+      <c r="G68" s="53">
+        <v>0.43964114779715263</v>
+      </c>
+      <c r="H68" s="52">
+        <v>39055.77825</v>
+      </c>
+      <c r="I68" s="52">
+        <v>30684.03</v>
+      </c>
+      <c r="J68" s="52">
+        <v>29537.289750000004</v>
+      </c>
+      <c r="K68" s="52">
+        <v>26364.309999999998</v>
+      </c>
+      <c r="L68" s="52">
+        <v>3172.979750000006</v>
+      </c>
+      <c r="M68" s="53">
+        <v>0.10742284674239638</v>
+      </c>
       <c r="N68" s="53"/>
-      <c r="O68" s="52"/>
-      <c r="P68" s="52"/>
-      <c r="Q68" s="52"/>
-      <c r="R68" s="53"/>
-      <c r="S68" s="54"/>
-      <c r="T68" s="54"/>
-      <c r="U68" s="54"/>
-      <c r="V68" s="53"/>
+      <c r="O68" s="52">
+        <v>9518.4885</v>
+      </c>
+      <c r="P68" s="52">
+        <v>4319.72</v>
+      </c>
+      <c r="Q68" s="52">
+        <v>5198.768499999999</v>
+      </c>
+      <c r="R68" s="53">
+        <v>0.5461758450409432</v>
+      </c>
+      <c r="S68" s="54">
+        <v>193.32</v>
+      </c>
+      <c r="T68" s="54">
+        <v>90.75</v>
+      </c>
+      <c r="U68" s="54">
+        <v>102.57</v>
+      </c>
+      <c r="V68" s="53">
+        <v>0.5305710738671633</v>
+      </c>
       <c r="W68" s="53"/>
-      <c r="X68" s="55"/>
-      <c r="Y68" s="55"/>
-      <c r="Z68" s="53"/>
-      <c r="AA68" s="56"/>
+      <c r="X68" s="55">
+        <v>-10.670633608815427</v>
+      </c>
+      <c r="Y68" s="55">
+        <v>72.28396616733912</v>
+      </c>
+      <c r="Z68" s="53">
+        <v>-0.0326</v>
+      </c>
+      <c r="AA68" s="56">
+        <v>0.2635</v>
+      </c>
       <c r="AB68" s="57"/>
       <c r="AD68" s="35" t="s">
         <v>99</v>
@@ -13267,30 +13619,74 @@
       <c r="C75" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D75" s="52"/>
-      <c r="E75" s="52"/>
-      <c r="F75" s="52"/>
-      <c r="G75" s="53"/>
-      <c r="H75" s="52"/>
-      <c r="I75" s="52"/>
-      <c r="J75" s="52"/>
-      <c r="K75" s="52"/>
-      <c r="L75" s="52"/>
-      <c r="M75" s="53"/>
+      <c r="D75" s="52">
+        <v>78753.06644148</v>
+      </c>
+      <c r="E75" s="52">
+        <v>61764.82</v>
+      </c>
+      <c r="F75" s="52">
+        <v>16988.246441479998</v>
+      </c>
+      <c r="G75" s="53">
+        <v>0.21571536460873764</v>
+      </c>
+      <c r="H75" s="52">
+        <v>55589.7822</v>
+      </c>
+      <c r="I75" s="52">
+        <v>49921.75</v>
+      </c>
+      <c r="J75" s="52">
+        <v>32594.7534</v>
+      </c>
+      <c r="K75" s="52">
+        <v>36088.43</v>
+      </c>
+      <c r="L75" s="52">
+        <v>-3493.676599999999</v>
+      </c>
+      <c r="M75" s="53">
+        <v>-0.10718524411355107</v>
+      </c>
       <c r="N75" s="53"/>
-      <c r="O75" s="52"/>
-      <c r="P75" s="52"/>
-      <c r="Q75" s="52"/>
-      <c r="R75" s="53"/>
-      <c r="S75" s="54"/>
-      <c r="T75" s="54"/>
-      <c r="U75" s="54"/>
-      <c r="V75" s="53"/>
+      <c r="O75" s="52">
+        <v>22995.0288</v>
+      </c>
+      <c r="P75" s="52">
+        <v>13833.32</v>
+      </c>
+      <c r="Q75" s="52">
+        <v>9161.7088</v>
+      </c>
+      <c r="R75" s="53">
+        <v>0.3984212796463208</v>
+      </c>
+      <c r="S75" s="54">
+        <v>472.14</v>
+      </c>
+      <c r="T75" s="54">
+        <v>275.25</v>
+      </c>
+      <c r="U75" s="54">
+        <v>196.89</v>
+      </c>
+      <c r="V75" s="53">
+        <v>0.4170161392807218</v>
+      </c>
       <c r="W75" s="53"/>
-      <c r="X75" s="55"/>
-      <c r="Y75" s="55"/>
-      <c r="Z75" s="53"/>
-      <c r="AA75" s="56"/>
+      <c r="X75" s="55">
+        <v>43.02659400544959</v>
+      </c>
+      <c r="Y75" s="55">
+        <v>49.060202993773025</v>
+      </c>
+      <c r="Z75" s="53">
+        <v>0.1917</v>
+      </c>
+      <c r="AA75" s="56">
+        <v>0.2941</v>
+      </c>
       <c r="AB75" s="57"/>
       <c r="AD75" s="35" t="s">
         <v>99</v>
@@ -13580,30 +13976,74 @@
       <c r="C82" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D82" s="52"/>
-      <c r="E82" s="52"/>
-      <c r="F82" s="52"/>
-      <c r="G82" s="53"/>
-      <c r="H82" s="52"/>
-      <c r="I82" s="52"/>
-      <c r="J82" s="52"/>
-      <c r="K82" s="52"/>
-      <c r="L82" s="52"/>
-      <c r="M82" s="53"/>
+      <c r="D82" s="52">
+        <v>26846.9041072</v>
+      </c>
+      <c r="E82" s="52">
+        <v>20977.47</v>
+      </c>
+      <c r="F82" s="52">
+        <v>5869.434107199999</v>
+      </c>
+      <c r="G82" s="53">
+        <v>0.21862610615225056</v>
+      </c>
+      <c r="H82" s="52">
+        <v>17678.176816</v>
+      </c>
+      <c r="I82" s="52">
+        <v>16373.33</v>
+      </c>
+      <c r="J82" s="52">
+        <v>10731.333616</v>
+      </c>
+      <c r="K82" s="52">
+        <v>7553.74</v>
+      </c>
+      <c r="L82" s="52">
+        <v>3177.593616</v>
+      </c>
+      <c r="M82" s="53">
+        <v>0.2961042615674842</v>
+      </c>
       <c r="N82" s="53"/>
-      <c r="O82" s="52"/>
-      <c r="P82" s="52"/>
-      <c r="Q82" s="52"/>
-      <c r="R82" s="53"/>
-      <c r="S82" s="54"/>
-      <c r="T82" s="54"/>
-      <c r="U82" s="54"/>
-      <c r="V82" s="53"/>
+      <c r="O82" s="52">
+        <v>6946.8432</v>
+      </c>
+      <c r="P82" s="52">
+        <v>8819.59</v>
+      </c>
+      <c r="Q82" s="52">
+        <v>-1872.7468</v>
+      </c>
+      <c r="R82" s="53">
+        <v>-0.26958241982487813</v>
+      </c>
+      <c r="S82" s="54">
+        <v>139.07</v>
+      </c>
+      <c r="T82" s="54">
+        <v>167.75</v>
+      </c>
+      <c r="U82" s="54">
+        <v>-28.680000000000007</v>
+      </c>
+      <c r="V82" s="53">
+        <v>-0.20622707988782632</v>
+      </c>
       <c r="W82" s="53"/>
-      <c r="X82" s="55"/>
-      <c r="Y82" s="55"/>
-      <c r="Z82" s="53"/>
-      <c r="AA82" s="56"/>
+      <c r="X82" s="55">
+        <v>27.446438152011925</v>
+      </c>
+      <c r="Y82" s="55">
+        <v>65.92886525634573</v>
+      </c>
+      <c r="Z82" s="53">
+        <v>0.2195</v>
+      </c>
+      <c r="AA82" s="56">
+        <v>0.3415</v>
+      </c>
       <c r="AB82" s="57"/>
       <c r="AD82" s="35" t="s">
         <v>99</v>
@@ -13899,30 +14339,74 @@
       <c r="C89" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D89" s="67"/>
-      <c r="E89" s="67"/>
-      <c r="F89" s="52"/>
-      <c r="G89" s="53"/>
-      <c r="H89" s="52"/>
-      <c r="I89" s="52"/>
-      <c r="J89" s="52"/>
-      <c r="K89" s="52"/>
-      <c r="L89" s="52"/>
-      <c r="M89" s="53"/>
+      <c r="D89" s="67">
+        <v>37218.0313712</v>
+      </c>
+      <c r="E89" s="67">
+        <v>36381.33</v>
+      </c>
+      <c r="F89" s="52">
+        <v>836.7013711999971</v>
+      </c>
+      <c r="G89" s="53">
+        <v>0.022481075445797277</v>
+      </c>
+      <c r="H89" s="52">
+        <v>27090.14646</v>
+      </c>
+      <c r="I89" s="52">
+        <v>26164.59</v>
+      </c>
+      <c r="J89" s="52">
+        <v>15515.12046</v>
+      </c>
+      <c r="K89" s="52">
+        <v>14571.4</v>
+      </c>
+      <c r="L89" s="52">
+        <v>943.7204600000005</v>
+      </c>
+      <c r="M89" s="53">
+        <v>0.060825854522562985</v>
+      </c>
       <c r="N89" s="53"/>
-      <c r="O89" s="52"/>
-      <c r="P89" s="52"/>
-      <c r="Q89" s="52"/>
-      <c r="R89" s="53"/>
-      <c r="S89" s="68"/>
-      <c r="T89" s="68"/>
-      <c r="U89" s="54"/>
-      <c r="V89" s="53"/>
+      <c r="O89" s="52">
+        <v>11575.026</v>
+      </c>
+      <c r="P89" s="52">
+        <v>11593.19</v>
+      </c>
+      <c r="Q89" s="52">
+        <v>-18.16400000000067</v>
+      </c>
+      <c r="R89" s="53">
+        <v>-0.0015692405356152693</v>
+      </c>
+      <c r="S89" s="68">
+        <v>232</v>
+      </c>
+      <c r="T89" s="68">
+        <v>234</v>
+      </c>
+      <c r="U89" s="54">
+        <v>-2</v>
+      </c>
+      <c r="V89" s="53">
+        <v>-0.008620689655172414</v>
+      </c>
       <c r="W89" s="53"/>
-      <c r="X89" s="55"/>
-      <c r="Y89" s="55"/>
-      <c r="Z89" s="53"/>
-      <c r="AA89" s="56"/>
+      <c r="X89" s="55">
+        <v>43.66128205128205</v>
+      </c>
+      <c r="Y89" s="55">
+        <v>43.65467634137931</v>
+      </c>
+      <c r="Z89" s="53">
+        <v>0.2808</v>
+      </c>
+      <c r="AA89" s="56">
+        <v>0.2721</v>
+      </c>
       <c r="AB89" s="57"/>
       <c r="AD89" s="35" t="s">
         <v>99</v>
@@ -14218,30 +14702,74 @@
       <c r="C96" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D96" s="52"/>
-      <c r="E96" s="52"/>
-      <c r="F96" s="52"/>
-      <c r="G96" s="53"/>
-      <c r="H96" s="52"/>
-      <c r="I96" s="52"/>
-      <c r="J96" s="52"/>
-      <c r="K96" s="52"/>
-      <c r="L96" s="52"/>
-      <c r="M96" s="53"/>
+      <c r="D96" s="52">
+        <v>26186.1354</v>
+      </c>
+      <c r="E96" s="52">
+        <v>5762.27</v>
+      </c>
+      <c r="F96" s="52">
+        <v>20423.8654</v>
+      </c>
+      <c r="G96" s="53">
+        <v>0.7799495835494686</v>
+      </c>
+      <c r="H96" s="52">
+        <v>19428.9760178</v>
+      </c>
+      <c r="I96" s="52">
+        <v>8019.36</v>
+      </c>
+      <c r="J96" s="52">
+        <v>12051.3142178</v>
+      </c>
+      <c r="K96" s="52">
+        <v>7687.129999999999</v>
+      </c>
+      <c r="L96" s="52">
+        <v>4364.184217800001</v>
+      </c>
+      <c r="M96" s="53">
+        <v>0.3621334685103493</v>
+      </c>
       <c r="N96" s="53"/>
-      <c r="O96" s="52"/>
-      <c r="P96" s="52"/>
-      <c r="Q96" s="52"/>
-      <c r="R96" s="53"/>
-      <c r="S96" s="54"/>
-      <c r="T96" s="54"/>
-      <c r="U96" s="54"/>
-      <c r="V96" s="53"/>
+      <c r="O96" s="52">
+        <v>7377.6618</v>
+      </c>
+      <c r="P96" s="52">
+        <v>332.23</v>
+      </c>
+      <c r="Q96" s="52">
+        <v>7045.4318</v>
+      </c>
+      <c r="R96" s="53">
+        <v>0.954968117405436</v>
+      </c>
+      <c r="S96" s="54">
+        <v>147.9</v>
+      </c>
+      <c r="T96" s="54">
+        <v>6.5</v>
+      </c>
+      <c r="U96" s="54">
+        <v>141.4</v>
+      </c>
+      <c r="V96" s="53">
+        <v>0.9560513860716701</v>
+      </c>
       <c r="W96" s="53"/>
-      <c r="X96" s="55"/>
-      <c r="Y96" s="55"/>
-      <c r="Z96" s="53"/>
-      <c r="AA96" s="56"/>
+      <c r="X96" s="55">
+        <v>-347.24461538461543</v>
+      </c>
+      <c r="Y96" s="55">
+        <v>45.687352144692355</v>
+      </c>
+      <c r="Z96" s="53">
+        <v>-0.3917</v>
+      </c>
+      <c r="AA96" s="56">
+        <v>0.258</v>
+      </c>
       <c r="AB96" s="57"/>
       <c r="AD96" s="35" t="s">
         <v>99</v>
@@ -15173,30 +15701,74 @@
       <c r="C117" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D117" s="52"/>
-      <c r="E117" s="52"/>
-      <c r="F117" s="52"/>
-      <c r="G117" s="53"/>
-      <c r="H117" s="52"/>
-      <c r="I117" s="52"/>
-      <c r="J117" s="52"/>
-      <c r="K117" s="52"/>
-      <c r="L117" s="52"/>
-      <c r="M117" s="53"/>
+      <c r="D117" s="52">
+        <v>20278.45679756</v>
+      </c>
+      <c r="E117" s="52">
+        <v>0</v>
+      </c>
+      <c r="F117" s="52">
+        <v>20278.45679756</v>
+      </c>
+      <c r="G117" s="53">
+        <v>1</v>
+      </c>
+      <c r="H117" s="52">
+        <v>16648.056795</v>
+      </c>
+      <c r="I117" s="52">
+        <v>3100.1</v>
+      </c>
+      <c r="J117" s="52">
+        <v>12536.982795</v>
+      </c>
+      <c r="K117" s="52">
+        <v>1650.85</v>
+      </c>
+      <c r="L117" s="52">
+        <v>10886.132795</v>
+      </c>
+      <c r="M117" s="53">
+        <v>0.8683215868607244</v>
+      </c>
       <c r="N117" s="53"/>
-      <c r="O117" s="52"/>
-      <c r="P117" s="52"/>
-      <c r="Q117" s="52"/>
-      <c r="R117" s="53"/>
-      <c r="S117" s="54"/>
-      <c r="T117" s="54"/>
-      <c r="U117" s="54"/>
-      <c r="V117" s="53"/>
+      <c r="O117" s="52">
+        <v>4111.074</v>
+      </c>
+      <c r="P117" s="52">
+        <v>1449.25</v>
+      </c>
+      <c r="Q117" s="52">
+        <v>2661.8239999999996</v>
+      </c>
+      <c r="R117" s="53">
+        <v>0.6474765474909963</v>
+      </c>
+      <c r="S117" s="54">
+        <v>82.37</v>
+      </c>
+      <c r="T117" s="54">
+        <v>31.75</v>
+      </c>
+      <c r="U117" s="54">
+        <v>50.620000000000005</v>
+      </c>
+      <c r="V117" s="53">
+        <v>0.6145441301444701</v>
+      </c>
       <c r="W117" s="53"/>
-      <c r="X117" s="55"/>
-      <c r="Y117" s="55"/>
-      <c r="Z117" s="53"/>
-      <c r="AA117" s="56"/>
+      <c r="X117" s="55">
+        <v>-97.64094488188977</v>
+      </c>
+      <c r="Y117" s="55">
+        <v>44.07429892630812</v>
+      </c>
+      <c r="Z117" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA117" s="56">
+        <v>0.179</v>
+      </c>
       <c r="AB117" s="57"/>
       <c r="AD117" s="35" t="s">
         <v>99</v>
@@ -15480,30 +16052,74 @@
       <c r="C124" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D124" s="52"/>
-      <c r="E124" s="52"/>
-      <c r="F124" s="52"/>
-      <c r="G124" s="53"/>
-      <c r="H124" s="52"/>
-      <c r="I124" s="52"/>
-      <c r="J124" s="52"/>
-      <c r="K124" s="52"/>
-      <c r="L124" s="52"/>
-      <c r="M124" s="53"/>
+      <c r="D124" s="52">
+        <v>105896.9567712</v>
+      </c>
+      <c r="E124" s="52">
+        <v>79457.73</v>
+      </c>
+      <c r="F124" s="52">
+        <v>26439.226771200003</v>
+      </c>
+      <c r="G124" s="53">
+        <v>0.2496693727311197</v>
+      </c>
+      <c r="H124" s="52">
+        <v>85934.2000148</v>
+      </c>
+      <c r="I124" s="52">
+        <v>64324.38</v>
+      </c>
+      <c r="J124" s="52">
+        <v>70065.71561479999</v>
+      </c>
+      <c r="K124" s="52">
+        <v>59442.78999999999</v>
+      </c>
+      <c r="L124" s="52">
+        <v>10622.925614799999</v>
+      </c>
+      <c r="M124" s="53">
+        <v>0.15161374606093533</v>
+      </c>
       <c r="N124" s="53"/>
-      <c r="O124" s="52"/>
-      <c r="P124" s="52"/>
-      <c r="Q124" s="52"/>
-      <c r="R124" s="53"/>
-      <c r="S124" s="54"/>
-      <c r="T124" s="54"/>
-      <c r="U124" s="54"/>
-      <c r="V124" s="53"/>
+      <c r="O124" s="52">
+        <v>15868.4844</v>
+      </c>
+      <c r="P124" s="52">
+        <v>4881.59</v>
+      </c>
+      <c r="Q124" s="52">
+        <v>10986.8944</v>
+      </c>
+      <c r="R124" s="53">
+        <v>0.6923720074993425</v>
+      </c>
+      <c r="S124" s="54">
+        <v>317.92</v>
+      </c>
+      <c r="T124" s="54">
+        <v>106</v>
+      </c>
+      <c r="U124" s="54">
+        <v>211.92000000000002</v>
+      </c>
+      <c r="V124" s="53">
+        <v>0.6665827881227983</v>
+      </c>
       <c r="W124" s="53"/>
-      <c r="X124" s="55"/>
-      <c r="Y124" s="55"/>
-      <c r="Z124" s="53"/>
-      <c r="AA124" s="56"/>
+      <c r="X124" s="55">
+        <v>142.7674528301887</v>
+      </c>
+      <c r="Y124" s="55">
+        <v>62.79176131227983</v>
+      </c>
+      <c r="Z124" s="53">
+        <v>0.1905</v>
+      </c>
+      <c r="AA124" s="56">
+        <v>0.1885</v>
+      </c>
       <c r="AB124" s="57"/>
       <c r="AD124" s="35" t="s">
         <v>99</v>
@@ -15797,30 +16413,74 @@
       <c r="C131" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D131" s="52"/>
-      <c r="E131" s="52"/>
-      <c r="F131" s="52"/>
-      <c r="G131" s="53"/>
-      <c r="H131" s="52"/>
-      <c r="I131" s="52"/>
-      <c r="J131" s="52"/>
-      <c r="K131" s="52"/>
-      <c r="L131" s="52"/>
-      <c r="M131" s="53"/>
+      <c r="D131" s="52">
+        <v>31802.4136956</v>
+      </c>
+      <c r="E131" s="52">
+        <v>16498.64</v>
+      </c>
+      <c r="F131" s="52">
+        <v>15303.7736956</v>
+      </c>
+      <c r="G131" s="53">
+        <v>0.48121421984134943</v>
+      </c>
+      <c r="H131" s="52">
+        <v>23448.14263</v>
+      </c>
+      <c r="I131" s="52">
+        <v>12360.83</v>
+      </c>
+      <c r="J131" s="52">
+        <v>15632.028429999998</v>
+      </c>
+      <c r="K131" s="52">
+        <v>11772.08</v>
+      </c>
+      <c r="L131" s="52">
+        <v>3859.9484299999986</v>
+      </c>
+      <c r="M131" s="53">
+        <v>0.24692562755273845</v>
+      </c>
       <c r="N131" s="53"/>
-      <c r="O131" s="52"/>
-      <c r="P131" s="52"/>
-      <c r="Q131" s="52"/>
-      <c r="R131" s="53"/>
-      <c r="S131" s="54"/>
-      <c r="T131" s="54"/>
-      <c r="U131" s="54"/>
-      <c r="V131" s="53"/>
+      <c r="O131" s="52">
+        <v>7816.1142</v>
+      </c>
+      <c r="P131" s="52">
+        <v>588.75</v>
+      </c>
+      <c r="Q131" s="52">
+        <v>7227.3642</v>
+      </c>
+      <c r="R131" s="53">
+        <v>0.92467484674162</v>
+      </c>
+      <c r="S131" s="54">
+        <v>156.69</v>
+      </c>
+      <c r="T131" s="54">
+        <v>11.5</v>
+      </c>
+      <c r="U131" s="54">
+        <v>145.19</v>
+      </c>
+      <c r="V131" s="53">
+        <v>0.9266066756015061</v>
+      </c>
       <c r="W131" s="53"/>
-      <c r="X131" s="55"/>
-      <c r="Y131" s="55"/>
-      <c r="Z131" s="53"/>
-      <c r="AA131" s="56"/>
+      <c r="X131" s="55">
+        <v>359.80956521739137</v>
+      </c>
+      <c r="Y131" s="55">
+        <v>53.31719360265494</v>
+      </c>
+      <c r="Z131" s="53">
+        <v>0.25079999999999997</v>
+      </c>
+      <c r="AA131" s="56">
+        <v>0.2627</v>
+      </c>
       <c r="AB131" s="57"/>
       <c r="AD131" s="35" t="s">
         <v>99</v>
@@ -17052,30 +17712,74 @@
       <c r="C159" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D159" s="52"/>
-      <c r="E159" s="52"/>
-      <c r="F159" s="52"/>
-      <c r="G159" s="53"/>
-      <c r="H159" s="52"/>
-      <c r="I159" s="52"/>
-      <c r="J159" s="52"/>
-      <c r="K159" s="52"/>
-      <c r="L159" s="52"/>
-      <c r="M159" s="53"/>
+      <c r="D159" s="52">
+        <v>19505.5188968</v>
+      </c>
+      <c r="E159" s="52">
+        <v>19505.52</v>
+      </c>
+      <c r="F159" s="52">
+        <v>-0.0011032000002160203</v>
+      </c>
+      <c r="G159" s="53">
+        <v>-5.655835182098165e-8</v>
+      </c>
+      <c r="H159" s="52">
+        <v>14923.5903884</v>
+      </c>
+      <c r="I159" s="52">
+        <v>14052.73</v>
+      </c>
+      <c r="J159" s="52">
+        <v>8915.0763884</v>
+      </c>
+      <c r="K159" s="52">
+        <v>8190.78</v>
+      </c>
+      <c r="L159" s="52">
+        <v>724.296388400001</v>
+      </c>
+      <c r="M159" s="53">
+        <v>0.08124399128452015</v>
+      </c>
       <c r="N159" s="53"/>
-      <c r="O159" s="52"/>
-      <c r="P159" s="52"/>
-      <c r="Q159" s="52"/>
-      <c r="R159" s="53"/>
-      <c r="S159" s="54"/>
-      <c r="T159" s="54"/>
-      <c r="U159" s="54"/>
-      <c r="V159" s="53"/>
+      <c r="O159" s="52">
+        <v>6008.514</v>
+      </c>
+      <c r="P159" s="52">
+        <v>5861.95</v>
+      </c>
+      <c r="Q159" s="52">
+        <v>146.5640000000003</v>
+      </c>
+      <c r="R159" s="53">
+        <v>0.02439272006356319</v>
+      </c>
+      <c r="S159" s="54">
+        <v>120.44</v>
+      </c>
+      <c r="T159" s="54">
+        <v>116.25</v>
+      </c>
+      <c r="U159" s="54">
+        <v>4.189999999999998</v>
+      </c>
+      <c r="V159" s="53">
+        <v>0.03478910660909995</v>
+      </c>
       <c r="W159" s="53"/>
-      <c r="X159" s="55"/>
-      <c r="Y159" s="55"/>
-      <c r="Z159" s="53"/>
-      <c r="AA159" s="56"/>
+      <c r="X159" s="55">
+        <v>46.90572043010753</v>
+      </c>
+      <c r="Y159" s="55">
+        <v>38.04324566921289</v>
+      </c>
+      <c r="Z159" s="53">
+        <v>0.2796</v>
+      </c>
+      <c r="AA159" s="56">
+        <v>0.2349</v>
+      </c>
       <c r="AB159" s="57"/>
       <c r="AD159" s="35" t="s">
         <v>99</v>
@@ -17359,30 +18063,74 @@
       <c r="C166" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D166" s="52"/>
-      <c r="E166" s="52"/>
-      <c r="F166" s="52"/>
-      <c r="G166" s="53"/>
-      <c r="H166" s="52"/>
-      <c r="I166" s="52"/>
-      <c r="J166" s="52"/>
-      <c r="K166" s="52"/>
-      <c r="L166" s="52"/>
-      <c r="M166" s="53"/>
+      <c r="D166" s="52">
+        <v>10827.20261235</v>
+      </c>
+      <c r="E166" s="52">
+        <v>0</v>
+      </c>
+      <c r="F166" s="52">
+        <v>10827.20261235</v>
+      </c>
+      <c r="G166" s="53">
+        <v>1</v>
+      </c>
+      <c r="H166" s="52">
+        <v>7687.765097</v>
+      </c>
+      <c r="I166" s="52">
+        <v>2097.39</v>
+      </c>
+      <c r="J166" s="52">
+        <v>4437.133697</v>
+      </c>
+      <c r="K166" s="52">
+        <v>1010.6899999999998</v>
+      </c>
+      <c r="L166" s="52">
+        <v>3426.4436970000006</v>
+      </c>
+      <c r="M166" s="53">
+        <v>0.7722200706543192</v>
+      </c>
       <c r="N166" s="53"/>
-      <c r="O166" s="52"/>
-      <c r="P166" s="52"/>
-      <c r="Q166" s="52"/>
-      <c r="R166" s="53"/>
-      <c r="S166" s="54"/>
-      <c r="T166" s="54"/>
-      <c r="U166" s="54"/>
-      <c r="V166" s="53"/>
+      <c r="O166" s="52">
+        <v>3250.6314</v>
+      </c>
+      <c r="P166" s="52">
+        <v>1086.7</v>
+      </c>
+      <c r="Q166" s="52">
+        <v>2163.9314000000004</v>
+      </c>
+      <c r="R166" s="53">
+        <v>0.6656957168382734</v>
+      </c>
+      <c r="S166" s="54">
+        <v>65.13</v>
+      </c>
+      <c r="T166" s="54">
+        <v>24.33</v>
+      </c>
+      <c r="U166" s="54">
+        <v>40.8</v>
+      </c>
+      <c r="V166" s="53">
+        <v>0.6264394288346384</v>
+      </c>
       <c r="W166" s="53"/>
-      <c r="X166" s="55"/>
-      <c r="Y166" s="55"/>
-      <c r="Z166" s="53"/>
-      <c r="AA166" s="56"/>
+      <c r="X166" s="55">
+        <v>53.18249075215784</v>
+      </c>
+      <c r="Y166" s="55">
+        <v>48.202633430830645</v>
+      </c>
+      <c r="Z166" s="53">
+        <v>0.3815</v>
+      </c>
+      <c r="AA166" s="56">
+        <v>0.29</v>
+      </c>
       <c r="AB166" s="57"/>
       <c r="AD166" s="35" t="s">
         <v>99</v>
@@ -17668,30 +18416,74 @@
       <c r="C173" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D173" s="52"/>
-      <c r="E173" s="52"/>
-      <c r="F173" s="52"/>
-      <c r="G173" s="53"/>
-      <c r="H173" s="52"/>
-      <c r="I173" s="52"/>
-      <c r="J173" s="52"/>
-      <c r="K173" s="52"/>
-      <c r="L173" s="52"/>
-      <c r="M173" s="53"/>
+      <c r="D173" s="52">
+        <v>146237.1072</v>
+      </c>
+      <c r="E173" s="52">
+        <v>129751.67</v>
+      </c>
+      <c r="F173" s="52">
+        <v>16485.4372</v>
+      </c>
+      <c r="G173" s="53">
+        <v>0.11273087601120163</v>
+      </c>
+      <c r="H173" s="52">
+        <v>114651.8653946</v>
+      </c>
+      <c r="I173" s="52">
+        <v>102580.79</v>
+      </c>
+      <c r="J173" s="52">
+        <v>82888.0783946</v>
+      </c>
+      <c r="K173" s="52">
+        <v>74954.88999999998</v>
+      </c>
+      <c r="L173" s="52">
+        <v>7933.188394600016</v>
+      </c>
+      <c r="M173" s="53">
+        <v>0.095709643030123</v>
+      </c>
       <c r="N173" s="53"/>
-      <c r="O173" s="52"/>
-      <c r="P173" s="52"/>
-      <c r="Q173" s="52"/>
-      <c r="R173" s="53"/>
-      <c r="S173" s="54"/>
-      <c r="T173" s="54"/>
-      <c r="U173" s="54"/>
-      <c r="V173" s="53"/>
+      <c r="O173" s="52">
+        <v>31763.787</v>
+      </c>
+      <c r="P173" s="52">
+        <v>27625.9</v>
+      </c>
+      <c r="Q173" s="52">
+        <v>4137.886999999999</v>
+      </c>
+      <c r="R173" s="53">
+        <v>0.1302705814013927</v>
+      </c>
+      <c r="S173" s="54">
+        <v>659.73</v>
+      </c>
+      <c r="T173" s="54">
+        <v>550.75</v>
+      </c>
+      <c r="U173" s="54">
+        <v>108.98000000000002</v>
+      </c>
+      <c r="V173" s="53">
+        <v>0.1651887893532203</v>
+      </c>
       <c r="W173" s="53"/>
-      <c r="X173" s="55"/>
-      <c r="Y173" s="55"/>
-      <c r="Z173" s="53"/>
-      <c r="AA173" s="56"/>
+      <c r="X173" s="55">
+        <v>49.33432591920109</v>
+      </c>
+      <c r="Y173" s="55">
+        <v>47.87601261940491</v>
+      </c>
+      <c r="Z173" s="53">
+        <v>0.2094</v>
+      </c>
+      <c r="AA173" s="56">
+        <v>0.216</v>
+      </c>
       <c r="AB173" s="57"/>
       <c r="AD173" s="35" t="s">
         <v>99</v>
@@ -17983,30 +18775,74 @@
       <c r="C180" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D180" s="52"/>
-      <c r="E180" s="52"/>
-      <c r="F180" s="52"/>
-      <c r="G180" s="53"/>
-      <c r="H180" s="52"/>
-      <c r="I180" s="52"/>
-      <c r="J180" s="52"/>
-      <c r="K180" s="52"/>
-      <c r="L180" s="52"/>
-      <c r="M180" s="53"/>
+      <c r="D180" s="52">
+        <v>16897.52982004</v>
+      </c>
+      <c r="E180" s="52">
+        <v>9293.64</v>
+      </c>
+      <c r="F180" s="52">
+        <v>7603.88982004</v>
+      </c>
+      <c r="G180" s="53">
+        <v>0.450000082912829</v>
+      </c>
+      <c r="H180" s="52">
+        <v>9226.2731</v>
+      </c>
+      <c r="I180" s="52">
+        <v>6976.46</v>
+      </c>
+      <c r="J180" s="52">
+        <v>2977.1135000000004</v>
+      </c>
+      <c r="K180" s="52">
+        <v>3448.13</v>
+      </c>
+      <c r="L180" s="52">
+        <v>-471.0164999999997</v>
+      </c>
+      <c r="M180" s="53">
+        <v>-0.15821247661535232</v>
+      </c>
       <c r="N180" s="53"/>
-      <c r="O180" s="52"/>
-      <c r="P180" s="52"/>
-      <c r="Q180" s="52"/>
-      <c r="R180" s="53"/>
-      <c r="S180" s="54"/>
-      <c r="T180" s="54"/>
-      <c r="U180" s="54"/>
-      <c r="V180" s="53"/>
+      <c r="O180" s="52">
+        <v>6249.1596</v>
+      </c>
+      <c r="P180" s="52">
+        <v>3528.33</v>
+      </c>
+      <c r="Q180" s="52">
+        <v>2720.8296</v>
+      </c>
+      <c r="R180" s="53">
+        <v>0.43539128045313485</v>
+      </c>
+      <c r="S180" s="54">
+        <v>125.17</v>
+      </c>
+      <c r="T180" s="54">
+        <v>65.75</v>
+      </c>
+      <c r="U180" s="54">
+        <v>59.42</v>
+      </c>
+      <c r="V180" s="53">
+        <v>0.47471438843173286</v>
+      </c>
       <c r="W180" s="53"/>
-      <c r="X180" s="55"/>
-      <c r="Y180" s="55"/>
-      <c r="Z180" s="53"/>
-      <c r="AA180" s="56"/>
+      <c r="X180" s="55">
+        <v>35.24228136882129</v>
+      </c>
+      <c r="Y180" s="55">
+        <v>61.286703843093385</v>
+      </c>
+      <c r="Z180" s="53">
+        <v>0.2493</v>
+      </c>
+      <c r="AA180" s="56">
+        <v>0.454</v>
+      </c>
       <c r="AB180" s="57"/>
       <c r="AD180" s="35" t="s">
         <v>99</v>
@@ -18298,30 +19134,74 @@
       <c r="C187" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D187" s="52"/>
-      <c r="E187" s="52"/>
-      <c r="F187" s="52"/>
-      <c r="G187" s="53"/>
-      <c r="H187" s="52"/>
-      <c r="I187" s="52"/>
-      <c r="J187" s="52"/>
-      <c r="K187" s="52"/>
-      <c r="L187" s="52"/>
-      <c r="M187" s="53"/>
+      <c r="D187" s="52">
+        <v>20992.11525559</v>
+      </c>
+      <c r="E187" s="52">
+        <v>14169.68</v>
+      </c>
+      <c r="F187" s="52">
+        <v>6822.43525559</v>
+      </c>
+      <c r="G187" s="53">
+        <v>0.3249998950807614</v>
+      </c>
+      <c r="H187" s="52">
+        <v>16299.085174</v>
+      </c>
+      <c r="I187" s="52">
+        <v>9699.51</v>
+      </c>
+      <c r="J187" s="52">
+        <v>9784.324774</v>
+      </c>
+      <c r="K187" s="52">
+        <v>8137.88</v>
+      </c>
+      <c r="L187" s="52">
+        <v>1646.4447740000005</v>
+      </c>
+      <c r="M187" s="53">
+        <v>0.16827372476178604</v>
+      </c>
       <c r="N187" s="53"/>
-      <c r="O187" s="52"/>
-      <c r="P187" s="52"/>
-      <c r="Q187" s="52"/>
-      <c r="R187" s="53"/>
-      <c r="S187" s="54"/>
-      <c r="T187" s="54"/>
-      <c r="U187" s="54"/>
-      <c r="V187" s="53"/>
+      <c r="O187" s="52">
+        <v>6514.7604</v>
+      </c>
+      <c r="P187" s="52">
+        <v>1561.63</v>
+      </c>
+      <c r="Q187" s="52">
+        <v>4953.1304</v>
+      </c>
+      <c r="R187" s="53">
+        <v>0.7602935635207705</v>
+      </c>
+      <c r="S187" s="54">
+        <v>130.62</v>
+      </c>
+      <c r="T187" s="54">
+        <v>34.75</v>
+      </c>
+      <c r="U187" s="54">
+        <v>95.87</v>
+      </c>
+      <c r="V187" s="53">
+        <v>0.7339611085591793</v>
+      </c>
       <c r="W187" s="53"/>
-      <c r="X187" s="55"/>
-      <c r="Y187" s="55"/>
-      <c r="Z187" s="53"/>
-      <c r="AA187" s="56"/>
+      <c r="X187" s="55">
+        <v>128.6379856115108</v>
+      </c>
+      <c r="Y187" s="55">
+        <v>35.92887828502527</v>
+      </c>
+      <c r="Z187" s="53">
+        <v>0.3155</v>
+      </c>
+      <c r="AA187" s="56">
+        <v>0.2236</v>
+      </c>
       <c r="AB187" s="57"/>
       <c r="AD187" s="35" t="s">
         <v>99</v>
@@ -18605,30 +19485,74 @@
       <c r="C194" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D194" s="52"/>
-      <c r="E194" s="52"/>
-      <c r="F194" s="52"/>
-      <c r="G194" s="53"/>
-      <c r="H194" s="52"/>
-      <c r="I194" s="52"/>
-      <c r="J194" s="52"/>
-      <c r="K194" s="52"/>
-      <c r="L194" s="52"/>
-      <c r="M194" s="53"/>
+      <c r="D194" s="52">
+        <v>23770.94615247</v>
+      </c>
+      <c r="E194" s="52">
+        <v>10204.54</v>
+      </c>
+      <c r="F194" s="52">
+        <v>13566.406152469997</v>
+      </c>
+      <c r="G194" s="53">
+        <v>0.5707137639980029</v>
+      </c>
+      <c r="H194" s="52">
+        <v>14310.9577</v>
+      </c>
+      <c r="I194" s="52">
+        <v>7116.73</v>
+      </c>
+      <c r="J194" s="52">
+        <v>7389.335500000001</v>
+      </c>
+      <c r="K194" s="52">
+        <v>6605.049999999999</v>
+      </c>
+      <c r="L194" s="52">
+        <v>784.2855000000018</v>
+      </c>
+      <c r="M194" s="53">
+        <v>0.10613748692287713</v>
+      </c>
       <c r="N194" s="53"/>
-      <c r="O194" s="52"/>
-      <c r="P194" s="52"/>
-      <c r="Q194" s="52"/>
-      <c r="R194" s="53"/>
-      <c r="S194" s="54"/>
-      <c r="T194" s="54"/>
-      <c r="U194" s="54"/>
-      <c r="V194" s="53"/>
+      <c r="O194" s="52">
+        <v>6921.6222</v>
+      </c>
+      <c r="P194" s="52">
+        <v>511.68</v>
+      </c>
+      <c r="Q194" s="52">
+        <v>6409.9421999999995</v>
+      </c>
+      <c r="R194" s="53">
+        <v>0.9260751330807971</v>
+      </c>
+      <c r="S194" s="54">
+        <v>140.15</v>
+      </c>
+      <c r="T194" s="54">
+        <v>9.25</v>
+      </c>
+      <c r="U194" s="54">
+        <v>130.9</v>
+      </c>
+      <c r="V194" s="53">
+        <v>0.9339992864787727</v>
+      </c>
       <c r="W194" s="53"/>
-      <c r="X194" s="55"/>
-      <c r="Y194" s="55"/>
-      <c r="Z194" s="53"/>
-      <c r="AA194" s="56"/>
+      <c r="X194" s="55">
+        <v>333.8172972972973</v>
+      </c>
+      <c r="Y194" s="55">
+        <v>67.49902570438813</v>
+      </c>
+      <c r="Z194" s="53">
+        <v>0.30260000000000004</v>
+      </c>
+      <c r="AA194" s="56">
+        <v>0.398</v>
+      </c>
       <c r="AB194" s="57"/>
       <c r="AD194" s="35" t="s">
         <v>99</v>
@@ -19490,30 +20414,74 @@
       <c r="C215" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D215" s="52"/>
-      <c r="E215" s="52"/>
-      <c r="F215" s="52"/>
-      <c r="G215" s="53"/>
-      <c r="H215" s="52"/>
-      <c r="I215" s="52"/>
-      <c r="J215" s="52"/>
-      <c r="K215" s="52"/>
-      <c r="L215" s="52"/>
-      <c r="M215" s="53"/>
+      <c r="D215" s="52">
+        <v>137109.56054889</v>
+      </c>
+      <c r="E215" s="52">
+        <v>42368.33</v>
+      </c>
+      <c r="F215" s="52">
+        <v>94741.23054889</v>
+      </c>
+      <c r="G215" s="53">
+        <v>0.6909892364151188</v>
+      </c>
+      <c r="H215" s="52">
+        <v>117394.569232</v>
+      </c>
+      <c r="I215" s="52">
+        <v>37161.14</v>
+      </c>
+      <c r="J215" s="52">
+        <v>99479.615032</v>
+      </c>
+      <c r="K215" s="52">
+        <v>37161.14</v>
+      </c>
+      <c r="L215" s="52">
+        <v>62318.475032</v>
+      </c>
+      <c r="M215" s="53">
+        <v>0.6264446742375689</v>
+      </c>
       <c r="N215" s="53"/>
-      <c r="O215" s="52"/>
-      <c r="P215" s="52"/>
-      <c r="Q215" s="52"/>
-      <c r="R215" s="53"/>
-      <c r="S215" s="54"/>
-      <c r="T215" s="54"/>
-      <c r="U215" s="54"/>
-      <c r="V215" s="53"/>
+      <c r="O215" s="52">
+        <v>17914.9542</v>
+      </c>
+      <c r="P215" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q215" s="52">
+        <v>17914.9542</v>
+      </c>
+      <c r="R215" s="53">
+        <v>1</v>
+      </c>
+      <c r="S215" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="T215" s="54">
+        <v>0</v>
+      </c>
+      <c r="U215" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="V215" s="53">
+        <v>1</v>
+      </c>
       <c r="W215" s="53"/>
-      <c r="X215" s="55"/>
-      <c r="Y215" s="55"/>
-      <c r="Z215" s="53"/>
-      <c r="AA215" s="56"/>
+      <c r="X215" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y215" s="55">
+        <v>54.93783457863793</v>
+      </c>
+      <c r="Z215" s="53">
+        <v>0.1229</v>
+      </c>
+      <c r="AA215" s="56">
+        <v>0.1438</v>
+      </c>
       <c r="AB215" s="57"/>
       <c r="AD215" s="35" t="s">
         <v>99</v>
@@ -19799,30 +20767,74 @@
       <c r="C222" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D222" s="52"/>
-      <c r="E222" s="52"/>
-      <c r="F222" s="52"/>
-      <c r="G222" s="53"/>
-      <c r="H222" s="52"/>
-      <c r="I222" s="52"/>
-      <c r="J222" s="52"/>
-      <c r="K222" s="52"/>
-      <c r="L222" s="52"/>
-      <c r="M222" s="53"/>
+      <c r="D222" s="52">
+        <v>412300.73261827</v>
+      </c>
+      <c r="E222" s="52">
+        <v>353667.87</v>
+      </c>
+      <c r="F222" s="52">
+        <v>58632.86261826998</v>
+      </c>
+      <c r="G222" s="53">
+        <v>0.1422089702483149</v>
+      </c>
+      <c r="H222" s="52">
+        <v>306356.278672</v>
+      </c>
+      <c r="I222" s="52">
+        <v>253033.2</v>
+      </c>
+      <c r="J222" s="52">
+        <v>186357.488872</v>
+      </c>
+      <c r="K222" s="52">
+        <v>180716.68</v>
+      </c>
+      <c r="L222" s="52">
+        <v>5640.808871999994</v>
+      </c>
+      <c r="M222" s="53">
+        <v>0.03026875338438583</v>
+      </c>
       <c r="N222" s="53"/>
-      <c r="O222" s="52"/>
-      <c r="P222" s="52"/>
-      <c r="Q222" s="52"/>
-      <c r="R222" s="53"/>
-      <c r="S222" s="54"/>
-      <c r="T222" s="54"/>
-      <c r="U222" s="54"/>
-      <c r="V222" s="53"/>
+      <c r="O222" s="52">
+        <v>119998.7898</v>
+      </c>
+      <c r="P222" s="52">
+        <v>72316.52</v>
+      </c>
+      <c r="Q222" s="52">
+        <v>47682.269799999995</v>
+      </c>
+      <c r="R222" s="53">
+        <v>0.3973562556711717</v>
+      </c>
+      <c r="S222" s="54">
+        <v>2412.45</v>
+      </c>
+      <c r="T222" s="54">
+        <v>1543.42</v>
+      </c>
+      <c r="U222" s="54">
+        <v>869.0299999999997</v>
+      </c>
+      <c r="V222" s="53">
+        <v>0.36022715496694224</v>
+      </c>
       <c r="W222" s="53"/>
-      <c r="X222" s="55"/>
-      <c r="Y222" s="55"/>
-      <c r="Z222" s="53"/>
-      <c r="AA222" s="56"/>
+      <c r="X222" s="55">
+        <v>65.2023882028223</v>
+      </c>
+      <c r="Y222" s="55">
+        <v>43.91570973337064</v>
+      </c>
+      <c r="Z222" s="53">
+        <v>0.2845</v>
+      </c>
+      <c r="AA222" s="56">
+        <v>0.257</v>
+      </c>
       <c r="AB222" s="57"/>
       <c r="AD222" s="35" t="s">
         <v>99</v>
@@ -20104,30 +21116,74 @@
       <c r="C229" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D229" s="52"/>
-      <c r="E229" s="52"/>
-      <c r="F229" s="52"/>
-      <c r="G229" s="53"/>
-      <c r="H229" s="52"/>
-      <c r="I229" s="52"/>
-      <c r="J229" s="52"/>
-      <c r="K229" s="52"/>
-      <c r="L229" s="52"/>
-      <c r="M229" s="53"/>
+      <c r="D229" s="52">
+        <v>8795.02836582</v>
+      </c>
+      <c r="E229" s="52">
+        <v>1740.2</v>
+      </c>
+      <c r="F229" s="52">
+        <v>7054.828365820001</v>
+      </c>
+      <c r="G229" s="53">
+        <v>0.8021382163174237</v>
+      </c>
+      <c r="H229" s="52">
+        <v>6369.1218</v>
+      </c>
+      <c r="I229" s="52">
+        <v>757.35</v>
+      </c>
+      <c r="J229" s="52">
+        <v>4527.894</v>
+      </c>
+      <c r="K229" s="52">
+        <v>311.34000000000003</v>
+      </c>
+      <c r="L229" s="52">
+        <v>4216.554</v>
+      </c>
+      <c r="M229" s="53">
+        <v>0.931239556403043</v>
+      </c>
       <c r="N229" s="53"/>
-      <c r="O229" s="52"/>
-      <c r="P229" s="52"/>
-      <c r="Q229" s="52"/>
-      <c r="R229" s="53"/>
-      <c r="S229" s="54"/>
-      <c r="T229" s="54"/>
-      <c r="U229" s="54"/>
-      <c r="V229" s="53"/>
+      <c r="O229" s="52">
+        <v>1841.2278</v>
+      </c>
+      <c r="P229" s="52">
+        <v>446.01</v>
+      </c>
+      <c r="Q229" s="52">
+        <v>1395.2178</v>
+      </c>
+      <c r="R229" s="53">
+        <v>0.7577649001389182</v>
+      </c>
+      <c r="S229" s="54">
+        <v>36.92</v>
+      </c>
+      <c r="T229" s="54">
+        <v>7.75</v>
+      </c>
+      <c r="U229" s="54">
+        <v>29.17</v>
+      </c>
+      <c r="V229" s="53">
+        <v>0.7900866738894908</v>
+      </c>
       <c r="W229" s="53"/>
-      <c r="X229" s="55"/>
-      <c r="Y229" s="55"/>
-      <c r="Z229" s="53"/>
-      <c r="AA229" s="56"/>
+      <c r="X229" s="55">
+        <v>126.81935483870969</v>
+      </c>
+      <c r="Y229" s="55">
+        <v>65.70711175027087</v>
+      </c>
+      <c r="Z229" s="53">
+        <v>0.5648</v>
+      </c>
+      <c r="AA229" s="56">
+        <v>0.2758</v>
+      </c>
       <c r="AB229" s="57"/>
       <c r="AD229" s="35"/>
       <c r="AE229" s="36"/>
@@ -20401,30 +21457,74 @@
       <c r="C236" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D236" s="52"/>
-      <c r="E236" s="52"/>
-      <c r="F236" s="52"/>
-      <c r="G236" s="53"/>
-      <c r="H236" s="52"/>
-      <c r="I236" s="52"/>
-      <c r="J236" s="52"/>
-      <c r="K236" s="52"/>
-      <c r="L236" s="52"/>
-      <c r="M236" s="53"/>
+      <c r="D236" s="52">
+        <v>27503.13664251</v>
+      </c>
+      <c r="E236" s="52">
+        <v>0</v>
+      </c>
+      <c r="F236" s="52">
+        <v>27503.13664251</v>
+      </c>
+      <c r="G236" s="53">
+        <v>1</v>
+      </c>
+      <c r="H236" s="52">
+        <v>19683.280628</v>
+      </c>
+      <c r="I236" s="52">
+        <v>0</v>
+      </c>
+      <c r="J236" s="52">
+        <v>10693.531628</v>
+      </c>
+      <c r="K236" s="52">
+        <v>0</v>
+      </c>
+      <c r="L236" s="52">
+        <v>10693.531628</v>
+      </c>
+      <c r="M236" s="53">
+        <v>1</v>
+      </c>
       <c r="N236" s="53"/>
-      <c r="O236" s="52"/>
-      <c r="P236" s="52"/>
-      <c r="Q236" s="52"/>
-      <c r="R236" s="53"/>
-      <c r="S236" s="54"/>
-      <c r="T236" s="54"/>
-      <c r="U236" s="54"/>
-      <c r="V236" s="53"/>
+      <c r="O236" s="52">
+        <v>8989.749</v>
+      </c>
+      <c r="P236" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q236" s="52">
+        <v>8989.749</v>
+      </c>
+      <c r="R236" s="53">
+        <v>1</v>
+      </c>
+      <c r="S236" s="54">
+        <v>180.16</v>
+      </c>
+      <c r="T236" s="54">
+        <v>0</v>
+      </c>
+      <c r="U236" s="54">
+        <v>180.16</v>
+      </c>
+      <c r="V236" s="53">
+        <v>1</v>
+      </c>
       <c r="W236" s="53"/>
-      <c r="X236" s="55"/>
-      <c r="Y236" s="55"/>
-      <c r="Z236" s="53"/>
-      <c r="AA236" s="56"/>
+      <c r="X236" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y236" s="55">
+        <v>43.40506224750221</v>
+      </c>
+      <c r="Z236" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA236" s="56">
+        <v>0.2843</v>
+      </c>
       <c r="AB236" s="57"/>
       <c r="AD236" s="35"/>
       <c r="AE236" s="36"/>
@@ -20698,30 +21798,74 @@
       <c r="C243" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D243" s="52"/>
-      <c r="E243" s="52"/>
-      <c r="F243" s="52"/>
-      <c r="G243" s="53"/>
-      <c r="H243" s="52"/>
-      <c r="I243" s="52"/>
-      <c r="J243" s="52"/>
-      <c r="K243" s="52"/>
-      <c r="L243" s="52"/>
-      <c r="M243" s="53"/>
+      <c r="D243" s="52">
+        <v>40670.1518342</v>
+      </c>
+      <c r="E243" s="52">
+        <v>0</v>
+      </c>
+      <c r="F243" s="52">
+        <v>40670.1518342</v>
+      </c>
+      <c r="G243" s="53">
+        <v>1</v>
+      </c>
+      <c r="H243" s="52">
+        <v>29498.3116992</v>
+      </c>
+      <c r="I243" s="52">
+        <v>0</v>
+      </c>
+      <c r="J243" s="52">
+        <v>24964.3288992</v>
+      </c>
+      <c r="K243" s="52">
+        <v>0</v>
+      </c>
+      <c r="L243" s="52">
+        <v>24964.3288992</v>
+      </c>
+      <c r="M243" s="53">
+        <v>1</v>
+      </c>
       <c r="N243" s="53"/>
-      <c r="O243" s="52"/>
-      <c r="P243" s="52"/>
-      <c r="Q243" s="52"/>
-      <c r="R243" s="53"/>
-      <c r="S243" s="54"/>
-      <c r="T243" s="54"/>
-      <c r="U243" s="54"/>
-      <c r="V243" s="53"/>
+      <c r="O243" s="52">
+        <v>4533.9828</v>
+      </c>
+      <c r="P243" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q243" s="52">
+        <v>4533.9828</v>
+      </c>
+      <c r="R243" s="53">
+        <v>1</v>
+      </c>
+      <c r="S243" s="54">
+        <v>90.88</v>
+      </c>
+      <c r="T243" s="54">
+        <v>0</v>
+      </c>
+      <c r="U243" s="54">
+        <v>90.88</v>
+      </c>
+      <c r="V243" s="53">
+        <v>1</v>
+      </c>
       <c r="W243" s="53"/>
-      <c r="X243" s="55"/>
-      <c r="Y243" s="55"/>
-      <c r="Z243" s="53"/>
-      <c r="AA243" s="56"/>
+      <c r="X243" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y243" s="55">
+        <v>122.92957895026407</v>
+      </c>
+      <c r="Z243" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA243" s="56">
+        <v>0.2747</v>
+      </c>
       <c r="AB243" s="57"/>
       <c r="AD243" s="35"/>
       <c r="AE243" s="36"/>
@@ -20995,30 +22139,74 @@
       <c r="C250" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D250" s="52"/>
-      <c r="E250" s="52"/>
-      <c r="F250" s="52"/>
-      <c r="G250" s="53"/>
-      <c r="H250" s="52"/>
-      <c r="I250" s="52"/>
-      <c r="J250" s="52"/>
-      <c r="K250" s="52"/>
-      <c r="L250" s="52"/>
-      <c r="M250" s="53"/>
+      <c r="D250" s="52">
+        <v>21396.50036782</v>
+      </c>
+      <c r="E250" s="52">
+        <v>0</v>
+      </c>
+      <c r="F250" s="52">
+        <v>21396.50036782</v>
+      </c>
+      <c r="G250" s="53">
+        <v>1</v>
+      </c>
+      <c r="H250" s="52">
+        <v>15378.244372</v>
+      </c>
+      <c r="I250" s="52">
+        <v>0</v>
+      </c>
+      <c r="J250" s="52">
+        <v>8344.608772</v>
+      </c>
+      <c r="K250" s="52">
+        <v>0</v>
+      </c>
+      <c r="L250" s="52">
+        <v>8344.608772</v>
+      </c>
+      <c r="M250" s="53">
+        <v>1</v>
+      </c>
       <c r="N250" s="53"/>
-      <c r="O250" s="52"/>
-      <c r="P250" s="52"/>
-      <c r="Q250" s="52"/>
-      <c r="R250" s="53"/>
-      <c r="S250" s="54"/>
-      <c r="T250" s="54"/>
-      <c r="U250" s="54"/>
-      <c r="V250" s="53"/>
+      <c r="O250" s="52">
+        <v>7033.6356</v>
+      </c>
+      <c r="P250" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q250" s="52">
+        <v>7033.6356</v>
+      </c>
+      <c r="R250" s="53">
+        <v>1</v>
+      </c>
+      <c r="S250" s="54">
+        <v>140.9</v>
+      </c>
+      <c r="T250" s="54">
+        <v>0</v>
+      </c>
+      <c r="U250" s="54">
+        <v>140.9</v>
+      </c>
+      <c r="V250" s="53">
+        <v>1</v>
+      </c>
       <c r="W250" s="53"/>
-      <c r="X250" s="55"/>
-      <c r="Y250" s="55"/>
-      <c r="Z250" s="53"/>
-      <c r="AA250" s="56"/>
+      <c r="X250" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y250" s="55">
+        <v>42.71295951611073</v>
+      </c>
+      <c r="Z250" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA250" s="56">
+        <v>0.2813</v>
+      </c>
       <c r="AB250" s="57"/>
       <c r="AD250" s="35"/>
       <c r="AE250" s="36"/>
@@ -21292,30 +22480,74 @@
       <c r="C257" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D257" s="52"/>
-      <c r="E257" s="52"/>
-      <c r="F257" s="52"/>
-      <c r="G257" s="53"/>
-      <c r="H257" s="52"/>
-      <c r="I257" s="52"/>
-      <c r="J257" s="52"/>
-      <c r="K257" s="52"/>
-      <c r="L257" s="52"/>
-      <c r="M257" s="53"/>
+      <c r="D257" s="52">
+        <v>239296.88379393</v>
+      </c>
+      <c r="E257" s="52">
+        <v>19872.16</v>
+      </c>
+      <c r="F257" s="52">
+        <v>219424.72379393</v>
+      </c>
+      <c r="G257" s="53">
+        <v>0.916956043534972</v>
+      </c>
+      <c r="H257" s="52">
+        <v>203192.691868</v>
+      </c>
+      <c r="I257" s="52">
+        <v>18292.87</v>
+      </c>
+      <c r="J257" s="52">
+        <v>175849.529668</v>
+      </c>
+      <c r="K257" s="52">
+        <v>16897.46</v>
+      </c>
+      <c r="L257" s="52">
+        <v>158952.069668</v>
+      </c>
+      <c r="M257" s="53">
+        <v>0.9039095524912576</v>
+      </c>
       <c r="N257" s="53"/>
-      <c r="O257" s="52"/>
-      <c r="P257" s="52"/>
-      <c r="Q257" s="52"/>
-      <c r="R257" s="53"/>
-      <c r="S257" s="54"/>
-      <c r="T257" s="54"/>
-      <c r="U257" s="54"/>
-      <c r="V257" s="53"/>
+      <c r="O257" s="52">
+        <v>27343.1622</v>
+      </c>
+      <c r="P257" s="52">
+        <v>1395.41</v>
+      </c>
+      <c r="Q257" s="52">
+        <v>25947.7522</v>
+      </c>
+      <c r="R257" s="53">
+        <v>0.9489667658117465</v>
+      </c>
+      <c r="S257" s="54">
+        <v>547.57</v>
+      </c>
+      <c r="T257" s="54">
+        <v>27.84</v>
+      </c>
+      <c r="U257" s="54">
+        <v>519.73</v>
+      </c>
+      <c r="V257" s="53">
+        <v>0.9491571853826908</v>
+      </c>
       <c r="W257" s="53"/>
-      <c r="X257" s="55"/>
-      <c r="Y257" s="55"/>
-      <c r="Z257" s="53"/>
-      <c r="AA257" s="56"/>
+      <c r="X257" s="55">
+        <v>56.727370689655174</v>
+      </c>
+      <c r="Y257" s="55">
+        <v>65.93529946112827</v>
+      </c>
+      <c r="Z257" s="53">
+        <v>0.0795</v>
+      </c>
+      <c r="AA257" s="56">
+        <v>0.1509</v>
+      </c>
       <c r="AB257" s="57"/>
       <c r="AD257" s="35"/>
       <c r="AE257" s="36"/>
@@ -22211,10 +23443,10 @@
         <v>0</v>
       </c>
       <c r="D6" s="52">
-        <v>0</v>
+        <v>44.070000000006985</v>
       </c>
       <c r="E6" s="52">
-        <v>0</v>
+        <v>-44.070000000006985</v>
       </c>
       <c r="F6" s="52">
         <v>7</v>
@@ -22238,13 +23470,13 @@
         <v>0</v>
       </c>
       <c r="M6" s="52">
-        <v>-20265.6</v>
+        <v>-20309.670000000006</v>
       </c>
       <c r="N6" s="54">
         <v>-52.5</v>
       </c>
       <c r="O6" s="58">
-        <v>-45.28625698324022</v>
+        <v>-45.38473743016761</v>
       </c>
       <c r="Q6" s="35" t="s">
         <v>120</v>
@@ -22278,10 +23510,10 @@
         <v>0</v>
       </c>
       <c r="D8" s="52">
-        <v>0</v>
+        <v>768.4200000000001</v>
       </c>
       <c r="E8" s="52">
-        <v>0</v>
+        <v>-768.4200000000001</v>
       </c>
       <c r="F8" s="52"/>
       <c r="G8" s="53">
@@ -22301,13 +23533,13 @@
         <v>0</v>
       </c>
       <c r="M8" s="52">
-        <v>-640</v>
+        <v>-1408.42</v>
       </c>
       <c r="N8" s="54">
         <v>-34.75</v>
       </c>
       <c r="O8" s="58">
-        <v>34.13333333333333</v>
+        <v>75.11573333333334</v>
       </c>
     </row>
     <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -22469,10 +23701,10 @@
         <v>0</v>
       </c>
       <c r="D14" s="52">
-        <v>0</v>
+        <v>1155.719999999994</v>
       </c>
       <c r="E14" s="52">
-        <v>0</v>
+        <v>-1155.719999999994</v>
       </c>
       <c r="F14" s="52">
         <v>0</v>
@@ -22496,13 +23728,13 @@
         <v>0</v>
       </c>
       <c r="M14" s="52">
-        <v>-3000</v>
+        <v>-4155.719999999994</v>
       </c>
       <c r="N14" s="54">
         <v>-112</v>
       </c>
       <c r="O14" s="58">
-        <v>26.785714285714285</v>
+        <v>37.1046428571428</v>
       </c>
     </row>
     <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -22533,10 +23765,10 @@
         <v>0</v>
       </c>
       <c r="D16" s="52">
-        <v>0</v>
+        <v>575.9099999999999</v>
       </c>
       <c r="E16" s="52">
-        <v>0</v>
+        <v>-575.9099999999999</v>
       </c>
       <c r="F16" s="52"/>
       <c r="G16" s="53">
@@ -22558,13 +23790,13 @@
         <v>0</v>
       </c>
       <c r="M16" s="52">
-        <v>-3000</v>
+        <v>-3575.91</v>
       </c>
       <c r="N16" s="54">
         <v>-86.75</v>
       </c>
       <c r="O16" s="58">
-        <v>34.5821325648415</v>
+        <v>41.22086455331412</v>
       </c>
     </row>
     <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -22595,10 +23827,10 @@
         <v>0</v>
       </c>
       <c r="D18" s="52">
-        <v>0</v>
+        <v>797.9000000000087</v>
       </c>
       <c r="E18" s="52">
-        <v>0</v>
+        <v>-797.9000000000087</v>
       </c>
       <c r="F18" s="52">
         <v>0</v>
@@ -22622,13 +23854,13 @@
         <v>0</v>
       </c>
       <c r="M18" s="52">
-        <v>-8200</v>
+        <v>-8997.900000000009</v>
       </c>
       <c r="N18" s="54">
         <v>-269</v>
       </c>
       <c r="O18" s="58">
-        <v>43.386243386243386</v>
+        <v>47.60793650793656</v>
       </c>
       <c r="Q18" s="35" t="s">
         <v>123</v>
@@ -22776,10 +24008,10 @@
         <v>0</v>
       </c>
       <c r="D24" s="52">
-        <v>0</v>
+        <v>1106.1800000000003</v>
       </c>
       <c r="E24" s="52">
-        <v>0</v>
+        <v>-1106.1800000000003</v>
       </c>
       <c r="F24" s="52">
         <v>3</v>
@@ -22797,7 +24029,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="52">
-        <v>3</v>
+        <v>-1103.1800000000003</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="58">
@@ -22894,10 +24126,10 @@
         <v>0</v>
       </c>
       <c r="D28" s="52">
-        <v>0</v>
+        <v>1060.7700000000004</v>
       </c>
       <c r="E28" s="52">
-        <v>0</v>
+        <v>-1060.7700000000004</v>
       </c>
       <c r="F28" s="52">
         <v>0</v>
@@ -22917,13 +24149,13 @@
         <v>0</v>
       </c>
       <c r="M28" s="52">
-        <v>0</v>
+        <v>-1060.7700000000004</v>
       </c>
       <c r="N28" s="54">
         <v>-148.5</v>
       </c>
       <c r="O28" s="58">
-        <v>0</v>
+        <v>7.1432323232323265</v>
       </c>
     </row>
     <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -23140,10 +24372,10 @@
         <v>0</v>
       </c>
       <c r="D36" s="52">
-        <v>0</v>
+        <v>3041.7799999999997</v>
       </c>
       <c r="E36" s="52">
-        <v>0</v>
+        <v>-3041.7799999999997</v>
       </c>
       <c r="F36" s="52">
         <v>0</v>
@@ -23165,11 +24397,11 @@
         <v>0</v>
       </c>
       <c r="M36" s="52">
-        <v>-3200</v>
+        <v>-6241.78</v>
       </c>
       <c r="N36" s="54"/>
       <c r="O36" s="58">
-        <v>-40</v>
+        <v>-78.02225</v>
       </c>
     </row>
     <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -23200,10 +24432,10 @@
         <v>0</v>
       </c>
       <c r="D38" s="52">
-        <v>0</v>
+        <v>48.57999999999447</v>
       </c>
       <c r="E38" s="52">
-        <v>0</v>
+        <v>-48.57999999999447</v>
       </c>
       <c r="F38" s="52">
         <v>0</v>
@@ -23223,7 +24455,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="52">
-        <v>0</v>
+        <v>-48.57999999999447</v>
       </c>
       <c r="N38" s="54"/>
       <c r="O38" s="58">
@@ -23608,17 +24840,17 @@
         <v>56</v>
       </c>
       <c r="C52" s="99">
-        <v>0</v>
+        <v>4365.459999999992</v>
       </c>
       <c r="D52" s="99">
         <v>0</v>
       </c>
       <c r="E52" s="99">
-        <v>0</v>
+        <v>4365.459999999992</v>
       </c>
       <c r="F52" s="99"/>
       <c r="G52" s="100">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H52" s="100">
         <v>0.215986489339129</v>
@@ -23633,16 +24865,16 @@
         <v>1280</v>
       </c>
       <c r="L52" s="100">
-        <v>0</v>
+        <v>0.7067892043450169</v>
       </c>
       <c r="M52" s="99">
-        <v>-1280</v>
+        <v>3085.459999999992</v>
       </c>
       <c r="N52" s="98">
         <v>-304.75</v>
       </c>
       <c r="O52" s="60">
-        <v>4.692942254812099</v>
+        <v>-11.312410632447266</v>
       </c>
     </row>
     <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -23981,10 +25213,10 @@
         <v>0</v>
       </c>
       <c r="D66" s="99">
-        <v>0</v>
+        <v>352.5</v>
       </c>
       <c r="E66" s="99">
-        <v>0</v>
+        <v>-352.5</v>
       </c>
       <c r="F66" s="99"/>
       <c r="G66" s="100">
@@ -24006,13 +25238,13 @@
         <v>0</v>
       </c>
       <c r="M66" s="99">
-        <v>-3200</v>
+        <v>-3552.5</v>
       </c>
       <c r="N66" s="98">
         <v>-1014.25</v>
       </c>
       <c r="O66" s="60">
-        <v>3.425207385603425</v>
+        <v>3.8025153866738024</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -24182,10 +25414,10 @@
         <v>0</v>
       </c>
       <c r="D71" s="99">
-        <v>0</v>
+        <v>172.5</v>
       </c>
       <c r="E71" s="99">
-        <v>0</v>
+        <v>-172.5</v>
       </c>
       <c r="F71" s="99"/>
       <c r="G71" s="100">
@@ -24203,7 +25435,7 @@
         <v>0</v>
       </c>
       <c r="M71" s="99">
-        <v>0</v>
+        <v>-172.5</v>
       </c>
       <c r="N71" s="98"/>
       <c r="O71" s="60">
@@ -24252,25 +25484,25 @@
         <v>126</v>
       </c>
       <c r="C74" s="104">
-        <v>0</v>
+        <v>4365.459999999992</v>
       </c>
       <c r="D74" s="104">
-        <v>0</v>
+        <v>9124.330000000005</v>
       </c>
       <c r="E74" s="105">
-        <v>0</v>
+        <v>-4758.8700000000135</v>
       </c>
       <c r="F74" s="106" t="s">
         <v>127</v>
       </c>
       <c r="G74" s="107">
-        <v>0</v>
+        <v>-1.0901187961864323</v>
       </c>
       <c r="H74" s="108" t="s">
         <v>128</v>
       </c>
       <c r="I74" s="109">
-        <v>0</v>
+        <v>-17.178366082841247</v>
       </c>
       <c r="J74" s="36"/>
       <c r="K74" s="36"/>
@@ -24939,10 +26171,10 @@
         <v>125.39</v>
       </c>
       <c r="D8" s="54">
-        <v>34.75</v>
+        <v>42.75</v>
       </c>
       <c r="E8" s="54">
-        <v>90.64</v>
+        <v>82.64</v>
       </c>
       <c r="F8" s="54"/>
       <c r="G8" s="54"/>
@@ -25110,10 +26342,10 @@
         <v>501.83</v>
       </c>
       <c r="D14" s="54">
-        <v>373.25</v>
+        <v>393.75</v>
       </c>
       <c r="E14" s="54">
-        <v>128.57999999999998</v>
+        <v>108.07999999999998</v>
       </c>
       <c r="F14" s="54"/>
       <c r="G14" s="54"/>
@@ -25221,10 +26453,10 @@
         <v>685.48</v>
       </c>
       <c r="D18" s="54">
-        <v>718.75</v>
+        <v>740.5</v>
       </c>
       <c r="E18" s="54">
-        <v>-33.26999999999998</v>
+        <v>-55.01999999999998</v>
       </c>
       <c r="F18" s="54"/>
       <c r="G18" s="54"/>
@@ -25379,10 +26611,10 @@
         <v>472.14</v>
       </c>
       <c r="D24" s="54">
-        <v>257.25</v>
+        <v>275.25</v>
       </c>
       <c r="E24" s="54">
-        <v>214.89</v>
+        <v>196.89</v>
       </c>
       <c r="F24" s="54"/>
       <c r="G24" s="54"/>
@@ -25483,10 +26715,10 @@
         <v>232</v>
       </c>
       <c r="D28" s="54">
-        <v>225.5</v>
+        <v>234</v>
       </c>
       <c r="E28" s="54">
-        <v>6.5</v>
+        <v>-2</v>
       </c>
       <c r="F28" s="54"/>
       <c r="G28" s="54"/>
@@ -25689,10 +26921,10 @@
         <v>82.37</v>
       </c>
       <c r="D36" s="54">
-        <v>0</v>
+        <v>31.75</v>
       </c>
       <c r="E36" s="54">
-        <v>82.37</v>
+        <v>50.620000000000005</v>
       </c>
       <c r="F36" s="54"/>
       <c r="G36" s="54"/>
@@ -26481,10 +27713,10 @@
         <v>2412.45</v>
       </c>
       <c r="D66" s="54">
-        <v>1535.92</v>
+        <v>1543.42</v>
       </c>
       <c r="E66" s="54">
-        <v>876.5299999999997</v>
+        <v>869.0299999999997</v>
       </c>
       <c r="F66" s="54"/>
       <c r="G66" s="54"/>
@@ -26660,10 +27892,10 @@
         <v>36.92</v>
       </c>
       <c r="D71" s="54">
-        <v>6</v>
+        <v>7.75</v>
       </c>
       <c r="E71" s="54">
-        <v>30.92</v>
+        <v>29.17</v>
       </c>
       <c r="F71" s="54"/>
       <c r="G71" s="54"/>

</xml_diff>

<commit_message>
Sync data files (2026-10-02T03:57:37Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -10829,54 +10829,54 @@
         <v>19565.829</v>
       </c>
       <c r="I19" s="52">
-        <v>8852.34</v>
+        <v>10428.02</v>
       </c>
       <c r="J19" s="52">
         <v>13767.337200000002</v>
       </c>
       <c r="K19" s="52">
-        <v>6787.5</v>
+        <v>6798.900000000001</v>
       </c>
       <c r="L19" s="52">
-        <v>6979.837200000002</v>
+        <v>6968.437200000001</v>
       </c>
       <c r="M19" s="53">
-        <v>0.506985272358986</v>
+        <v>0.5061572255236111</v>
       </c>
       <c r="N19" s="53"/>
       <c r="O19" s="52">
         <v>5798.4918</v>
       </c>
       <c r="P19" s="52">
-        <v>2064.84</v>
+        <v>3629.12</v>
       </c>
       <c r="Q19" s="52">
-        <v>3733.6517999999996</v>
+        <v>2169.3718</v>
       </c>
       <c r="R19" s="53">
-        <v>0.643900505300361</v>
+        <v>0.37412690658629544</v>
       </c>
       <c r="S19" s="54">
         <v>125.39</v>
       </c>
       <c r="T19" s="54">
-        <v>42.75</v>
+        <v>71.75</v>
       </c>
       <c r="U19" s="54">
-        <v>82.64</v>
+        <v>53.64</v>
       </c>
       <c r="V19" s="53">
-        <v>0.6590637211898875</v>
+        <v>0.42778530983332</v>
       </c>
       <c r="W19" s="53"/>
       <c r="X19" s="55">
-        <v>73.60795321637427</v>
+        <v>21.89630662020906</v>
       </c>
       <c r="Y19" s="55">
         <v>63.27846478985563</v>
       </c>
       <c r="Z19" s="53">
-        <v>0.2622</v>
+        <v>0.1309</v>
       </c>
       <c r="AA19" s="56">
         <v>0.2885</v>
@@ -11513,7 +11513,7 @@
         <v>328046.93216</v>
       </c>
       <c r="I33" s="65">
-        <v>278861.56</v>
+        <v>280258.12</v>
       </c>
       <c r="J33" s="52">
         <v>271925.57216000004</v>
@@ -11532,35 +11532,35 @@
         <v>56121.36</v>
       </c>
       <c r="P33" s="52">
-        <v>35476.05</v>
+        <v>36872.61</v>
       </c>
       <c r="Q33" s="52">
-        <v>20645.309999999998</v>
+        <v>19248.75</v>
       </c>
       <c r="R33" s="53">
-        <v>0.367869025269523</v>
+        <v>0.3429843824169621</v>
       </c>
       <c r="S33" s="54">
         <v>1124.47</v>
       </c>
       <c r="T33" s="54">
-        <v>821.5</v>
+        <v>854.5</v>
       </c>
       <c r="U33" s="54">
-        <v>302.97</v>
+        <v>269.97</v>
       </c>
       <c r="V33" s="53">
-        <v>0.2694335998292529</v>
+        <v>0.24008644072318516</v>
       </c>
       <c r="W33" s="53"/>
       <c r="X33" s="55">
-        <v>89.78968959220937</v>
+        <v>84.68773551784669</v>
       </c>
       <c r="Y33" s="55">
         <v>61.532703026350184</v>
       </c>
       <c r="Z33" s="53">
-        <v>0.20920000000000002</v>
+        <v>0.2052</v>
       </c>
       <c r="AA33" s="56">
         <v>0.1742</v>
@@ -11876,54 +11876,54 @@
         <v>94098.31685</v>
       </c>
       <c r="I40" s="52">
-        <v>75059.27</v>
+        <v>76478.01</v>
       </c>
       <c r="J40" s="52">
         <v>69042.08885</v>
       </c>
       <c r="K40" s="52">
-        <v>57501.850000000006</v>
+        <v>57617.119999999995</v>
       </c>
       <c r="L40" s="52">
-        <v>11540.238849999994</v>
+        <v>11424.968850000005</v>
       </c>
       <c r="M40" s="53">
-        <v>0.16714788098419467</v>
+        <v>0.16547831967862028</v>
       </c>
       <c r="N40" s="53"/>
       <c r="O40" s="52">
         <v>25056.228</v>
       </c>
       <c r="P40" s="52">
-        <v>17557.42</v>
+        <v>18860.89</v>
       </c>
       <c r="Q40" s="52">
-        <v>7498.808000000001</v>
+        <v>6195.338</v>
       </c>
       <c r="R40" s="53">
-        <v>0.29927920515410383</v>
+        <v>0.24725740841757984</v>
       </c>
       <c r="S40" s="54">
         <v>501.83</v>
       </c>
       <c r="T40" s="54">
-        <v>393.75</v>
+        <v>420.5</v>
       </c>
       <c r="U40" s="54">
-        <v>108.07999999999998</v>
+        <v>81.32999999999998</v>
       </c>
       <c r="V40" s="53">
-        <v>0.21537173943367274</v>
+        <v>0.16206683538250002</v>
       </c>
       <c r="W40" s="53"/>
       <c r="X40" s="55">
-        <v>102.23563174603174</v>
+        <v>92.35800237812128</v>
       </c>
       <c r="Y40" s="55">
         <v>68.07122423898531</v>
       </c>
       <c r="Z40" s="53">
-        <v>0.34909999999999997</v>
+        <v>0.3368</v>
       </c>
       <c r="AA40" s="56">
         <v>0.2663</v>
@@ -12241,19 +12241,19 @@
         <v>50582.36785</v>
       </c>
       <c r="I47" s="52">
-        <v>46298.69</v>
+        <v>46423.2</v>
       </c>
       <c r="J47" s="52">
         <v>39438.99025</v>
       </c>
       <c r="K47" s="52">
-        <v>36941.96000000001</v>
+        <v>37066.47</v>
       </c>
       <c r="L47" s="52">
-        <v>2497.030249999996</v>
+        <v>2372.5202500000014</v>
       </c>
       <c r="M47" s="53">
-        <v>0.06331374698417884</v>
+        <v>0.060156718895712634</v>
       </c>
       <c r="N47" s="53"/>
       <c r="O47" s="52">
@@ -12282,13 +12282,13 @@
       </c>
       <c r="W47" s="53"/>
       <c r="X47" s="55">
-        <v>69.18836027713625</v>
+        <v>68.61325635103927</v>
       </c>
       <c r="Y47" s="55">
         <v>67.69550512136009</v>
       </c>
       <c r="Z47" s="53">
-        <v>0.2444</v>
+        <v>0.24239999999999998</v>
       </c>
       <c r="AA47" s="56">
         <v>0.23</v>
@@ -12604,54 +12604,54 @@
         <v>109364.9721</v>
       </c>
       <c r="I54" s="52">
-        <v>115851.63</v>
+        <v>116901.15</v>
       </c>
       <c r="J54" s="52">
         <v>75135.0159</v>
       </c>
       <c r="K54" s="52">
-        <v>81019.67000000001</v>
+        <v>81019.66999999998</v>
       </c>
       <c r="L54" s="52">
-        <v>-5884.654100000014</v>
+        <v>-5884.654099999985</v>
       </c>
       <c r="M54" s="53">
-        <v>-0.07832106015432433</v>
+        <v>-0.07832106015432394</v>
       </c>
       <c r="N54" s="53"/>
       <c r="O54" s="52">
         <v>34229.9562</v>
       </c>
       <c r="P54" s="52">
-        <v>34831.96</v>
+        <v>35881.48</v>
       </c>
       <c r="Q54" s="52">
-        <v>-602.0037999999986</v>
+        <v>-1651.5238000000027</v>
       </c>
       <c r="R54" s="53">
-        <v>-0.01758704558319004</v>
+        <v>-0.04824790865493432</v>
       </c>
       <c r="S54" s="54">
         <v>685.48</v>
       </c>
       <c r="T54" s="54">
-        <v>740.5</v>
+        <v>768.75</v>
       </c>
       <c r="U54" s="54">
-        <v>-55.01999999999998</v>
+        <v>-83.26999999999998</v>
       </c>
       <c r="V54" s="53">
-        <v>-0.0802649238489817</v>
+        <v>-0.12147692128143779</v>
       </c>
       <c r="W54" s="53"/>
       <c r="X54" s="55">
-        <v>53.26829169480081</v>
+        <v>49.94556097560976</v>
       </c>
       <c r="Y54" s="55">
         <v>67.00679527854935</v>
       </c>
       <c r="Z54" s="53">
-        <v>0.254</v>
+        <v>0.24719999999999998</v>
       </c>
       <c r="AA54" s="56">
         <v>0.2958</v>
@@ -13280,19 +13280,19 @@
         <v>39055.77825</v>
       </c>
       <c r="I68" s="52">
-        <v>30684.03</v>
+        <v>30284.51</v>
       </c>
       <c r="J68" s="52">
         <v>29537.289750000004</v>
       </c>
       <c r="K68" s="52">
-        <v>26364.309999999998</v>
+        <v>25964.789999999997</v>
       </c>
       <c r="L68" s="52">
-        <v>3172.979750000006</v>
+        <v>3572.4997500000063</v>
       </c>
       <c r="M68" s="53">
-        <v>0.10742284674239638</v>
+        <v>0.12094879998257138</v>
       </c>
       <c r="N68" s="53"/>
       <c r="O68" s="52">
@@ -13321,13 +13321,13 @@
       </c>
       <c r="W68" s="53"/>
       <c r="X68" s="55">
-        <v>-10.670633608815427</v>
+        <v>-6.268209366391185</v>
       </c>
       <c r="Y68" s="55">
         <v>72.28396616733912</v>
       </c>
       <c r="Z68" s="53">
-        <v>-0.0326</v>
+        <v>-0.0191</v>
       </c>
       <c r="AA68" s="56">
         <v>0.2635</v>
@@ -15717,19 +15717,19 @@
         <v>16648.056795</v>
       </c>
       <c r="I117" s="52">
-        <v>3100.1</v>
+        <v>2122.39</v>
       </c>
       <c r="J117" s="52">
         <v>12536.982795</v>
       </c>
       <c r="K117" s="52">
-        <v>1650.85</v>
+        <v>673.1399999999999</v>
       </c>
       <c r="L117" s="52">
-        <v>10886.132795</v>
+        <v>11863.842795</v>
       </c>
       <c r="M117" s="53">
-        <v>0.8683215868607244</v>
+        <v>0.9463076554377612</v>
       </c>
       <c r="N117" s="53"/>
       <c r="O117" s="52">
@@ -15758,7 +15758,7 @@
       </c>
       <c r="W117" s="53"/>
       <c r="X117" s="55">
-        <v>-97.64094488188977</v>
+        <v>-66.84692913385827</v>
       </c>
       <c r="Y117" s="55">
         <v>44.07429892630812</v>
@@ -20430,19 +20430,19 @@
         <v>117394.569232</v>
       </c>
       <c r="I215" s="52">
-        <v>37161.14</v>
+        <v>38162.19</v>
       </c>
       <c r="J215" s="52">
         <v>99479.615032</v>
       </c>
       <c r="K215" s="52">
-        <v>37161.14</v>
+        <v>38162.19</v>
       </c>
       <c r="L215" s="52">
-        <v>62318.475032</v>
+        <v>61317.425032</v>
       </c>
       <c r="M215" s="53">
-        <v>0.6264446742375689</v>
+        <v>0.6163818085974275</v>
       </c>
       <c r="N215" s="53"/>
       <c r="O215" s="52">
@@ -20477,7 +20477,7 @@
         <v>54.93783457863793</v>
       </c>
       <c r="Z215" s="53">
-        <v>0.1229</v>
+        <v>0.0993</v>
       </c>
       <c r="AA215" s="56">
         <v>0.1438</v>
@@ -20768,72 +20768,72 @@
         <v>98</v>
       </c>
       <c r="D222" s="52">
-        <v>412300.73261827</v>
+        <v>415822.30048988</v>
       </c>
       <c r="E222" s="52">
         <v>353667.87</v>
       </c>
       <c r="F222" s="52">
-        <v>58632.86261826998</v>
+        <v>62154.43048988003</v>
       </c>
       <c r="G222" s="53">
-        <v>0.1422089702483149</v>
+        <v>0.14947353813553513</v>
       </c>
       <c r="H222" s="52">
-        <v>306356.278672</v>
+        <v>309419.878672</v>
       </c>
       <c r="I222" s="52">
-        <v>253033.2</v>
+        <v>253132.82</v>
       </c>
       <c r="J222" s="52">
-        <v>186357.488872</v>
+        <v>189421.08887200002</v>
       </c>
       <c r="K222" s="52">
-        <v>180716.68</v>
+        <v>180794.42</v>
       </c>
       <c r="L222" s="52">
-        <v>5640.808871999994</v>
+        <v>8626.66887200001</v>
       </c>
       <c r="M222" s="53">
-        <v>0.03026875338438583</v>
+        <v>0.045542283192287106</v>
       </c>
       <c r="N222" s="53"/>
       <c r="O222" s="52">
         <v>119998.7898</v>
       </c>
       <c r="P222" s="52">
-        <v>72316.52</v>
+        <v>72338.4</v>
       </c>
       <c r="Q222" s="52">
-        <v>47682.269799999995</v>
+        <v>47660.389800000004</v>
       </c>
       <c r="R222" s="53">
-        <v>0.3973562556711717</v>
+        <v>0.39717392049898825</v>
       </c>
       <c r="S222" s="54">
         <v>2412.45</v>
       </c>
       <c r="T222" s="54">
-        <v>1543.42</v>
+        <v>1543.92</v>
       </c>
       <c r="U222" s="54">
-        <v>869.0299999999997</v>
+        <v>868.5299999999997</v>
       </c>
       <c r="V222" s="53">
-        <v>0.36022715496694224</v>
+        <v>0.3600198967854255</v>
       </c>
       <c r="W222" s="53"/>
       <c r="X222" s="55">
-        <v>65.2023882028223</v>
+        <v>65.1167482771128</v>
       </c>
       <c r="Y222" s="55">
-        <v>43.91570973337064</v>
+        <v>44.10554490989659</v>
       </c>
       <c r="Z222" s="53">
-        <v>0.2845</v>
+        <v>0.2843</v>
       </c>
       <c r="AA222" s="56">
-        <v>0.257</v>
+        <v>0.2559</v>
       </c>
       <c r="AB222" s="57"/>
       <c r="AD222" s="35" t="s">
@@ -21473,19 +21473,19 @@
         <v>19683.280628</v>
       </c>
       <c r="I236" s="52">
-        <v>0</v>
+        <v>2975.43</v>
       </c>
       <c r="J236" s="52">
         <v>10693.531628</v>
       </c>
       <c r="K236" s="52">
-        <v>0</v>
+        <v>2975.43</v>
       </c>
       <c r="L236" s="52">
-        <v>10693.531628</v>
+        <v>7718.101628</v>
       </c>
       <c r="M236" s="53">
-        <v>1</v>
+        <v>0.7217542245623403</v>
       </c>
       <c r="N236" s="53"/>
       <c r="O236" s="52">
@@ -22155,19 +22155,19 @@
         <v>15378.244372</v>
       </c>
       <c r="I250" s="52">
-        <v>0</v>
+        <v>4730.33</v>
       </c>
       <c r="J250" s="52">
         <v>8344.608772</v>
       </c>
       <c r="K250" s="52">
-        <v>0</v>
+        <v>4730.33</v>
       </c>
       <c r="L250" s="52">
-        <v>8344.608772</v>
+        <v>3614.2787719999997</v>
       </c>
       <c r="M250" s="53">
-        <v>1</v>
+        <v>0.4331274084565315</v>
       </c>
       <c r="N250" s="53"/>
       <c r="O250" s="52">
@@ -23510,10 +23510,10 @@
         <v>0</v>
       </c>
       <c r="D8" s="52">
-        <v>768.4200000000001</v>
+        <v>2344.1000000000004</v>
       </c>
       <c r="E8" s="52">
-        <v>-768.4200000000001</v>
+        <v>-2344.1000000000004</v>
       </c>
       <c r="F8" s="52"/>
       <c r="G8" s="53">
@@ -23533,13 +23533,13 @@
         <v>0</v>
       </c>
       <c r="M8" s="52">
-        <v>-1408.42</v>
+        <v>-2984.1000000000004</v>
       </c>
       <c r="N8" s="54">
         <v>-34.75</v>
       </c>
       <c r="O8" s="58">
-        <v>75.11573333333334</v>
+        <v>159.15200000000002</v>
       </c>
     </row>
     <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -23634,10 +23634,10 @@
         <v>0</v>
       </c>
       <c r="D12" s="52">
-        <v>0</v>
+        <v>1396.5599999999977</v>
       </c>
       <c r="E12" s="52">
-        <v>0</v>
+        <v>-1396.5599999999977</v>
       </c>
       <c r="F12" s="52">
         <v>3</v>
@@ -23661,13 +23661,13 @@
         <v>0</v>
       </c>
       <c r="M12" s="52">
-        <v>-2637</v>
+        <v>-4033.5599999999977</v>
       </c>
       <c r="N12" s="54">
         <v>53</v>
       </c>
       <c r="O12" s="58">
-        <v>-38.21739130434783</v>
+        <v>-58.457391304347794</v>
       </c>
       <c r="Q12" s="35" t="s">
         <v>122</v>
@@ -23701,10 +23701,10 @@
         <v>0</v>
       </c>
       <c r="D14" s="52">
-        <v>16449.9</v>
+        <v>17868.639999999992</v>
       </c>
       <c r="E14" s="52">
-        <v>-16449.9</v>
+        <v>-17868.639999999992</v>
       </c>
       <c r="F14" s="52">
         <v>0</v>
@@ -23728,13 +23728,13 @@
         <v>0</v>
       </c>
       <c r="M14" s="52">
-        <v>-19449.9</v>
+        <v>-20868.639999999992</v>
       </c>
       <c r="N14" s="54">
         <v>-112</v>
       </c>
       <c r="O14" s="58">
-        <v>173.65982142857143</v>
+        <v>186.32714285714277</v>
       </c>
     </row>
     <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -23765,10 +23765,10 @@
         <v>0</v>
       </c>
       <c r="D16" s="52">
-        <v>16697.65</v>
+        <v>16822.159999999996</v>
       </c>
       <c r="E16" s="52">
-        <v>-16697.65</v>
+        <v>-16822.159999999996</v>
       </c>
       <c r="F16" s="52"/>
       <c r="G16" s="53">
@@ -23790,13 +23790,13 @@
         <v>0</v>
       </c>
       <c r="M16" s="52">
-        <v>-19697.65</v>
+        <v>-19822.159999999996</v>
       </c>
       <c r="N16" s="54">
         <v>-86.75</v>
       </c>
       <c r="O16" s="58">
-        <v>227.06224783861674</v>
+        <v>228.49752161383282</v>
       </c>
     </row>
     <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -23827,10 +23827,10 @@
         <v>0</v>
       </c>
       <c r="D18" s="52">
-        <v>797.9000000000087</v>
+        <v>1847.4199999999983</v>
       </c>
       <c r="E18" s="52">
-        <v>-797.9000000000087</v>
+        <v>-1847.4199999999983</v>
       </c>
       <c r="F18" s="52">
         <v>0</v>
@@ -23854,13 +23854,13 @@
         <v>0</v>
       </c>
       <c r="M18" s="52">
-        <v>-8997.900000000009</v>
+        <v>-10047.419999999998</v>
       </c>
       <c r="N18" s="54">
         <v>-269</v>
       </c>
       <c r="O18" s="58">
-        <v>47.60793650793656</v>
+        <v>53.160952380952374</v>
       </c>
       <c r="Q18" s="35" t="s">
         <v>123</v>
@@ -23950,10 +23950,10 @@
         <v>0</v>
       </c>
       <c r="D22" s="52">
-        <v>0</v>
+        <v>-399.52000000000044</v>
       </c>
       <c r="E22" s="52">
-        <v>0</v>
+        <v>399.52000000000044</v>
       </c>
       <c r="F22" s="52">
         <v>3</v>
@@ -23973,7 +23973,7 @@
         <v>0</v>
       </c>
       <c r="M22" s="52">
-        <v>3</v>
+        <v>402.52000000000044</v>
       </c>
       <c r="N22" s="54"/>
       <c r="O22" s="58">
@@ -24372,10 +24372,10 @@
         <v>0</v>
       </c>
       <c r="D36" s="52">
-        <v>3041.7799999999997</v>
+        <v>2064.0699999999997</v>
       </c>
       <c r="E36" s="52">
-        <v>-3041.7799999999997</v>
+        <v>-2064.0699999999997</v>
       </c>
       <c r="F36" s="52">
         <v>0</v>
@@ -24397,11 +24397,11 @@
         <v>0</v>
       </c>
       <c r="M36" s="52">
-        <v>-6241.78</v>
+        <v>-5264.07</v>
       </c>
       <c r="N36" s="54"/>
       <c r="O36" s="58">
-        <v>-78.02225</v>
+        <v>-65.80087499999999</v>
       </c>
     </row>
     <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -25155,10 +25155,10 @@
         <v>0</v>
       </c>
       <c r="D64" s="99">
-        <v>0</v>
+        <v>1001.0500000000029</v>
       </c>
       <c r="E64" s="99">
-        <v>0</v>
+        <v>-1001.0500000000029</v>
       </c>
       <c r="F64" s="99"/>
       <c r="G64" s="100">
@@ -25178,7 +25178,7 @@
         <v>0</v>
       </c>
       <c r="M64" s="99">
-        <v>-1750</v>
+        <v>-2751.050000000003</v>
       </c>
       <c r="N64" s="98"/>
       <c r="O64" s="60">
@@ -25213,10 +25213,10 @@
         <v>0</v>
       </c>
       <c r="D66" s="99">
-        <v>352.5</v>
+        <v>452.11999999999534</v>
       </c>
       <c r="E66" s="99">
-        <v>-352.5</v>
+        <v>-452.11999999999534</v>
       </c>
       <c r="F66" s="99"/>
       <c r="G66" s="100">
@@ -25238,13 +25238,13 @@
         <v>0</v>
       </c>
       <c r="M66" s="99">
-        <v>-3552.5</v>
+        <v>-3652.1199999999953</v>
       </c>
       <c r="N66" s="98">
         <v>-1014.25</v>
       </c>
       <c r="O66" s="60">
-        <v>3.8025153866738024</v>
+        <v>3.909146374096864</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -25297,10 +25297,10 @@
         <v>0</v>
       </c>
       <c r="D68" s="99">
-        <v>0</v>
+        <v>4730.33</v>
       </c>
       <c r="E68" s="99">
-        <v>0</v>
+        <v>-4730.33</v>
       </c>
       <c r="F68" s="99"/>
       <c r="G68" s="100">
@@ -25318,7 +25318,7 @@
         <v>0</v>
       </c>
       <c r="M68" s="99">
-        <v>0</v>
+        <v>-4730.33</v>
       </c>
       <c r="N68" s="98"/>
       <c r="O68" s="60">
@@ -25375,10 +25375,10 @@
         <v>0</v>
       </c>
       <c r="D70" s="99">
-        <v>0</v>
+        <v>2975.43</v>
       </c>
       <c r="E70" s="99">
-        <v>0</v>
+        <v>-2975.43</v>
       </c>
       <c r="F70" s="99"/>
       <c r="G70" s="100">
@@ -25396,7 +25396,7 @@
         <v>0</v>
       </c>
       <c r="M70" s="99">
-        <v>0</v>
+        <v>-2975.43</v>
       </c>
       <c r="N70" s="98"/>
       <c r="O70" s="60">
@@ -25487,22 +25487,22 @@
         <v>4365.459999999992</v>
       </c>
       <c r="D74" s="104">
-        <v>40931.45000000001</v>
+        <v>53925.65999999999</v>
       </c>
       <c r="E74" s="105">
-        <v>-36565.99000000002</v>
+        <v>-49560.2</v>
       </c>
       <c r="F74" s="106" t="s">
         <v>127</v>
       </c>
       <c r="G74" s="107">
-        <v>-8.37620548579075</v>
+        <v>-11.352801308453197</v>
       </c>
       <c r="H74" s="108" t="s">
         <v>128</v>
       </c>
       <c r="I74" s="109">
-        <v>-24.46445277244557</v>
+        <v>-27.441048595108015</v>
       </c>
       <c r="J74" s="36"/>
       <c r="K74" s="36"/>
@@ -26171,10 +26171,10 @@
         <v>125.39</v>
       </c>
       <c r="D8" s="54">
-        <v>42.75</v>
+        <v>71.75</v>
       </c>
       <c r="E8" s="54">
-        <v>82.64</v>
+        <v>53.64</v>
       </c>
       <c r="F8" s="54"/>
       <c r="G8" s="54"/>
@@ -26283,10 +26283,10 @@
         <v>1124.47</v>
       </c>
       <c r="D12" s="54">
-        <v>821.5</v>
+        <v>854.5</v>
       </c>
       <c r="E12" s="54">
-        <v>302.97</v>
+        <v>269.97</v>
       </c>
       <c r="F12" s="54"/>
       <c r="G12" s="54"/>
@@ -26342,10 +26342,10 @@
         <v>501.83</v>
       </c>
       <c r="D14" s="54">
-        <v>393.75</v>
+        <v>420.5</v>
       </c>
       <c r="E14" s="54">
-        <v>108.07999999999998</v>
+        <v>81.32999999999998</v>
       </c>
       <c r="F14" s="54"/>
       <c r="G14" s="54"/>
@@ -26453,10 +26453,10 @@
         <v>685.48</v>
       </c>
       <c r="D18" s="54">
-        <v>740.5</v>
+        <v>768.75</v>
       </c>
       <c r="E18" s="54">
-        <v>-55.01999999999998</v>
+        <v>-83.26999999999998</v>
       </c>
       <c r="F18" s="54"/>
       <c r="G18" s="54"/>
@@ -27713,10 +27713,10 @@
         <v>2412.45</v>
       </c>
       <c r="D66" s="54">
-        <v>1543.42</v>
+        <v>1543.92</v>
       </c>
       <c r="E66" s="54">
-        <v>869.0299999999997</v>
+        <v>868.5299999999997</v>
       </c>
       <c r="F66" s="54"/>
       <c r="G66" s="54"/>

</xml_diff>

<commit_message>
Sync data files (2026-10-03T01:10:19Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -10103,19 +10103,19 @@
         <v>225410.5455298</v>
       </c>
       <c r="I5" s="52">
-        <v>189455.97</v>
+        <v>201489.31</v>
       </c>
       <c r="J5" s="52">
         <v>193787.2413298</v>
       </c>
       <c r="K5" s="52">
-        <v>158286.35</v>
+        <v>170319.69</v>
       </c>
       <c r="L5" s="52">
-        <v>35500.89132979998</v>
+        <v>23467.551329799986</v>
       </c>
       <c r="M5" s="53">
-        <v>0.18319519430787606</v>
+        <v>0.12109956862361929</v>
       </c>
       <c r="N5" s="53"/>
       <c r="O5" s="52">
@@ -10144,13 +10144,13 @@
       </c>
       <c r="W5" s="53"/>
       <c r="X5" s="55">
-        <v>78.81167532986805</v>
+        <v>59.56602958816474</v>
       </c>
       <c r="Y5" s="55">
         <v>66.57519091683645</v>
       </c>
       <c r="Z5" s="53">
-        <v>0.2064</v>
+        <v>0.156</v>
       </c>
       <c r="AA5" s="56">
         <v>0.1586</v>
@@ -10829,7 +10829,7 @@
         <v>19565.829</v>
       </c>
       <c r="I19" s="52">
-        <v>10428.02</v>
+        <v>11127.1</v>
       </c>
       <c r="J19" s="52">
         <v>13767.337200000002</v>
@@ -10848,35 +10848,35 @@
         <v>5798.4918</v>
       </c>
       <c r="P19" s="52">
-        <v>3629.12</v>
+        <v>4328.2</v>
       </c>
       <c r="Q19" s="52">
-        <v>2169.3718</v>
+        <v>1470.2918</v>
       </c>
       <c r="R19" s="53">
-        <v>0.37412690658629544</v>
+        <v>0.25356452172614957</v>
       </c>
       <c r="S19" s="54">
         <v>125.39</v>
       </c>
       <c r="T19" s="54">
-        <v>71.75</v>
+        <v>85.25</v>
       </c>
       <c r="U19" s="54">
-        <v>53.64</v>
+        <v>40.14</v>
       </c>
       <c r="V19" s="53">
-        <v>0.42778530983332</v>
+        <v>0.3201212217880214</v>
       </c>
       <c r="W19" s="53"/>
       <c r="X19" s="55">
-        <v>21.89630662020906</v>
+        <v>10.22850439882698</v>
       </c>
       <c r="Y19" s="55">
         <v>63.27846478985563</v>
       </c>
       <c r="Z19" s="53">
-        <v>0.1309</v>
+        <v>0.0727</v>
       </c>
       <c r="AA19" s="56">
         <v>0.2885</v>
@@ -11876,19 +11876,19 @@
         <v>94098.31685</v>
       </c>
       <c r="I40" s="52">
-        <v>76478.01</v>
+        <v>76764.25</v>
       </c>
       <c r="J40" s="52">
         <v>69042.08885</v>
       </c>
       <c r="K40" s="52">
-        <v>57617.119999999995</v>
+        <v>57903.36</v>
       </c>
       <c r="L40" s="52">
-        <v>11424.968850000005</v>
+        <v>11138.72885</v>
       </c>
       <c r="M40" s="53">
-        <v>0.16547831967862028</v>
+        <v>0.1613324427973184</v>
       </c>
       <c r="N40" s="53"/>
       <c r="O40" s="52">
@@ -11917,13 +11917,13 @@
       </c>
       <c r="W40" s="53"/>
       <c r="X40" s="55">
-        <v>92.35800237812128</v>
+        <v>91.67728894173604</v>
       </c>
       <c r="Y40" s="55">
         <v>68.07122423898531</v>
       </c>
       <c r="Z40" s="53">
-        <v>0.3368</v>
+        <v>0.3343</v>
       </c>
       <c r="AA40" s="56">
         <v>0.2663</v>
@@ -12241,19 +12241,19 @@
         <v>50582.36785</v>
       </c>
       <c r="I47" s="52">
-        <v>46423.2</v>
+        <v>46355.29</v>
       </c>
       <c r="J47" s="52">
         <v>39438.99025</v>
       </c>
       <c r="K47" s="52">
-        <v>37066.47</v>
+        <v>36998.56</v>
       </c>
       <c r="L47" s="52">
-        <v>2372.5202500000014</v>
+        <v>2440.430250000005</v>
       </c>
       <c r="M47" s="53">
-        <v>0.060156718895712634</v>
+        <v>0.061878618963881936</v>
       </c>
       <c r="N47" s="53"/>
       <c r="O47" s="52">
@@ -12282,13 +12282,13 @@
       </c>
       <c r="W47" s="53"/>
       <c r="X47" s="55">
-        <v>68.61325635103927</v>
+        <v>68.92692840646652</v>
       </c>
       <c r="Y47" s="55">
         <v>67.69550512136009</v>
       </c>
       <c r="Z47" s="53">
-        <v>0.24239999999999998</v>
+        <v>0.24350000000000002</v>
       </c>
       <c r="AA47" s="56">
         <v>0.23</v>
@@ -13635,54 +13635,54 @@
         <v>55589.7822</v>
       </c>
       <c r="I75" s="52">
-        <v>51465.45</v>
+        <v>51952.35</v>
       </c>
       <c r="J75" s="52">
         <v>32594.7534</v>
       </c>
       <c r="K75" s="52">
-        <v>36088.42999999999</v>
+        <v>36088.43</v>
       </c>
       <c r="L75" s="52">
-        <v>-3493.6765999999916</v>
+        <v>-3493.676599999999</v>
       </c>
       <c r="M75" s="53">
-        <v>-0.10718524411355085</v>
+        <v>-0.10718524411355107</v>
       </c>
       <c r="N75" s="53"/>
       <c r="O75" s="52">
         <v>22995.0288</v>
       </c>
       <c r="P75" s="52">
-        <v>15377.02</v>
+        <v>15863.92</v>
       </c>
       <c r="Q75" s="52">
-        <v>7618.0088</v>
+        <v>7131.1088</v>
       </c>
       <c r="R75" s="53">
-        <v>0.33128937851123713</v>
+        <v>0.31011523673325425</v>
       </c>
       <c r="S75" s="54">
         <v>472.14</v>
       </c>
       <c r="T75" s="54">
-        <v>307.75</v>
+        <v>316.75</v>
       </c>
       <c r="U75" s="54">
-        <v>164.39</v>
+        <v>155.39</v>
       </c>
       <c r="V75" s="53">
-        <v>0.34818062439107045</v>
+        <v>0.32911848180624387</v>
       </c>
       <c r="W75" s="53"/>
       <c r="X75" s="55">
-        <v>33.46667749796914</v>
+        <v>30.978595106550905</v>
       </c>
       <c r="Y75" s="55">
         <v>49.060202993773025</v>
       </c>
       <c r="Z75" s="53">
-        <v>0.1668</v>
+        <v>0.1589</v>
       </c>
       <c r="AA75" s="56">
         <v>0.2941</v>
@@ -20430,19 +20430,19 @@
         <v>117394.569232</v>
       </c>
       <c r="I215" s="52">
-        <v>38162.19</v>
+        <v>38171.51</v>
       </c>
       <c r="J215" s="52">
         <v>99479.615032</v>
       </c>
       <c r="K215" s="52">
-        <v>38162.19</v>
+        <v>38171.51</v>
       </c>
       <c r="L215" s="52">
-        <v>61317.425032</v>
+        <v>61308.105032</v>
       </c>
       <c r="M215" s="53">
-        <v>0.6163818085974275</v>
+        <v>0.616288121061574</v>
       </c>
       <c r="N215" s="53"/>
       <c r="O215" s="52">
@@ -20477,7 +20477,7 @@
         <v>54.93783457863793</v>
       </c>
       <c r="Z215" s="53">
-        <v>0.0993</v>
+        <v>0.09910000000000001</v>
       </c>
       <c r="AA215" s="56">
         <v>0.1438</v>
@@ -20783,54 +20783,54 @@
         <v>309419.878672</v>
       </c>
       <c r="I222" s="52">
-        <v>253132.82</v>
+        <v>253989.54</v>
       </c>
       <c r="J222" s="52">
         <v>189421.08887200002</v>
       </c>
       <c r="K222" s="52">
-        <v>180794.42</v>
+        <v>180917.58000000002</v>
       </c>
       <c r="L222" s="52">
-        <v>8626.66887200001</v>
+        <v>8503.508872000006</v>
       </c>
       <c r="M222" s="53">
-        <v>0.045542283192287106</v>
+        <v>0.044892091596760865</v>
       </c>
       <c r="N222" s="53"/>
       <c r="O222" s="52">
         <v>119998.7898</v>
       </c>
       <c r="P222" s="52">
-        <v>72338.4</v>
+        <v>73071.96</v>
       </c>
       <c r="Q222" s="52">
-        <v>47660.389800000004</v>
+        <v>46926.82979999999</v>
       </c>
       <c r="R222" s="53">
-        <v>0.39717392049898825</v>
+        <v>0.3910608588487614</v>
       </c>
       <c r="S222" s="54">
         <v>2412.45</v>
       </c>
       <c r="T222" s="54">
-        <v>1543.92</v>
+        <v>1559.67</v>
       </c>
       <c r="U222" s="54">
-        <v>868.5299999999997</v>
+        <v>852.7799999999997</v>
       </c>
       <c r="V222" s="53">
-        <v>0.3600198967854255</v>
+        <v>0.35349126406764897</v>
       </c>
       <c r="W222" s="53"/>
       <c r="X222" s="55">
-        <v>65.1167482771128</v>
+        <v>63.90988478331955</v>
       </c>
       <c r="Y222" s="55">
         <v>44.10554490989659</v>
       </c>
       <c r="Z222" s="53">
-        <v>0.2843</v>
+        <v>0.2818</v>
       </c>
       <c r="AA222" s="56">
         <v>0.2559</v>
@@ -22155,7 +22155,7 @@
         <v>15378.244372</v>
       </c>
       <c r="I250" s="52">
-        <v>4730.33</v>
+        <v>4993.07</v>
       </c>
       <c r="J250" s="52">
         <v>8344.608772</v>
@@ -22174,29 +22174,29 @@
         <v>7033.6356</v>
       </c>
       <c r="P250" s="52">
-        <v>0</v>
+        <v>262.74</v>
       </c>
       <c r="Q250" s="52">
-        <v>7033.6356</v>
+        <v>6770.8956</v>
       </c>
       <c r="R250" s="53">
-        <v>1</v>
+        <v>0.9626452072666375</v>
       </c>
       <c r="S250" s="54">
         <v>140.9</v>
       </c>
       <c r="T250" s="54">
-        <v>0</v>
+        <v>5.75</v>
       </c>
       <c r="U250" s="54">
-        <v>140.9</v>
+        <v>135.15</v>
       </c>
       <c r="V250" s="53">
-        <v>1</v>
+        <v>0.9591909155429382</v>
       </c>
       <c r="W250" s="53"/>
       <c r="X250" s="55">
-        <v>0</v>
+        <v>-868.3599999999999</v>
       </c>
       <c r="Y250" s="55">
         <v>42.71295951611073</v>
@@ -23379,10 +23379,10 @@
         <v>0</v>
       </c>
       <c r="D4" s="52">
-        <v>0</v>
+        <v>12033.339999999997</v>
       </c>
       <c r="E4" s="52">
-        <v>0</v>
+        <v>-12033.339999999997</v>
       </c>
       <c r="F4" s="52">
         <v>0</v>
@@ -23406,13 +23406,13 @@
         <v>0</v>
       </c>
       <c r="M4" s="52">
-        <v>-7000</v>
+        <v>-19033.339999999997</v>
       </c>
       <c r="N4" s="54">
         <v>20</v>
       </c>
       <c r="O4" s="58">
-        <v>-100</v>
+        <v>-271.9048571428571</v>
       </c>
     </row>
     <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -23510,10 +23510,10 @@
         <v>0</v>
       </c>
       <c r="D8" s="52">
-        <v>2344.1000000000004</v>
+        <v>3043.1800000000003</v>
       </c>
       <c r="E8" s="52">
-        <v>-2344.1000000000004</v>
+        <v>-3043.1800000000003</v>
       </c>
       <c r="F8" s="52"/>
       <c r="G8" s="53">
@@ -23533,13 +23533,13 @@
         <v>0</v>
       </c>
       <c r="M8" s="52">
-        <v>-2984.1000000000004</v>
+        <v>-3683.1800000000003</v>
       </c>
       <c r="N8" s="54">
         <v>-34.75</v>
       </c>
       <c r="O8" s="58">
-        <v>159.15200000000002</v>
+        <v>196.43626666666668</v>
       </c>
     </row>
     <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -23701,10 +23701,10 @@
         <v>0</v>
       </c>
       <c r="D14" s="52">
-        <v>17868.639999999992</v>
+        <v>18154.879999999997</v>
       </c>
       <c r="E14" s="52">
-        <v>-17868.639999999992</v>
+        <v>-18154.879999999997</v>
       </c>
       <c r="F14" s="52">
         <v>0</v>
@@ -23728,13 +23728,13 @@
         <v>0</v>
       </c>
       <c r="M14" s="52">
-        <v>-20868.639999999992</v>
+        <v>-21154.879999999997</v>
       </c>
       <c r="N14" s="54">
         <v>-112</v>
       </c>
       <c r="O14" s="58">
-        <v>186.32714285714277</v>
+        <v>188.88285714285712</v>
       </c>
     </row>
     <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -23765,10 +23765,10 @@
         <v>0</v>
       </c>
       <c r="D16" s="52">
-        <v>16822.159999999996</v>
+        <v>16754.25</v>
       </c>
       <c r="E16" s="52">
-        <v>-16822.159999999996</v>
+        <v>-16754.25</v>
       </c>
       <c r="F16" s="52"/>
       <c r="G16" s="53">
@@ -23790,13 +23790,13 @@
         <v>0</v>
       </c>
       <c r="M16" s="52">
-        <v>-19822.159999999996</v>
+        <v>-19754.25</v>
       </c>
       <c r="N16" s="54">
         <v>-86.75</v>
       </c>
       <c r="O16" s="58">
-        <v>228.49752161383282</v>
+        <v>227.71469740634006</v>
       </c>
     </row>
     <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -24008,10 +24008,10 @@
         <v>0</v>
       </c>
       <c r="D24" s="52">
-        <v>2649.8799999999974</v>
+        <v>3136.779999999999</v>
       </c>
       <c r="E24" s="52">
-        <v>-2649.8799999999974</v>
+        <v>-3136.779999999999</v>
       </c>
       <c r="F24" s="52">
         <v>3</v>
@@ -24029,7 +24029,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="52">
-        <v>-2646.8799999999974</v>
+        <v>-3133.779999999999</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="58">
@@ -25155,10 +25155,10 @@
         <v>0</v>
       </c>
       <c r="D64" s="99">
-        <v>1001.0500000000029</v>
+        <v>1010.3700000000026</v>
       </c>
       <c r="E64" s="99">
-        <v>-1001.0500000000029</v>
+        <v>-1010.3700000000026</v>
       </c>
       <c r="F64" s="99"/>
       <c r="G64" s="100">
@@ -25178,7 +25178,7 @@
         <v>0</v>
       </c>
       <c r="M64" s="99">
-        <v>-2751.050000000003</v>
+        <v>-2760.3700000000026</v>
       </c>
       <c r="N64" s="98"/>
       <c r="O64" s="60">
@@ -25213,10 +25213,10 @@
         <v>0</v>
       </c>
       <c r="D66" s="99">
-        <v>452.11999999999534</v>
+        <v>1308.8399999999965</v>
       </c>
       <c r="E66" s="99">
-        <v>-452.11999999999534</v>
+        <v>-1308.8399999999965</v>
       </c>
       <c r="F66" s="99"/>
       <c r="G66" s="100">
@@ -25238,13 +25238,13 @@
         <v>0</v>
       </c>
       <c r="M66" s="99">
-        <v>-3652.1199999999953</v>
+        <v>-4508.8399999999965</v>
       </c>
       <c r="N66" s="98">
         <v>-1014.25</v>
       </c>
       <c r="O66" s="60">
-        <v>3.909146374096864</v>
+        <v>4.826160021407542</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -25297,10 +25297,10 @@
         <v>0</v>
       </c>
       <c r="D68" s="99">
-        <v>4730.33</v>
+        <v>4993.07</v>
       </c>
       <c r="E68" s="99">
-        <v>-4730.33</v>
+        <v>-4993.07</v>
       </c>
       <c r="F68" s="99"/>
       <c r="G68" s="100">
@@ -25318,7 +25318,7 @@
         <v>0</v>
       </c>
       <c r="M68" s="99">
-        <v>-4730.33</v>
+        <v>-4993.07</v>
       </c>
       <c r="N68" s="98"/>
       <c r="O68" s="60">
@@ -25487,22 +25487,22 @@
         <v>4365.459999999992</v>
       </c>
       <c r="D74" s="104">
-        <v>55469.359999999986</v>
+        <v>70035.78999999998</v>
       </c>
       <c r="E74" s="105">
-        <v>-51103.899999999994</v>
+        <v>-65670.32999999999</v>
       </c>
       <c r="F74" s="106" t="s">
         <v>127</v>
       </c>
       <c r="G74" s="107">
-        <v>-11.706418109431787</v>
+        <v>-15.043163836113516</v>
       </c>
       <c r="H74" s="108" t="s">
         <v>128</v>
       </c>
       <c r="I74" s="109">
-        <v>-27.794665396086604</v>
+        <v>-31.131411122768334</v>
       </c>
       <c r="J74" s="36"/>
       <c r="K74" s="36"/>
@@ -26171,10 +26171,10 @@
         <v>125.39</v>
       </c>
       <c r="D8" s="54">
-        <v>71.75</v>
+        <v>85.25</v>
       </c>
       <c r="E8" s="54">
-        <v>53.64</v>
+        <v>40.14</v>
       </c>
       <c r="F8" s="54"/>
       <c r="G8" s="54"/>
@@ -26611,10 +26611,10 @@
         <v>472.14</v>
       </c>
       <c r="D24" s="54">
-        <v>307.75</v>
+        <v>316.75</v>
       </c>
       <c r="E24" s="54">
-        <v>164.39</v>
+        <v>155.39</v>
       </c>
       <c r="F24" s="54"/>
       <c r="G24" s="54"/>
@@ -27713,10 +27713,10 @@
         <v>2412.45</v>
       </c>
       <c r="D66" s="54">
-        <v>1543.92</v>
+        <v>1559.67</v>
       </c>
       <c r="E66" s="54">
-        <v>868.5299999999997</v>
+        <v>852.7799999999997</v>
       </c>
       <c r="F66" s="54"/>
       <c r="G66" s="54"/>
@@ -27789,10 +27789,10 @@
         <v>140.9</v>
       </c>
       <c r="D68" s="54">
-        <v>0</v>
+        <v>5.75</v>
       </c>
       <c r="E68" s="54">
-        <v>140.9</v>
+        <v>135.15</v>
       </c>
       <c r="F68" s="54"/>
       <c r="G68" s="54"/>

</xml_diff>